<commit_message>
Mise à jour manuelle des frises de courants de pensée
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -3228,7 +3228,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3354,18 +3354,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF1E1208"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="10"/>
@@ -3512,7 +3500,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3522,7 +3510,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -3542,7 +3530,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -3562,7 +3550,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -3574,7 +3562,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -3582,7 +3570,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -3606,7 +3594,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -3621,35 +3609,27 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3908,16 +3888,16 @@
   <dimension ref="A1:L177"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="22.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="107.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="33.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="21.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="101.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="15.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="3" width="6.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="3" width="46.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="3" width="4.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="3" width="37.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="3" width="20.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
@@ -5867,7 +5847,7 @@
       <c r="D69" s="12" t="s">
         <v>388</v>
       </c>
-      <c r="E69" s="27" t="s">
+      <c r="E69" s="26" t="s">
         <v>389</v>
       </c>
       <c r="F69" s="11" t="s">
@@ -5878,7 +5858,7 @@
       </c>
       <c r="H69" s="11"/>
       <c r="I69" s="13"/>
-      <c r="J69" s="28" t="s">
+      <c r="J69" s="22" t="s">
         <v>392</v>
       </c>
       <c r="K69" s="3" t="s">
@@ -5925,7 +5905,7 @@
       <c r="D71" s="15" t="s">
         <v>399</v>
       </c>
-      <c r="E71" s="29" t="s">
+      <c r="E71" s="27" t="s">
         <v>400</v>
       </c>
       <c r="F71" s="14" t="s">
@@ -6157,7 +6137,7 @@
       <c r="D79" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="E79" s="30" t="s">
+      <c r="E79" s="28" t="s">
         <v>444</v>
       </c>
       <c r="F79" s="11" t="s">
@@ -6416,7 +6396,7 @@
       <c r="D88" s="12" t="s">
         <v>493</v>
       </c>
-      <c r="E88" s="30" t="s">
+      <c r="E88" s="28" t="s">
         <v>494</v>
       </c>
       <c r="F88" s="11" t="s">
@@ -6445,7 +6425,7 @@
       <c r="D89" s="15" t="s">
         <v>499</v>
       </c>
-      <c r="E89" s="31" t="s">
+      <c r="E89" s="29" t="s">
         <v>500</v>
       </c>
       <c r="F89" s="14" t="s">
@@ -6652,7 +6632,7 @@
       <c r="D96" s="12" t="s">
         <v>543</v>
       </c>
-      <c r="E96" s="30" t="s">
+      <c r="E96" s="28" t="s">
         <v>544</v>
       </c>
       <c r="F96" s="11" t="s">
@@ -6797,7 +6777,7 @@
       <c r="D101" s="12" t="s">
         <v>571</v>
       </c>
-      <c r="E101" s="30" t="s">
+      <c r="E101" s="28" t="s">
         <v>572</v>
       </c>
       <c r="F101" s="11" t="s">
@@ -7029,7 +7009,7 @@
       <c r="D109" s="15" t="s">
         <v>613</v>
       </c>
-      <c r="E109" s="31" t="s">
+      <c r="E109" s="29" t="s">
         <v>614</v>
       </c>
       <c r="F109" s="14" t="s">
@@ -7841,7 +7821,7 @@
       <c r="D138" s="15" t="s">
         <v>769</v>
       </c>
-      <c r="E138" s="31" t="s">
+      <c r="E138" s="29" t="s">
         <v>770</v>
       </c>
       <c r="F138" s="14" t="s">
@@ -8707,7 +8687,7 @@
       </c>
     </row>
     <row r="169" customFormat="false" ht="251.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D169" s="1"/>
+      <c r="D169" s="3"/>
       <c r="E169" s="1"/>
       <c r="I169" s="1"/>
       <c r="J169" s="1"/>
@@ -8729,17 +8709,17 @@
       <c r="J173" s="1"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D174" s="1"/>
+      <c r="D174" s="3"/>
       <c r="I174" s="1"/>
       <c r="J174" s="1"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D175" s="1"/>
+      <c r="D175" s="3"/>
       <c r="I175" s="1"/>
       <c r="J175" s="1"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D176" s="1"/>
+      <c r="D176" s="3"/>
       <c r="I176" s="1"/>
       <c r="J176" s="1"/>
     </row>
@@ -8817,192 +8797,192 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="30" t="s">
         <v>935</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="30" t="s">
         <v>936</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="31" t="s">
         <v>937</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="32" t="s">
         <v>938</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="31" t="s">
         <v>939</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="32" t="s">
         <v>940</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="31" t="s">
         <v>941</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="32" t="s">
         <v>942</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="31" t="s">
         <v>943</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="32" t="s">
         <v>944</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="31" t="s">
         <v>945</v>
       </c>
-      <c r="C10" s="34" t="s">
+      <c r="C10" s="32" t="s">
         <v>946</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="31" t="s">
         <v>947</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C11" s="32" t="s">
         <v>948</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="31" t="s">
         <v>949</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="32" t="s">
         <v>950</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="31" t="s">
         <v>951</v>
       </c>
-      <c r="C13" s="34" t="s">
+      <c r="C13" s="32" t="s">
         <v>952</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="31" t="s">
         <v>953</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C14" s="32" t="s">
         <v>954</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="30" t="s">
         <v>955</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="31" t="s">
         <v>956</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="32" t="s">
         <v>957</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="31" t="s">
         <v>958</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="32" t="s">
         <v>959</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="31" t="s">
         <v>960</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="C19" s="32" t="s">
         <v>961</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="30" t="s">
         <v>962</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="33" t="s">
+      <c r="B22" s="31" t="s">
         <v>963</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="32" t="s">
         <v>964</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="33" t="s">
+      <c r="B23" s="31" t="s">
         <v>965</v>
       </c>
-      <c r="C23" s="34" t="s">
+      <c r="C23" s="32" t="s">
         <v>966</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="30" t="s">
         <v>967</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="33" t="s">
+      <c r="B26" s="31" t="s">
         <v>968</v>
       </c>
-      <c r="C26" s="34" t="s">
+      <c r="C26" s="32" t="s">
         <v>969</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="33" t="s">
+      <c r="B27" s="31" t="s">
         <v>970</v>
       </c>
-      <c r="C27" s="34" t="s">
+      <c r="C27" s="32" t="s">
         <v>971</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="95.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="33" t="s">
+      <c r="B28" s="31" t="s">
         <v>972</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C28" s="32" t="s">
         <v>973</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="33" t="s">
+      <c r="B29" s="31" t="s">
         <v>974</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="32" t="s">
         <v>975</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="30" t="s">
         <v>976</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="33" t="s">
+      <c r="B32" s="31" t="s">
         <v>977</v>
       </c>
-      <c r="C32" s="34" t="s">
+      <c r="C32" s="32" t="s">
         <v>978</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="33" t="s">
+      <c r="B33" s="31" t="s">
         <v>979</v>
       </c>
-      <c r="C33" s="34" t="s">
+      <c r="C33" s="32" t="s">
         <v>980</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Harmonise les noms « Tous les Philosophes … » sur /frises/ et met à jour les données des frises
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -1455,7 +1455,7 @@
     <t xml:space="preserve">philosophie des lumières concentrée sur l'examen critique des idées et des croyances.</t>
   </si>
   <si>
-    <t xml:space="preserve">Constructivisme</t>
+    <t xml:space="preserve">Constructivisme (politique)</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_(politique)"  title=" Wikipedia"&gt; Le Constructivisme (politique) &lt;/a&gt; est un courant de pensée multidisciplinaire postulant que nos connaissances et notre vision du monde ne sont pas un reflet passif de la réalité, mais une construction active élaborée par l'esprit humain. Dans cette approche, le sujet connaissant interagit avec son environnement pour structurer ses propres modèles mentaux, intégrant de nouvelles expériences à des structures cognitives déjà existantes. &lt;/p&gt;&lt;p&gt; Emmanuel Kant a joué un rôle charnière au XVIIIe siècle, en proposant dans sa Critique de la raison pure une vision où l'expérience naît de l'interaction entre les impressions sensibles et la structure propre à l'esprit humain. Cette perspective a posé les jalons d'un constructivisme empirique qui rejette l'idée d'une perception passive et directe de la réalité. &lt;/p&gt;  &lt;p&gt; Dans le domaine de la philosophie politique et du libéralisme, le « rationalisme constructiviste » est souvent dénoncé comme une volonté d'édifier la société selon un dessein rationnel préconçu. Les critiques, notamment Friedrich Hayek, soutiennent que cette approche tend à imposer des plans collectifs par la coercition, négligeant la liberté individuelle et les mécanismes d'ordre spontané issus des interactions humaines. &lt;/p&gt; &lt;p&gt; À l'inverse, en relations internationales, le constructivisme est une théorie scientifique qui analyse la réalité mondiale comme une construction sociale. Pour ses partisans, les intérêts des États et les structures du système international ne sont pas des données fixes ou matérielles, mais le fruit de normes, d'idées et d'interactions partagées entre les acteurs. &lt;/p&gt; 
@@ -6072,7 +6072,7 @@
         <v>431</v>
       </c>
       <c r="K76" s="3" t="s">
-        <v>100</v>
+        <v>251</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Remplace « Immanuel Kant » par « Emmanuel Kant »
Nom de la fiche et mentions dans les textes (fiche de Kant, Marcus Herz,
courants Idéalisme, Illuminisme, Néo-kantisme). La fiche passe à
/philosophes/emmanuel-kant/ ; l'ancienne adresse redirige (301).
Friedrich Immanuel Niethammer n'est pas concerné.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -1471,10 +1471,10 @@
       <c r="E18" s="50" t="inlineStr">
         <is>
           <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Id%C3%A9alisme_(philosophie)"  style="color:#d35400"  title=" Wikipedia"&gt; L'Idéalisme&lt;/a&gt; est une approche philosophique qui accorde une importance primordiale à l'esprit, à la conscience et aux idées en tant que réalités fondamentales. Il soutient que la réalité ultime est de nature mentale ou conceptuelle, plutôt que matérielle et remet en question la conception selon laquelle le monde extérieur existe indépendamment de notre perception et propose que notre conscience joue un rôle actif dans la construction de la réalité. &lt;/p&gt; &lt;p&gt; 
-L'idéalisme a une longue histoire et a été développé par de nombreux philosophes à travers les âges. Parmi les penseurs majeurs associés à l'idéalisme, on trouve Platon, George Berkeley, Immanuel Kant, Friedrich Hegel et Arthur Schopenhauer. &lt;/p&gt; &lt;p&gt; 
+L'idéalisme a une longue histoire et a été développé par de nombreux philosophes à travers les âges. Parmi les penseurs majeurs associés à l'idéalisme, on trouve Platon, George Berkeley, Emmanuel Kant, Friedrich Hegel et Arthur Schopenhauer. &lt;/p&gt; &lt;p&gt; 
 Une des formes les plus célèbres d'idéalisme est l'idéalisme platonicien. Selon Platon, le monde des idées, qui est constitué de concepts abstraits et éternels tels que la beauté, la justice et la vérité, est plus réel que le monde matériel sensible que nous percevons avec nos sens. Pour Platon, les objets physiques ne sont que des reflets imparfaits des idées parfaites et immuables. &lt;/p&gt; &lt;p&gt; 
 L'idéalisme subjectif, également connu sous le nom de solipsisme, soutient que seule notre conscience individuelle est certaine et que tout le reste du monde est une construction de notre esprit. Cependant, cette forme d'idéalisme est souvent considérée comme extrême et controversée. &lt;/p&gt; &lt;p&gt; 
-Une autre forme importante d'idéalisme est l'idéalisme transcendantal d'Immanuel Kant qui a soutenu que notre perception de la réalité est structurée par les catégories de l'esprit humain et que nous ne pouvons connaître que la réalité telle qu'elle est filtrée par nos facultés cognitives. Il a distingué entre le "noumène", la réalité en soi, et le "phénomène", la réalité telle que nous la percevons. &lt;/p&gt; &lt;p&gt;  
+Une autre forme importante d'idéalisme est l'idéalisme transcendantal d'Emmanuel Kant qui a soutenu que notre perception de la réalité est structurée par les catégories de l'esprit humain et que nous ne pouvons connaître que la réalité telle qu'elle est filtrée par nos facultés cognitives. Il a distingué entre le "noumène", la réalité en soi, et le "phénomène", la réalité telle que nous la percevons. &lt;/p&gt; &lt;p&gt;  
 L'idéalisme allemand, représenté principalement par Hegel, a proposé que l'esprit absolu est à la fois la source et la réalité ultime de tout ce qui existe. Selon lui, l'histoire est le processus dialectique de développement de l'esprit vers une compréhension plus complète de lui-même. L'idéalisme de Hegel a eu une influence significative sur d'autres courants de pensée, y compris le marxisme.&lt;/p&gt; &lt;p&gt; 
 Il convient de noter que l'idéalisme est souvent critiqué pour son éloignement de la réalité matérielle et sa propension à négliger l'importance des facteurs matériels et physiques dans la construction de la réalité. Cependant, l'idéalisme a également apporté des contributions importantes à la philosophie en mettant l'accent sur l'importance de la conscience, de la pensée et des idées dans notre compréhension du monde. &lt;/p&gt; &lt;p&gt; &lt;/p&gt;</t>
         </is>
@@ -3762,7 +3762,7 @@
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Illuminisme"  title=" Wikipedia"&gt; L'Illuminisme&lt;/a&gt; , également connu sous le nom de mouvement des Lumières, était un mouvement intellectuel et philosophique qui s'est développé en Europe aux XVIIe et XVIIIe siècles. Les penseurs illuministes remettaient en question les dogmes religieux et l'autorité absolue des monarchies, tout en prônant la raison, la science et la tolérance. &lt;/p&gt; &lt;p&gt;
 Ils cherchaient à éclairer l'esprit des individus en promouvant les idées de liberté, d'égalité, de démocratie, de progrès et de droits de l'homme et ils s'opposaient aux préjugés, à l'obscurantisme et à l'intolérance, et plaçaient la raison au centre de leurs réflexions. &lt;/p&gt; &lt;p&gt;
-Parmi les philosophes les plus influents de ce courant de pensée, on retrouve des figures telles que René Descartes, Voltaire, John Locke, Jean-Jacques Rousseau, Denis Diderot, Montesquieu et Immanuel Kant. Ces penseurs ont produit une grande quantité d'écrits dans lesquels ils ont exposé leurs idées sur des sujets tels que la liberté individuelle, les droits de l'homme, la séparation des pouvoirs, la laïcité, la science et la rationalité. &lt;/p&gt; &lt;p&gt;
+Parmi les philosophes les plus influents de ce courant de pensée, on retrouve des figures telles que René Descartes, Voltaire, John Locke, Jean-Jacques Rousseau, Denis Diderot, Montesquieu et Emmanuel Kant. Ces penseurs ont produit une grande quantité d'écrits dans lesquels ils ont exposé leurs idées sur des sujets tels que la liberté individuelle, les droits de l'homme, la séparation des pouvoirs, la laïcité, la science et la rationalité. &lt;/p&gt; &lt;p&gt;
 L'un des principaux objectifs des Lumières était de réformer les institutions et les pratiques sociales à travers l'éducation et la diffusion des connaissances. Ils croyaient en l'idée que l'ignorance était la source de l'oppression et de l'injustice, et qu'en encourageant la diffusion des savoirs, on pouvait améliorer la condition humaine et favoriser le progrès social. &lt;/p&gt; &lt;p&gt;
 Ce mouvement a exercé une influence considérable sur les événements qui ont suivi, notamment la Révolution française et les mouvements d'indépendance en Amérique du Nord et en Amérique latine. Les idées des philosophes des Lumières ont contribué à façonner les fondements de la démocratie moderne, des droits de l'homme et de la séparation des pouvoirs. &lt;/p&gt;  &lt;audio controls title="Qui a allumé les Lumières par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23497-22.04.2023-ITEMA_23353768-2023F49012S0112-22.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
 </t>
@@ -5215,7 +5215,7 @@
       </c>
       <c r="E103" s="47" t="inlineStr">
         <is>
-          <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/N%C3%A9okantisme"  title=" Wikipedia"&gt;Le Néo-kantisme&lt;/a&gt;  est un courant philosophique apparu en Allemagne et visant à revitaliser la pensée critique d’Immanuel Kant face à l’hégélianisme spéculatif et au positivisme matérialiste. Né en réaction à la crise de la philosophie post-hégélienne, il s’appuie sur les progrès scientifiques (physique newtonienne, puis relativité) pour repenser les conditions de possibilité du savoir. Dominant les universités allemandes jusqu’aux années 1920, il influence épistémologie, éthique, esthétique et sciences humaines avant d’être supplanté par phénoménologie et existentialisme. &lt;/p&gt; &lt;p&gt; Les concepts centraux sont : - Méthode critique actualisée : priorité à "Que puis-je savoir ?" kantien, appliquée aux sciences positives ; rejet du noumène comme fiction, primauté de la production conceptuelle sur l’intuition sensible. - Philosophie des valeurs (Axiologie) : vérité, bien, beauté comme exigences normatives objectives, unifiant savoir et culture sans relativisme historiciste. - Unité du savoir : réponse à la spécialisation scientifique, via une critique de la raison étendue à la culture (Cassirer : "critique de la raison devient critique de la culture"). &lt;/p&gt; &lt;p&gt;</t>
+          <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/N%C3%A9okantisme"  title=" Wikipedia"&gt;Le Néo-kantisme&lt;/a&gt;  est un courant philosophique apparu en Allemagne et visant à revitaliser la pensée critique d’Emmanuel Kant face à l’hégélianisme spéculatif et au positivisme matérialiste. Né en réaction à la crise de la philosophie post-hégélienne, il s’appuie sur les progrès scientifiques (physique newtonienne, puis relativité) pour repenser les conditions de possibilité du savoir. Dominant les universités allemandes jusqu’aux années 1920, il influence épistémologie, éthique, esthétique et sciences humaines avant d’être supplanté par phénoménologie et existentialisme. &lt;/p&gt; &lt;p&gt; Les concepts centraux sont : - Méthode critique actualisée : priorité à "Que puis-je savoir ?" kantien, appliquée aux sciences positives ; rejet du noumène comme fiction, primauté de la production conceptuelle sur l’intuition sensible. - Philosophie des valeurs (Axiologie) : vérité, bien, beauté comme exigences normatives objectives, unifiant savoir et culture sans relativisme historiciste. - Unité du savoir : réponse à la spécialisation scientifique, via une critique de la raison étendue à la culture (Cassirer : "critique de la raison devient critique de la culture"). &lt;/p&gt; &lt;p&gt;</t>
         </is>
       </c>
       <c r="F103" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Recherche : couleurs des drapeaux et ordre des traditions ; Constructivisme en Épistémologie
- Pastilles aux couleurs des drapeaux : Américains (bleu, rayures rouges
  et blanches), Français (bleu, blanc, rouge), Russes (blanc, bleu, rouge).
- « Juifs » placé juste après « Russes ».
- Courant « Constructivisme » classé en Épistémologie : il passe de la
  frise « Politique & Éthique » à « Connaissance & Sciences ».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -6067,8 +6067,10 @@
       <c r="J76" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="K76" s="3" t="s">
-        <v>251</v>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Épistémologie</t>
+        </is>
       </c>
     </row>
     <row r="77" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Ajoute les colonnes Groupe et Importance pour la future frise du monde
- 12 xlsx de philosophes : colonne « Groupe » (8 grandes traditions :
  occident, islam-juif, inde, asie-est, asie-se, sud, russe, orient-ancien)
  et « Importance » (3 = incontournable, 2 = important). Groupes secondaires
  en tags dans « Traditions » (26 fiches : Kojève russe, Byung-Chul Han
  occident, Edward Saïd sud…).
- build-data.py lit ces colonnes et signale un groupe manquant ou inconnu.
  Une nationalité saisie l'emporte sur celle imposée par le fichier.
- Les 13 Latino-Américains du fichier américains reçoivent leur vraie
  nationalité : ils quittent la frise « américains » (85 -> 72) pour la
  frise « hispaniques » (18 -> 31), qui accepte aussi les nationalités
  vénézuélienne, péruvienne et brésilienne (idem dans la recherche).
- Inclut les modifications déjà faites dans autre-actif, coreens,
  greco-romains et courant-occidental.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -3508,131 +3508,131 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3902,6 +3902,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="3" width="4.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="3" width="37.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="3" width="20.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -6067,10 +6068,8 @@
       <c r="J76" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="K76" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Épistémologie</t>
-        </is>
+      <c r="K76" s="3" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Courants par tradition : colonne Groupe, frises par tradition et par grande question, frise « Courants des autres traditions du monde », thèmes harmonisés ; médias Proche-Orient ancien
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -3888,7 +3888,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1048576"/>
+  <dimension ref="A1:N1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -3969,6 +3969,16 @@
       <c r="L3" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groupe</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Traditions</t>
+        </is>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="198" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="n">
@@ -3998,6 +4008,16 @@
       <c r="K4" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien;asie-est</t>
+        </is>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="n">
@@ -4027,6 +4047,11 @@
       <c r="K5" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="205.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
@@ -4053,6 +4078,11 @@
       </c>
       <c r="K6" s="3" t="s">
         <v>27</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="7" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4083,6 +4113,16 @@
       <c r="K7" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident;orient-ancien</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="212.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="n">
@@ -4112,6 +4152,11 @@
       <c r="K8" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="153.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="n">
@@ -4141,6 +4186,11 @@
       <c r="K9" s="3" t="s">
         <v>51</v>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
@@ -4170,6 +4220,11 @@
       <c r="K10" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
@@ -4199,6 +4254,11 @@
       <c r="K11" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="n">
@@ -4228,6 +4288,11 @@
       <c r="K12" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="n">
@@ -4257,6 +4322,11 @@
       <c r="K13" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="n">
@@ -4286,6 +4356,11 @@
       <c r="K14" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="n">
@@ -4315,6 +4390,11 @@
       <c r="K15" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="186" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="n">
@@ -4344,6 +4424,16 @@
       <c r="K16" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="235.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="n">
@@ -4373,6 +4463,11 @@
       <c r="K17" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="257.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="n">
@@ -4402,6 +4497,11 @@
       <c r="K18" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="n">
@@ -4431,6 +4531,11 @@
       <c r="K19" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="n">
@@ -4460,6 +4565,11 @@
       <c r="K20" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="n">
@@ -4489,6 +4599,11 @@
       <c r="K21" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="296.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="n">
@@ -4518,6 +4633,11 @@
       <c r="K22" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="217.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="n">
@@ -4547,6 +4667,11 @@
       <c r="K23" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="219" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="n">
@@ -4576,6 +4701,11 @@
       <c r="K24" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="n">
@@ -4605,6 +4735,11 @@
       <c r="K25" s="3" t="s">
         <v>149</v>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="n">
@@ -4634,6 +4769,16 @@
       <c r="K26" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="n">
@@ -4663,6 +4808,16 @@
       <c r="K27" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="n">
@@ -4692,6 +4847,11 @@
       <c r="K28" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="n">
@@ -4721,6 +4881,11 @@
       <c r="K29" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="n">
@@ -4750,6 +4915,11 @@
       <c r="K30" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="n">
@@ -4778,6 +4948,11 @@
       </c>
       <c r="K31" s="3" t="s">
         <v>20</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="32" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4806,6 +4981,11 @@
       <c r="K32" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="n">
@@ -4835,6 +5015,11 @@
       <c r="K33" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="n">
@@ -4864,6 +5049,11 @@
       <c r="K34" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="n">
@@ -4893,6 +5083,11 @@
       <c r="K35" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="n">
@@ -4921,6 +5116,11 @@
       </c>
       <c r="K36" s="3" t="s">
         <v>20</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="37" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4947,6 +5147,11 @@
       <c r="K37" s="3" t="s">
         <v>51</v>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="n">
@@ -4972,6 +5177,11 @@
       <c r="K38" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="n">
@@ -5001,6 +5211,16 @@
       <c r="K39" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="n">
@@ -5030,6 +5250,11 @@
       <c r="K40" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="n">
@@ -5059,6 +5284,16 @@
       <c r="K41" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud;russe;inde</t>
+        </is>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="n">
@@ -5084,6 +5319,11 @@
       </c>
       <c r="K42" s="3" t="s">
         <v>20</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="43" customFormat="false" ht="127.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5114,6 +5354,11 @@
       <c r="K43" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="208.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="n">
@@ -5143,6 +5388,11 @@
       <c r="K44" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="n">
@@ -5172,6 +5422,11 @@
       <c r="K45" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="n">
@@ -5201,6 +5456,11 @@
       <c r="K46" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="n">
@@ -5230,6 +5490,11 @@
       <c r="K47" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="253.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="n">
@@ -5259,6 +5524,11 @@
       <c r="K48" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="n">
@@ -5288,6 +5558,11 @@
       <c r="K49" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="165.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="n">
@@ -5317,6 +5592,16 @@
       <c r="K50" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe;sud</t>
+        </is>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="n">
@@ -5346,6 +5631,11 @@
       <c r="K51" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="140.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="n">
@@ -5375,6 +5665,11 @@
       <c r="K52" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="168" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="n">
@@ -5404,6 +5699,11 @@
       <c r="K53" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="281.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="n">
@@ -5433,6 +5733,11 @@
       <c r="K54" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="147" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="n">
@@ -5462,6 +5767,11 @@
       <c r="K55" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="250.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="n">
@@ -5491,6 +5801,11 @@
       <c r="K56" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="228.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="n">
@@ -5520,6 +5835,11 @@
       <c r="K57" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="228.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="n">
@@ -5549,6 +5869,11 @@
       <c r="K58" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="223.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="n">
@@ -5578,6 +5903,11 @@
       <c r="K59" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="116.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="14" t="n">
@@ -5607,6 +5937,11 @@
       <c r="K60" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="n">
@@ -5636,6 +5971,11 @@
       <c r="K61" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="14" t="n">
@@ -5665,6 +6005,16 @@
       <c r="K62" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe;sud</t>
+        </is>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="204.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="n">
@@ -5694,6 +6044,11 @@
       <c r="K63" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="11" t="n">
@@ -5723,6 +6078,11 @@
       <c r="K64" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="n">
@@ -5752,6 +6112,11 @@
       <c r="K65" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="117" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="n">
@@ -5781,6 +6146,11 @@
       <c r="K66" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="n">
@@ -5810,6 +6180,11 @@
       <c r="K67" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="n">
@@ -5839,6 +6214,11 @@
       <c r="K68" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="266.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="n">
@@ -5868,6 +6248,11 @@
       <c r="K69" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="202.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="14" t="n">
@@ -5897,6 +6282,11 @@
       <c r="K70" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="162.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="14" t="n">
@@ -5926,6 +6316,16 @@
       <c r="K71" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe;sud</t>
+        </is>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="11" t="n">
@@ -5955,6 +6355,11 @@
       <c r="K72" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="14" t="n">
@@ -5984,6 +6389,16 @@
       <c r="K73" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="11" t="n">
@@ -6013,6 +6428,11 @@
       <c r="K74" s="3" t="s">
         <v>420</v>
       </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="14" t="n">
@@ -6042,6 +6462,11 @@
       <c r="K75" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="182.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="14" t="n">
@@ -6071,6 +6496,11 @@
       <c r="K76" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="n">
@@ -6100,6 +6530,11 @@
       <c r="K77" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="222" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="14" t="n">
@@ -6129,6 +6564,11 @@
       <c r="K78" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="195" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="n">
@@ -6158,6 +6598,11 @@
       <c r="K79" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="222" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="11" t="n">
@@ -6187,6 +6632,11 @@
       <c r="K80" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="14" t="n">
@@ -6216,6 +6666,16 @@
       <c r="K81" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="136.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="14" t="n">
@@ -6245,6 +6705,16 @@
       <c r="K82" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">asie-est</t>
+        </is>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="151.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="n">
@@ -6271,6 +6741,16 @@
       </c>
       <c r="K83" s="3" t="s">
         <v>27</v>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
       </c>
     </row>
     <row r="84" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6301,6 +6781,11 @@
       <c r="K84" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="n">
@@ -6330,6 +6815,11 @@
       <c r="K85" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="14" t="n">
@@ -6359,6 +6849,11 @@
       <c r="K86" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="n">
@@ -6388,6 +6883,16 @@
       <c r="K87" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="99" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="11" t="n">
@@ -6417,6 +6922,11 @@
       <c r="K88" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="14" t="n">
@@ -6446,6 +6956,11 @@
       <c r="K89" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="11" t="n">
@@ -6475,6 +6990,11 @@
       <c r="K90" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="n">
@@ -6504,6 +7024,16 @@
       <c r="K91" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="11" t="n">
@@ -6533,6 +7063,11 @@
       <c r="K92" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="14" t="n">
@@ -6565,6 +7100,16 @@
       <c r="L93" s="1" t="s">
         <v>528</v>
       </c>
+      <c r="M93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="191.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="n">
@@ -6597,6 +7142,16 @@
       <c r="L94" s="1" t="s">
         <v>536</v>
       </c>
+      <c r="M94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe;asie-est</t>
+        </is>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="n">
@@ -6623,6 +7178,11 @@
       </c>
       <c r="K95" s="3" t="s">
         <v>251</v>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="96" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6653,6 +7213,11 @@
       <c r="K96" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="14" t="n">
@@ -6682,6 +7247,11 @@
       <c r="K97" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="11" t="n">
@@ -6711,6 +7281,11 @@
       <c r="K98" s="3" t="s">
         <v>559</v>
       </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="288" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="n">
@@ -6740,6 +7315,11 @@
       <c r="K99" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="165.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="14" t="n">
@@ -6769,6 +7349,16 @@
       <c r="K100" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="172.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="n">
@@ -6798,6 +7388,11 @@
       <c r="K101" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="248.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="14" t="n">
@@ -6827,6 +7422,11 @@
       <c r="K102" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="189" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="n">
@@ -6856,6 +7456,16 @@
       <c r="K103" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="198" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="14" t="n">
@@ -6885,6 +7495,16 @@
       <c r="K104" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="208.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="n">
@@ -6914,6 +7534,11 @@
       <c r="K105" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="222.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="11" t="n">
@@ -6943,6 +7568,11 @@
       <c r="K106" s="3" t="s">
         <v>559</v>
       </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="224.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="n">
@@ -6972,6 +7602,11 @@
       <c r="K107" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="14" t="n">
@@ -7001,6 +7636,11 @@
       <c r="K108" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="173.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="14" t="n">
@@ -7030,6 +7670,11 @@
       <c r="K109" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="150.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="14" t="n">
@@ -7059,6 +7704,11 @@
       <c r="K110" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="155.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="n">
@@ -7088,6 +7738,16 @@
       <c r="K111" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="215.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="n">
@@ -7115,6 +7775,16 @@
       <c r="K112" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="n">
@@ -7141,6 +7811,11 @@
       </c>
       <c r="K113" s="3" t="s">
         <v>251</v>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="114" customFormat="false" ht="279" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7171,6 +7846,16 @@
       <c r="K114" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe;sud;islam-juif</t>
+        </is>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="177.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="n">
@@ -7200,6 +7885,11 @@
       <c r="K115" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="217.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="n">
@@ -7226,6 +7916,11 @@
       <c r="K116" s="3" t="s">
         <v>559</v>
       </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="175.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="n">
@@ -7253,6 +7948,11 @@
       <c r="K117" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="319.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="1" t="n">
@@ -7280,6 +7980,11 @@
       <c r="K118" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="n">
@@ -7306,6 +8011,11 @@
       <c r="K119" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="n">
@@ -7332,6 +8042,11 @@
       <c r="K120" s="3" t="s">
         <v>559</v>
       </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="190.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="n">
@@ -7357,6 +8072,11 @@
       </c>
       <c r="K121" s="3" t="s">
         <v>680</v>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="122" customFormat="false" ht="232.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7387,6 +8107,11 @@
       <c r="K122" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="204.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="n">
@@ -7416,6 +8141,11 @@
       <c r="K123" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="124" customFormat="false" ht="128.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="11" t="n">
@@ -7445,6 +8175,11 @@
       <c r="K124" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="125" customFormat="false" ht="290.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="n">
@@ -7474,6 +8209,11 @@
       <c r="K125" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="290.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="11" t="n">
@@ -7503,6 +8243,11 @@
       <c r="K126" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="243" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="14" t="n">
@@ -7532,6 +8277,11 @@
       <c r="K127" s="3" t="s">
         <v>51</v>
       </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="128" customFormat="false" ht="141.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="14" t="n">
@@ -7561,6 +8311,11 @@
       <c r="K128" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="129" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="n">
@@ -7588,6 +8343,11 @@
       <c r="K129" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="1" t="n">
@@ -7614,6 +8374,11 @@
       </c>
       <c r="K130" s="3" t="s">
         <v>730</v>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="131" customFormat="false" ht="242.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7644,6 +8409,11 @@
       <c r="K131" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="155.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="1" t="n">
@@ -7670,6 +8440,11 @@
       </c>
       <c r="K132" s="3" t="s">
         <v>100</v>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="133" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7700,6 +8475,11 @@
       <c r="K133" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="213.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="14" t="n">
@@ -7729,6 +8509,11 @@
       <c r="K134" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="14" t="n">
@@ -7758,6 +8543,11 @@
       <c r="K135" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="296.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="14" t="n">
@@ -7787,6 +8577,11 @@
       <c r="K136" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="172.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="n">
@@ -7816,6 +8611,11 @@
       <c r="K137" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="288.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="14" t="n">
@@ -7845,6 +8645,11 @@
       <c r="K138" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="14" t="n">
@@ -7874,6 +8679,11 @@
       <c r="K139" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="155.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="11" t="n">
@@ -7903,6 +8713,11 @@
       <c r="K140" s="3" t="s">
         <v>680</v>
       </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="14" t="n">
@@ -7932,6 +8747,16 @@
       <c r="K141" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident;islam-juif</t>
+        </is>
+      </c>
     </row>
     <row r="142" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="14" t="n">
@@ -7961,6 +8786,11 @@
       <c r="K142" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="143" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="n">
@@ -7987,6 +8817,11 @@
       </c>
       <c r="K143" s="3" t="s">
         <v>70</v>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="144" customFormat="false" ht="256.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8017,6 +8852,11 @@
       <c r="K144" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="145" customFormat="false" ht="184.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="14" t="n">
@@ -8046,6 +8886,11 @@
       <c r="K145" s="3" t="s">
         <v>559</v>
       </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="146" customFormat="false" ht="151.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="1" t="n">
@@ -8071,6 +8916,11 @@
       </c>
       <c r="K146" s="3" t="s">
         <v>251</v>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="147" customFormat="false" ht="146.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8101,6 +8951,11 @@
       <c r="K147" s="3" t="s">
         <v>559</v>
       </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="148" customFormat="false" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="11" t="n">
@@ -8130,6 +8985,11 @@
       <c r="K148" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="149" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="n">
@@ -8159,6 +9019,11 @@
       <c r="K149" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="150" customFormat="false" ht="149.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="11" t="n">
@@ -8188,6 +9053,11 @@
       <c r="K150" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="151" customFormat="false" ht="177.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="14" t="n">
@@ -8217,6 +9087,11 @@
       <c r="K151" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="152" customFormat="false" ht="201" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="11" t="n">
@@ -8246,6 +9121,11 @@
       <c r="K152" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="153" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="n">
@@ -8273,6 +9153,11 @@
       <c r="K153" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="154" customFormat="false" ht="170.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="1" t="n">
@@ -8299,6 +9184,11 @@
       <c r="K154" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="155" customFormat="false" ht="149.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="1" t="n">
@@ -8324,6 +9214,11 @@
       </c>
       <c r="K155" s="3" t="s">
         <v>251</v>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="156" customFormat="false" ht="246" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8355,6 +9250,11 @@
         <v>70</v>
       </c>
       <c r="L156" s="1"/>
+      <c r="M156" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="157" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="14" t="n">
@@ -8384,6 +9284,11 @@
       <c r="K157" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="158" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="1" t="n">
@@ -8410,6 +9315,11 @@
       <c r="K158" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="159" customFormat="false" ht="133.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="1" t="n">
@@ -8436,6 +9346,11 @@
       <c r="K159" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="160" customFormat="false" ht="168" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="n">
@@ -8462,6 +9377,11 @@
       </c>
       <c r="K160" s="3" t="s">
         <v>70</v>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="161" customFormat="false" ht="190.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8492,6 +9412,11 @@
       <c r="K161" s="3" t="s">
         <v>559</v>
       </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="162" customFormat="false" ht="150.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="1" t="n">
@@ -8517,6 +9442,11 @@
       </c>
       <c r="K162" s="3" t="s">
         <v>232</v>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="163" customFormat="false" ht="151.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8547,6 +9477,11 @@
       <c r="K163" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="164" customFormat="false" ht="155.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="11" t="n">
@@ -8576,6 +9511,11 @@
       <c r="K164" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="165" customFormat="false" ht="147.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="14" t="n">
@@ -8605,6 +9545,11 @@
       <c r="K165" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="166" customFormat="false" ht="161.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="11" t="n">
@@ -8634,6 +9579,11 @@
       <c r="K166" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="167" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="14" t="n">
@@ -8663,6 +9613,11 @@
       <c r="K167" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="168" customFormat="false" ht="222.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="11" t="n">
@@ -8691,6 +9646,11 @@
       </c>
       <c r="K168" s="3" t="s">
         <v>251</v>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Courants, lot D : Éléatisme, École mégarique, École du Yin-Yang, Xuanxue, Mystique rhénane, Jeunes hégéliens, Darwinisme social, Opéraïsme ; « Illuminisme » devient « Lumières » ; 7 fiches
- Lumières : nom, lien Wikipédia (Lumières (philosophie)), texte retouché, branche, 15 philosophes rattachés ; 301 depuis /courants/illuminisme/
- Fiches : Zou Yan, Guo Xiang, Ji Kang, Henri Suso, Jan van Ruusbroec, William Graham Sumner, Mario Tronti
- Figures clés des courants concernés

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -6262,11 +6262,20 @@
       <c r="C70" s="14" t="s">
         <v>393</v>
       </c>
-      <c r="D70" s="15" t="s">
-        <v>394</v>
-      </c>
-      <c r="E70" s="16" t="s">
-        <v>395</v>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Lumi%C3%A8res_(philosophie)" title=" Wikipedia"&gt;Les Lumières&lt;/a&gt; sont un mouvement intellectuel et philosophique qui s'est développé en Europe aux XVIIe et XVIIIe siècles. Leurs penseurs remettaient en question les dogmes religieux et l'autorité absolue des monarchies, tout en prônant la raison, la science et la tolérance. &lt;/p&gt; &lt;p&gt;
+Ils cherchaient à éclairer l'esprit des individus en promouvant les idées de liberté, d'égalité, de démocratie, de progrès et de droits de l'homme et ils s'opposaient aux préjugés, à l'obscurantisme et à l'intolérance, et plaçaient la raison au centre de leurs réflexions. &lt;/p&gt; &lt;p&gt;
+Parmi les philosophes les plus influents de ce courant de pensée, on retrouve Voltaire, Montesquieu, Jean-Jacques Rousseau, Denis Diderot, d'Holbach, Condorcet, David Hume, Adam Smith et Emmanuel Kant, héritiers de Descartes, de Spinoza et de John Locke. Ces penseurs ont produit une grande quantité d'écrits dans lesquels ils ont exposé leurs idées sur des sujets tels que la liberté individuelle, les droits de l'homme, la séparation des pouvoirs, la laïcité, la science et la rationalité. &lt;/p&gt; &lt;p&gt;
+L'un des principaux objectifs des Lumières était de réformer les institutions et les pratiques sociales à travers l'éducation et la diffusion des connaissances. Ils croyaient en l'idée que l'ignorance était la source de l'oppression et de l'injustice, et qu'en encourageant la diffusion des savoirs, on pouvait améliorer la condition humaine et favoriser le progrès social. L'&lt;a href="https://fr.wikipedia.org/wiki/Encyclop%C3%A9die_ou_Dictionnaire_raisonn%C3%A9_des_sciences%2C_des_arts_et_des_m%C3%A9tiers" title=" Wikipedia"&gt;&lt;em&gt;Encyclopédie&lt;/em&gt;&lt;/a&gt; de Diderot et d'Alembert en fut le grand chantier collectif, et Kant en donna la devise en 1784 dans &lt;a href="https://fr.wikipedia.org/wiki/Qu%27est-ce_que_les_Lumi%C3%A8res_%3F" title=" Wikipedia"&gt;« Qu'est-ce que les Lumières ? »&lt;/a&gt; : « Aie le courage de te servir de ton propre entendement ! » &lt;/p&gt; &lt;p&gt;
+Ce mouvement a exercé une influence considérable sur les événements qui ont suivi, notamment la Révolution française et les mouvements d'indépendance en Amérique du Nord et en Amérique latine. Les idées des philosophes des Lumières ont contribué à façonner les fondements de la démocratie moderne, des droits de l'homme et de la séparation des pouvoirs. &lt;/p&gt;  &lt;audio controls title="Qui a allumé les Lumières par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23497-22.04.2023-ITEMA_23353768-2023F49012S0112-22.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+</t>
+        </is>
       </c>
       <c r="F70" s="14" t="s">
         <v>396</v>
@@ -6276,11 +6285,20 @@
       </c>
       <c r="H70" s="14"/>
       <c r="I70" s="16"/>
-      <c r="J70" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="K70" s="3" t="s">
-        <v>20</v>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement philosophique européen du XVIIIe siècle qui prône la raison, la tolérance, la liberté et le progrès contre les préjugés et l'arbitraire.</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique;Épistémologie</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VOLTAIRE;Denis DIDEROT;MONTESQUIEU;Emmanuel KANT</t>
+        </is>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -9654,30 +9672,256 @@
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A169" s="11">
+        <v>-540</v>
+      </c>
+      <c r="C169" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-540</t>
+        </is>
+      </c>
+      <c r="D169" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Éléatisme</t>
+        </is>
+      </c>
+      <c r="E169" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89cole_%C3%A9l%C3%A9atique" title=" Wikipedia"&gt;L’éléatisme&lt;/a&gt;, ou école d’Élée, est un courant de la philosophie grecque présocratique né au VIe siècle avant notre ère à &lt;a href="https://fr.wikipedia.org/wiki/%C3%89l%C3%A9e" title=" Wikipedia"&gt;Élée&lt;/a&gt;, colonie grecque du sud de l’Italie. La tradition en fait remonter l’origine au poète Xénophane de Colophon, qui critiquait les dieux à forme humaine et concevait un dieu unique et immobile. Mais son véritable fondateur est Parménide.&lt;/p&gt; &lt;p&gt;Dans son poème &lt;em&gt;De la nature&lt;/em&gt;, Parménide oppose deux voies : celle de la vérité, qui affirme que « l’être est » et que « le non-être n’est pas », et celle de l’opinion, qui suit les sens et croit au devenir. Car si seul l’être est, rien ne peut naître du néant ni y retourner : l’être est un, sans commencement ni fin, continu, immobile, semblable à « une sphère bien arrondie ». Le changement et la multiplicité que nous percevons ne sont qu’apparence, et « c’est la même chose que penser et être ». Son disciple Zénon défend cette thèse par l’absurde, avec des &lt;a href="https://fr.wikipedia.org/wiki/Paradoxes_de_Z%C3%A9non" title=" Wikipedia"&gt;paradoxes&lt;/a&gt; restés célèbres : Achille ne rattrapera jamais la tortue, car il doit d’abord atteindre le point d’où elle est partie, et elle a déjà avancé ; la flèche en vol est immobile à chaque instant. Aristote voit en lui l’inventeur de la dialectique. Mélissos de Samos, amiral qui battit la flotte athénienne, ajoute que l’être est infini.&lt;/p&gt; &lt;p&gt;Toute la philosophie grecque a dû répondre à l’éléatisme : les atomistes, en admettant le vide, et Platon, qui dans le &lt;em&gt;Sophiste&lt;/em&gt; ose le « parricide » de son « père Parménide » en montrant que le non-être est en un sens. Au XXe siècle, Heidegger a vu en Parménide le premier penseur de l’être.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="I169" s="1"/>
-      <c r="J169" s="1"/>
+      <c r="J169" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">école grecque d’Élée pour qui l’être est un, immobile et éternel, et le changement une illusion des sens.</t>
+        </is>
+      </c>
+      <c r="K169" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Logique</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARMÉNIDE;ZÉNON d'Élée;MÉLISSOS</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N169"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A170" s="11">
+        <v>-400</v>
+      </c>
+      <c r="C170" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-400</t>
+        </is>
+      </c>
+      <c r="D170" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">École mégarique</t>
+        </is>
+      </c>
+      <c r="E170" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89cole_m%C3%A9garique" title=" Wikipedia"&gt;L’école mégarique&lt;/a&gt; est une école de philosophie grecque fondée vers 400 avant notre ère à Mégare, près d’Athènes, par Euclide de Mégare, disciple de Socrate, présent à sa mort selon le &lt;em&gt;Phédon&lt;/em&gt;. Après l’exécution de leur maître, Platon et d’autres socratiques trouvent d’ailleurs refuge auprès de lui.&lt;/p&gt; &lt;p&gt;Euclide unit l’enseignement moral de Socrate et la doctrine de Parménide : le Bien est un, même si on l’appelle de plusieurs noms, sagesse, Dieu ou intelligence, et ce qui s’oppose au Bien n’existe pas. Mais l’école est surtout restée célèbre pour son art de la discussion et ses paradoxes, qui mettent la logique à l’épreuve. Eubulide de Milet invente le &lt;a href="https://fr.wikipedia.org/wiki/Paradoxe_du_menteur" title=" Wikipedia"&gt;paradoxe du menteur&lt;/a&gt; (« celui qui dit qu’il ment dit-il vrai ? ») et le &lt;a href="https://fr.wikipedia.org/wiki/Paradoxe_sorite" title=" Wikipedia"&gt;paradoxe du tas&lt;/a&gt; : un grain de blé ne fait pas un tas, ni deux, ni trois ; à partir de combien en fait-on un ? Diodore Cronos, surnommé « le dialecticien », forge l’« argument dominateur » sur le possible et le nécessaire : n’est possible que ce qui est ou sera vrai. Son élève Philon de Mégare définit l’implication logique comme le feront les logiciens modernes. Stilpon, enfin, connu pour son calme face aux malheurs, enseigne une morale proche des cyniques.&lt;/p&gt; &lt;p&gt;Zénon de Kition, le fondateur du stoïcisme, fut l’élève de Stilpon et de Diodore : la logique stoïcienne prolonge celle des Mégariques. Leurs paradoxes, longtemps tenus pour de simples jeux, sont aujourd’hui étudiés par les logiciens comme de vrais problèmes sur la vérité, le vague et la modalité.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="I170" s="1"/>
-      <c r="J170" s="1"/>
+      <c r="J170" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">école socratique de Mégare, célèbre pour ses paradoxes logiques : le menteur, le tas, l’argument dominateur.</t>
+        </is>
+      </c>
+      <c r="K170" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Logique;Éthique</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EUCLIDE de Mégare;EUBULIDE de Milet;Diodore CRONOS</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N170"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A171" s="11">
+        <v>1300</v>
+      </c>
+      <c r="C171" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1300</t>
+        </is>
+      </c>
+      <c r="D171" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mystique rhénane</t>
+        </is>
+      </c>
+      <c r="E171" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Mystique_rh%C3%A9nane" title=" Wikipedia"&gt;La mystique rhénane&lt;/a&gt; est un grand courant spirituel chrétien des XIIIe et XIVe siècles, qui s’étend le long du Rhin, de la Suisse aux Flandres. Il naît dans l’ordre dominicain et dans les communautés de béguines, ces femmes qui menaient une vie religieuse sans prononcer de vœux, comme Mechtilde de Magdebourg ou &lt;a href="https://fr.wikipedia.org/wiki/Marguerite_Porete" title=" Wikipedia"&gt;Marguerite Porete&lt;/a&gt;, brûlée à Paris en 1310. Fait nouveau, ses maîtres prêchent et écrivent dans la langue du peuple, l’allemand ou le flamand, et non en latin.&lt;/p&gt; &lt;p&gt;Sa figure majeure est Maître Eckhart. Dans ses sermons, il enseigne que Dieu n’est pas à chercher au-dehors : au fond de l’âme se trouve un lieu où Dieu et l’âme ne font qu’un, et où le Verbe divin naît sans cesse. Pour y parvenir, il faut le « détachement », se défaire de tout attachement aux choses, aux images et même à sa propre volonté, jusqu’à « prier Dieu d’être libre de Dieu », c’est-à-dire des représentations que l’on se fait de lui. Au-delà du Dieu que l’on nomme, il y a la « déité », abîme silencieux et sans nom. Accusé d’hérésie, il meurt pendant son procès, et le pape condamne en 1329 vingt-huit de ses propositions. Ses disciples Jean Tauler, prédicateur à Strasbourg, et &lt;a href="https://fr.wikipedia.org/wiki/Henri_Suso" title=" Wikipedia"&gt;Henri Suso&lt;/a&gt; poursuivent son œuvre de manière plus pratique et plus prudente, tandis que le Brabançon &lt;a href="https://fr.wikipedia.org/wiki/Jan_Van_Ruysbroeck_%28religieux%29" title=" Wikipedia"&gt;Jan van Ruusbroec&lt;/a&gt; décrit les étapes de l’union à Dieu dans &lt;em&gt;Les Noces spirituelles&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;La mystique rhénane a inspiré Luther, Nicolas de Cues, Angelus Silesius, puis Hegel et Schopenhauer. Au XXe siècle, Heidegger reprend le mot d’Eckhart, la « sérénité », pour penser une autre relation au monde.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="I171" s="1"/>
-      <c r="J171" s="1"/>
+      <c r="J171" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mystique chrétienne des XIIIe et XIVe siècles, de Maître Eckhart à Ruusbroec : le détachement et la naissance de Dieu dans l’âme.</t>
+        </is>
+      </c>
+      <c r="K171" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Métaphysique</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maître ECKHART;Jean TAULER;Henri SUSO;Jan van RUUSBROEC</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N171"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A172" s="11">
+        <v>1835</v>
+      </c>
+      <c r="C172" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1835</t>
+        </is>
+      </c>
+      <c r="D172" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jeunes hégéliens</t>
+        </is>
+      </c>
+      <c r="E172" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;On appelle &lt;a href="https://fr.wikipedia.org/wiki/Jeunes_h%C3%A9g%C3%A9liens" title=" Wikipedia"&gt;jeunes hégéliens&lt;/a&gt;, ou hégéliens de gauche, les disciples de Hegel qui, après sa mort en 1831, tirent de sa philosophie des conclusions radicales. Hegel avait voulu réconcilier la raison, la religion et l’État ; ses héritiers « de droite » y voient une justification du christianisme et de la monarchie prussienne, ceux « de gauche » une méthode critique qui doit tout remettre en cause.&lt;/p&gt; &lt;p&gt;La rupture éclate en 1835 avec la &lt;em&gt;Vie de Jésus&lt;/em&gt; de David Strauss, qui lit les Évangiles comme des mythes nés de la foi des premières communautés. Bruno Bauer va plus loin et en conteste toute valeur historique, ce qui lui coûte son poste à l’université. Dans &lt;a href="https://fr.wikipedia.org/wiki/L%27Essence_du_christianisme" title=" Wikipedia"&gt;&lt;em&gt;L’Essence du christianisme&lt;/em&gt;&lt;/a&gt; (1841), Ludwig Feuerbach soutient que Dieu n’est que la projection de l’essence humaine : en adorant Dieu, l’homme adore sans le savoir ses propres qualités, dont il s’est dépouillé. La critique de la religion doit donc rendre à l’homme ce qu’il a donné au ciel. Réunis à Berlin dans le cercle des « Affranchis », ces penseurs passent de la critique religieuse à la critique politique. Max Stirner, dans &lt;a href="https://fr.wikipedia.org/wiki/L%27Unique_et_sa_propri%C3%A9t%C3%A9" title=" Wikipedia"&gt;&lt;em&gt;L’Unique et sa propriété&lt;/em&gt;&lt;/a&gt; (1844), retourne l’argument contre Feuerbach lui-même : « l’Homme » n’est qu’un nouveau dieu, et seul compte l’individu unique.&lt;/p&gt; &lt;p&gt;Le jeune Karl Marx et Friedrich Engels appartiennent à ce milieu avant de rompre avec lui : dans les &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A8ses_sur_Feuerbach" title=" Wikipedia"&gt;Thèses sur Feuerbach&lt;/a&gt; (1845), Marx écrit que « les philosophes n’ont fait qu’interpréter le monde ; il s’agit maintenant de le transformer ». Le mouvement se dissout après la révolution de 1848.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="I172" s="1"/>
-      <c r="J172" s="1"/>
+      <c r="J172" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">disciples radicaux de Hegel des années 1835-1848 : critique de la religion et de l’État prussien, de Feuerbach à Marx et Stirner.</t>
+        </is>
+      </c>
+      <c r="K172" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique;Théologie et spiritualité</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ludwig FEUERBACH;Max STIRNER;Bruno BAUER;Karl MARX</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N172"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D173" s="3"/>
+      <c r="A173" s="11">
+        <v>1860</v>
+      </c>
+      <c r="C173" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1860</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darwinisme social</t>
+        </is>
+      </c>
+      <c r="E173" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;On appelle &lt;a href="https://fr.wikipedia.org/wiki/Darwinisme_social" title=" Wikipedia"&gt;darwinisme social&lt;/a&gt; les doctrines de la seconde moitié du XIXe siècle qui appliquent aux sociétés humaines la théorie de l’évolution et la sélection naturelle. Le mot, apparu vers 1880, est surtout employé par ses adversaires : rares sont ceux qui s’en sont réclamés.&lt;/p&gt; &lt;p&gt;Son principal inspirateur est le philosophe anglais Herbert Spencer, qui avait conçu une philosophie de l’évolution universelle avant même la parution de &lt;em&gt;L’Origine des espèces&lt;/em&gt; de Darwin, en 1859, et qui invente en 1864 l’expression « survie du plus apte ». Pour lui, la société évolue comme un organisme, et la concurrence entre individus est le moteur du progrès : l’État ne doit pas aider les pauvres, car il entraverait la sélection. Aux États-Unis, le sociologue &lt;a href="https://fr.wikipedia.org/wiki/William_Graham_Sumner" title=" Wikipedia"&gt;William Graham Sumner&lt;/a&gt; défend de même un libéralisme sans pitié. D’autres transposent la lutte pour la vie aux nations et aux « races », pour justifier la colonisation et les guerres. Le cousin de Darwin, &lt;a href="https://fr.wikipedia.org/wiki/Francis_Galton" title=" Wikipedia"&gt;Francis Galton&lt;/a&gt;, fonde l’&lt;a href="https://fr.wikipedia.org/wiki/Eug%C3%A9nisme" title=" Wikipedia"&gt;eugénisme&lt;/a&gt;, qui veut améliorer l’espèce humaine en favorisant la reproduction des « meilleurs » ; il conduira à des stérilisations forcées et nourrira l’idéologie nazie.&lt;/p&gt; &lt;p&gt;Darwin lui-même voyait dans la sympathie et l’entraide des instincts sociaux sélectionnés par l’évolution. Le géographe anarchiste Pierre Kropotkine répond en 1902, dans &lt;a href="https://fr.wikipedia.org/wiki/L%27Entraide%2C_un_facteur_de_l%27%C3%A9volution" title=" Wikipedia"&gt;&lt;em&gt;L’Entraide&lt;/em&gt;&lt;/a&gt;, que la coopération compte autant que la lutte. Aujourd’hui, le darwinisme social est rejeté par les biologistes comme une confusion entre ce qui est et ce qui doit être.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="I173" s="1"/>
-      <c r="J173" s="1"/>
+      <c r="J173" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">application de la sélection naturelle aux sociétés humaines, qui a servi à justifier inégalités, colonialisme et eugénisme.</t>
+        </is>
+      </c>
+      <c r="K173" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique;Philosophie des sciences et du vivant</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Herbert SPENCER;William Graham SUMNER</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N173"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D174" s="3"/>
+      <c r="A174" s="11">
+        <v>1961</v>
+      </c>
+      <c r="C174" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1961</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opéraïsme</t>
+        </is>
+      </c>
+      <c r="E174" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Op%C3%A9ra%C3%AFsme" title=" Wikipedia"&gt;L’opéraïsme&lt;/a&gt;, de l’italien &lt;em&gt;operaio&lt;/em&gt;, « ouvrier », est un courant marxiste italien né au début des années 1960, en marge du Parti communiste, autour de la revue &lt;em&gt;Quaderni rossi&lt;/em&gt; fondée en 1961 par &lt;a href="https://fr.wikipedia.org/wiki/Raniero_Panzieri" title=" Wikipedia"&gt;Raniero Panzieri&lt;/a&gt;. Dans l’Italie du « miracle économique », de grandes usines comme celles de Fiat à Turin attirent des centaines de milliers d’ouvriers venus du Sud.&lt;/p&gt; &lt;p&gt;Plutôt que de partir des théories des partis, les opéraïstes partent de l’enquête auprès des ouvriers eux-mêmes, de leurs conditions de travail et de leurs luttes. Dans &lt;em&gt;Ouvriers et capital&lt;/em&gt; (1966), &lt;a href="https://fr.wikipedia.org/wiki/Mario_Tronti" title=" Wikipedia"&gt;Mario Tronti&lt;/a&gt; opère ce qu’il appelle une « révolution copernicienne » : ce n’est pas le capital qui fait l’histoire et les ouvriers qui réagissent, ce sont les luttes ouvrières qui contraignent le capital à se transformer, à innover et à s’automatiser. L’ouvrier ne cherche pas à être reconnu comme travailleur, mais à se libérer du travail lui-même : d’où le mot d’ordre du « refus du travail ». Les opéraïstes étudient la « composition de classe », c’est-à-dire la manière dont les ouvriers sont organisés et se pensent, et voient dans l’« ouvrier-masse » des chaînes de montage, peu qualifié et sans attache au métier, le nouveau sujet révolutionnaire.&lt;/p&gt; &lt;p&gt;Après « l’automne chaud » des grèves de 1969, le courant inspire des groupes comme &lt;a href="https://fr.wikipedia.org/wiki/Potere_operaio" title=" Wikipedia"&gt;Potere operaio&lt;/a&gt;, animé par Antonio Negri, puis l’Autonomie des années 1970. Il se prolonge dans le « post-opéraïsme » de Negri et de Paolo Virno, qui pensent le travail immatériel et la « multitude ».&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="I174" s="1"/>
-      <c r="J174" s="1"/>
+      <c r="J174" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">marxisme italien des années 1960 qui part des luttes ouvrières et du refus du travail plutôt que des partis.</t>
+        </is>
+      </c>
+      <c r="K174" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mario TRONTI;Antonio NEGRI</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N174"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D175" s="3"/>

</xml_diff>

<commit_message>
Courants : 10 textes enrichis ; /frises/ : cartes des courants refaites ; frises de courants sans boutons de thème
- Textes : Platonisme, Socratisme, Ontologie Orientée Objet, Monisme, Cynisme, Transcendantalisme, Keynésianisme, Psychanalyse, Confucianisme coréen, Mimamsa (liens et audios gardés, HTML cassé réparé)
- /frises/ : carte Occident à part entière, plus de carte « Reste du monde » ; 4 philosophes représentatifs en vignettes ; jalons = courant le plus fourni de chaque époque ; « → aujourd'hui »
- Frises occidentale et orientale : boutons de filtre par thème retirés ; la recherche filtrée par thème ouvre la sous-frise du thème

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -4305,8 +4305,10 @@
       <c r="D13" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="13" t="s">
-        <v>73</v>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Socrate"  style="color:#d35400"  title=" Wikipedia"&gt;Le Socratisme&lt;/a&gt; désigne la philosophie de Socrate (vers 470-399 av. J.-C.) et de ceux qui s’en sont réclamés. Socrate n’a rien écrit : nous le connaissons surtout par les dialogues de son disciple Platon, par Xénophon et par la caricature qu’en fait Aristophane dans &lt;em&gt;Les Nuées&lt;/em&gt;. Il passe sa vie à interroger ses concitoyens sur l’agora d’Athènes et fait « descendre la philosophie du ciel sur la terre », selon le mot de Cicéron : au lieu d’étudier la nature, comme les présocratiques, il s’intéresse à la manière dont l’être humain doit vivre.&lt;/p&gt; &lt;p&gt;Sa méthode est le dialogue. Par l’&lt;a href="https://fr.wikipedia.org/wiki/Ironie_socratique" title=" Wikipedia"&gt;ironie&lt;/a&gt;, il feint l’ignorance et pousse ses interlocuteurs à définir le courage, la justice ou la piété, puis montre les contradictions de leurs réponses. Par la &lt;a href="https://fr.wikipedia.org/wiki/Ma%C3%AFeutique_%28philosophie%29" title=" Wikipedia"&gt;maïeutique&lt;/a&gt;, l’« art d’accoucher les esprits », comme sa mère sage-femme accouchait les corps, il les aide à découvrir par eux-mêmes la vérité qu’ils portent en eux. Sa devise est le « &lt;a href="https://fr.wikipedia.org/wiki/Gnothi_seauton" title=" Wikipedia"&gt;Connais-toi toi-même&lt;/a&gt; » inscrit au temple de Delphes, et sa sagesse consiste à savoir qu’il ne sait rien. Pour lui, nul n’est méchant volontairement : le mal vient de l’ignorance, et la vertu est un savoir ; c’est en se connaissant soi-même qu’on devient juste et heureux. Mieux vaut subir l’injustice que la commettre.&lt;/p&gt; &lt;p&gt;Accusé d’impiété et de corruption de la jeunesse, Socrate est condamné à mort en 399 lors d’un &lt;a href="https://fr.wikipedia.org/wiki/Proc%C3%A8s_de_Socrate" title=" Wikipedia"&gt;procès&lt;/a&gt; resté célèbre, et boit la ciguë, refusant de s’enfuir pour ne pas désobéir aux lois. Sa mort fait de lui le modèle du philosophe. De son enseignement naissent les écoles dites socratiques : l’Académie de Platon, les cyniques d’Antisthène, les cyrénaïques d’Aristippe et l’école de Mégare.&lt;/p&gt;  &lt;audio controls title="La pensée de Socrate par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-21.11.2016-ITEMA_21141871-2.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F13" s="11" t="s">
         <v>74</v>
@@ -4339,14 +4341,20 @@
       <c r="D14" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="G14" s="16" t="s">
-        <v>81</v>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Platonisme"  style="color:#d35400" title=" Wikipedia"&gt;Le Platonisme&lt;/a&gt; est la philosophie issue de l’enseignement de Platon (vers 428-348 av. J.-C.), disciple de Socrate et fondateur de l’&lt;a href="https://fr.wikipedia.org/wiki/Acad%C3%A9mie_de_Platon" title=" Wikipedia"&gt;Académie&lt;/a&gt; d’Athènes, la première grande école de philosophie. Son idée centrale est la distinction entre deux mondes : le monde sensible, que nous percevons par les sens, changeant et imparfait, et le monde intelligible des Idées, ou Formes, éternelles et immuables, que seule la raison peut saisir. La beauté d’un visage passe, mais l’Idée du Beau demeure ; les cercles que nous traçons sont imparfaits, mais le Cercle en soi est parfait.&lt;/p&gt; &lt;p&gt;Platon illustre cette doctrine par l’&lt;a href="https://fr.wikipedia.org/wiki/All%C3%A9gorie_de_la_caverne" title=" Wikipedia"&gt;allégorie de la caverne&lt;/a&gt;, dans &lt;em&gt;La République&lt;/em&gt; : des prisonniers enchaînés au fond d’une caverne prennent pour la réalité les ombres projetées sur la paroi ; le philosophe est celui qui se libère, monte vers la lumière et découvre le soleil, image du Bien, source de toute vérité. Connaître, c’est donc se détourner des apparences ; c’est aussi se ressouvenir, car l’âme, immortelle, a contemplé les Idées avant de naître : c’est la théorie de la réminiscence. De cette métaphysique découle une politique, où la cité juste doit être gouvernée par ceux qui connaissent le Bien, les philosophes-rois, et une éthique de l’harmonie de l’âme.&lt;/p&gt; &lt;p&gt;Le platonisme a traversé toute l’histoire de la pensée : l’Académie dure près de trois siècles, le néoplatonisme de &lt;a href="https://fr.wikipedia.org/wiki/Plotin" title=" Wikipedia"&gt;Plotin&lt;/a&gt; le prolonge et les Pères de l’Église, comme saint Augustin, s’en inspirent. Descartes, Leibniz ou Hegel en héritent à leur manière. En mathématiques, on appelle encore « platoniciens » ceux qui pensent que les nombres existent indépendamment de nous. Il a aussi marqué la théologie, la littérature et les arts.&lt;/p&gt;  &lt;audio controls title="Raison et réalité: les idées de Platon par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13915-06.05.2022-ITEMA_23017794-2020C3372E0466-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1QRzyfS0-Jg</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Le platonisme en 3 minutes | Derrière les ombres, que cherches-tu vraiment ?" par Échos de Philosophie</t>
+        </is>
       </c>
       <c r="H14" s="14"/>
       <c r="I14" s="16"/>
@@ -4548,8 +4556,10 @@
       <c r="D20" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="E20" s="16" t="s">
-        <v>115</v>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Cynisme"   title=" Wikipedia"&gt;Le Cynisme&lt;/a&gt; est une école de philosophie grecque née au IVe siècle avant notre ère, à Athènes. Elle se réclame d’Antisthène, disciple de Socrate, et surtout de &lt;a href="https://fr.wikipedia.org/wiki/Diog%C3%A8ne_de_Sinope" title=" Wikipedia"&gt;Diogène de Sinope&lt;/a&gt;, qui en devient la figure légendaire. Son nom viendrait du gymnase du Cynosarge, où enseignait Antisthène, ou du mot grec qui signifie « chien » : les cyniques vivent comme des chiens, sans honte et sans maison, et revendiquent fièrement ce surnom.&lt;/p&gt; &lt;p&gt;Leur philosophie est d’abord une manière de vivre. Pour être heureux, il faut suivre la nature et se libérer de tout ce qui est artificiel : les richesses, le pouvoir, la réputation, les conventions. Diogène dort dans une jarre et jette son écuelle en voyant un enfant boire dans le creux de ses mains. Il cherche « un homme » en plein jour avec une lanterne, et répond à Alexandre le Grand, qui lui propose ce qu’il désire : « Ôte-toi de mon soleil. » Par la provocation et l’insolence, les cyniques pratiquent le « franc-parler » et dénoncent l’hypocrisie de la société. Ils se disent citoyens du monde, « cosmopolites », plutôt que d’une cité. La vertu, qui s’acquiert par l’effort et l’entraînement, suffit au bonheur. Cratès et Hipparchia, couple de philosophes, mènent ensemble cette vie libre.&lt;/p&gt; &lt;p&gt;Le cynisme a profondément influencé le stoïcisme. Au XXe siècle, Michel Foucault y voit une forme exemplaire du « courage de la vérité ». Le sens moderne du mot, le mépris des valeurs morales, en est éloigné, et &lt;a href="https://www.youtube.com/watch?v=_ITGtKs056M&amp;t=105s&amp;ab_channel=Kosmos" title="Le cynisme, vidéo de Kosmos"&gt;certains penseurs&lt;/a&gt; ont proposé de retrouver dans le cynisme antique une critique joyeuse et constructive de la société.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F20" s="14" t="s">
         <v>116</v>
@@ -6317,8 +6327,10 @@
       <c r="D71" s="15" t="s">
         <v>399</v>
       </c>
-      <c r="E71" s="27" t="s">
-        <v>400</v>
+      <c r="E71" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Monisme"  title=" Wikipedia"&gt;Le Monisme&lt;/a&gt; désigne toute doctrine qui ramène la diversité du réel à une seule substance ou à un seul principe. Le mot est forgé en 1734 par le philosophe allemand Christian Wolff dans sa &lt;em&gt;Psychologia rationalis&lt;/em&gt;, pour désigner ceux qui n’admettent qu’une seule sorte de substance, par opposition au &lt;a href="https://fr.wikipedia.org/wiki/Dualisme_%28philosophie_de_l%27esprit%29" title=" Wikipedia"&gt;dualisme&lt;/a&gt; de Descartes, qui distinguait l’âme et le corps. Il entre en français à la fin du XIXe siècle.&lt;/p&gt; &lt;p&gt;Les idées monistes sont pourtant bien plus anciennes. Parménide affirme que l’Être est un, éternel et immobile ; Héraclite voit dans le Logos l’unité des contraires. En Inde, l’Advaita Védanta enseigne que l’âme individuelle et l’absolu, le Brahman, ne font qu’un. Le premier grand monisme moderne est celui de Spinoza : dans l’&lt;em&gt;Éthique&lt;/em&gt; (1677), il n’existe qu’une seule substance infinie, « Dieu, c’est-à-dire la Nature », dont la pensée et l’étendue ne sont que deux attributs. On distingue ensuite plusieurs formes de monisme : matérialiste, quand tout se ramène à la matière, comme chez d’Holbach ou chez le biologiste &lt;a href="https://fr.wikipedia.org/wiki/Ernst_Haeckel" title=" Wikipedia"&gt;Ernst Haeckel&lt;/a&gt;, qui fonde en 1906 une Ligue moniste ; idéaliste, quand tout est esprit, comme chez Hegel, pour qui le réel est le déploiement de l’Esprit absolu ; ou neutre, quand matière et esprit sont deux aspects d’une réalité plus fondamentale, comme chez William James ou Bertrand Russell.&lt;/p&gt; &lt;p&gt;En philosophie de l’esprit, le débat entre monisme et dualisme reste vif : la plupart des philosophes contemporains sont monistes et cherchent à expliquer la conscience comme un phénomène naturel, tandis que d’autres jugent cette réduction impossible. Le monisme s’oppose ainsi au dualisme, qui admet deux principes, et au pluralisme, qui en admet plusieurs.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F71" s="14" t="s">
         <v>401</v>
@@ -7064,8 +7076,10 @@
       <c r="D92" s="12" t="s">
         <v>516</v>
       </c>
-      <c r="E92" s="13" t="s">
-        <v>517</v>
+      <c r="E92" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Transcendantalisme_(%C3%89tats-Unis)"  style="color:#d35400"  title=" Wikipedia"&gt;Le Transcendantalisme&lt;/a&gt; est un mouvement philosophique, littéraire et spirituel né en Nouvelle-Angleterre dans les années 1830, autour de &lt;a href="https://fr.wikipedia.org/wiki/Ralph_Waldo_Emerson" title=" Wikipedia"&gt;Ralph Waldo Emerson&lt;/a&gt;. Il réagit contre le rationalisme de l’Église unitarienne et contre l’empirisme de Locke, pour qui toute connaissance vient des sens. Les transcendantalistes affirment au contraire, en s’inspirant de Kant, de l’idéalisme allemand, du romantisme anglais et même des textes sacrés de l’Inde, que l’esprit humain a une intuition directe des vérités spirituelles.&lt;/p&gt; &lt;p&gt;Son manifeste est l’essai &lt;em&gt;Nature&lt;/em&gt; d’Emerson (1836) : la nature est le langage de l’esprit, et chacun peut y rencontrer le divin sans passer par les Églises ni les dogmes. Emerson parle d’une « surâme » (&lt;em&gt;Over-Soul&lt;/em&gt;), âme universelle à laquelle participent tous les êtres. Il en tire une éthique de la « confiance en soi » : chacun doit suivre sa voix intérieure plutôt que la tradition et le conformisme. Le « Transcendental Club » fonde une revue, &lt;em&gt;The Dial&lt;/em&gt;, dirigée par la féministe &lt;a href="https://fr.wikipedia.org/wiki/Margaret_Fuller" title=" Wikipedia"&gt;Margaret Fuller&lt;/a&gt;, et des communautés utopiques comme Brook Farm. &lt;a href="https://fr.wikipedia.org/wiki/Henry_David_Thoreau" title=" Wikipedia"&gt;Henry David Thoreau&lt;/a&gt;, ami d’Emerson, vit deux ans dans une cabane au bord de l’étang de Walden, expérience racontée dans &lt;em&gt;Walden ou la Vie dans les bois&lt;/em&gt; (1854) ; il refuse de payer l’impôt qui finance l’esclavage et la guerre, et en tire &lt;a href="https://fr.wikipedia.org/wiki/La_D%C3%A9sob%C3%A9issance_civile" title=" Wikipedia"&gt;&lt;em&gt;La Désobéissance civile&lt;/em&gt;&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Mouvement bref, qui décline après 1850, le transcendantalisme a pourtant profondément marqué la culture américaine : il a nourri l’abolitionnisme, inspiré Walt Whitman et, plus tard, Gandhi, Martin Luther King et la pensée écologique.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F92" s="11" t="s">
         <v>518</v>
@@ -7919,8 +7933,10 @@
       <c r="D116" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="E116" s="3" t="s">
-        <v>651</v>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Psychanalyse" title=" Wikipedia"&gt;La Psychanalyse&lt;/a&gt; est à la fois une théorie du psychisme, une méthode d’investigation et une pratique thérapeutique, fondées par le médecin viennois &lt;a href="https://fr.wikipedia.org/wiki/Sigmund_Freud" title=" Wikipedia"&gt;Sigmund Freud&lt;/a&gt; à la fin du XIXe siècle. Elle naît de son travail avec des malades hystériques et de la découverte que leurs symptômes ont un sens : ils expriment des souvenirs et des désirs refoulés. Le patient, allongé sur le divan, dit tout ce qui lui vient à l’esprit : c’est la méthode des « associations libres ».&lt;/p&gt; &lt;p&gt;Son concept central est l’&lt;a href="https://fr.wikipedia.org/wiki/Inconscient" title=" Wikipedia"&gt;inconscient&lt;/a&gt; : une grande part de notre vie psychique échappe à la conscience, et des désirs refoulés, souvent d’origine sexuelle et infantile, déterminent en secret nos actes, nos rêves, nos lapsus et nos symptômes. « Le rêve est la voie royale qui mène à l’inconscient », écrit Freud dans &lt;a href="https://fr.wikipedia.org/wiki/L%27Interpr%C3%A9tation_du_r%C3%AAve" title=" Wikipedia"&gt;&lt;em&gt;L’Interprétation du rêve&lt;/em&gt;&lt;/a&gt; (1900). Il décrit le psychisme comme le lieu d’un conflit entre le ça, réservoir des pulsions, le surmoi, gardien des interdits, et le moi, qui tente de les concilier avec la réalité. Le &lt;a href="https://fr.wikipedia.org/wiki/Complexe_d%27%C5%92dipe" title=" Wikipedia"&gt;complexe d’Œdipe&lt;/a&gt; structure le développement de l’enfant. Après Copernic et Darwin, Freud inflige à l’humanité une troisième « blessure narcissique » : le moi « n’est pas maître dans sa propre maison ».&lt;/p&gt; &lt;p&gt;Ses disciples se séparent souvent de lui, comme Carl Gustav Jung, avec l’inconscient collectif, ou Alfred Adler. En France, Jacques Lacan relit Freud à la lumière de la linguistique structurale : l’inconscient est « structuré comme un langage ». Sartre, Ricœur, Derrida ou Deleuze ont débattu avec la psychanalyse, et des penseurs comme Slavoj Žižek ou Judith Butler s’en servent pour penser l’idéologie, le genre et le pouvoir. Sa scientificité a aussi été contestée, notamment par Karl Popper.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F116" s="1" t="s">
         <v>652</v>
@@ -8410,8 +8426,10 @@
       <c r="D131" s="12" t="s">
         <v>732</v>
       </c>
-      <c r="E131" s="13" t="s">
-        <v>733</v>
+      <c r="E131" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Keyn%C3%A9sianisme" title=" Wikipedia"&gt;Le Keynésianisme&lt;/a&gt; n’est pas un courant philosophique au sens strict, mais une école de pensée économique, née de l’œuvre de l’économiste britannique &lt;a href="https://fr.wikipedia.org/wiki/John_Maynard_Keynes" title=" Wikipedia"&gt;John Maynard Keynes&lt;/a&gt;. Elle a pourtant profondément transformé la philosophie politique du XXe siècle, en redéfinissant le rôle de l’État face au marché. Figure de Cambridge et du groupe de Bloomsbury, Keynes avait déjà dénoncé en 1919 les conséquences économiques désastreuses du traité de Versailles.&lt;/p&gt; &lt;p&gt;Son œuvre majeure, la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9orie_g%C3%A9n%C3%A9rale_de_l%27emploi%2C_de_l%27int%C3%A9r%C3%AAt_et_de_la_monnaie" title=" Wikipedia"&gt;&lt;em&gt;Théorie générale de l’emploi, de l’intérêt et de la monnaie&lt;/em&gt;&lt;/a&gt; (1936), répond à la Grande Dépression. Contre les économistes classiques, pour qui les marchés s’équilibrent d’eux-mêmes et le chômage n’est que passager, Keynes montre qu’une économie peut rester durablement bloquée dans le chômage de masse, parce que la demande globale, consommation et investissement, est insuffisante. Dans l’incertitude, les entrepreneurs, mus par leurs « esprits animaux », cessent d’investir, et les ménages épargnent : chacun agit raisonnablement, mais tous ensemble aggravent la crise. L’État doit alors relancer l’activité par la dépense publique, les grands travaux et la baisse des taux d’intérêt, quitte à accepter un déficit, car chaque dépense en entraîne d’autres : c’est l’effet « multiplicateur ». « À long terme, nous serons tous morts », répond-il à ceux qui attendent que le marché se corrige seul.&lt;/p&gt; &lt;p&gt;Formalisé dès 1937 par John Hicks, le keynésianisme inspire les politiques des Trente Glorieuses, l’État-providence et les &lt;a href="https://fr.wikipedia.org/wiki/Accords_de_Bretton_Woods" title=" Wikipedia"&gt;accords de Bretton Woods&lt;/a&gt;, que Keynes négocie en 1944. Contesté dans les années 1970 par le monétarisme de Milton Friedman, il fait un retour remarqué lors des crises de 2008 et de 2020.&lt;/p&gt;  &lt;audio controls title="Keynésianisme : l’héritage de la discorde par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10081-12.11.2020-ITEMA_22481657-2020C29629S0317.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F131" s="11" t="s">
         <v>734</v>
@@ -9546,8 +9564,10 @@
       <c r="D165" s="15" t="s">
         <v>913</v>
       </c>
-      <c r="E165" s="16" t="s">
-        <v>914</v>
+      <c r="E165" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Object-oriented_ontology#:~:text=Object-oriented_ontology_holds_that,at_any_specific_spatiotemporal_location."  style="color:#d35400"  title=" Wikipedia"&gt;L'Ontologie Orientée Objet&lt;/a&gt;, ou « OOO », est un courant de la philosophie contemporaine né au début des années 2000 autour du philosophe américain &lt;a href="https://fr.wikipedia.org/wiki/Graham_Harman" title=" Wikipedia"&gt;Graham Harman&lt;/a&gt;, dont le livre &lt;em&gt;Tool-Being&lt;/em&gt; (2002) en pose les bases. Elle appartient à la mouvance plus large du &lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9alisme_sp%C3%A9culatif" title=" Wikipedia"&gt;réalisme spéculatif&lt;/a&gt;, qui veut rompre avec ce que Quentin Meillassoux appelle le « corrélationnisme » : l’idée, dominante depuis Kant, que nous ne pouvons jamais connaître les choses en elles-mêmes, mais seulement dans leur rapport à nous.&lt;/p&gt; &lt;p&gt;L’OOO propose une ontologie « plate » : tous les objets, humains ou non, naturels ou artificiels, réels ou imaginaires, un caillou, une tempête, une entreprise ou un personnage de roman, ont le même statut d’êtres. L’humain n’est plus au centre. Partant d’une lecture originale de Heidegger et de son analyse de l’outil, Harman soutient que tout objet est « en retrait » : il ne s’épuise jamais dans ses relations, ni dans la perception que nous en avons, ni dans son utilité, ni même dans ses effets sur les autres objets. Le feu qui brûle le coton n’en touche que certaines qualités. Les objets n’interagissent donc jamais directement, mais de manière indirecte, « vicariante » : le monde est fait d’objets qui se dérobent les uns aux autres.&lt;/p&gt; &lt;p&gt;Autour de Harman se rassemblent des penseurs comme Levi Bryant, Ian Bogost ou &lt;a href="https://fr.wikipedia.org/wiki/Timothy_Morton" title=" Wikipedia"&gt;Timothy Morton&lt;/a&gt;, qui forge la notion d’« hyperobjets » pour désigner des réalités si vastes, comme le réchauffement climatique, qu’on ne peut jamais les saisir d’un seul regard. Critiquée par certains comme une métaphysique sans politique, l’OOO a eu une grande influence dans l’art contemporain, l’architecture et la pensée écologique.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F165" s="14" t="s">
         <v>915</v>

</xml_diff>

<commit_message>
Courants, textes lot 2 : Silhak, Martinisme, Donghak, Anarcho-syndicalisme, Patristique, Herméneutique juive, Vitalisme, Saint-Simonisme, Hésychasme, Théisme
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -4874,8 +4874,10 @@
       <c r="D29" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="E29" s="16" t="s">
-        <v>169</v>
+      <c r="E29" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Patristique"  style="color:#d35400"  title=" Wikipedia"&gt;La Patristique&lt;/a&gt; désigne la pensée des Pères de l’Église, ces écrivains chrétiens des premiers siècles, du IIe au VIIIe siècle environ, dont l’autorité a fixé la doctrine chrétienne. Évêques, moines ou professeurs, ils écrivent en grec ou en latin dans un monde imprégné de philosophie grecque, et doivent à la fois défendre leur foi contre les païens, combattre les hérésies et expliquer la Bible. Ils empruntent pour cela les outils de la philosophie, surtout du platonisme et du stoïcisme, au point de présenter le christianisme comme la « vraie philosophie ».&lt;/p&gt; &lt;p&gt;Au IIe siècle, Justin, philosophe converti, voit dans la raison des Grecs une semence du Verbe divin, tandis que Tertullien demande : « Qu’y a-t-il de commun entre Athènes et Jérusalem ? » À Alexandrie, Clément et Origène bâtissent une théologie savante nourrie de Platon. Au IVe siècle, âge d’or des Pères, les conciles de Nicée (325) puis de Chalcédoine (451) définissent la Trinité et l’incarnation ; en Orient brillent Basile de Césarée, Grégoire de Nysse et Jean Chrysostome, en Occident Ambroise de Milan, Jérôme et surtout &lt;a href="https://fr.wikipedia.org/wiki/Augustin_d%27Hippone" title=" Wikipedia"&gt;Augustin d’Hippone&lt;/a&gt; (354-430), dont les &lt;em&gt;Confessions&lt;/em&gt; et &lt;em&gt;La Cité de Dieu&lt;/em&gt; marquent tout le Moyen Âge. Les Pères pensent la création à partir de rien, contre l’éternité du monde des Grecs, la liberté et le mal, le temps, la personne, et le rapport entre la foi et la raison : « Crois pour comprendre », dit Augustin.&lt;/p&gt; &lt;p&gt;La période s’achève avec Isidore de Séville en Occident et Jean Damascène en Orient. La patristique transmet au Moyen Âge une part de la philosophie antique et prépare la scolastique.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F29" s="14" t="s">
         <v>170</v>
@@ -5760,8 +5762,10 @@
       <c r="D55" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="E55" s="13" t="s">
-        <v>313</v>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9isme"  title=" Wikipedia"&gt;Le Théisme&lt;/a&gt; est la doctrine qui affirme l’existence d’un Dieu personnel et unique, créateur du monde, qui continue d’agir en lui. Le mot, apparu en anglais au XVIIe siècle, s’oppose à l’athéisme, qui nie l’existence de Dieu, et au panthéisme, qui confond Dieu et la nature, comme chez Spinoza. Il se distingue aussi du déisme : le Dieu des déistes, connu par la seule raison, a créé le monde comme un horloger, puis le laisse suivre ses lois, tandis que celui des théistes intervient par sa providence, entend les prières et se révèle aux humains.&lt;/p&gt; &lt;p&gt;Le théisme est la conception de Dieu des trois monothéismes, judaïsme, christianisme et islam, mais aussi une position philosophique, qui veut démontrer l’existence de Dieu par la raison. L’&lt;a href="https://fr.wikipedia.org/wiki/Argument_ontologique" title=" Wikipedia"&gt;argument ontologique&lt;/a&gt; d’Anselme de Cantorbéry, repris par Descartes, part de l’idée d’un être parfait ; les « cinq voies » de Thomas d’Aquin remontent des effets à une cause première ; l’argument du dessein, popularisé par William Paley en 1802, voit dans l’ordre du monde la marque d’un créateur intelligent. Voltaire décrit le théiste comme un homme persuadé de l’existence d’un Être suprême « aussi bon que puissant ». La grande objection reste le &lt;a href="https://fr.wikipedia.org/wiki/Probl%C3%A8me_du_mal" title=" Wikipedia"&gt;problème du mal&lt;/a&gt; : si Dieu est tout-puissant et bon, pourquoi la souffrance ? Leibniz y répond par sa &lt;em&gt;Théodicée&lt;/em&gt; (1710).&lt;/p&gt; &lt;p&gt;Hume et Kant ont critiqué ces preuves, mais le théisme connaît un renouveau dans la philosophie analytique depuis les années 1960, avec Alvin Plantinga et Richard Swinburne.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F55" s="11" t="s">
         <v>314</v>
@@ -6441,8 +6445,10 @@
       <c r="D74" s="12" t="s">
         <v>415</v>
       </c>
-      <c r="E74" s="26" t="s">
-        <v>416</v>
+      <c r="E74" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Vitalisme"  title=" Wikipedia"&gt;Le Vitalisme&lt;/a&gt; est une doctrine philosophique et médicale selon laquelle la vie ne s’explique pas seulement par les lois de la physique et de la chimie : les êtres vivants seraient animés par un principe propre, une « force vitale », qui les distingue de la matière inerte. Il s’oppose au mécanisme de Descartes, pour qui l’animal n’est qu’une machine, plus compliquée qu’une horloge. Le vivant, au contraire, se développe, se répare, se reproduit et résiste à sa propre destruction ; en lui, c’est le tout qui commande aux parties.&lt;/p&gt; &lt;p&gt;L’idée remonte à Aristote, pour qui l’âme est le principe qui organise le corps vivant. Le vitalisme moderne naît au XVIIIe siècle à l’école de médecine de Montpellier, avec Théophile de Bordeu puis Paul-Joseph Barthez, qui parle en 1778 d’un « principe vital » distinct à la fois de l’âme et du corps. &lt;a href="https://fr.wikipedia.org/wiki/Xavier_Bichat" title=" Wikipedia"&gt;Xavier Bichat&lt;/a&gt; définit la vie comme « l’ensemble des fonctions qui résistent à la mort ». Au XIXe siècle, la chimie l’affaiblit : en 1828, Friedrich Wöhler fabrique en laboratoire l’urée, qu’on croyait réservée aux êtres vivants. Le biologiste Hans Driesch le relance pourtant vers 1900 sous le nom d’« entéléchie ». En 1907, dans &lt;em&gt;L’Évolution créatrice&lt;/em&gt;, &lt;a href="https://fr.wikipedia.org/wiki/Henri_Bergson" title=" Wikipedia"&gt;Henri Bergson&lt;/a&gt; en donne une version philosophique avec l’« élan vital », poussée créatrice et imprévisible qui traverse toute l’évolution.&lt;/p&gt; &lt;p&gt;Rejeté par la biologie moderne, le vitalisme a été réhabilité comme attitude par &lt;a href="https://fr.wikipedia.org/wiki/Georges_Canguilhem" title=" Wikipedia"&gt;Georges Canguilhem&lt;/a&gt;, qui y voit l’exigence de respecter l’originalité du vivant face au réductionnisme.&lt;/p&gt;  &lt;audio controls title="Qu’est ce que le vitalisme par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-02.04.2013-ITEMA_20465724-2013C12410S0092-NET_FC_A749DB22-ACB1-4BF2-9A16-61DE07750CA9-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F74" s="11" t="s">
         <v>417</v>
@@ -6645,8 +6651,10 @@
       <c r="D80" s="12" t="s">
         <v>449</v>
       </c>
-      <c r="E80" s="13" t="s">
-        <v>450</v>
+      <c r="E80" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Saint-simonisme"  title=" Wikipedia"&gt;Le Saint-simonisme&lt;/a&gt; est un courant de pensée politique, économique et religieux né des idées de Claude-Henri de Rouvroy, comte de &lt;a href="https://fr.wikipedia.org/wiki/Claude-Henri_de_Rouvroy_de_Saint-Simon" title=" Wikipedia"&gt;Saint-Simon&lt;/a&gt; (1760-1825), et développé après sa mort par ses disciples. Aristocrate ruiné, ancien combattant de la guerre d’indépendance américaine, Saint-Simon voit naître la révolution industrielle et en tire une conviction : la société doit être dirigée par ceux qui produisent, les « industriels », savants, ingénieurs, banquiers, artisans et ouvriers, et non plus par les nobles, les militaires et les rentiers, qu’il appelle les « oisifs ».&lt;/p&gt; &lt;p&gt;Dans sa célèbre « parabole » de 1819, il montre que la France perdrait tout si disparaissaient ses trois mille meilleurs savants, artistes et producteurs, mais rien si mouraient les princes et les grands dignitaires. La politique doit devenir une science de la production, qui remplace le gouvernement des hommes par l’administration des choses. Dans le &lt;em&gt;Nouveau Christianisme&lt;/em&gt; (1825), il propose une religion sans dogme, tournée vers l’amélioration du sort de « la classe la plus pauvre ». Ses disciples Saint-Amand Bazard et Prosper Enfantin en font une doctrine : « à chacun selon sa capacité, à chaque capacité selon ses œuvres », suppression de l’héritage, crédit organisé, émancipation des femmes. Enfantin fonde même en 1832 une communauté à Ménilmontant, vite condamnée par la justice.&lt;/p&gt; &lt;p&gt;Les saint-simoniens ont surtout bâti la France industrielle : chemins de fer, banques comme le Crédit mobilier des frères Pereire, libre-échange avec Michel Chevalier, projet du &lt;a href="https://fr.wikipedia.org/wiki/Canal_de_Suez" title=" Wikipedia"&gt;canal de Suez&lt;/a&gt;. Auguste Comte, secrétaire de Saint-Simon, et Marx leur doivent beaucoup.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F80" s="11" t="s">
         <v>451</v>
@@ -7791,8 +7799,10 @@
       <c r="D112" s="17" t="s">
         <v>629</v>
       </c>
-      <c r="E112" s="3" t="s">
-        <v>630</v>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Anarcho-syndicalisme" title=" Wikipedia"&gt;L’Anarcho-syndicalisme&lt;/a&gt; est un courant politique né en France à la fin du XIXe siècle, qui fait du syndicat ouvrier, et non du parti ou de l’État, l’instrument de la révolution et la base de la société future. Il hérite de l’anarchisme de Proudhon et de Bakounine le rejet de l’État, même socialiste : toute prise du pouvoir centralisée, fût-ce au nom du prolétariat, reproduit selon lui la domination qu’elle prétend abolir. Les travailleurs doivent donc s’émanciper eux-mêmes, sur leur lieu de travail.&lt;/p&gt; &lt;p&gt;Dans les années 1890, des anarchistes français entrent dans les syndicats. &lt;a href="https://fr.wikipedia.org/wiki/Fernand_Pelloutier" title=" Wikipedia"&gt;Fernand Pelloutier&lt;/a&gt; anime les Bourses du travail, à la fois lieux d’entraide, d’éducation et d’organisation, et Émile Pouget défend l’« action directe » : grève, boycott, sabotage, sans passer par les élus. La CGT, fondée en 1895, adopte en 1906 la &lt;a href="https://fr.wikipedia.org/wiki/Charte_d%27Amiens" title=" Wikipedia"&gt;Charte d’Amiens&lt;/a&gt;, qui affirme l’indépendance du syndicat envers les partis et fait de la grève générale l’arme de l’émancipation ; Georges Sorel y voit un « mythe » qui mobilise les masses. Le syndicat prépare dès aujourd’hui la gestion de la production par les producteurs eux-mêmes : la société future sera une fédération libre de syndicats et de communes autogérées, sans patrons ni État.&lt;/p&gt; &lt;p&gt;Le courant gagne l’Italie, l’Argentine, les États-Unis et surtout l’Espagne, où la CNT, fondée en 1910, dépasse le million de membres. Pendant la guerre civile, en 1936, elle organise l’autogestion des usines et des terres en Catalogne et en Aragon. Rudolf Rocker en a fait la théorie, et Noam Chomsky s’en réclame.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F112" s="1" t="s">
         <v>631</v>

</xml_diff>

<commit_message>
Courants, textes lot 3 : Biopolitique, Consciencisme, Philosophie vietnamienne, Minjung, Pythagorisme, Réalisme scientifique, Confucianisme, Social-démocratie, Logique paraconsistante, Symbolisme ; Shuruppak retouché
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -4063,8 +4063,10 @@
       <c r="D6" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>30</v>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89cole_pythagoricienne" title=" Wikipedia"&gt;Le Pythagorisme&lt;/a&gt; est l’école philosophique et religieuse fondée par Pythagore (vers 570-495 av. J.-C.). Né à Samos, en Ionie, il s’installe vers 530 à Crotone, en Italie du Sud, où il réunit une communauté d’hommes et de femmes liés par le secret, la vie commune et des règles strictes. Les pythagoriciens ont exercé une influence politique dans les cités grecques d’Italie, avant d’en être chassés par des révoltes vers le milieu du Ve siècle.&lt;/p&gt; &lt;p&gt;Leur thèse centrale est que « tout est nombre » : le nombre est le principe de toutes choses. Ils l’ont découvert dans la musique, où les accords harmonieux, l’octave, la quinte et la quarte, correspondent à des rapports simples entre les longueurs des cordes : 2/1, 3/2, 4/3. Le cosmos tout entier serait ainsi ordonné par des proportions mathématiques, jusqu’à l’« harmonie des sphères » que produiraient les astres en tournant. La tétraktys, triangle de dix points formé par 1 + 2 + 3 + 4, est leur symbole sacré. On leur attribue aussi la découverte, troublante pour eux, de grandeurs « irrationnelles », comme la diagonale du carré. Le pythagorisme est enfin une voie de salut : l’âme est immortelle et passe de corps en corps, y compris animaux, c’est la métempsycose ; on la purifie par une vie ascétique, des interdits alimentaires, la musique et l’étude. Parmi ses figures, on compte &lt;a href="https://fr.wikipedia.org/wiki/Philolaos_de_Crotone" title=" Wikipedia"&gt;Philolaos&lt;/a&gt;, qui fait tourner la Terre autour d’un feu central, Archytas de Tarente et &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9ano_%28pythagoricienne%29" title=" Wikipedia"&gt;Théano&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Platon, ami d’Archytas, reprend l’idée d’une réalité mathématique supérieure au monde sensible. Le néopythagorisme renaît à Rome, et Kepler comme Galilée y puisent la conviction que la nature est écrite en langage mathématique.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F6" s="1" t="s">
         <v>31</v>
@@ -7838,8 +7840,10 @@
       <c r="D113" s="17" t="s">
         <v>634</v>
       </c>
-      <c r="E113" s="3" t="s">
-        <v>635</v>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Social-d%C3%A9mocratie" title=" Wikipedia"&gt;La Social-démocratie&lt;/a&gt; est un courant politique qui veut atteindre les buts du socialisme, l’égalité et la justice sociale, par des réformes progressives et par la démocratie parlementaire plutôt que par la révolution. À l’origine, au XIXe siècle, le mot désigne les partis ouvriers marxistes, comme le Parti social-démocrate allemand (SPD). Son sens actuel naît d’une rupture au sein de ce parti, avec &lt;a href="https://fr.wikipedia.org/wiki/Eduard_Bernstein" title=" Wikipedia"&gt;Eduard Bernstein&lt;/a&gt; et ses &lt;em&gt;Présupposés du socialisme&lt;/em&gt; (1899).&lt;/p&gt; &lt;p&gt;Bernstein constate que le capitalisme ne s’effondre pas comme Marx l’avait annoncé : les classes moyennes ne disparaissent pas, la condition ouvrière s’améliore, et les syndicats et le suffrage universel permettent de conquérir des droits. « Le but final n’est rien, le mouvement est tout », écrit-il. Ce « révisionnisme » provoque une vive controverse dans la IIe Internationale : Karl Kautsky le combat et &lt;a href="https://fr.wikipedia.org/wiki/Rosa_Luxemburg" title=" Wikipedia"&gt;Rosa Luxemburg&lt;/a&gt; lui répond par &lt;em&gt;Réforme sociale ou révolution ?&lt;/em&gt; (1899). Après la Révolution russe de 1917, la séparation devient définitive entre les communistes et les sociaux-démocrates, qui acceptent l’économie de marché et le cadre de l’État libéral tout en voulant les corriger : impôt progressif, sécurité sociale, droit du travail, négociation collective, services publics.&lt;/p&gt; &lt;p&gt;Ce courant a façonné l’Europe du XXe siècle, du « foyer du peuple » suédois des années 1930 aux États-providence de l’après-guerre. En 1959, le SPD renonce officiellement au marxisme. Dans les années 1990, la « troisième voie » de Tony Blair et Gerhard Schröder le rapproche du libéralisme.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F113" s="1" t="s">
         <v>636</v>
@@ -9183,8 +9187,10 @@
       <c r="D153" s="17" t="s">
         <v>849</v>
       </c>
-      <c r="E153" s="3" t="s">
-        <v>850</v>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9alisme_scientifique" title=" Wikipedia"&gt;Le Réalisme scientifique&lt;/a&gt; est la thèse selon laquelle nos meilleures théories scientifiques décrivent, au moins approximativement, le monde tel qu’il est réellement, y compris ce que nous ne pouvons pas observer : les électrons, les gènes, les champs ou les trous noirs. Il s’oppose à l’instrumentalisme, défendu par Ernst Mach ou Pierre Duhem, pour qui les théories ne sont que des outils commodes pour prédire les phénomènes, et qui refusaient de croire à la réalité des atomes.&lt;/p&gt; &lt;p&gt;Son argument le plus célèbre est formulé en 1975 par &lt;a href="https://fr.wikipedia.org/wiki/Hilary_Putnam" title=" Wikipedia"&gt;Hilary Putnam&lt;/a&gt; : le réalisme est « la seule philosophie qui ne fasse pas du succès de la science un miracle ». Si les théories permettent de prédire des phénomènes inconnus, comme l’existence d’une planète ou d’une particule, c’est qu’elles saisissent quelque chose du réel. En 1980, &lt;a href="https://fr.wikipedia.org/wiki/Bas_van_Fraassen" title=" Wikipedia"&gt;Bas van Fraassen&lt;/a&gt; lui oppose un « empirisme constructif » : une théorie n’a pas besoin d’être vraie, il suffit qu’elle sauve les phénomènes observables. En 1981, Larry Laudan oppose l’argument dit de la « méta-induction pessimiste » : l’histoire des sciences est un cimetière de théories qui marchaient bien et se sont révélées fausses, comme l’éther ou le phlogistique ; pourquoi les nôtres échapperaient-elles à ce sort ?&lt;/p&gt; &lt;p&gt;Pour répondre, des versions plus modestes sont nées. Le réalisme structural de John Worrall soutient que ce qui survit aux révolutions scientifiques, ce sont les structures mathématiques des théories. Le réalisme des entités de Ian Hacking croit aux électrons parce qu’on sait s’en servir : « si on peut les projeter, ils sont réels ».&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F153" s="1" t="s">
         <v>851</v>
@@ -9215,8 +9221,10 @@
       <c r="D154" s="17" t="s">
         <v>855</v>
       </c>
-      <c r="E154" s="3" t="s">
-        <v>856</v>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Biopolitique" style="color:#d35400" title=" Wikipedia"&gt;La Biopolitique&lt;/a&gt; désigne la manière dont le pouvoir moderne prend en charge la vie biologique des populations : la natalité, la santé, l’hygiène, la sexualité, la durée de vie. Le concept est forgé par &lt;a href="https://fr.wikipedia.org/wiki/Michel_Foucault" title=" Wikipedia"&gt;Michel Foucault&lt;/a&gt; au milieu des années 1970, notamment dans &lt;em&gt;La Volonté de savoir&lt;/em&gt; (1976) et dans ses cours au Collège de France. Pendant des siècles, explique-t-il, le souverain exerçait surtout un droit de mort : il pouvait « faire mourir et laisser vivre ». À partir du XVIIIe siècle, le pouvoir cherche au contraire à « faire vivre et laisser mourir ».&lt;/p&gt; &lt;p&gt;Ce « biopouvoir » a deux faces. La première, née aux XVIIe et XVIIIe siècles, est la discipline des corps individuels, à l’école, à l’armée, à l’usine ou en prison, qu’il décrit dans &lt;em&gt;Surveiller et punir&lt;/em&gt; (1975). La seconde, la biopolitique proprement dite, vise l’espèce humaine prise en masse : elle mesure, compte et régule grâce aux statistiques, à la démographie, à la médecine sociale et aux assurances. Le pouvoir ne se contente plus d’interdire : il gère, il normalise, il protège. Foucault montre aussi le revers de ce souci de la vie : le racisme d’État, qui trie entre ceux qu’il faut faire vivre et ceux qu’on peut laisser mourir, au nom de la santé de la population.&lt;/p&gt; &lt;p&gt;Le philosophe italien &lt;a href="https://fr.wikipedia.org/wiki/Giorgio_Agamben" title=" Wikipedia"&gt;Giorgio Agamben&lt;/a&gt; prolonge cette analyse dans &lt;em&gt;Homo sacer&lt;/em&gt; (1995) : il distingue la « vie nue », simple fait de vivre, de la vie politique, et voit dans l’état d’exception et dans le camp le paradigme du pouvoir moderne. Roberto Esposito oppose la logique de l’immunité à celle de la communauté. La pandémie de 2020 a relancé ces débats.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F154" s="1" t="s">
         <v>857</v>

</xml_diff>

<commit_message>
Courants, textes lot 4 ; « Particuliarisme » devient « Particularisme » (301) ; familles des courants : colonnes Nature, Famille, Issu_de (données, vérifications, éditeur)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -3888,7 +3888,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N1048576"/>
+  <dimension ref="A1:Q1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -3979,6 +3979,21 @@
           <t xml:space="preserve">Traditions</t>
         </is>
       </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nature</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Famille</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Issu_de</t>
+        </is>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="198" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="n">
@@ -4018,6 +4033,16 @@
           <t xml:space="preserve">orient-ancien;asie-est</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
+        </is>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="195.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="n">
@@ -4052,6 +4077,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les débuts de la philosophie grecque</t>
+        </is>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="205.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
@@ -4084,6 +4119,21 @@
       <c r="M6" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les débuts de la philosophie grecque</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Présocratique</t>
         </is>
       </c>
     </row>
@@ -4125,6 +4175,16 @@
           <t xml:space="preserve">occident;orient-ancien</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="212.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="n">
@@ -4159,6 +4219,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les débuts de la philosophie grecque</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Présocratique</t>
+        </is>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="153.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="n">
@@ -4193,6 +4268,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les débuts de la philosophie grecque</t>
+        </is>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
@@ -4227,6 +4312,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
+        </is>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
@@ -4239,8 +4334,10 @@
       <c r="D11" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>60</v>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Solipsisme" title=" Wikipedia"&gt;Le Solipsisme&lt;/a&gt;, du latin &lt;em&gt;solus&lt;/em&gt;, « seul », et &lt;em&gt;ipse&lt;/em&gt;, « soi-même », est la thèse selon laquelle seul existe, ou du moins seul peut être connu avec certitude, mon propre esprit. Le monde extérieur et les autres personnes ne me sont donnés que par mes perceptions : rien ne garantit qu’ils existent indépendamment de moi. On distingue un solipsisme métaphysique, qui nie l’existence de ce qui n’est pas moi, et un solipsisme épistémologique, qui affirme seulement qu’on ne peut la prouver.&lt;/p&gt; &lt;p&gt;Presque aucun philosophe ne s’est déclaré solipsiste : la position sert plutôt d’épreuve. Dans l’Antiquité, le sophiste &lt;a href="https://fr.wikipedia.org/wiki/Gorgias" title=" Wikipedia"&gt;Gorgias&lt;/a&gt; soutenait que rien n’existe, que si quelque chose existait on ne pourrait le connaître, et que si on le connaissait on ne pourrait le communiquer. &lt;a href="https://fr.wikipedia.org/wiki/Ren%C3%A9_Descartes" title=" Wikipedia"&gt;Descartes&lt;/a&gt; traverse un moment proche du solipsisme : après avoir douté de tout, il ne trouve d’abord qu’une certitude, celle de sa propre pensée, « je pense, donc je suis » (&lt;em&gt;Discours de la méthode&lt;/em&gt;, 1637). Mais il en sort en prouvant l’existence de Dieu, garant de celle du monde. Berkeley, pour qui être, c’est être perçu, n’est pas davantage solipsiste : il admet l’existence des autres esprits et de Dieu.&lt;/p&gt; &lt;p&gt;Le problème reparaît au XXe siècle. Husserl consacre la cinquième de ses &lt;em&gt;Méditations cartésiennes&lt;/em&gt; (1931) à montrer comment autrui se donne à ma conscience, et Sartre nomme « écueil du solipsisme » la difficulté de prouver l’existence d’autrui. Wittgenstein, par sa critique d’un « langage privé », suggère que le solipsiste ne peut même pas formuler sa thèse, puisque tout langage est partagé.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F11" s="11" t="s">
         <v>61</v>
@@ -4261,6 +4358,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que pouvons-nous connaître ?</t>
+        </is>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="n">
@@ -4295,6 +4402,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
+        </is>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="n">
@@ -4331,6 +4448,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socrate et ses héritiers</t>
+        </is>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="n">
@@ -4371,6 +4498,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socrate et ses héritiers</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socratisme;Pythagorisme</t>
+        </is>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="n">
@@ -4405,6 +4547,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les débuts de la philosophie grecque</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Éléatisme</t>
+        </is>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="186" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="n">
@@ -4417,8 +4574,10 @@
       <c r="D16" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="E16" s="16" t="s">
-        <v>91</v>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Mat%C3%A9rialisme"  style="color:#d35400"  title=" Wikipedia"&gt;Le Matérialisme&lt;/a&gt; est la doctrine selon laquelle la matière est la seule réalité : tout ce qui existe, y compris la pensée, les sentiments et la conscience, est matériel ou dépend de processus matériels. Il s’oppose au spiritualisme et à l’idéalisme, qui accordent à l’esprit une existence propre ou première. Le mot date de la fin du XVIIe siècle, mais l’idée remonte aux présocratiques grecs.&lt;/p&gt; &lt;p&gt;Au Ve siècle av. J.-C., Leucippe et &lt;a href="https://fr.wikipedia.org/wiki/D%C3%A9mocrite" title=" Wikipedia"&gt;Démocrite&lt;/a&gt; affirment que tout est fait d’atomes, corps indivisibles en mouvement dans le vide, dont les assemblages expliquent la naissance et la disparition des choses, sans intervention divine. &lt;a href="https://fr.wikipedia.org/wiki/%C3%89picure" title=" Wikipedia"&gt;Épicure&lt;/a&gt; reprend cet atomisme pour délivrer les hommes de la peur des dieux et de la mort, et Lucrèce l’expose à Rome dans &lt;em&gt;De la nature des choses&lt;/em&gt;. Après une longue éclipse, le matérialisme renaît à l’époque moderne avec Hobbes, puis au XVIIIe siècle avec La Mettrie, auteur de &lt;em&gt;L’Homme-machine&lt;/em&gt; (1747), d’Holbach et Diderot, souvent liés à l’athéisme.&lt;/p&gt; &lt;p&gt;Au XIXe siècle, Marx et Engels développent une conception matérialiste de l’histoire : ce sont les conditions matérielles de la production qui expliquent les idées et les institutions ; leurs successeurs parleront de « matérialisme dialectique ». Aujourd’hui, en philosophie de l’esprit, le physicalisme soutient que les états mentaux sont des états du cerveau. Ses adversaires objectent qu’il peine à rendre compte de l’expérience subjective, de ce que cela fait d’être conscient : c’est le « problème difficile » de la conscience.&lt;/p&gt;  &lt;audio controls title="Qu'est ce que le Matérialisme ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-30.09.2016-ITEMA_21090944-2.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F16" s="14" t="s">
         <v>92</v>
@@ -4444,6 +4603,16 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matière ou esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="235.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="n">
@@ -4478,6 +4647,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que pouvons-nous connaître ?</t>
+        </is>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="257.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="n">
@@ -4512,6 +4691,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matière ou esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="n">
@@ -4546,6 +4735,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socrate et ses héritiers</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Platonisme</t>
+        </is>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="n">
@@ -4582,6 +4786,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socrate et ses héritiers</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socratisme</t>
+        </is>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="n">
@@ -4616,6 +4835,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socrate et ses héritiers</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socratisme</t>
+        </is>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="296.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="n">
@@ -4650,6 +4884,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Écoles hellénistiques et romaines</t>
+        </is>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="217.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="n">
@@ -4684,6 +4928,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Écoles hellénistiques et romaines</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atomisme;Cyrénaïsme</t>
+        </is>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="219" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="n">
@@ -4718,6 +4977,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Écoles hellénistiques et romaines</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cynisme</t>
+        </is>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="n">
@@ -4752,6 +5026,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sommes-nous libres ?</t>
+        </is>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="n">
@@ -4791,6 +5075,21 @@
           <t xml:space="preserve">islam-juif</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Écoles hellénistiques et romaines</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Platonisme</t>
+        </is>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="n">
@@ -4830,6 +5129,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ésotérismes et gnoses</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Platonisme</t>
+        </is>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="n">
@@ -4864,6 +5178,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Écoles hellénistiques et romaines</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Platonisme;Stoïcisme</t>
+        </is>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="n">
@@ -4900,6 +5229,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Platonisme;Stoïcisme</t>
+        </is>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="n">
@@ -4934,6 +5278,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patristique;Néoplatonisme</t>
+        </is>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="n">
@@ -4966,6 +5325,21 @@
       <c r="M31" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patristique</t>
         </is>
       </c>
     </row>
@@ -5000,6 +5374,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Augustinisme;Aristotélisme</t>
+        </is>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="n">
@@ -5034,6 +5423,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Le réel est-il un ou multiple ?</t>
+        </is>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="n">
@@ -5068,6 +5467,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scolastique</t>
+        </is>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="n">
@@ -5102,6 +5516,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scolastique</t>
+        </is>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="n">
@@ -5134,6 +5563,21 @@
       <c r="M36" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scolastique;Aristotélisme</t>
         </is>
       </c>
     </row>
@@ -5166,6 +5610,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scolastique</t>
+        </is>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="n">
@@ -5196,6 +5655,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scolastique</t>
+        </is>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="n">
@@ -5235,6 +5709,21 @@
           <t xml:space="preserve">islam-juif</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Falsafa;Aristotélisme</t>
+        </is>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="n">
@@ -5269,6 +5758,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matière ou esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="178.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="n">
@@ -5308,6 +5807,16 @@
           <t xml:space="preserve">sud;russe;inde</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Renaissance et Réformes</t>
+        </is>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="203.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="n">
@@ -5337,6 +5846,21 @@
       <c r="M42" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Renaissance et Réformes</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Augustinisme;Humanisme</t>
         </is>
       </c>
     </row>
@@ -5373,6 +5897,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Renaissance et Réformes</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Humanisme</t>
+        </is>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="208.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="n">
@@ -5407,6 +5946,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matière ou esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="14" t="n">
@@ -5441,6 +5990,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que pouvons-nous connaître ?</t>
+        </is>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="180.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="n">
@@ -5475,6 +6034,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Renaissance et Réformes</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Humanisme</t>
+        </is>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="n">
@@ -5509,6 +6083,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="253.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="n">
@@ -5543,6 +6127,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Humanisme</t>
+        </is>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="14" t="n">
@@ -5577,6 +6176,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
+        </is>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="165.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="n">
@@ -5616,6 +6225,16 @@
           <t xml:space="preserve">russe;sud</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matière ou esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="n">
@@ -5650,6 +6269,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée chrétienne moderne</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Augustinisme</t>
+        </is>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="140.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="11" t="n">
@@ -5684,6 +6318,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descartes et ses héritiers</t>
+        </is>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="168" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="14" t="n">
@@ -5718,6 +6362,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que pouvons-nous connaître ?</t>
+        </is>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="281.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="n">
@@ -5752,6 +6406,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sommes-nous libres ?</t>
+        </is>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="147" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="n">
@@ -5788,6 +6452,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
+        </is>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="250.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="14" t="n">
@@ -5822,6 +6496,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="228.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="14" t="n">
@@ -5856,6 +6540,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
+        </is>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="228.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="14" t="n">
@@ -5890,6 +6584,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sommes-nous libres ?</t>
+        </is>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="223.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="n">
@@ -5924,6 +6628,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sommes-nous libres ?</t>
+        </is>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="116.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="14" t="n">
@@ -5958,6 +6672,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descartes et ses héritiers</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cartésianisme</t>
+        </is>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="n">
@@ -5992,6 +6721,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
+        </is>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="259.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="14" t="n">
@@ -6031,6 +6770,21 @@
           <t xml:space="preserve">russe;sud</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contractualisme</t>
+        </is>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="204.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="n">
@@ -6065,6 +6819,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descartes et ses héritiers</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Empirisme</t>
+        </is>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="11" t="n">
@@ -6099,6 +6868,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment les sociétés pensent-elles la nature ? (Descola)</t>
+        </is>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="n">
@@ -6133,6 +6912,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment les sociétés pensent-elles la nature ? (Descola)</t>
+        </is>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="117" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="n">
@@ -6167,6 +6956,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment les sociétés pensent-elles la nature ? (Descola)</t>
+        </is>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="n">
@@ -6201,6 +7000,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment les sociétés pensent-elles la nature ? (Descola)</t>
+        </is>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="11" t="n">
@@ -6235,6 +7044,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Le réel est-il un ou multiple ?</t>
+        </is>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="266.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="n">
@@ -6267,6 +7086,16 @@
       <c r="M69" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que pouvons-nous connaître ?</t>
         </is>
       </c>
     </row>
@@ -6321,6 +7150,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cartésianisme;Empirisme</t>
+        </is>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="162.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="14" t="n">
@@ -6362,6 +7206,16 @@
           <t xml:space="preserve">russe;sud</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Le réel est-il un ou multiple ?</t>
+        </is>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="11" t="n">
@@ -6396,6 +7250,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libéralisme</t>
+        </is>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="14" t="n">
@@ -6435,6 +7304,16 @@
           <t xml:space="preserve">islam-juif</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anticolonialisme et décolonisation</t>
+        </is>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="11" t="n">
@@ -6471,6 +7350,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matière ou esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="14" t="n">
@@ -6505,6 +7394,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand et romantisme</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rationalisme;Empirisme</t>
+        </is>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="182.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="14" t="n">
@@ -6539,6 +7443,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que pouvons-nous connaître ?</t>
+        </is>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="n">
@@ -6573,6 +7487,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hédonisme</t>
+        </is>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="222" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="14" t="n">
@@ -6607,6 +7536,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
+        </is>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="195" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="n">
@@ -6641,6 +7580,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utilitarisme</t>
+        </is>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="222" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="11" t="n">
@@ -6677,6 +7631,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières</t>
+        </is>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="14" t="n">
@@ -6716,6 +7685,16 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="136.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="14" t="n">
@@ -6755,6 +7734,21 @@
           <t xml:space="preserve">asie-est</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières</t>
+        </is>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="151.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="n">
@@ -6790,6 +7784,21 @@
       <c r="N83" t="inlineStr">
         <is>
           <t xml:space="preserve">russe</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand et romantisme</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criticisme</t>
         </is>
       </c>
     </row>
@@ -6826,6 +7835,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand et romantisme</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand</t>
+        </is>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="n">
@@ -6860,6 +7884,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée chrétienne moderne</t>
+        </is>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="14" t="n">
@@ -6894,6 +7928,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Volonté, vie et soupçon</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand;Bouddhisme</t>
+        </is>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="n">
@@ -6933,6 +7982,21 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivismes</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saint-Simonisme</t>
+        </is>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="99" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="11" t="n">
@@ -6967,6 +8031,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand et romantisme</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Romantisme</t>
+        </is>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="14" t="n">
@@ -7001,6 +8080,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée chrétienne moderne</t>
+        </is>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="11" t="n">
@@ -7035,6 +8124,16 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="n">
@@ -7074,6 +8173,21 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jeunes hégéliens</t>
+        </is>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="11" t="n">
@@ -7110,6 +8224,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand et romantisme</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Romantisme;Idéalisme allemand</t>
+        </is>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="14" t="n">
@@ -7152,6 +8281,21 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phénoménologie, existence et herméneutique</t>
+        </is>
+      </c>
+      <c r="Q93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand</t>
+        </is>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="191.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="11" t="n">
@@ -7194,6 +8338,21 @@
           <t xml:space="preserve">russe;asie-est</t>
         </is>
       </c>
+      <c r="O94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jeunes hégéliens;Saint-Simonisme</t>
+        </is>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="n">
@@ -7224,6 +8383,16 @@
       <c r="M95" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
         </is>
       </c>
     </row>
@@ -7260,6 +8429,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée chrétienne moderne</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Occasionalisme</t>
+        </is>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="14" t="n">
@@ -7294,6 +8478,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qui existe vraiment ?</t>
+        </is>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="11" t="n">
@@ -7328,6 +8522,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce que l’esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="288" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="n">
@@ -7362,6 +8566,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivismes</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivisme</t>
+        </is>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="165.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="14" t="n">
@@ -7401,6 +8620,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Slavophiles, occidentalistes et nihilistes</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matérialisme</t>
+        </is>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="172.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="n">
@@ -7435,6 +8669,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libertarianisme</t>
+        </is>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="248.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="14" t="n">
@@ -7469,6 +8718,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
+        </is>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="189" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="n">
@@ -7481,8 +8740,10 @@
       <c r="D103" s="12" t="s">
         <v>582</v>
       </c>
-      <c r="E103" s="13" t="s">
-        <v>583</v>
+      <c r="E103" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/N%C3%A9okantisme"  title=" Wikipedia"&gt;Le Néo-kantisme&lt;/a&gt; est un vaste mouvement philosophique qui domine les universités allemandes des années 1870 à la Première Guerre mondiale. Face au déclin des grands systèmes idéalistes, celui de Hegel en tête, et à la montée d’un matérialisme scientifique sûr de lui, il prône un « retour à Kant » : en 1865, Otto Liebmann termine chaque chapitre de &lt;em&gt;Kant et les épigones&lt;/em&gt; par la formule « Il faut donc revenir à Kant ». Friedrich Albert Lange, avec son &lt;em&gt;Histoire du matérialisme&lt;/em&gt; (1866), ouvre aussi la voie.&lt;/p&gt; &lt;p&gt;Deux écoles se distinguent. L’école de Marbourg, avec &lt;a href="https://fr.wikipedia.org/wiki/Hermann_Cohen_%28philosophe%29" title=" Wikipedia"&gt;Hermann Cohen&lt;/a&gt;, Paul Natorp puis Ernst Cassirer, fait de la philosophie une théorie de la connaissance scientifique : elle cherche dans la physique mathématique les conditions qui rendent le savoir possible, et réinterprète la chose en soi comme une simple idée-limite, l’objet étant construit par la pensée plutôt que reçu. L’école de Bade, avec &lt;a href="https://fr.wikipedia.org/wiki/Wilhelm_Windelband" title=" Wikipedia"&gt;Wilhelm Windelband&lt;/a&gt; et Heinrich Rickert, s’attache aux valeurs, le vrai, le bien, le beau, et distingue les sciences de la nature, qui cherchent des lois, des sciences de la culture, comme l’histoire, qui s’intéressent à l’individuel.&lt;/p&gt; &lt;p&gt;Dans sa &lt;em&gt;Philosophie des formes symboliques&lt;/em&gt; (1923-1929), &lt;a href="https://fr.wikipedia.org/wiki/Ernst_Cassirer" title=" Wikipedia"&gt;Cassirer&lt;/a&gt; étend l’entreprise au langage, au mythe et à l’art : « la critique de la raison devient ainsi critique de la culture ». Après la guerre, le courant décline ; le débat de Davos qui oppose Cassirer à Heidegger en 1929 marque son effacement devant la phénoménologie. En France, Charles Renouvier avait développé un néocriticisme parallèle.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F103" s="11" t="s">
         <v>584</v>
@@ -7508,6 +8769,21 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand et romantisme</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criticisme</t>
+        </is>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="198" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="14" t="n">
@@ -7547,6 +8823,21 @@
           <t xml:space="preserve">sud</t>
         </is>
       </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Volonté, vie et soupçon</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pessimisme</t>
+        </is>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="208.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="n">
@@ -7581,6 +8872,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luttes et éthiques contemporaines</t>
+        </is>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="222.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="11" t="n">
@@ -7615,6 +8916,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce que l’esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="224.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="n">
@@ -7649,6 +8960,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qui existe vraiment ?</t>
+        </is>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="14" t="n">
@@ -7683,6 +9004,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie analytique et pragmatisme</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Empirisme</t>
+        </is>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="173.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="14" t="n">
@@ -7717,6 +9053,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Volonté, vie et soupçon</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Romantisme</t>
+        </is>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="150.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="14" t="n">
@@ -7751,6 +9102,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée chrétienne moderne</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thomisme</t>
+        </is>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="155.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="n">
@@ -7790,6 +9156,21 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie analytique et pragmatisme</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Empirisme</t>
+        </is>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="215.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="n">
@@ -7829,6 +9210,21 @@
           <t xml:space="preserve">russe</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anarchisme</t>
+        </is>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="n">
@@ -7861,6 +9257,21 @@
       <c r="M113" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marxisme</t>
         </is>
       </c>
     </row>
@@ -7902,6 +9313,21 @@
           <t xml:space="preserve">russe;sud;islam-juif</t>
         </is>
       </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phénoménologie, existence et herméneutique</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Romantisme</t>
+        </is>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="177.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="n">
@@ -7936,6 +9362,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qui existe vraiment ?</t>
+        </is>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="217.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="n">
@@ -7969,6 +9405,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Psychanalyse et sciences cognitives</t>
+        </is>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="175.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="n">
@@ -8001,6 +9447,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qu’une théorie scientifique ?</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pragmatisme</t>
+        </is>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="319.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="1" t="n">
@@ -8033,6 +9494,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qu’une théorie scientifique ?</t>
+        </is>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="n">
@@ -8064,6 +9535,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie analytique et pragmatisme</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Analytique</t>
+        </is>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="n">
@@ -8095,6 +9581,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Psychanalyse et sciences cognitives</t>
+        </is>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="190.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="n">
@@ -8124,6 +9620,21 @@
       <c r="M121" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Individualisme</t>
         </is>
       </c>
     </row>
@@ -8160,6 +9671,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phénoménologie, existence et herméneutique</t>
+        </is>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="204.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="n">
@@ -8194,6 +9715,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ésotérismes et gnoses</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théosophisme</t>
+        </is>
+      </c>
     </row>
     <row r="124" customFormat="false" ht="128.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="11" t="n">
@@ -8228,6 +9764,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
+      <c r="Q124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conservatisme</t>
+        </is>
+      </c>
     </row>
     <row r="125" customFormat="false" ht="290.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="n">
@@ -8262,6 +9813,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce que l’esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="290.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="11" t="n">
@@ -8296,6 +9857,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Psychanalyse et sciences cognitives</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Béhaviorisme</t>
+        </is>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="243" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="14" t="n">
@@ -8330,6 +9906,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivismes</t>
+        </is>
+      </c>
+      <c r="Q127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivisme;Analytique</t>
+        </is>
+      </c>
     </row>
     <row r="128" customFormat="false" ht="141.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="14" t="n">
@@ -8364,6 +9955,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Le réel est-il un ou multiple ?</t>
+        </is>
+      </c>
     </row>
     <row r="129" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="n">
@@ -8396,6 +9997,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qui existe vraiment ?</t>
+        </is>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="1" t="n">
@@ -8426,6 +10037,16 @@
       <c r="M130" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce que l’esprit ?</t>
         </is>
       </c>
     </row>
@@ -8464,6 +10085,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libéralisme</t>
+        </is>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="155.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="1" t="n">
@@ -8494,6 +10130,21 @@
       <c r="M132" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qu’une théorie scientifique ?</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivisme Logique</t>
         </is>
       </c>
     </row>
@@ -8530,6 +10181,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Individualisme</t>
+        </is>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="213.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="14" t="n">
@@ -8564,6 +10230,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phénoménologie, existence et herméneutique</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Existentialisme</t>
+        </is>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="14" t="n">
@@ -8598,6 +10279,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que pouvons-nous connaître ?</t>
+        </is>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="296.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="14" t="n">
@@ -8607,11 +10298,15 @@
       <c r="C136" s="14" t="n">
         <v>1945</v>
       </c>
-      <c r="D136" s="15" t="s">
-        <v>758</v>
-      </c>
-      <c r="E136" s="16" t="s">
-        <v>759</v>
+      <c r="D136" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Particularisme</t>
+        </is>
+      </c>
+      <c r="E136" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Particularisme_(%C3%A9pist%C3%A9mologie)" title=" Wikipedia"&gt;Le Particularisme&lt;/a&gt; épistémologique est la position selon laquelle on peut savoir certaines choses avant d’avoir expliqué, de manière générale, comment on les sait. À la question « Que savons-nous ? », il répond avant de se demander « Comment le savons-nous ? ». Il part donc de cas concrets de connaissance, que nous tenons pour assurés, et cherche ensuite à en dégager les critères.&lt;/p&gt; &lt;p&gt;Le débat a été mis en forme par le philosophe américain &lt;a href="https://fr.wikipedia.org/wiki/Roderick_Chisholm" title=" Wikipedia"&gt;Roderick Chisholm&lt;/a&gt; dans &lt;em&gt;The Problem of the Criterion&lt;/em&gt; (1973). Pour savoir si une croyance est une connaissance, il faut un critère ; mais pour savoir si ce critère est bon, il faut déjà connaître des cas où il réussit. Ce cercle, relevé dès l’Antiquité par les sceptiques comme Sextus Empiricus, laisse trois issues. Le sceptique conclut qu’on ne peut rien savoir. Le méthodiste, comme Descartes ou Locke, pose d’abord un critère, l’évidence ou l’expérience sensible, et en déduit ce que nous savons. Le particulariste, que Chisholm préfère, part au contraire de connaissances particulières, par exemple que j’ai deux mains, et juge les critères à leur aune.&lt;/p&gt; &lt;p&gt;Cette position s’inspire de &lt;a href="https://fr.wikipedia.org/wiki/George_Edward_Moore" title=" Wikipedia"&gt;G. E. Moore&lt;/a&gt;, qui opposait aux sceptiques, dans sa « Preuve d’un monde extérieur » (1939), la certitude de faits ordinaires, et avant lui de Thomas Reid et de sa philosophie du sens commun. Ernest Sosa l’a discutée et nuancée. On lui reproche de trancher la question plutôt que de la résoudre ; ses défenseurs répondent qu’une théorie de la connaissance doit rendre compte de ce que nous savons déjà, sans céder au scepticisme.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F136" s="14" t="s">
         <v>760</v>
@@ -8632,6 +10327,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Que pouvons-nous connaître ?</t>
+        </is>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="172.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="n">
@@ -8666,6 +10371,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qui existe vraiment ?</t>
+        </is>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="288.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="14" t="n">
@@ -8700,6 +10415,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Structuralisme et pensée française</t>
+        </is>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="14" t="n">
@@ -8734,6 +10459,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qu’une théorie scientifique ?</t>
+        </is>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="155.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="11" t="n">
@@ -8768,6 +10503,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marxisme;Psychanalyse</t>
+        </is>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="14" t="n">
@@ -8807,6 +10557,21 @@
           <t xml:space="preserve">occident;islam-juif</t>
         </is>
       </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anticolonialisme et décolonisation</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anticolonialisme;Marxisme</t>
+        </is>
+      </c>
     </row>
     <row r="142" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="14" t="n">
@@ -8841,6 +10606,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marxisme</t>
+        </is>
+      </c>
     </row>
     <row r="143" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="n">
@@ -8871,6 +10651,21 @@
       <c r="M143" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aristotélisme</t>
         </is>
       </c>
     </row>
@@ -8907,6 +10702,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Structuralisme et pensée française</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-structuralisme;Phénoménologie</t>
+        </is>
+      </c>
     </row>
     <row r="145" customFormat="false" ht="184.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="14" t="n">
@@ -8941,6 +10751,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Psychanalyse et sciences cognitives</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cognitivisme</t>
+        </is>
+      </c>
     </row>
     <row r="146" customFormat="false" ht="151.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="1" t="n">
@@ -8970,6 +10795,16 @@
       <c r="M146" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luttes et éthiques contemporaines</t>
         </is>
       </c>
     </row>
@@ -9006,6 +10841,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce que l’esprit ?</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Physicalisme</t>
+        </is>
+      </c>
     </row>
     <row r="148" customFormat="false" ht="76.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="11" t="n">
@@ -9040,6 +10890,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Structuralisme et pensée française</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Structuralisme</t>
+        </is>
+      </c>
     </row>
     <row r="149" customFormat="false" ht="231.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="n">
@@ -9074,6 +10939,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libertarianisme</t>
+        </is>
+      </c>
     </row>
     <row r="150" customFormat="false" ht="149.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="11" t="n">
@@ -9108,6 +10988,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libertarianisme;Anarchisme</t>
+        </is>
+      </c>
     </row>
     <row r="151" customFormat="false" ht="177.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="14" t="n">
@@ -9142,6 +11037,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Structuralisme et pensée française</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-structuralisme</t>
+        </is>
+      </c>
     </row>
     <row r="152" customFormat="false" ht="201" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="11" t="n">
@@ -9176,6 +11086,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ésotérismes et gnoses</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Néoplatonisme</t>
+        </is>
+      </c>
     </row>
     <row r="153" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="n">
@@ -9210,6 +11135,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce qu’une théorie scientifique ?</t>
+        </is>
+      </c>
     </row>
     <row r="154" customFormat="false" ht="170.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="1" t="n">
@@ -9243,6 +11178,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Structuralisme et pensée française</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-structuralisme</t>
+        </is>
+      </c>
     </row>
     <row r="155" customFormat="false" ht="149.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="1" t="n">
@@ -9272,6 +11222,21 @@
       <c r="M155" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marxisme</t>
         </is>
       </c>
     </row>
@@ -9309,6 +11274,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luttes et éthiques contemporaines</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utilitarisme</t>
+        </is>
+      </c>
     </row>
     <row r="157" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="14" t="n">
@@ -9343,6 +11323,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Structuralisme et pensée française</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-structuralisme</t>
+        </is>
+      </c>
     </row>
     <row r="158" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="1" t="n">
@@ -9354,8 +11349,10 @@
       <c r="D158" s="2" t="s">
         <v>876</v>
       </c>
-      <c r="E158" s="3" t="s">
-        <v>877</v>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Communautarisme_(concept_politique)"  title=" Wikipedia"&gt;Le Communautarisme philosophique&lt;/a&gt; est un courant de philosophie politique et morale apparu dans le monde anglophone au début des années 1980, en réaction au libéralisme de John Rawls et à sa &lt;em&gt;Théorie de la justice&lt;/em&gt; (1971). Il reproche à ce libéralisme de penser l’individu comme un sujet abstrait, qui choisirait ses valeurs et ses fins hors de toute appartenance, et de vouloir un État neutre à l’égard des conceptions de la vie bonne.&lt;/p&gt; &lt;p&gt;Ses figures majeures affirment au contraire que l’identité des personnes est constituée par les communautés dont elles font partie : famille, peuple, religion, tradition culturelle. Pour &lt;a href="https://fr.wikipedia.org/wiki/Alasdair_MacIntyre" title=" Wikipedia"&gt;Alasdair MacIntyre&lt;/a&gt;, dans &lt;em&gt;Après la vertu&lt;/em&gt; (1981), la morale moderne est en ruine parce qu’elle a perdu le cadre des traditions et des pratiques qui donnaient sens aux vertus, comme chez Aristote. &lt;a href="https://fr.wikipedia.org/wiki/Michael_Sandel" title=" Wikipedia"&gt;Michael Sandel&lt;/a&gt;, dans &lt;em&gt;Le Libéralisme et les limites de la justice&lt;/em&gt; (1982), juge fictif le « moi désengagé » de Rawls : nous sommes des êtres situés, liés par des attachements qui précèdent nos choix. &lt;a href="https://fr.wikipedia.org/wiki/Charles_Taylor_%28philosophe%29" title=" Wikipedia"&gt;Charles Taylor&lt;/a&gt;, dans &lt;em&gt;Les Sources du moi&lt;/em&gt; (1989), montre que l’individu ne se comprend qu’à l’intérieur d’« horizons de signification » hérités. Michael Walzer, dans &lt;em&gt;Sphères de justice&lt;/em&gt; (1983), soutient que chaque bien social doit être réparti selon le sens que lui donne une communauté.&lt;/p&gt; &lt;p&gt;Ces penseurs ne rejettent pas la liberté individuelle, et plusieurs ont refusé l’étiquette. Rawls leur a en partie répondu dans &lt;em&gt;Libéralisme politique&lt;/em&gt; (1993). En français courant, « communautarisme » désigne plutôt, de façon péjorative, le repli d’un groupe sur lui-même, un sens bien différent.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F158" s="1" t="s">
         <v>878</v>
@@ -9372,6 +11369,16 @@
       <c r="M158" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
         </is>
       </c>
     </row>
@@ -9405,6 +11412,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce que l’esprit ?</t>
+        </is>
+      </c>
     </row>
     <row r="160" customFormat="false" ht="168" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="n">
@@ -9435,6 +11452,21 @@
       <c r="M160" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luttes et éthiques contemporaines</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Féminisme</t>
         </is>
       </c>
     </row>
@@ -9471,6 +11503,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Psychanalyse et sciences cognitives</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cognitivisme</t>
+        </is>
+      </c>
     </row>
     <row r="162" customFormat="false" ht="150.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="1" t="n">
@@ -9500,6 +11547,16 @@
       <c r="M162" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Technique et avenir de l’humain</t>
         </is>
       </c>
     </row>
@@ -9536,6 +11593,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nouveaux réalismes</t>
+        </is>
+      </c>
     </row>
     <row r="164" customFormat="false" ht="155.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="11" t="n">
@@ -9570,6 +11637,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Technique et avenir de l’humain</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marxisme;Post-structuralisme</t>
+        </is>
+      </c>
     </row>
     <row r="165" customFormat="false" ht="147.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="14" t="n">
@@ -9606,6 +11688,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nouveaux réalismes</t>
+        </is>
+      </c>
+      <c r="Q165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phénoménologie</t>
+        </is>
+      </c>
     </row>
     <row r="166" customFormat="false" ht="161.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="11" t="n">
@@ -9640,6 +11737,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pessimisme</t>
+        </is>
+      </c>
     </row>
     <row r="167" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="14" t="n">
@@ -9674,6 +11786,21 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Technique et avenir de l’humain</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transhumanisme</t>
+        </is>
+      </c>
     </row>
     <row r="168" customFormat="false" ht="222.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="11" t="n">
@@ -9708,6 +11835,16 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luttes et éthiques contemporaines</t>
+        </is>
+      </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11">
@@ -9750,6 +11887,21 @@
         </is>
       </c>
       <c r="N169"/>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les débuts de la philosophie grecque</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Présocratique</t>
+        </is>
+      </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="11">
@@ -9792,6 +11944,21 @@
         </is>
       </c>
       <c r="N170"/>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socrate et ses héritiers</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socratisme;Éléatisme</t>
+        </is>
+      </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11">
@@ -9834,6 +12001,21 @@
         </is>
       </c>
       <c r="N171"/>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mysticisme;Thomisme</t>
+        </is>
+      </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="11">
@@ -9876,6 +12058,21 @@
         </is>
       </c>
       <c r="N172"/>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand et romantisme</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Idéalisme allemand</t>
+        </is>
+      </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11">
@@ -9918,6 +12115,21 @@
         </is>
       </c>
       <c r="N173"/>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivismes</t>
+        </is>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivisme</t>
+        </is>
+      </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="11">
@@ -9960,6 +12172,21 @@
         </is>
       </c>
       <c r="N174"/>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marxisme</t>
+        </is>
+      </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D175" s="3"/>

</xml_diff>

<commit_message>
Histoire des courants : 7 nouveaux cartouches (ésotérismes, Inde moderne, pensée juive, réveils de l'islam, pensée russe, anticolonialisme, libération) ; courant Déontologisme ; fiches Jean Bodin et Antoine de Montchrestien (Mercantilisme) ; Oecuménisme daté de 1910 et rattaché à 6 philosophes ; dates du Dualisme (1641) et du Personnalisme (1932) ; 3 descriptions courtes ; paragraphes égarés et coquilles corrigés
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -5551,12 +5551,14 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14" t="n">
-        <v>1055</v>
+      <c r="A35" s="14">
+        <v>1641</v>
       </c>
       <c r="B35" s="14"/>
-      <c r="C35" s="14" t="s">
-        <v>190</v>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1641</t>
+        </is>
       </c>
       <c r="D35" s="15" t="s">
         <v>191</v>
@@ -6725,8 +6727,12 @@
       <c r="D59" s="15" t="s">
         <v>317</v>
       </c>
-      <c r="E59" s="21" t="s">
-        <v>318</v>
+      <c r="E59" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Mercantilisme" title=" Wikipedia"&gt; Le Mercantilisme&lt;/a&gt; est une doctrine économique dominante en Europe du XVIᵉ au milieu du XVIIIᵉ siècle, qui prône le développement économique par l'enrichissement des nations grâce au commerce extérieur. Cette conception de l'économie vise à renforcer la puissance de l'État en accumulant des métaux précieux (or et argent), considérés comme la richesse essentielle des nations. &lt;/p&gt; &lt;p&gt; Ses principes fondamentaux reposent sur l'accumulation de réserves de métaux précieux, le développement des activités économiques et des exportations, et l'adoption de mesures protectionnistes. Pour réaliser un excédent de la balance commerciale, les États mercantilistes établissent des barrières tarifaires, encadrent le commerce et la production, et encouragent activement les exportations.  L'État joue un rôle primordial dans le développement mercantile, en adoptant des politiques protectionnistes et en encadrant strictement l'activité nationale. En France, le mercantilisme a inspiré la politique de Colbert (colbertisme), qui donnait à l'État un rôle prépondérant dans la conduite des affaires de la Nation. &lt;/p&gt; &lt;p&gt; Le terme « mercantilisme » est forgé a posteriori, notamment au XVIIIᵉ siècle par Adam Smith, pour critiquer certaines politiques orientées vers le commerce extérieur et le rôle central de l'État. Les détracteurs du mercantilisme (Adam Smith, Marx) considèrent qu'il ne représente pas un système théorique homogène, mais plutôt les conceptions économiques européennes ayant cours pendant plus de deux siècles. &lt;/p&gt; &lt;p&gt;Ses principaux auteurs sont, en France, &lt;a href="https://fr.wikipedia.org/wiki/Jean_Bodin" title=" Wikipedia"&gt;Jean Bodin&lt;/a&gt;, qui explique dès 1568 la hausse des prix par l’afflux de l’or d’Amérique, et &lt;a href="https://fr.wikipedia.org/wiki/Antoine_de_Montchrestien" title=" Wikipedia"&gt;Antoine de Montchrestien&lt;/a&gt;, qui invente en 1615 l’expression « économie politique » ; en Angleterre, &lt;a href="https://fr.wikipedia.org/wiki/Thomas_Mun" title=" Wikipedia"&gt;Thomas Mun&lt;/a&gt;, pour qui la richesse du royaume vient de l’excédent du commerce extérieur ; en Allemagne et en Autriche, les caméralistes, qui en font une science de l’administration. Les physiocrates, puis Adam Smith, lui opposeront la liberté du commerce.&lt;/p&gt; 
+&lt;audio controls title="XVIIe, grand siecle du mercantilisme par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10081-25.03.2024-ITEMA_23688783-2024C29629S0085-NET_MFC_57DAA2F8-478A-4A5B-A77B-CDF7D6FF4505-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+</t>
+        </is>
       </c>
       <c r="F59" s="14" t="s">
         <v>319</v>
@@ -6741,6 +6747,11 @@
       </c>
       <c r="K59" s="3" t="s">
         <v>251</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jean BODIN;Antoine de MONTCHRESTIEN</t>
+        </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -8138,18 +8149,23 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="11" t="n">
-        <v>1800</v>
+      <c r="A88" s="11">
+        <v>1932</v>
       </c>
       <c r="B88" s="11"/>
-      <c r="C88" s="11" t="n">
-        <v>1800</v>
+      <c r="C88" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1932</t>
+        </is>
       </c>
       <c r="D88" s="12" t="s">
         <v>476</v>
       </c>
-      <c r="E88" s="13" t="s">
-        <v>477</v>
+      <c r="E88" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Personnalisme"  title=" Wikipedia"&gt; Le Personnalisme&lt;/a&gt; est un courant philosophique qui place la personne humaine au centre de toute réflexion. Il affirme que chaque être humain possède une dignité propre, irréductible à sa fonction sociale, à son utilité économique ou à une simple appartenance au groupe. &lt;/p&gt; &lt;p&gt; Ce courant s’est développé surtout au début du XXe siècle, dans un contexte de crise des valeurs et de montée des idéologies qui tendaient à écraser l’individu, comme certaines formes de collectivisme ou de matérialisme. Il s’agit donc d’une réaction contre tout ce qui réduit l’être humain à un rouage, un objet ou un numéro. &lt;/p&gt; &lt;p&gt; Le personnalisme insiste sur le fait que la personne n’est pas un individu isolé. Elle est au contraire un être libre, conscient, responsable et fondamentalement relationnel, c’est-à-dire défini aussi par ses liens avec autrui. Cette idée mène à une éthique de la solidarité, du respect et de la reconnaissance de l’autre. &lt;/p&gt; &lt;p&gt; En France, Emmanuel Mounier est la figure la plus connue du personnalisme chrétien. Il a donné à ce courant une portée morale et politique en défendant une société plus humaine, où l’économie et les institutions doivent rester au service de la personne. Le personnalisme propose une vision de l’homme qui refuse à la fois l’individualisme absolu et le collectivisme excessif. Son message essentiel est simple : la personne humaine a une valeur absolue et doit toujours être traitée comme une fin, jamais comme un moyen.  &lt;/p&gt;  
+</t>
+        </is>
       </c>
       <c r="F88" s="11" t="s">
         <v>478</v>
@@ -8336,18 +8352,22 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="14" t="n">
-        <v>1830</v>
+      <c r="A92" s="14">
+        <v>1910</v>
       </c>
       <c r="B92" s="14"/>
-      <c r="C92" s="14" t="s">
-        <v>498</v>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1910</t>
+        </is>
       </c>
       <c r="D92" s="15" t="s">
         <v>499</v>
       </c>
-      <c r="E92" s="29" t="s">
-        <v>500</v>
+      <c r="E92" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C5%92cum%C3%A9nisme"  title=" Wikipedia"&gt;L'Oecuménisme&lt;/a&gt;  désigne le mouvement au sein du christianisme visant à promouvoir l'unité visible entre les différentes Églises et confessions chrétiennes, en surmontant les divisions historiques et doctrinales. Issu du grec oikoumenê "terre habitée" ou "monde entier", il s'agit d'un effort spirituel et pratique pour réaliser la prière de Jésus « que tous soient un » (Jean 17:21), en favorisant le dialogue, la prière commune et la coopération. &lt;/p&gt; &lt;p&gt; Le mouvement moderne émerge avec des initiatives protestantes comme la Conférence missionnaire mondiale d'Édimbourg en 1910. Le Conseil œcuménique des Églises (COE) est fondé en 1948 à Amsterdam, regroupant protestants, anglicans et orthodoxes. L'Église catholique s'engage officiellement lors du Concile Vatican II (1962-1965), avec le décret Unitatis redintegratio qui définit l'œcuménisme comme une priorité. &lt;/p&gt; &lt;p&gt; Le COE réunit aujourd'hui plus de 350 Églises, tandis que des organismes bilatéraux comme le Groupe des Dombes (catholiques-protestants) avancent sur des consensus. Les obstacles persistent : divergences sur le rôle du pape, l'ordination des femmes ou le mariage homosexuel, mais des progrès marquent 2025, comme des déclarations conjointes sur la synodalité. &lt;/p&gt; &lt;p&gt;Le rêve de l’unité des chrétiens est pourtant plus ancien. Après les déchirements de la Réforme, des penseurs « iréniques » cherchent la paix entre les confessions : Hugo Grotius, Comenius, ou &lt;a href="https://fr.wikipedia.org/wiki/Gottfried_Wilhelm_Leibniz" title=" Wikipedia"&gt;Leibniz&lt;/a&gt;, qui négocie avec Bossuet, à la fin du XVIIe siècle, un projet de réunion des catholiques et des protestants. En Russie, Vladimir Soloviev plaide pour l’union de l’Église orthodoxe et de Rome. Au XXe siècle, des théologiens orthodoxes de l’émigration, comme Sergueï Boulgakov et &lt;a href="https://fr.wikipedia.org/wiki/Georges_Florovsky" title=" Wikipedia"&gt;Georges Florovsky&lt;/a&gt;, deviennent des acteurs majeurs du dialogue avec les anglicans et les protestants, et Florovsky participe à la fondation du COE.&lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F92" s="14" t="s">
         <v>501</v>
@@ -8363,6 +8383,11 @@
       <c r="K92" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vladimir SOLOVIEV;Sergueï BOULGAKOV;Georges FLOROVSKY</t>
+        </is>
+      </c>
       <c r="M92" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
@@ -12420,9 +12445,61 @@
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D175" s="3"/>
+      <c r="A175" s="11">
+        <v>1785</v>
+      </c>
+      <c r="C175" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1785</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Déontologisme</t>
+        </is>
+      </c>
+      <c r="E175" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/D%C3%A9ontologisme" title=" Wikipedia"&gt;Le Déontologisme&lt;/a&gt;, du grec &lt;em&gt;deon&lt;/em&gt;, « ce qu’il faut faire », désigne les morales du devoir : certaines actions sont obligatoires ou interdites en elles-mêmes, quelles qu’en soient les conséquences. On ne doit pas mentir, ni tuer un innocent, même pour obtenir un plus grand bien. Le déontologisme s’oppose ainsi au conséquentialisme et à l’utilitarisme, pour qui seuls comptent les effets d’une action, et à l’éthique de la vertu, qui juge le caractère plutôt que les actes.&lt;/p&gt; &lt;p&gt;Sa forme la plus célèbre est la morale de &lt;a href="https://fr.wikipedia.org/wiki/Emmanuel_Kant" title=" Wikipedia"&gt;Kant&lt;/a&gt;, exposée dans les &lt;em&gt;Fondements de la métaphysique des mœurs&lt;/em&gt; (1785) et la &lt;em&gt;Critique de la raison pratique&lt;/em&gt; (1788). Pour Kant, une action n’a de valeur morale que si elle est faite par devoir, et non par intérêt ou par inclination. La raison donne à chacun une loi inconditionnelle, l’&lt;a href="https://fr.wikipedia.org/wiki/Imp%C3%A9ratif_cat%C3%A9gorique" title=" Wikipedia"&gt;impératif catégorique&lt;/a&gt; : « Agis uniquement d’après la maxime qui fait que tu peux vouloir en même temps qu’elle devienne une loi universelle. » Une autre formule ordonne de traiter l’humanité, en soi et en autrui, toujours comme une fin et jamais simplement comme un moyen : c’est le fondement moderne de la dignité humaine. Kant va jusqu’à refuser le mensonge pour sauver un ami poursuivi par un assassin, ce que Benjamin Constant lui reproche.&lt;/p&gt; &lt;p&gt;Au XXe siècle, W. D. Ross propose plusieurs devoirs qui peuvent entrer en conflit ; &lt;a href="https://fr.wikipedia.org/wiki/John_Rawls_%28philosophe%29" title=" Wikipedia"&gt;John Rawls&lt;/a&gt; fonde sa théorie de la justice sur une inspiration kantienne ; Habermas et Apel en tirent une éthique de la discussion ; Robert Nozick fait des droits individuels des « contraintes » qu’aucun calcul ne peut violer ; Christine Korsgaard renouvelle la lecture de Kant.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="I175" s="1"/>
-      <c r="J175" s="1"/>
+      <c r="J175" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">morale selon laquelle certaines actions sont obligatoires ou interdites en elles-mêmes, quelles qu’en soient les conséquences (Kant).</t>
+        </is>
+      </c>
+      <c r="K175" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Éthique</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emmanuel KANT;John RAWLS;Jürgen HABERMAS;Christine KORSGAARD</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N175"/>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
+        </is>
+      </c>
+      <c r="Q175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Criticisme</t>
+        </is>
+      </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="I176" s="1"/>

</xml_diff>

<commit_message>
Données : dates des 4 ontologies de Descola et de l'Ubuntu (1980, paragraphe sur sa forme écrite) ; Zera Yacob rattaché au Rationalisme, Pak Chong-hong au Confucianisme coréen et à la Phénoménologie ; 47 coquilles visibles (mots doublés, phrases sans majuscule ou sans sujet, points égarés) ; espaces en trop avant virgule et point dans 197 textes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -6921,8 +6921,10 @@
       <c r="D63" s="15" t="s">
         <v>340</v>
       </c>
-      <c r="E63" s="16" t="s">
-        <v>341</v>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Occasionnalisme"  title=" Wikipedia"&gt;L'occasionalisme&lt;/a&gt; est une théorie philosophique qui émerge principalement au XVIIe siècle, en réponse aux problèmes posés par la métaphysique cartésienne, notamment la question de l'interaction entre l'âme et le corps. Cette doctrine soutient que Dieu est la seule cause véritable de tous les événements dans le monde, et que les causes naturelles ne sont que des "occasions" pour Dieu d'intervenir. Il trouve ses racines dans la philosophie de René Descartes, qui a introduit une distinction radicale entre l'âme (la substance pensante) et le corps (la substance étendue). Cette dualité pose un problème majeur : comment l'âme, qui est immatérielle, peut-elle agir sur le corps, qui est matériel, et vice versa ? &lt;/p&gt; &lt;p&gt; Selon l'occasionalisme, Dieu est la seule cause efficiente dans l'univers. Les événements naturels (comme une boule de billard qui en frappe une autre) ne sont pas causés par les objets eux-mêmes, mais par l'intervention directe de Dieu. Les causes naturelles ne sont que des "occasions" qui déclenchent l'action divine. Ils soutiennent que Dieu a établi une harmonie entre les événements du monde. Par exemple, quand je décide de lever mon bras (action de l'âme), Dieu intervient pour faire en sorte que mon bras se lève (action du corps). Il n'y a pas de causalité directe entre l'âme et le corps, mais une coordination divine. L'occasionalisme résout le problème cartésien de l'interaction entre l'âme et le corps en niant toute causalité directe entre les deux. Dieu agit comme médiateur entre les deux substances. Ils s'appuient sur l'idée que Dieu doit continuellement maintenir l'existence du monde. Si Dieu doit constamment soutenir l'univers, il est cohérent de penser qu'il intervient aussi dans chaque événement. &lt;/p&gt; &lt;p&gt; Malebranche est le plus célèbre des occasionalistes. Dans De la recherche de la vérité, il développe une version sophistiquée de l'occasionalisme, en insistant sur la "vision en Dieu" (l'idée que nous percevons les objets à travers les idées divines). &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F63" s="14" t="s">
         <v>342</v>
@@ -7109,12 +7111,14 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="11" t="n">
-        <v>1720</v>
+      <c r="A67" s="11">
+        <v>1871</v>
       </c>
       <c r="B67" s="11"/>
-      <c r="C67" s="11" t="n">
-        <v>1720</v>
+      <c r="C67" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1871</t>
+        </is>
       </c>
       <c r="D67" s="23" t="s">
         <v>362</v>
@@ -7155,12 +7159,14 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="11" t="n">
-        <v>1720</v>
+      <c r="A68" s="11">
+        <v>1869</v>
       </c>
       <c r="B68" s="11"/>
-      <c r="C68" s="11" t="n">
-        <v>1720</v>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1869</t>
+        </is>
       </c>
       <c r="D68" s="23" t="s">
         <v>367</v>
@@ -7201,12 +7207,14 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="117" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="11" t="n">
-        <v>1720</v>
+      <c r="A69" s="11">
+        <v>2005</v>
       </c>
       <c r="B69" s="11"/>
-      <c r="C69" s="11" t="s">
-        <v>372</v>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2005</t>
+        </is>
       </c>
       <c r="D69" s="23" t="s">
         <v>373</v>
@@ -7247,12 +7255,14 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="11" t="n">
-        <v>1720</v>
+      <c r="A70" s="11">
+        <v>2005</v>
       </c>
       <c r="B70" s="11"/>
-      <c r="C70" s="11" t="s">
-        <v>372</v>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2005</t>
+        </is>
       </c>
       <c r="D70" s="23" t="s">
         <v>378</v>
@@ -8821,8 +8831,10 @@
       <c r="D101" s="12" t="s">
         <v>554</v>
       </c>
-      <c r="E101" s="13" t="s">
-        <v>555</v>
+      <c r="E101" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Fonctionnalisme_(philosophie)"  title=" Wikipedia"&gt;Le Fonctionnalisme&lt;/a&gt; est un courant philosophique, principalement en philosophie de l'esprit, qui définit les états mentaux par leur rôle fonctionnel ou causal plutôt que par leur composition matérielle intrinsèque. Il considère que ce qui importe pour identifier une douleur ou une croyance, par exemple, c'est sa place dans le système cognitif global : ses interactions avec les stimuli, d'autres états mentaux et les comportements. &lt;/p&gt; &lt;p&gt; Émergé aux États-Unis à la fin du XIXe siècle avec des psychologues comme William James, il s'oppose au structuralisme (qui analyse la structure de la conscience) en se focalisant sur l'utilité adaptative des processus mentaux, influencé par Darwin. En philosophie analytique du XXe siècle (Hilary Putnam, 1960s), il devient une théorie anti-matérialiste : un état mental est réalisé par tout substrat (cerveau humain, silicone d'IA, etc.) accomplissant la même fonction causale. &lt;/p&gt; &lt;p&gt; En philosophie de l'esprit, il englobe le computationnalisme, voyant l'esprit comme un programme informatique multiple-réalisable ; en sciences sociales, chez Durkheim ou Parsons, il analyse les institutions par leur contribution à l'équilibre social (ex. : famille pour la socialisation).  Critiqué pour ignorer les qualia (expériences subjectives) et pour son risque de panpsychisme extrême.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F101" s="11" t="s">
         <v>556</v>
@@ -10298,8 +10310,12 @@
       <c r="D131" s="15" t="s">
         <v>709</v>
       </c>
-      <c r="E131" s="16" t="s">
-        <v>710</v>
+      <c r="E131" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Empirisme_logique"  title=" Wikipedia"&gt;Le positivisme logique&lt;/a&gt;, également connu sous le nom "d'empirisme logique" est un courant philosophique majeur qui a cherché à définir les critères de la connaissance scientifique et à éliminer la métaphysique jugée dépourvue de sens. Né au sein du Cercle de Vienne, il a eu une influence considérable sur la philosophie des sciences et la philosophie analytique. Voici les points essentiels: &lt;/p&gt; &lt;p&gt; - Le principe de vérification (ou vérifiabilité) : C'est le critère central du positivisme logique pour déterminer la signification d'un énoncé. Selon ce principe, un énoncé n'a de sens que s'il est : &lt;/p&gt; 
+&lt;dd&gt; - Analytiquement vrai : vrai en vertu de sa structure logique ou de la définition de ses termes (par exemple, "Tous les célibataires sont non mariés"). Ces énoncés sont tautologiques et n'apportent pas d'information sur le monde. &lt;/dd&gt; 
+&lt;dd&gt; - Empiriquement vérifiable : sa vérité ou sa fausseté peut être établie par l'observation et l'expérience sensorielle (par exemple, "Cette table est marron"). &lt;/dd&gt; &lt;p&gt; - Le rejet de la métaphysique : Les énoncés qui ne sont ni analytiques ni empiriquement vérifiables sont considérés comme dépourvus de sens cognitif. Cela inclut la plupart des affirmations traditionnelles de la métaphysique (sur l'existence de Dieu, l'âme, le sens de la vie, etc.), de l'éthique normative (les jugements de valeur ne pouvant être vérifiés empiriquement) et de la théologie. Pour les positivistes logiques, ces énoncés peuvent avoir une valeur émotive ou poétique, mais pas une valeur de vérité. &lt;/p&gt; &lt;p&gt; - L'empirisme radical : Toute connaissance du monde provient de l'expérience sensorielle. La science est considérée comme le modèle de la connaissance rationnelle. &lt;/p&gt; &lt;p&gt; - La logique et les mathématiques comme outils : La logique et les mathématiques sont vues comme des outils formels essentiels pour analyser et structurer la connaissance scientifique. Leurs énoncés sont analytiques. &lt;/p&gt; &lt;p&gt;  - L'unité de la science : Les positivistes logiques aspiraient à unifier toutes les sciences (physique, biologie, psychologie, sciences sociales) sur la base d'un langage commun (idéalement le langage de la physique) et d'une méthodologie commune fondée sur la vérification empirique. &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F131" s="14" t="s">
         <v>711</v>
@@ -10925,8 +10941,13 @@
       <c r="D144" s="12" t="s">
         <v>781</v>
       </c>
-      <c r="E144" s="13" t="s">
-        <v>782</v>
+      <c r="E144" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9orie_critique"   title=" Wikipedia"&gt; La Théorie Critique&lt;/a&gt;, également connue sous le nom d'École de Francfort, est un courant de pensée philosophique et sociologique développé par un groupe de chercheurs associés à l'Institut de recherche sociale de l'Université de Francfort en Allemagne. Ce courant a émergé dans les années 1920 et s'est développé principalement dans les décennies suivantes. &lt;/p&gt; &lt;p&gt;  Un concept central de la Théorie critique est celui d'idéologie. Les penseurs de l'École de Francfort soutiennent que les idées et les croyances dominantes dans une société donnée peuvent être instrumentalisées pour maintenir l'ordre établi et perpétuer les inégalités. Ils cherchent à dévoiler les idéologies qui opèrent dans la société afin de permettre une prise de conscience critique et de favoriser la transformation sociale en analysant et à critiquant les structures sociales, politiques et culturelles afin de promouvoir l'émancipation et la libération des individus. Elle s'inspire à la fois de la philosophie, de la sociologie et de la psychologie pour comprendre les processus de domination et d'aliénation qui existent dans les sociétés modernes. &lt;/p&gt; &lt;p&gt; 
+La Théorie critique analyse et critique la société capitaliste et ses formes d'oppression, en mettant en lumière les mécanismes de domination économique, politique et culturelle avec une dimension psychologique de l'aliénation. &lt;/p&gt; &lt;p&gt;
+Un autre aspect important de la Théorie critique est sa réflexion sur la culture de masse et les industries culturelles. Ils analysent comment la culture de masse peut renforcer l'aliénation et la conformité, en transformant les individus en consommateurs passifs et en renforçant les normes sociales dominantes.  &lt;/p&gt; &lt;p&gt;  Max Horkheimer, Theodor Adorno ou Jürgen Habermas, chacun a contribué a en développer différents aspects, mais ils partagent certains points communs dans leur approche. &lt;/p&gt;
+ </t>
+        </is>
       </c>
       <c r="F144" s="11" t="s">
         <v>783</v>
@@ -11130,8 +11151,12 @@
       <c r="D148" s="12" t="s">
         <v>802</v>
       </c>
-      <c r="E148" s="13" t="s">
-        <v>803</v>
+      <c r="E148" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/D%C3%A9construction_(analyse_de_texte)#:~:text=La%20d%C3%A9construction%20(ou%20le%20d%C3%A9constructionnisme,sous%2Dentendus%20et%20les%20omissions."   title=" Wikipedia"&gt;Le Déconstructionnisme&lt;/a&gt;, tel que développé principalement par Jacques Derrida, n'est pas une doctrine ou une méthode fixe, mais plutôt une approche critique et philosophique qui vise à déconstruire les systèmes de pensée et les textes en révélant les tensions, les contradictions et les hiérarchies cachées qui les sous-tendent. Pour le comprendre, imaginez un bâtiment que vous analysez non seulement pour sa structure apparente, mais aussi pour les fondations invisibles, les matériaux utilisés, les fissures potentielles et les différentes manières dont il pourrait être interprété ou utilisé. Le déconstructionnisme fait quelque chose d'analogue avec les idées et les textes.  Voici les principaux aspects du déconstructionnisme : &lt;/p&gt; &lt;p&gt; 
+-  Déconstruction des Oppositions Binaires : La pensée occidentale est souvent structurée autour d'oppositions binaires (par exemple, bien/mal, vrai/faux). Le déconstructionnisme ne cherche pas simplement à inverser ces oppositions, mais à montrer comment chaque terme d'une paire dépend de l'autre pour sa définition et comment la hiérarchie implicite entre eux est instable et arbitraire. &lt;/p&gt; &lt;p&gt; -  Mise en Lumière de l'Instabilité du Sens : Le déconstructionnisme souligne que le sens n'est pas fixe et transparent, mais qu'il est toujours en jeu, différé et dépendant du contexte et des interprétations. Le concept clé de différance (un néologisme de Derrida) exprime cette idée : il combine à la fois la "différence" (le sens émerge des distinctions entre les éléments) et le "différer" (le sens est toujours renvoyé à plus tard, à d'autres contextes et interprétations). &lt;/p&gt; &lt;p&gt; 
+- Révélation des Tensions Internes : Les textes et les systèmes de pensée contiennent souvent des contradictions internes, des non-dits et des présupposés implicites qui minent leur cohérence apparente. Le déconstructionnisme cherche à identifier ces tensions et à montrer comment elles déstabilisent les affirmations centrales du texte ou du système. &lt;/p&gt; &lt;p&gt; - Attention au Langage : Le langage n'est pas un outil neutre pour transmettre des idées, mais il est intrinsèquement ambigu et porteur d'une histoire et de préjugés. Le déconstructionnisme examine attentivement le langage utilisé dans un texte pour révéler les jeux de sens, les métaphores et les implications qui peuvent échapper à une lecture superficielle. &lt;/p&gt; &lt;p&gt; -  Pas une Méthode, mais une Stratégie de Lecture :  Derrida insistait sur le fait que la déconstruction n'est pas une méthode que l'on peut appliquer mécaniquement. C'est plutôt une attitude critique, une manière d'aborder les textes et les idées avec une sensibilité aux complexités et aux non-dits. &lt;/p&gt; &lt;p&gt; Il est important de noter que le déconstructionnisme a souvent été mal compris et critiqué pour son apparente négation du sens ou son relativisme. Cependant, pour Derrida, il ne s'agissait pas de détruire le sens, mais de montrer sa complexité et de nous rendre plus conscients des forces qui le façonnent. &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F148" s="11" t="s">
         <v>804</v>
@@ -12354,8 +12379,10 @@
       <c r="D173" s="12" t="s">
         <v>931</v>
       </c>
-      <c r="E173" s="13" t="s">
-        <v>932</v>
+      <c r="E173" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Woke#:~:text=Par%20exemple%2C%20MTV%20News%20l,ne%20l'es%20pas%20%C2%BB."  style="color:#d35400"  title=" Wikipedia"&gt;Le Wokisme&lt;/a&gt;, diré du mot "woke" (éveillé en anglais) était utilisé dans les communautés afro-américaines pour désigner une prise de conscience des injustices raciales et sociales. Il invitait à rester vigilant face aux discriminations. &lt;/p&gt;  Aujourd'hui, le terme "wokisme" a pris une connotation plus large et plus complexe. Il est souvent utilisé pour décrire les questions d'injustice sociale, Il encourage à remettre en question les normes sociales et les stéréotypes, en particulier ceux liés à la race, au genre, à l'orientation sexuelle. Les personnes considérées comme "woke" cherchent à créer une société plus juste et équitable pour tous, en dénonçant les discriminations et en promouvant la diversité. Ils s'intéressent aux mécanismes qui perpétuent les inégalités, comme le racisme systémique, le sexisme, l'homophobie. &lt;/p&gt; &lt;p&gt; Certains accusent les personnes "woke" d'être trop radicales et de vouloir censurer les opinions dissidentes. On leur reproche de diviser la société en groupes identitaires et de nier l'existence d'une humanité universelle. Ses détracteurs estiment que les personnes "woke" exagèrent les problèmes et se présentent comme des victimes. &lt;/p&gt;  &lt;p&gt;  &lt;p&gt; Il remet en question les valeurs traditionnelles et propose une vision plus inclusive de la société, contribuant à l'émergence de nouveaux mots et expressions pour décrire les expériences des personnes marginalisées. &lt;/p&gt;   &lt;p&gt; Des philosophes comme Judith Butler, philosophe féministe et queer qui a développé la théorie du genre et a questionné les normes de genre et de sexualité. Michel Foucault, historien et philosophe, il a analysé les rapports de pouvoir et les mécanismes de domination dans la société. Kimberlé Crenshaw, juriste et théoricienne féministe, elle a développé le concept d'intersectionnalité, qui permet d'analyser les différentes formes de discrimination qui se croisent et s'additionnent. &lt;/p&gt; &lt;audio controls title="Dieu, un homme en trop ?  "Qu'est ce que le Wokisme? " par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13397-11.06.2022-ITEMA_23055745-2022C3397E0022-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F173" s="11" t="s">
         <v>933</v>

</xml_diff>

<commit_message>
Vidéos : Anticolonialisme (Césaire, France Culture) et Haskala (Henry Abramson) à la place de vidéos orientées ; crédit du Kalâm corrigé (non écrits au commit précédent)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -7577,11 +7577,15 @@
       <c r="E76" s="16" t="s">
         <v>411</v>
       </c>
-      <c r="F76" s="14" t="s">
-        <v>412</v>
-      </c>
-      <c r="G76" s="16" t="s">
-        <v>413</v>
+      <c r="F76" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1E_GadDJvKI</t>
+        </is>
+      </c>
+      <c r="G76" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Le Temps des archives / 1950 : le Discours sur le colonialisme d'Aimé Césaire" par France Culture</t>
+        </is>
       </c>
       <c r="H76" s="14"/>
       <c r="I76" s="16"/>

</xml_diff>

<commit_message>
Courants à un seul philosophe, lots 1 à 3 : fiches Charles Maurras et Serge Ier de Constantinople ; 6 rattachements faux retirés ; 105 penseurs déjà présents rattachés à 50 courants (Wokisme : Butler et hooks) ; figures clés de 8 courants ; dates d'Akshapada Gautama et de Patañjali
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -5482,6 +5482,11 @@
       <c r="K33" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SERGE Ier de Constantinople</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
@@ -8900,6 +8905,11 @@
       <c r="K102" s="3" t="s">
         <v>232</v>
       </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ernest RENAN</t>
+        </is>
+      </c>
       <c r="M102" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
@@ -9462,6 +9472,11 @@
       <c r="K113" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Friedrich Heinrich JACOBI;Arthur SCHOPENHAUER;Soren KIERKEGAARD;Friedrich NIETZSCHE</t>
+        </is>
+      </c>
       <c r="M113" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
@@ -9775,6 +9790,11 @@
       <c r="K119" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stanislaw LESNIEWSKI;Nelson GOODMAN</t>
+        </is>
+      </c>
       <c r="M119" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
@@ -10185,6 +10205,11 @@
       <c r="K128" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Charles MAURRAS</t>
+        </is>
+      </c>
       <c r="M128" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
@@ -10728,6 +10753,11 @@
       <c r="K139" s="3" t="s">
         <v>100</v>
       </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">René DESCARTES;John LOCKE;David HUME</t>
+        </is>
+      </c>
       <c r="M139" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
@@ -10779,6 +10809,11 @@
       </c>
       <c r="K140" s="3" t="s">
         <v>27</v>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thomas REID;Georges Edward MOORE;Roderick CHISHOLM</t>
+        </is>
       </c>
       <c r="M140" t="inlineStr">
         <is>
@@ -12401,6 +12436,11 @@
       </c>
       <c r="K173" s="3" t="s">
         <v>251</v>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Judith BUTLER;Bell HOOKS</t>
+        </is>
       </c>
       <c r="M173" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Textes des courants, lots 8 et 9 : 20 textes portés à 1 410-1 525 caractères (Cartésianisme, Tiers-mondisme, Béhaviorisme, Sophisme, Maurrassisme, Cyrénaïsme, Lokayata, Réductionnisme, Éclectisme, Négritude, Anticolonialisme, Mazdakisme, Taoïsme, Bushido, Averroïsme, Agnosticisme, Populisme, Advaïta Védanta, Individualisme méthodologique, Meinongianisme) ; lien du Sophisme vers la page « Sophiste » ; HTML du Populisme réparé
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -4321,8 +4321,10 @@
       <c r="D10" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>47</v>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Sophiste" title=" Wikipedia"&gt;Le Sophisme&lt;/a&gt; désigne ici le mouvement des sophistes, maîtres itinérants qui, dans la Grèce du Ve siècle av. J.-C., enseignent contre rémunération l’art de bien parler et de réussir dans la cité. Dans l’Athènes démocratique, où tout se décide par le débat, à l’Assemblée comme au tribunal, savoir convaincre devient une force politique, et les jeunes gens fortunés se pressent à leurs leçons.&lt;/p&gt; &lt;p&gt;Le plus célèbre, &lt;a href="https://fr.wikipedia.org/wiki/Protagoras" title=" Wikipedia"&gt;Protagoras&lt;/a&gt; d’Abdère, affirme que « l’homme est la mesure de toutes choses » : il n’y a pas de vérité absolue, seulement ce qui paraît vrai à chacun. Sur tout sujet, on peut soutenir deux thèses opposées, et l’habileté consiste à rendre fort l’argument le plus faible. &lt;a href="https://fr.wikipedia.org/wiki/Gorgias" title=" Wikipedia"&gt;Gorgias&lt;/a&gt; de Léontinoi va plus loin dans un traité paradoxal : rien n’existe ; si quelque chose existait, on ne pourrait le connaître ; et si on le connaissait, on ne pourrait le communiquer. Le discours est pour lui un « puissant tyran » qui agit sur l’âme comme un remède sur le corps. D’autres, comme Prodicos ou Hippias, s’intéressent au sens exact des mots ou au savoir encyclopédique. Beaucoup opposent la nature (&lt;em&gt;physis&lt;/em&gt;) aux lois humaines (&lt;em&gt;nomos&lt;/em&gt;), conventionnelles et variables d’un peuple à l’autre.&lt;/p&gt; &lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Socrate" title=" Wikipedia"&gt;Socrate&lt;/a&gt; puis Platon les combattent, leur reprochant de vendre l’apparence du savoir et de préférer la persuasion à la vérité : de là vient le sens péjoratif de « sophisme », raisonnement trompeur. Le XIXe siècle les a réhabilités comme les premiers penseurs du langage, de la relativité des valeurs et de l’éducation.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F10" s="14" t="s">
         <v>48</v>
@@ -4969,8 +4971,10 @@
       <c r="D23" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="E23" s="16" t="s">
-        <v>121</v>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Cyr%C3%A9na%C3%AFsme"  style="color:#d35400"  title=" Wikipedia"&gt;Le Cyrénaïsme&lt;/a&gt; est l’école philosophique fondée à Cyrène, dans l’actuelle Libye, par &lt;a href="https://fr.wikipedia.org/wiki/Aristippe_de_Cyr%C3%A8ne" title=" Wikipedia"&gt;Aristippe&lt;/a&gt; (vers 435-356 av. J.-C.), disciple de Socrate. C’est la première grande philosophie du plaisir : pour les cyrénaïques, le plaisir est le bien suprême, et le but de la vie est de jouir du plaisir présent. L’école est surtout organisée par le petit-fils d’Aristippe, qui porte le même nom, et se maintient jusqu’au IIIe siècle av. J.-C.&lt;/p&gt; &lt;p&gt;Les cyrénaïques fondent leur morale sur une théorie de la connaissance : nous ne connaissons que nos propres sensations, non les choses qui les causent. Nous savons que nous éprouvons une impression de blanc ou de sucré, pas ce qu’est l’objet. Seuls nos états sont certains, et parmi eux le plaisir, « mouvement doux », et la douleur, « mouvement rude » ; entre les deux, l’absence de mouvement est un état neutre. Le plaisir corporel et présent est le plus vif, car le passé n’est plus et l’avenir est incertain. Aristippe n’est pourtant pas un débauché : il veut maîtriser le plaisir sans en être l’esclave, et s’adapter à toute situation avec aisance. Familier de la cour de Denys de Syracuse, il disait de la courtisane Laïs : « je la possède, je ne suis pas possédé ».&lt;/p&gt; &lt;p&gt;Contre eux, &lt;a href="https://fr.wikipedia.org/wiki/%C3%89picure" title=" Wikipedia"&gt;Épicure&lt;/a&gt; définira le plaisir comme l’absence de douleur. Les derniers cyrénaïques divergent : Hégésias, surnommé « l’avocat de la mort », jugeait le bonheur impossible. Michel Onfray a contribué à faire redécouvrir cette école.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F23" s="14" t="s">
         <v>122</v>
@@ -5316,8 +5320,10 @@
       <c r="D30" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="E30" s="13" t="s">
-        <v>163</v>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89clectisme"  title=" Wikipedia"&gt;L’Éclectisme&lt;/a&gt;, du grec &lt;em&gt;eklegein&lt;/em&gt;, « choisir », est l’attitude qui consiste à emprunter à plusieurs écoles ce qu’elles ont de meilleur, plutôt que d’adhérer à un seul système. Le mot vient de l’Antiquité : &lt;a href="https://fr.wikipedia.org/wiki/Diog%C3%A8ne_La%C3%ABrce" title=" Wikipedia"&gt;Diogène Laërce&lt;/a&gt; mentionne au IIIe siècle une « école éclectique » fondée par Potamon d’Alexandrie, qui mêlait les doctrines de Platon, d’Aristote et des stoïciens.&lt;/p&gt; &lt;p&gt;Dès le Ier siècle av. J.-C., &lt;a href="https://fr.wikipedia.org/wiki/Cic%C3%A9ron" title=" Wikipedia"&gt;Cicéron&lt;/a&gt; pratique ce choix raisonné : sceptique en théorie de la connaissance, il retient de chaque école ce qui lui paraît le plus probable. Aux XVIIe et XVIIIe siècles, l’éclectisme devient un idéal de liberté intellectuelle : dans l’&lt;em&gt;Encyclopédie&lt;/em&gt;, Diderot loue l’éclectique qui, « foulant aux pieds le préjugé, la tradition, l’ancienneté », n’admet rien que sur le témoignage de sa raison. Au XIXe siècle, &lt;a href="https://fr.wikipedia.org/wiki/Victor_Cousin" title=" Wikipedia"&gt;Victor Cousin&lt;/a&gt; en fait une doctrine : l’histoire de la philosophie montre que chaque grand système, sensualisme, idéalisme, scepticisme et mysticisme, contient une part de vérité, et qu’il faut les concilier. Devenu ministre et maître de l’enseignement de la philosophie en France, il en fait la base des programmes du lycée et de l’université.&lt;/p&gt; &lt;p&gt;On reproche à l’éclectisme de juxtaposer sans cohérence des idées incompatibles, ou de servir de philosophie officielle prudente. Il a pourtant encouragé l’étude de l’histoire de la philosophie, et beaucoup de penseurs, sans se dire éclectiques, ont procédé de même, en empruntant librement à plusieurs traditions.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F30" s="11" t="s">
         <v>164</v>
@@ -5853,8 +5859,10 @@
       <c r="D41" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="E41" s="16" t="s">
-        <v>222</v>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Averro%C3%AFsme"  title=" Wikipedia"&gt;L’Averroïsme&lt;/a&gt; désigne le courant de pensée qui, dans l’Europe latine du XIIIe au XVIe siècle, se réclame des commentaires d’Aristote écrits par &lt;a href="https://fr.wikipedia.org/wiki/Averro%C3%A8s" title=" Wikipedia"&gt;Averroès&lt;/a&gt; (1126-1198). Juge et médecin à Cordoue, celui-ci est pour les Latins « le Commentateur » par excellence. Traduites en latin à partir des années 1220, ses œuvres donnent accès à un Aristote complet et rigoureux, débarrassé des ajouts néoplatoniciens.&lt;/p&gt; &lt;p&gt;Vers 1260-1270, à la faculté des arts de Paris, des maîtres comme &lt;a href="https://fr.wikipedia.org/wiki/Siger_de_Brabant" title=" Wikipedia"&gt;Siger de Brabant&lt;/a&gt; et Boèce de Dacie veulent pratiquer la philosophie de façon autonome, en suivant la raison et Aristote jusqu’au bout. Ils en tirent des thèses contraires à la foi : le monde est éternel, et il n’existe qu’un seul intellect pour tous les hommes, de sorte que l’âme individuelle ne survit pas à la mort. Leurs adversaires leur prêtent la doctrine de la « double vérité » : une thèse pourrait être vraie en philosophie et fausse en théologie. En réalité, ils distinguent plutôt ce que conclut la raison et ce qu’enseigne la foi, à laquelle ils déclarent se soumettre. &lt;a href="https://fr.wikipedia.org/wiki/Thomas_d%27Aquin" title=" Wikipedia"&gt;Thomas d’Aquin&lt;/a&gt; les réfute dans &lt;em&gt;L’Unité de l’intellect&lt;/em&gt; (1270), et l’évêque de Paris, Étienne Tempier, condamne 219 thèses en 1277.&lt;/p&gt; &lt;p&gt;L’averroïsme se maintient pourtant, surtout à Padoue, jusqu’au XVIe siècle. Il a fait d’Averroès le symbole de l’indépendance de la raison, alors qu’il était presque oublié dans le monde musulman. Ernest Renan lui consacre en 1852 une étude célèbre, &lt;em&gt;Averroès et l’averroïsme&lt;/em&gt;.&lt;/p&gt;  &lt;audio controls title="S'inspirer de l'audace intellectuelle d'Averroes par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10073-12.05.2019-ITEMA_22059483-0.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F41" s="14" t="s">
         <v>223</v>
@@ -6548,8 +6556,10 @@
       <c r="D55" s="12" t="s">
         <v>295</v>
       </c>
-      <c r="E55" s="13" t="s">
-        <v>296</v>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Cart%C3%A9sianisme"   title=" Wikipedia"&gt;Le Cartésianisme&lt;/a&gt; désigne la philosophie de &lt;a href="https://fr.wikipedia.org/wiki/Ren%C3%A9_Descartes" title=" Wikipedia"&gt;René Descartes&lt;/a&gt; (1596-1650) et le mouvement qui la prolonge aux XVIIe et XVIIIe siècles. Contre l’autorité d’Aristote et de la scolastique, Descartes veut reconstruire tout le savoir sur des bases certaines, à partir de la seule raison. Le &lt;em&gt;Discours de la méthode&lt;/em&gt; (1637) et les &lt;em&gt;Méditations métaphysiques&lt;/em&gt; (1641) en posent les fondements.&lt;/p&gt; &lt;p&gt;Sa méthode commence par le doute : il faut rejeter tout ce qui peut être mis en question, les sens, qui nous trompent parfois, et même les mathématiques, qu’un « malin génie » pourrait fausser. Une certitude résiste : « je pense, donc je suis ». À partir d’elle, Descartes prouve l’existence de Dieu, garant de la vérité des idées claires et distinctes, puis celle du monde. Il distingue deux substances : la pensée, dont l’essence est de penser, et l’étendue, la matière, qui n’est que figure et mouvement. Le monde physique devient une immense machine, explicable par les mathématiques, et les animaux eux-mêmes sont des automates. Ce dualisme pose une difficulté célèbre, soulevée par la princesse Élisabeth : comment l’âme, qui n’est pas étendue, peut-elle mouvoir le corps ?&lt;/p&gt; &lt;p&gt;Ses successeurs tentent d’y répondre : &lt;a href="https://fr.wikipedia.org/wiki/Nicolas_Malebranche" title=" Wikipedia"&gt;Malebranche&lt;/a&gt; fait de Dieu la seule vraie cause, &lt;a href="https://fr.wikipedia.org/wiki/Baruch_Spinoza" title=" Wikipedia"&gt;Spinoza&lt;/a&gt; voit dans la pensée et l’étendue deux attributs d’une substance unique. Enseigné malgré les interdictions, le cartésianisme marque durablement la science et l’esprit français, associé à la clarté et à la méthode.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F55" s="11" t="s">
         <v>297</v>
@@ -7652,8 +7662,10 @@
       <c r="D77" s="15" t="s">
         <v>410</v>
       </c>
-      <c r="E77" s="16" t="s">
-        <v>411</v>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Anticolonialisme" title=" Wikipedia"&gt;L’Anticolonialisme&lt;/a&gt; désigne l’ensemble des pensées et des luttes qui contestent la colonisation, c’est-à-dire la domination d’un peuple par une puissance étrangère qui s’empare de ses terres, exploite ses ressources et lui impose ses lois. Il en conteste la légitimité morale, au nom de l’égalité des êtres humains, mais aussi l’utilité économique et les justifications culturelles, comme la prétendue « mission civilisatrice ».&lt;/p&gt; &lt;p&gt;Dès le XVIe siècle, &lt;a href="https://fr.wikipedia.org/wiki/Bartolom%C3%A9_de_las_Casas" title=" Wikipedia"&gt;Bartolomé de las Casas&lt;/a&gt; dénonce les massacres des Indiens d’Amérique et, lors de la controverse de Valladolid (1550), défend leur pleine humanité. Au XVIIIe siècle, les Lumières s’en prennent à l’esclavage et aux conquêtes : l’&lt;em&gt;Histoire des deux Indes&lt;/em&gt; de l’abbé Raynal, à laquelle &lt;a href="https://fr.wikipedia.org/wiki/Denis_Diderot" title=" Wikipedia"&gt;Diderot&lt;/a&gt; prête ses pages les plus violentes, appelle les colonisés à la révolte, et la révolution haïtienne, menée par Toussaint Louverture, fonde en 1804 la première république noire. Au XIXe siècle, des libéraux comme Bastiat jugent les colonies ruineuses, tandis que des socialistes et des anarchistes dénoncent leur violence. Au XXe siècle, Lénine lie l’impérialisme au capitalisme, et Gandhi oppose à l’Empire britannique la résistance non violente. Après 1945, l’anticolonialisme porte les luttes d’indépendance, en Asie puis en Afrique.&lt;/p&gt; &lt;p&gt;Ses grands textes sont le &lt;em&gt;Discours sur le colonialisme&lt;/em&gt; (1950) d’&lt;a href="https://fr.wikipedia.org/wiki/Aim%C3%A9_C%C3%A9saire" title=" Wikipedia"&gt;Aimé Césaire&lt;/a&gt; et &lt;em&gt;Les Damnés de la terre&lt;/em&gt; (1961) de &lt;a href="https://fr.wikipedia.org/wiki/Frantz_Fanon" title=" Wikipedia"&gt;Frantz Fanon&lt;/a&gt;. Les études postcoloniales et la pensée décoloniale prolongent aujourd’hui son analyse des effets durables de la colonisation.&lt;/p&gt;  &lt;audio controls title=" "Fanon": le biopic sur la figure de l'anticolonialisme est peu diffusé dans les cinémas mais agite les réseaux par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23694-08.04.2025-ITEMA_24096522-2025J49319S0098-NET_MLM_8C70D14C-38CF-46CE-811B-6AFD802BAF4A-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F77" s="14" t="inlineStr">
         <is>
@@ -8509,8 +8521,10 @@
       <c r="D94" s="12" t="s">
         <v>504</v>
       </c>
-      <c r="E94" s="13" t="s">
-        <v>505</v>
+      <c r="E94" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Populisme_(politique)"  style="color:#d35400"  title=" Wikipedia"&gt;Le Populisme&lt;/a&gt; désigne une conception de la politique qui oppose un « peuple » vertueux et uni à des « élites » jugées corrompues, et prétend exprimer directement la volonté populaire. Pour le politologue Cas Mudde, c’est une « idéologie mince » : elle ne propose pas de programme complet et se combine avec d’autres doctrines, le nationalisme à droite, le socialisme à gauche.&lt;/p&gt; &lt;p&gt;Le mot a d’abord désigné, en Russie, les &lt;a href="https://fr.wikipedia.org/wiki/Narodniki" title=" Wikipedia"&gt;narodniki&lt;/a&gt; des années 1860-1870 : de jeunes intellectuels qui « allaient au peuple » pour éveiller les paysans et fonder un socialisme sur la commune rurale, sans passer par le capitalisme. Aux États-Unis, le People’s Party des années 1890 défend les fermiers contre les banques et les compagnies de chemin de fer. Au XXe siècle, le péronisme, en Argentine, associe autour de &lt;a href="https://fr.wikipedia.org/wiki/Juan_Per%C3%B3n" title=" Wikipedia"&gt;Juan Perón&lt;/a&gt; un chef charismatique, les masses ouvrières et un nationalisme social. Depuis les années 1990, et plus encore après la crise de 2008, des partis populistes progressent en Europe et en Amérique. Leurs traits communs sont la méfiance envers les institutions représentatives, les médias et les experts, le goût du référendum et du lien direct entre le chef et le peuple, et une conception du peuple comme un tout homogène.&lt;/p&gt; &lt;p&gt;Pour Jan-Werner Müller, le populisme est dangereux parce qu’il refuse le pluralisme : ses adversaires sont exclus du « vrai peuple ». À l’inverse, &lt;a href="https://fr.wikipedia.org/wiki/Ernesto_Laclau" title=" Wikipedia"&gt;Ernesto Laclau&lt;/a&gt; y voit la logique même de toute construction politique d’un « nous ».&lt;/p&gt;  &lt;audio controls title=" Le populiste par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23497-01.09.2023-ITEMA_23473557-2023F49012S0245-27.m4a" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F94" s="11" t="s">
         <v>506</v>
@@ -9189,8 +9203,10 @@
       <c r="D107" s="15" t="s">
         <v>576</v>
       </c>
-      <c r="E107" s="16" t="s">
-        <v>577</v>
+      <c r="E107" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Agnosticisme" title=" Wikipedia"&gt;L’Agnosticisme&lt;/a&gt; est la position selon laquelle l’existence ou l’inexistence de Dieu, et plus largement toute réalité au-delà de l’expérience, ne peut pas être connue. L’agnostique ne croit pas en Dieu, comme le croyant, mais il n’affirme pas non plus qu’il n’existe pas, comme l’athée : il suspend son jugement, faute de preuves accessibles à la raison.&lt;/p&gt; &lt;p&gt;Le mot est forgé en 1869 par le biologiste anglais &lt;a href="https://fr.wikipedia.org/wiki/Thomas_Henry_Huxley" title=" Wikipedia"&gt;Thomas Huxley&lt;/a&gt;, ardent défenseur de Darwin, à partir du grec &lt;em&gt;agnôstos&lt;/em&gt;, « inconnu » : il voulait se distinguer des « gnostiques » de toute sorte, religieux ou matérialistes, qui prétendaient savoir. Mais l’attitude est ancienne. &lt;a href="https://fr.wikipedia.org/wiki/Protagoras" title=" Wikipedia"&gt;Protagoras&lt;/a&gt; déclarait déjà : « Des dieux, je ne puis savoir ni qu’ils sont, ni qu’ils ne sont pas. » Au XVIIIe siècle, &lt;a href="https://fr.wikipedia.org/wiki/David_Hume" title=" Wikipedia"&gt;David Hume&lt;/a&gt; montre la faiblesse des preuves de Dieu tirées de l’ordre du monde, et &lt;a href="https://fr.wikipedia.org/wiki/Emmanuel_Kant" title=" Wikipedia"&gt;Kant&lt;/a&gt; établit que la raison ne peut connaître ce qui dépasse l’expérience possible : l’existence de Dieu ne peut être ni démontrée ni réfutée, elle reste objet de foi. Au XIXe siècle, Herbert Spencer place l’« Inconnaissable » au fondement de toute chose.&lt;/p&gt; &lt;p&gt;On distingue un agnosticisme faible, qui dit simplement « je ne sais pas », et un agnosticisme fort, qui affirme que personne ne peut savoir. Bertrand Russell se disait agnostique en philosophie et athée dans la vie courante, faute d’avoir plus de raisons de croire en Dieu qu’aux dieux de l’Olympe. Pour ses critiques, croyants ou athées, l’agnosticisme est une manière commode d’éviter de choisir.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F107" s="14" t="s">
         <v>578</v>
@@ -9437,8 +9453,10 @@
       <c r="D112" s="12" t="s">
         <v>602</v>
       </c>
-      <c r="E112" s="13" t="s">
-        <v>603</v>
+      <c r="E112" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Meinongianisme" title=" Wikipedia"&gt;Le Meinongianisme&lt;/a&gt; désigne la théorie de l’objet du philosophe autrichien &lt;a href="https://fr.wikipedia.org/wiki/Alexius_Meinong" title=" Wikipedia"&gt;Alexius Meinong&lt;/a&gt; (1853-1920) et les doctrines qui s’en inspirent. Sa thèse paraît paradoxale : il y a des objets qui n’existent pas. Quand je pense à la montagne d’or ou au cercle carré, ma pensée porte bien sur quelque chose, même si cela n’existe nulle part.&lt;/p&gt; &lt;p&gt;Élève de &lt;a href="https://fr.wikipedia.org/wiki/Franz_Brentano" title=" Wikipedia"&gt;Franz Brentano&lt;/a&gt;, Meinong part de l’intentionnalité : toute pensée est pensée de quelque chose. Il en conclut que le domaine des objets est plus vaste que celui de l’existence. Certains objets existent, comme les choses physiques ; d’autres « subsistent » sans être dans l’espace et le temps, comme les nombres ou les relations ; d’autres enfin ne sont d’aucune façon, comme la montagne d’or, et même le cercle carré, qui est impossible. Tous ont pourtant des propriétés : la montagne d’or est dorée, le cercle carré est rond et carré. C’est le principe d’indépendance de l’être-tel à l’égard de l’être, exposé dans la &lt;em&gt;Théorie de l’objet&lt;/em&gt; (1904). Il permet d’expliquer comment on peut dire des choses vraies de Sherlock Holmes ou nier l’existence de Pégase.&lt;/p&gt; &lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bertrand_Russell" title=" Wikipedia"&gt;Bertrand Russell&lt;/a&gt; le critique en 1905 avec sa théorie des descriptions, qui analyse « la montagne d’or » sans lui supposer d’objet, et Quine raille cette « jungle » d’entités. Depuis les années 1970, des néo-meinongiens comme Terence Parsons, Richard Routley ou Graham Priest l’ont réhabilité grâce à la logique moderne.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F112" s="11" t="s">
         <v>604</v>
@@ -10086,8 +10104,10 @@
       <c r="D125" s="17" t="s">
         <v>670</v>
       </c>
-      <c r="E125" s="25" t="s">
-        <v>671</v>
+      <c r="E125" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Comportementalisme" title=" Wikipedia"&gt;Le Béhaviorisme&lt;/a&gt;, ou comportementalisme, de l’anglais &lt;em&gt;behavior&lt;/em&gt;, « comportement », est un courant de la psychologie selon lequel celle-ci doit étudier uniquement les comportements observables, et non la conscience ou les états mentaux, qui échappent à la mesure. Il naît aux États-Unis avec le manifeste de &lt;a href="https://fr.wikipedia.org/wiki/John_Broadus_Watson" title=" Wikipedia"&gt;John B. Watson&lt;/a&gt;, &lt;em&gt;La psychologie telle que le béhavioriste la voit&lt;/em&gt; (1913), et domine la psychologie américaine jusqu’aux années 1950.&lt;/p&gt; &lt;p&gt;Il s’appuie sur les travaux du physiologiste russe &lt;a href="https://fr.wikipedia.org/wiki/Ivan_Pavlov" title=" Wikipedia"&gt;Ivan Pavlov&lt;/a&gt; sur le réflexe conditionné : un chien qui entend une sonnerie avant chaque repas finit par saliver au seul son de la sonnerie. Watson en tire un schéma stimulus-réponse et soutient que l’éducation peut tout : qu’on lui donne une douzaine d’enfants bien portants, il en fera ce qu’on voudra. &lt;a href="https://fr.wikipedia.org/wiki/Burrhus_Frederic_Skinner" title=" Wikipedia"&gt;B. F. Skinner&lt;/a&gt; développe ensuite le conditionnement opérant : un comportement suivi d’une récompense tend à se répéter, un comportement puni tend à disparaître. Il en tire des méthodes d’enseignement programmé et même, dans &lt;em&gt;Walden Two&lt;/em&gt; (1948), l’utopie d’une société réglée par le conditionnement. En philosophie, un béhaviorisme logique, chez Gilbert Ryle ou Carl Hempel, analyse les mots qui désignent des états mentaux comme des dispositions à agir.&lt;/p&gt; &lt;p&gt;En 1959, &lt;a href="https://fr.wikipedia.org/wiki/Noam_Chomsky" title=" Wikipedia"&gt;Noam Chomsky&lt;/a&gt; montre que l’apprentissage du langage ne s’explique pas par le seul conditionnement : c’est le début de la révolution cognitive. Le béhaviorisme survit dans les thérapies comportementales.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F125" s="1" t="s">
         <v>672</v>
@@ -10127,8 +10147,10 @@
       <c r="D126" s="17" t="s">
         <v>675</v>
       </c>
-      <c r="E126" s="3" t="s">
-        <v>676</v>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Individualisme_m%C3%A9thodologique" title=" Wikipedia"&gt;L’Individualisme méthodologique&lt;/a&gt; est un principe des sciences sociales selon lequel tout phénomène collectif, une institution, un marché, une révolution ou une mode, doit être expliqué à partir des actions, des croyances et des raisons des individus qui y participent. Il ne nie pas l’existence de la société, mais refuse de la traiter comme un sujet qui agirait par lui-même. L’expression est forgée en 1908 par l’économiste autrichien Joseph Schumpeter.&lt;/p&gt; &lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Max_Weber" title=" Wikipedia"&gt;Max Weber&lt;/a&gt; en pose les bases : la sociologie doit comprendre l’action sociale à partir du sens que les acteurs lui donnent. L’école autrichienne d’économie, de Carl Menger à Friedrich Hayek, explique les prix ou la monnaie comme des résultats non voulus d’actions individuelles. &lt;a href="https://fr.wikipedia.org/wiki/Karl_Popper" title=" Wikipedia"&gt;Karl Popper&lt;/a&gt; en fait une règle de méthode contre les grandes philosophies de l’histoire : la « société », la « classe » ou la « nation » n’agissent jamais, seuls les individus agissent. En France, &lt;a href="https://fr.wikipedia.org/wiki/Raymond_Boudon" title=" Wikipedia"&gt;Raymond Boudon&lt;/a&gt; en donne une version influente : les individus ont de bonnes raisons d’agir comme ils le font, et l’agrégation de leurs choix produit souvent des « effets pervers » que personne n’a voulus, comme les embouteillages ou l’inflation des diplômes.&lt;/p&gt; &lt;p&gt;Il s’oppose au holisme d’&lt;a href="https://fr.wikipedia.org/wiki/%C3%89mile_Durkheim" title=" Wikipedia"&gt;Émile Durkheim&lt;/a&gt;, pour qui les faits sociaux s’imposent aux individus et doivent être expliqués par d’autres faits sociaux. Le débat traverse toujours l’économie, la sociologie et la théorie du choix rationnel.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F126" s="1" t="s">
         <v>677</v>
@@ -10267,8 +10289,10 @@
       <c r="D129" s="12" t="s">
         <v>693</v>
       </c>
-      <c r="E129" s="26" t="s">
-        <v>694</v>
+      <c r="E129" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Nationalisme_int%C3%A9gral"  title=" Wikipedia"&gt;Le Maurrassisme&lt;/a&gt; désigne la doctrine de l’écrivain &lt;a href="https://fr.wikipedia.org/wiki/Charles_Maurras" title=" Wikipedia"&gt;Charles Maurras&lt;/a&gt; (1868-1952), qu’il appelle lui-même « nationalisme intégral ». Née dans le contexte de l’affaire Dreyfus, où Maurras prend parti contre Dreyfus, elle devient celle de l’&lt;a href="https://fr.wikipedia.org/wiki/Action_fran%C3%A7aise" title=" Wikipedia"&gt;Action française&lt;/a&gt;, mouvement et quotidien qui exercent une forte influence sur la droite française, de la Belle Époque aux années 1930.&lt;/p&gt; &lt;p&gt;Maurras se veut positiviste, disciple d’Auguste Comte : il entend fonder la politique sur l’observation des faits, un « empirisme organisateur », et non sur des principes abstraits. Il en conclut que la Révolution française et ses idées, la démocratie, l’individualisme, le romantisme, ont affaibli la France, et que seule une monarchie héréditaire, antiparlementaire et décentralisée peut garantir l’ordre et la continuité de la nation. Agnostique, il défend pourtant l’Église catholique comme facteur d’ordre. Sa formule « politique d’abord » subordonne tout à l’intérêt national. Le maurrassisme désigne aussi des ennemis intérieurs, les « quatre États confédérés » : juifs, protestants, francs-maçons et « métèques ». Cet antisémitisme d’État est au cœur de la doctrine.&lt;/p&gt; &lt;p&gt;Condamnée par le pape en 1926, l’Action française soutient le régime de Vichy, dont Maurras salue l’avènement comme une « divine surprise » ; il est condamné en 1945 à la réclusion à perpétuité. Son influence sur des écrivains comme Bernanos ou Maritain, dans leur jeunesse, reste un sujet d’étude et de controverse.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F129" s="11" t="s">
         <v>695</v>
@@ -11015,8 +11039,10 @@
       <c r="D144" s="15" t="s">
         <v>775</v>
       </c>
-      <c r="E144" s="29" t="s">
-        <v>776</v>
+      <c r="E144" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/R%C3%A9ductionnisme" title=" Wikipedia"&gt;Le Réductionnisme&lt;/a&gt; est la thèse selon laquelle un phénomène complexe peut être expliqué entièrement à partir de ses éléments les plus simples : le vivant par la chimie, la chimie par la physique, l’esprit par le cerveau. Il prend deux formes : un réductionnisme de méthode, qui décompose un problème pour l’étudier, et un réductionnisme de principe, qui affirme que le tout n’est rien d’autre que ses parties.&lt;/p&gt; &lt;p&gt;L’idée remonte à l’atomisme antique et à Descartes, qui conseille de diviser chaque difficulté « en autant de parcelles qu’il se pourrait ». Elle triomphe avec la science moderne : la physique explique la chaleur par le mouvement des molécules, et la biologie moléculaire, après la découverte de la structure de l’ADN en 1953, explique l’hérédité par la chimie. Au milieu du XXe siècle, les positivistes logiques rêvent d’une science unifiée, et le philosophe &lt;a href="https://fr.wikipedia.org/wiki/Ernest_Nagel" title=" Wikipedia"&gt;Ernest Nagel&lt;/a&gt; définit en 1961 la réduction d’une théorie à une autre, comme celle de la thermodynamique à la mécanique statistique. En philosophie de l’esprit, la théorie de l’identité, chez J. J. C. Smart, affirme que les états mentaux sont des états du cerveau.&lt;/p&gt; &lt;p&gt;Ses adversaires lui opposent l’&lt;a href="https://fr.wikipedia.org/wiki/%C3%89mergence" title=" Wikipedia"&gt;émergence&lt;/a&gt; : à chaque niveau d’organisation apparaissent des propriétés nouvelles. Le &lt;a href="https://fr.wikipedia.org/wiki/Holisme" title=" Wikipedia"&gt;holisme&lt;/a&gt; soutient que le tout est plus que la somme de ses parties, et &lt;a href="https://fr.wikipedia.org/wiki/Thomas_Nagel" title=" Wikipedia"&gt;Thomas Nagel&lt;/a&gt; objecte que l’expérience vécue échappe à toute description physique : savoir tout du cerveau d’une chauve-souris ne dit pas ce que cela fait d’être une chauve-souris.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F144" s="14" t="s">
         <v>777</v>
@@ -11117,8 +11143,10 @@
       <c r="D146" s="15" t="s">
         <v>786</v>
       </c>
-      <c r="E146" s="16" t="s">
-        <v>787</v>
+      <c r="E146" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Tiers-mondisme"  title=" Wikipedia"&gt;Le Tiers-mondisme&lt;/a&gt; est un courant de pensée politique né dans les années 1950, qui place au centre de l’histoire les peuples d’Asie, d’Afrique et d’Amérique latine, alors en pleine décolonisation, et défend leur émancipation face aux deux blocs de la guerre froide. L’expression « tiers-monde » est forgée en 1952 par le démographe &lt;a href="https://fr.wikipedia.org/wiki/Alfred_Sauvy" title=" Wikipedia"&gt;Alfred Sauvy&lt;/a&gt;, par allusion au tiers état de 1789 : ce tiers-monde « ignoré, exploité, méprisé » veut « lui aussi être quelque chose ».&lt;/p&gt; &lt;p&gt;En 1955, la &lt;a href="https://fr.wikipedia.org/wiki/Conf%C3%A9rence_de_Bandung" title=" Wikipedia"&gt;conférence de Bandung&lt;/a&gt; réunit 29 pays d’Asie et d’Afrique autour de Nehru, Nasser, Sukarno et Zhou Enlai ; elle annonce le mouvement des non-alignés, fondé en 1961. Le tiers-mondisme y ajoute une analyse : la pauvreté du Sud ne vient pas d’un simple retard, mais de la domination du Nord, par la colonisation, puis par l’échange inégal, la dette et les firmes multinationales. Les théoriciens de la dépendance, comme Samir Amin ou André Gunder Frank, le formulent en termes économiques. &lt;a href="https://fr.wikipedia.org/wiki/Frantz_Fanon" title=" Wikipedia"&gt;Frantz Fanon&lt;/a&gt;, dans &lt;em&gt;Les Damnés de la terre&lt;/em&gt; (1961), préfacé par Sartre, voit dans les paysans colonisés la nouvelle force révolutionnaire. En France, le courant marque la gauche après la guerre d’Algérie et Mai 68, de Che Guevara à la solidarité avec le Vietnam.&lt;/p&gt; &lt;p&gt;À partir des années 1980, il recule, avec l’échec de plusieurs régimes révolutionnaires, l’essor des pays d’Asie et des critiques comme &lt;em&gt;Le Sanglot de l’homme blanc&lt;/em&gt; (1983) de Pascal Bruckner. L’altermondialisme et la pensée décoloniale en ont repris certains thèmes.&lt;/p&gt;  &lt;audio controls title=" Agronomie et tiers-mondisme par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/17362-04.07.2023-ITEMA_23431389-2023C35448S0185-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F146" s="14" t="s">
         <v>788</v>

</xml_diff>

<commit_message>
Corrections de forme sur 342 fiches (bilan, point 2) : adresses web collées en clair retirées (26), listes à tirets et lignes <dd> remises en paragraphes (188), formules de remplissage « Voici… : » / « On peut dire qu'il… » supprimées (37), paragraphes vides retirés ; liens du nom corrigés (Morioka, Massignon, Persaios, Olympiodore, Pomponazzi, Huxley ; courants Occidentalisme, Jdanovisme, Wokisme) ; lien cassé de Gersonide et trois titres de liens réparés ; noms corrigés Leo Strauss, Carlos Vaz-Ferreira, Marilyn McCord-Adams, Bonaventure, Javier Muguerza, Jacob Osis (301 depuis les anciennes adresses)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -4059,8 +4059,13 @@
       <c r="D5" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="16" t="s">
-        <v>23</v>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pr%C3%A9socratiques"  style="color:#d35400"  title=" Wikipedia"&gt; Le courant Présocratique&lt;/a&gt; est une période importante de l'histoire de la philosophie occidentale qui s'étend du VIe siècle av. J.-C. jusqu'à l'avènement de Socrate au Ve siècle av. J.-C.&lt;/p&gt; &lt;p&gt; Les philosophes présocratiques ont jeté les bases de la philosophie grecque en posant des questions sur la nature, l'existence, la réalité et la connaissance et en cherchant à répondre à ces questions par le raisonnement logique et la spéculation philosophique.&lt;/p&gt;
+&lt;p&gt;Les philosophes présocratiques ont abordé des sujets variés, allant de la cosmologie à la métaphysique en passant par la philosophie de la connaissance. Parmi les plus célèbres, on peut citer Pittacos de Mytilene, Thalès de Milet, Anaximandre, Héraclite, Parménide.&lt;/p&gt;
+&lt;p&gt;Thalès de Milet a cherché à comprendre la nature de l'univers en affirmant que tout était constitué d'eau. Anaximandre a proposé l'idée que la réalité ultime était quelque chose d'indéfini et d'illimité, qu'il a appelé l'apeiron. Héraclite, quant à lui, a affirmé que tout était en mouvement constant et que le changement était la seule constante de l'univers.&lt;/p&gt;
+&lt;p&gt;Parménide a proposé une philosophie de la permanence et de l'immuabilité en affirmant que le monde sensible était une illusion, tandis que la réalité ultime était immuable et éternelle. Empédocle, pour sa part, a développé une théorie de la nature basée sur les quatre éléments : la terre, l'eau, l'air et le feu.&lt;/p&gt; &lt;audio controls title="Les présocratiques sont ils à l'origine de la philosophie ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/22788-01.09.2021-ITEMA_22759722-2021C45539E0003.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
+        </is>
       </c>
       <c r="F5" s="14" t="s">
         <v>24</v>
@@ -4461,8 +4466,12 @@
       <c r="D13" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="E13" s="16" t="s">
-        <v>66</v>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/H%C3%A9donisme"  style="color:#d35400"  title=" Wikipedia"&gt; L'hédonisme&lt;/a&gt; est une philosophie qui met l'accent sur la recherche du plaisir et l'évitement de la douleur. Le terme "hédonisme" vient du mot grec "hedone", qui signifie plaisir. &lt;/p&gt; &lt;p&gt; L'une des premières écoles hédonistes était l'école cyrénaïque, fondée par Aristippe de Cyrène au IVe siècle avant notre ère. Les cyrénaïques considéraient que le plaisir était le but ultime de la vie et qu'il fallait chercher à maximiser les plaisirs immédiats. Ils distinguaient les plaisirs corporels des plaisirs de l'esprit, mais accordaient une importance particulière aux plaisirs sensoriels. &lt;/p&gt; &lt;p&gt;  Cependant, il existe différentes variantes de l'hédonisme et des débats sur la nature du plaisir et sur la manière de le poursuivre de façon éthique et équilibrée. Certains hédonistes soutiennent que le plaisir physique, comme les sensations agréables, les plaisirs sensoriels ou sexuels, est le seul type de plaisir qui compte. D'autres formes d'hédonisme accordent de l'importance aux plaisirs intellectuels, esthétiques ou émotionnels, tels que l'appréciation de la beauté, la satisfaction intellectuelle ou les émotions positives. &lt;/p&gt; &lt;p&gt; 
+l'hédonisme ne se limite pas à une quête égoïste de plaisir immédiat mais soutiennent qu'une vie agréable et satisfaisante implique également une recherche du bien-être à long terme, en évitant les plaisirs fugaces qui pourraient entraîner des souffrances futures. &lt;/p&gt;   &lt;audio controls title="L'hédonisme antique ou le calcul des plaisirs par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-27.06.2016-ITEMA_21019965-1.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+</t>
+        </is>
       </c>
       <c r="F13" s="14" t="s">
         <v>67</v>
@@ -4608,8 +4617,15 @@
       <c r="D16" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="13" t="s">
-        <v>85</v>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Atomisme"  style="color:#d35400"  title=" Wikipedia"&gt; L'Atomisme&lt;/a&gt; est une théorie philosophique qui remonte à l'Antiquité grecque et qui soutient que tout ce qui existe est constitué d'atomes, c'est-à-dire de particules indivisibles et immuables. Cette théorie est souvent associée aux philosophes grecs Leucippe et Démocrite.&lt;/p&gt;
+&lt;p&gt;Selon l'atomisme, les atomes sont les éléments fondamentaux de l'univers, et tout ce qui existe peut être expliqué en termes de la manière dont les atomes interagissent entre eux. Les atomes sont considérés comme étant éternels et indestructibles, et ils sont en constante mouvement dans le vide.&lt;/p&gt;
+&lt;p&gt;Les atomistes considéraient que les propriétés des objets, telles que leur couleur, leur goût ou leur odeur, ne sont que des perceptions subjectives de l'observateur et ne reflètent pas les propriétés réelles des atomes qui les composent. Cette théorie a conduit à la distinction entre les qualités primaires, telles que la taille, la forme et la position, qui sont considérées comme des propriétés objectives des atomes, et les qualités secondaires, telles que la couleur et le goût, qui sont considérées comme des propriétés subjectives des observateurs.&lt;/p&gt;
+&lt;p&gt;Il eu des implications importantes en physique, car il a permis aux atomistes de développer des théories sur la nature de la matière, de l'espace et du mouvement. Par exemple, Épicure a proposé une théorie selon laquelle les atomes se déplacent dans le vide par leur propre poids, ce qui a influencé la théorie de la gravité développée par Isaac Newton des siècles plus tard.&lt;/p&gt;
+&lt;audio controls title="L'atomisme est il une philosophie encore valable ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/21713-13.10.2020-ITEMA_22454354-2020C41495S0287-1779455909.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+</t>
+        </is>
       </c>
       <c r="F16" s="11" t="s">
         <v>86</v>
@@ -4710,8 +4726,10 @@
       <c r="D18" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="E18" s="13" t="s">
-        <v>96</v>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Relativisme"  title=" Wikipedia Le relativisme"&gt;Le Relativisme&lt;/a&gt; est une perspective philosophique qui affirme que la vérité, la moralité, la réalité, ou d'autres concepts similaires sont relatifs et dépendent du contexte, de la culture, de la perspective individuelle ou d'autres facteurs.&lt;/p&gt; &lt;p&gt;Il existe plusieurs formes de relativisme, notamment le relativisme épistémique, le relativisme moral et le relativisme culturel. &lt;/p&gt; &lt;p&gt;RELATIVISME ÉPISTÉMIQUE : Cela concerne la vérité et la connaissance. Les relativistes épistémiques soutiennent que la vérité dépend du point de vue de l'observateur ou de la culture dans laquelle il se trouve. Ils remettent en question l'existence d'une vérité objective et universelle. &lt;/p&gt; &lt;p&gt;RELATIVISME MORAL : Cela concerne la moralité et l'éthique. Les relativistes moraux affirment que les jugements moraux dépendent des croyances culturelles, individuelles ou sociales, et qu'il n'y a pas de normes morales objectives qui s'appliquent universellement. &lt;/p&gt; &lt;p&gt;RELATIVISME CULTUREL : C'est l'idée que les différentes cultures ont des systèmes de valeurs et de normes morales qui leur sont propres, et qu'il n'est pas approprié de juger une culture en utilisant les critères d'une autre. &lt;/p&gt; &lt;p&gt;Cependant, le relativisme philosophique suscite également des critiques. Certains estiment qu'il peut conduire au scepticisme excessif, rendant difficile voire impossible le dialogue interculturel ou la recherche d'une vérité partagée. D'autres soutiennent que certaines valeurs universelles existent malgré les différences culturelles.. Cependant, il convient de noter que le relativisme a également été un moyen de promouvoir la tolérance culturelle et le respect des différences, en reconnaissant la diversité des valeurs et des perspectives à travers le monde. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F18" s="11" t="s">
         <v>97</v>
@@ -4823,8 +4841,16 @@
       <c r="D20" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="E20" s="16" t="s">
-        <v>103</v>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Id%C3%A9alisme_(philosophie)"  style="color:#d35400"  title=" Wikipedia"&gt; L'Idéalisme&lt;/a&gt; est une approche philosophique qui accorde une importance primordiale à l'esprit, à la conscience et aux idées en tant que réalités fondamentales. Il soutient que la réalité ultime est de nature mentale ou conceptuelle, plutôt que matérielle et remet en question la conception selon laquelle le monde extérieur existe indépendamment de notre perception et propose que notre conscience joue un rôle actif dans la construction de la réalité. &lt;/p&gt; &lt;p&gt; 
+L'idéalisme a une longue histoire et a été développé par de nombreux philosophes à travers les âges. Parmi les penseurs majeurs associés à l'idéalisme, on trouve Platon, George Berkeley, Emmanuel Kant, Friedrich Hegel et Arthur Schopenhauer. &lt;/p&gt; &lt;p&gt; 
+Une des formes les plus célèbres d'idéalisme est l'idéalisme platonicien. Selon Platon, le monde des idées, qui est constitué de concepts abstraits et éternels tels que la beauté, la justice et la vérité, est plus réel que le monde matériel sensible que nous percevons avec nos sens. Pour Platon, les objets physiques ne sont que des reflets imparfaits des idées parfaites et immuables. &lt;/p&gt; &lt;p&gt; 
+L'idéalisme subjectif, également connu sous le nom de solipsisme, soutient que seule notre conscience individuelle est certaine et que tout le reste du monde est une construction de notre esprit. Cependant, cette forme d'idéalisme est souvent considérée comme extrême et controversée. &lt;/p&gt; &lt;p&gt; 
+Une autre forme importante d'idéalisme est l'idéalisme transcendantal d'Emmanuel Kant qui a soutenu que notre perception de la réalité est structurée par les catégories de l'esprit humain et que nous ne pouvons connaître que la réalité telle qu'elle est filtrée par nos facultés cognitives. Il a distingué entre le "noumène", la réalité en soi, et le "phénomène", la réalité telle que nous la percevons. &lt;/p&gt; &lt;p&gt;  
+L'idéalisme allemand, représenté principalement par Hegel, a proposé que l'esprit absolu est à la fois la source et la réalité ultime de tout ce qui existe. Selon lui, l'histoire est le processus dialectique de développement de l'esprit vers une compréhension plus complète de lui-même. L'idéalisme de Hegel a eu une influence significative sur d'autres courants de pensée, y compris le marxisme.&lt;/p&gt; &lt;p&gt; 
+Il convient de noter que l'idéalisme est souvent critiqué pour son éloignement de la réalité matérielle et sa propension à négliger l'importance des facteurs matériels et physiques dans la construction de la réalité. Cependant, l'idéalisme a également apporté des contributions importantes à la philosophie en mettant l'accent sur l'importance de la conscience, de la pensée et des idées dans notre compréhension du monde. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F20" s="14" t="s">
         <v>104</v>
@@ -5022,8 +5048,13 @@
       <c r="D24" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="E24" s="13" t="s">
-        <v>127</v>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Scepticisme_(philosophie)"  style="color:#d35400"  title=" Wikipedia"&gt; Le Scepticisme&lt;/a&gt;  est une position philosophique qui remet en question la capacité de la raison humaine à atteindre une connaissance certaine et indubitable.&lt;/p&gt; &lt;p&gt;Les sceptiques affirment que toutes les croyances et les connaissances que nous possédons sont sujettes à une certaine incertitude et qu'il est impossible de savoir avec certitude si quelque chose est vrai ou non.&lt;/p&gt;
+&lt;p&gt;Il existe plusieurs types de scepticisme en philosophie, le scepticisme radical, par exemple, nie la possibilité de toute connaissance certaine, tandis que le scepticisme mitigé admet qu'il est possible d'acquérir une certaine connaissance, mais seulement dans des domaines limités.&lt;/p&gt;
+&lt;p&gt;Les sceptiques remettent souvent en question les méthodes et les critères utilisés pour parvenir à la connaissance. Par exemple, ils peuvent soutenir que les sens ne sont pas fiables, que les raisonnements logiques ne sont pas infaillibles, ou que les croyances sont influencées par des préjugés et des perspectives individuelles.&lt;/p&gt;
+&lt;p&gt;Le scepticisme a eu une influence importante sur la philosophie occidentale, notamment dans l'Antiquité grecque avec les philosophes Pyrrhon et Sextus Empiricus, ainsi que dans la période moderne avec des penseurs tels que David Hume et a joué un rôle important dans la naissance de la méthode scientifique, en remettant en question les idées reçues et en encourageant une approche critique et rigoureuse de la recherche de la vérité.&lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F24" s="11" t="s">
         <v>128</v>
@@ -5422,8 +5453,17 @@
       <c r="D32" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="E32" s="13" t="s">
-        <v>175</v>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Augustinisme"  style="color:#d35400"  title=" Wikipedia"&gt;  L'Augustinisme&lt;/a&gt; est une école de pensée philosophique et théologique qui se base sur les idées de Saint Augustin d'Hippone, l'un des Pères de l'Église les plus influents de l'histoire du christianisme.&lt;/p&gt;
+&lt;p&gt; Il  a développé une vision de l'existence humaine qui mettait l'accent sur la condition pécheresse de l'humanité et la nécessité d'une grâce divine pour atteindre la vie éternelle.
+Parmi les idées clés de l'augustinisme, on peut citer :&lt;/p&gt;
+&lt;p&gt;Le concept de "péché originel", qui est l'idée que tous les êtres humains sont nés dans le péché à cause de la désobéissance d'Adam et Ève dans le jardin d'Eden. Selon cette conception, le péché est hérité de génération en génération et ne peut être surmonté que par la grâce divine.&lt;/p&gt;
+&lt;p&gt;La doctrine de la "prédestination", qui est l'idée que Dieu a choisi à l'avance ceux qui seront sauvés et ceux qui ne le seront pas. Cela est basé sur  Dieu et la totale dépendance de l'homme envers lui.&lt;/p&gt;
+&lt;p&gt;La distinction entre la "cité de Dieu" et la "cité des hommes", qui sont deux communautés qui coexistent dans le monde. La "cité de Dieu" représente ceux qui sont destinés à la vie éternelle, tandis que la "cité des hommes" représente ceux qui ne sont pas destinés à la vie éternelle.&lt;/p&gt;
+&lt;p&gt;La philosophie de l'histoire, qui est l'idée que l'histoire est guidée par la volonté de Dieu et que les événements historiques sont le résultat de son plan divin.&lt;/p&gt;
+&lt;p&gt;La conception de la trinité, qui est l'idée que Dieu existe en trois personnes distinctes : le Père, le Fils et le Saint-Esprit. Cette conception est basée sur les enseignements bibliques et a été développée plus tard par d'autres penseurs chrétiens.&lt;/p&gt; &lt;p&gt; L'Augustinisme a eu une influence considérable sur la théologie chrétienne, la philosophie et la pensée politique occidentale. Ses idées ont façonné notre compréhension de la nature humaine, de la relation entre l'homme et Dieu, de la destinée humaine et de l'histoire.&lt;/p&gt; &lt;audio controls title="Sacré Saint Augustin:qu'est ce que le temps ? par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2013/09/s38/NET_FC_deace614-efd1-4d2e-a113-a95f532c9f74.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
+        </is>
       </c>
       <c r="F32" s="11" t="s">
         <v>176</v>
@@ -5525,8 +5565,14 @@
       <c r="D34" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="E34" s="13" t="s">
-        <v>187</v>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Scolastique"  style="color:#d35400"  title=" Wikipedia"&gt; La Scolastique&lt;/a&gt; était un mouvement intellectuel et philosophique qui a émergé en Europe occidentale au Moyen Âge, principalement dans les universités médiévales entre le 11ème et le 14ème siècle. Les scolastiques cherchaient à intégrer la philosophie aristotélicienne avec la théologie chrétienne.&lt;/p&gt; &lt;p&gt;
+Les scolastiques croyaient que la raison et la foi étaient complémentaires et pouvaient être utilisées pour comprendre la vérité divine. Ils ont cherché à développer une méthode de raisonnement rigoureuse qui pourrait être utilisée pour résoudre les questions théologiques complexes. Cette méthode était appelée la « dispute » et impliquait l'utilisation de raisonnements logiques pour débattre d'un sujet particulier.&lt;/p&gt; &lt;p&gt; 
+Les scolastiques ont produit de nombreuses œuvres importantes, notamment la Summa Theologica de Thomas d'Aquin et les Commentaires sur Aristote de Saint Albert le Grand. Ils ont également contribué à développer la logique formelle et l'analyse sémantique, ainsi qu'à influencer le développement de la science moderne.&lt;/p&gt; &lt;p&gt;
+La scolastique a été largement remplacée par la Renaissance et la Réforme protestante, mais elle a laissé un héritage important dans la pensée occidentale et a influencé de nombreux domaines de la connaissance, notamment la philosophie, la théologie, la science et la littérature. &lt;/p&gt;   &lt;audio controls title="La scolastique et les démons par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2011/04/s13/RF_5A85A561-0848-4E1F-8A5C-9D1F13AAD9F6_GENE.MP3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+</t>
+        </is>
       </c>
       <c r="F34" s="11" t="s">
         <v>188</v>
@@ -5574,8 +5620,12 @@
       <c r="D35" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="E35" s="16" t="s">
-        <v>192</v>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Dualisme_(philosophie)"  style="color:#d35400"  title=" Wikipedia"&gt; Le Dualisme&lt;/a&gt; est une théorie philosophique qui postule l'existence de deux substances fondamentales distinctes : le corps et l'esprit.  A partir du XIe siècle, une forme de philosophie dualiste commence à se développer avec le renouveau en Chine du confucianisme. Zhu Xi est l'un des principaux représentants de ce courant néoconfucianiste dont il clarifie les thèses vers la seconde moitié du XIIe siècle. Cependant, c'est René Descartes, philosophe français du XVIIe siècle, qui est souvent considéré comme le fondateur du dualisme moderne. &lt;/p&gt; &lt;p&gt; 
+Descartes croyait que l'esprit était une substance non physique, immatérielle et indépendante du corps, tandis que le corps était une substance physique qui pouvait être étudiée scientifiquement. Cette distinction entre l'esprit et le corps est souvent appelée la dualité cartésienne. Selon lui, l'esprit est responsable de la pensée, de la conscience et de la volonté, tandis que le corps est responsable des mouvements et des sensations physiques. &lt;/p&gt; &lt;p&gt; 
+Le dualisme a suscité des débats et des critiques depuis sa formulation par Descartes. Certains philosophes ont argumenté que la théorie du dualisme est problématique car elle ne peut pas expliquer comment l'esprit et le corps interagissent. D'autres ont soutenu que la distinction entre l'esprit et le corps est artificielle et que les deux sont en fait étroitement liés. Malgré ces critiques, le dualisme reste une théorie importante dans la philosophie de l'esprit et continue d'être discuté et étudié par les philosophes contemporains.  &lt;/p&gt;  </t>
+        </is>
       </c>
       <c r="F35" s="14" t="s">
         <v>193</v>
@@ -5620,8 +5670,13 @@
       <c r="D36" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="E36" s="13" t="s">
-        <v>198</v>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Conceptualisme"  style="color:#d35400"  title=" Wikipedia"&gt; Le Conceptualisme&lt;/a&gt; est une théorie philosophique qui a émergé pendant la période médiévale, principalement en réaction aux débats entre les réalistes et les nominalistes. Le conceptualisme affirme que les concepts ou les universaux (c'est-à-dire les idées générales qui se réfèrent à plusieurs objets particuliers) existent, mais qu'ils ne sont pas des entités indépendantes de l'esprit humain. &lt;/p&gt; &lt;p&gt;
+Selon les conceptualistes, les concepts sont des créations mentales qui résultent de l'activité de l'esprit humain lorsqu'il catégorise ou généralise les objets particuliers. Les universaux ne sont donc pas des réalités indépendantes, mais plutôt des produits de l'activité mentale humaine. &lt;/p&gt; &lt;p&gt; 
+Le conceptualisme a été développé par des philosophes tels que Pierre Abélard, Jean Buridan et Guillaume d'Ockham. Cette théorie a eu une influence importante sur la pensée médiévale et a été largement adoptée par les universités européennes. &lt;/p&gt; &lt;p&gt; 
+Le conceptualisme a également eu un impact sur le développement de la philosophie moderne. Par exemple, la distinction entre les idées innées et les idées acquises a été remise en question par les conceptualistes, qui ont affirmé que toutes les idées étaient acquises par l'expérience et l'activité mentale. Cette idée a ensuite été développée par des philosophes tels que John Locke et David Hume. &lt;/p&gt;   </t>
+        </is>
       </c>
       <c r="F36" s="11" t="s">
         <v>199</v>
@@ -5669,8 +5724,14 @@
       <c r="D37" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="E37" s="16" t="s">
-        <v>204</v>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Nominalisme"  title=" Wikipedia"&gt; Le Nominalisme&lt;/a&gt; est une position philosophique donc Jean Roscelin est le principal fondateur et qui traite de la nature des universaux. &lt;a href="https://fr.wikipedia.org/wiki/Universaux"  style="color:#6A142A"  title=" Wikipedia"&gt; Les Universaux&lt;/a&gt; sont des concepts abstraits tels que les idées, les propriétés ou les relations qui peuvent être appliqués à des objets particuliers. &lt;/p&gt; &lt;p&gt; 
+Selon les nominalistes, les universaux n'ont pas d'existence réelle ou indépendante en dehors de l'esprit humain. Ils soutiennent que les universaux ne sont que des noms ou des étiquettes que nous attribuons aux regroupements d'objets similaires en raison de leurs caractéristiques communes et qu' il est important de le comparer avec une autre position philosophique appelée réalisme. Les réalistes soutiennent que les universaux ont une existence indépendante et objective dans le monde. Selon leur perspective, il existe une réalité universelle ou une essence partagée entre les objets qui justifie notre capacité à les classer et à leur attribuer des propriétés communes. &lt;/p&gt; &lt;p&gt; 
+Le nominalisme a été défendu par des philosophes importants tels que Guillaume d'Ockham, John Locke et David Hume. Ils ont remis en question l'idée selon laquelle les universaux existent en dehors de notre esprit et ont soutenu que notre connaissance est basée sur nos expériences individuelles des objets particuliers. &lt;/p&gt; &lt;p&gt; 
+Il a des implications dans divers domaines de la philosophie, notamment en épistémologie, en métaphysique et en philosophie du langage. Par exemple, en épistémologie, le nominalisme remet en question la possibilité de connaître des vérités universelles et insiste sur l'importance de l'expérience individuelle dans la formation de nos concepts. &lt;/p&gt; &lt;p&gt; 
+En métaphysique, le nominalisme remet en question l'idée de l'existence d'entités abstraites et soulève des questions sur la nature de la réalité. Les nominalistes peuvent également avoir une vision particulière du langage, considérant les mots comme des étiquettes arbitraires que nous utilisons pour communiquer, plutôt que comme des reflets de réalités universelles. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F37" s="14" t="s">
         <v>205</v>
@@ -5718,8 +5779,15 @@
       <c r="D38" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="E38" s="13" t="s">
-        <v>210</v>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Thomisme" title=" Wikipedia"&gt; Le Thomisme&lt;/a&gt; est un système philosophique et théologique basé sur les enseignements de Thomas d'Aquin, un théologien et philosophe catholique du XIIIe siècle qui chercha à concilier la philosophie aristotélicienne avec la théologie chrétienne. &lt;/p&gt; &lt;p&gt;
+Thomas d'Aquin a développé une approche philosophique appelée "scholastique", qui cherchait à intégrer la raison et la foi. Selon le thomisme, la raison et la révélation divine sont complémentaires et peuvent être utilisées pour approfondir la compréhension de la vérité. &lt;/p&gt; &lt;p&gt; 
+Dans le cadre du thomisme, la philosophie naturelle et la philosophie de la connaissance sont importantes pour comprendre le monde matériel et la nature de la réalité. La théologie, quant à elle, est considérée comme la reine des sciences, car elle se concentre sur la connaissance de Dieu et des vérités révélées. &lt;/p&gt; &lt;p&gt;
+Le thomisme affirme que la raison humaine est capable de connaître Dieu jusqu'à un certain point, mais que la révélation divine est nécessaire pour une compréhension plus complète et profonde. Il met également l'accent sur l'importance de la pensée logique et de l'argumentation rationnelle dans l'élaboration de la théologie et de la philosophie. &lt;/p&gt; &lt;p&gt;
+Dans le domaine de l'éthique, le thomisme propose une approche dite "éthique naturelle" basée sur la nature humaine et les principes moraux fondamentaux. Selon cette perspective, l'homme a des inclinations naturelles qui le guident vers le bien et la vertu. La loi naturelle, qui découle de la nature humaine elle-même, est considérée comme une norme objective pour le comportement moral.
+&lt;/p&gt; &lt;audio controls title="Redécouvrir Saint Thomas d'Aquin par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18292-21.03.2019-ITEMA_22014608-0.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
+        </is>
       </c>
       <c r="F38" s="11" t="s">
         <v>211</v>
@@ -5767,8 +5835,11 @@
       <c r="D39" s="15" t="s">
         <v>214</v>
       </c>
-      <c r="E39" s="16" t="s">
-        <v>215</v>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Modistes" title=" Wikipedia"&gt; Les Modistes&lt;/a&gt;  forment une école de grammairiens et philosophes médiévaux actifs à Paris entre la seconde moitié du XIIIe et le début du XIVe siècle. Ils développent la "grammaire spéculative", cherchant à fonder la grammaire sur des principes universels appelés "modes de signifier". Cette école émerge dans le milieu averroïste de l'université de Paris vers 1270, marquant une distinction entre grammaire et logique. Les Modistes visent à expliquer les règles de construction des énoncés au-delà d'une simple norme prescriptive, affirmant l'autonomie de la grammaire. Ils s'inscrivent dans la philosophie médiévale, influencée par Aristote et les débats scolastiques.  &lt;/p&gt; &lt;p&gt; Leur œuvre structurée en trois parties : un proemium posant les modes de signifier, l'etymologia analysant les parties du discours, et la dyasynthetica traitant de la syntaxe. Ils étudient comment les mots "signifient" par essence (modes essentiels), qualité (accidentels) ou combinaison (syntaxe), sans aborder la sémantique logique.  Cette approche spéculative préfigure des réflexions modernes sur le langage. &lt;/p&gt; &lt;p&gt; Les Figures principales : Thomas d'Erfurt, auteur d'un traité majeur utilisant le terme "grammatica speculativa". Martin de Dacie et Boèce de Dacie comptent aussi parmi les représentants éminents de ce courant. Leur influence s'étend jusqu'à la fin du Moyen Âge, avant le déclin de la scolastique.&lt;/p&gt;
+</t>
+        </is>
       </c>
       <c r="F39" s="14"/>
       <c r="G39" s="16"/>
@@ -5982,8 +6053,13 @@
       <c r="D43" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="E43" s="13" t="s">
-        <v>228</v>
+      <c r="E43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Naturalisme_(philosophie)"  style="color:#d35400"  title=" Wikipedia"&gt; Le Naturalisme&lt;/a&gt;  est une philosophie qui affirme que la réalité peut être expliquée entièrement par des lois naturelles, sans recourir à des entités ou des forces surnaturelles. Il cherche à comprendre et à interpréter le monde en se basant sur les méthodes et les principes de la science. &lt;/p&gt; &lt;p&gt; 
+Le naturalisme affirme que le monde naturel est le seul domaine d'existence réel et que tout phénomène, y compris les êtres humains, peut être expliqué en termes de processus naturels. Il rejette l'idée d'un esprit distinct du corps, d'une âme immatérielle ou d'une volonté libre indépendante des lois de la nature. &lt;/p&gt; &lt;p&gt; 
+En ce qui concerne la connaissance, il soutient que la méthode scientifique est le meilleur moyen d'acquérir des connaissances sur le monde et met l'accent sur l'observation, l'expérimentation, la mesure et la recherche empirique pour comprendre les phénomènes naturels et les lois qui les régissent. &lt;/p&gt; &lt;p&gt; En éthique, le naturalisme moral affirme que les valeurs morales et éthiques peuvent être dérivées de l'étude des comportements humains et des sciences sociales. Il nie l'existence de normes morales absolues ou d'un ordre moral transcendant, mais cherche plutôt à fonder l'éthique sur des bases empiriques et naturelles. &lt;/p&gt; &lt;p&gt; 
+Le naturalisme a également des implications en esthétique, où il considère que l'art et la beauté peuvent être expliqués par des processus naturels et des caractéristiques humaines.                            &lt;/p&gt;  &lt;audio controls title="Naturalisme, Lumières et droit naturel par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/11921-03.02.2020-ITEMA_22272038-0.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
+        </is>
       </c>
       <c r="F43" s="11" t="s">
         <v>229</v>
@@ -6028,8 +6104,14 @@
       <c r="D44" s="15" t="s">
         <v>234</v>
       </c>
-      <c r="E44" s="16" t="s">
-        <v>235</v>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Humanisme"  style="color:#d35400"  title=" Wikipedia"&gt; L'Humanisme&lt;/a&gt; est une philosophie qui met l'accent sur la valeur et la dignité de l'être humain. Il place l'homme au centre de ses préoccupations et cherche à promouvoir son développement, son bien-être et son épanouissement. &lt;/p&gt; &lt;p&gt; 
+L'humanisme est né pendant la Renaissance en Europe, mais ses racines remontent à l'Antiquité, en particulier à la philosophie grecque et romaine. Les penseurs humanistes de la Renaissance ont redécouvert et étudié les textes anciens, ce qui a contribué à un renouveau des connaissances et de la pensée critique. &lt;/p&gt; &lt;p&gt;  
+Il se distingue par son rejet des conceptions théocentriques et anthropocentriques du monde et  remet en question l'autorité absolue de la religion et la place de l'homme en tant que simple sujet de Dieu. Au lieu de cela, il souligne la capacité de l'homme à raisonner, à penser de manière autonome et à agir moralement. &lt;/p&gt; &lt;p&gt;
+L'humanisme met également l'accent sur les valeurs telles que la liberté, la tolérance, la justice, l'égalité et la dignité humaine et il prône la reconnaissance et le respect des droits de l'homme, ainsi que la responsabilité individuelle et collective dans la construction d'une société meilleure. &lt;/p&gt; &lt;p&gt;
+Il englobe divers courants de pensée, y compris l'humanisme séculier, l'humanisme religieux et l'humanisme laïque. L'humanisme séculier se concentre sur l'homme en tant qu'être autonome, sans référence à une transcendance religieuse. L'humanisme religieux, quant à lui, intègre des valeurs humanistes dans le cadre d'une croyance religieuse. L'humanisme laïque met l'accent sur les valeurs humanistes dans le contexte de la séparation entre l'État et la religion. &lt;/p&gt;  &lt;audio controls title="La naissance de l'humanisme par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-26.10.2017-ITEMA_21475272-1.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
+        </is>
       </c>
       <c r="F44" s="14" t="s">
         <v>236</v>
@@ -6801,7 +6883,7 @@
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ath%C3%A9isme"  title=" Wikipedia"&gt;L'Athéisme&lt;/a&gt; est une position métaphysique qui nie l'existence de Dieu ou de divinités.&lt;/p&gt; &lt;p&gt;  C'est une perspective qui a été explorée et discutée par de nombreux philosophes à travers l'histoire de la philosophie occidentale et orientale. &lt;/p&gt;  &lt;p&gt;Voici quelques éléments clés liés à l'athéisme en philosophie : &lt;/p&gt;&lt;p&gt; Les premières traces de pensée athée se trouvent dans la Grèce antique, notamment avec des philosophes présocratiques tels que Diagoras de Mélos et Protagoras. Ils remettaient en question l'existence des dieux olympiens et avaient des doutes quant à leur réalité. &lt;/p&gt; &lt;dd&gt;&lt;strong&gt;Matérialisme :&lt;/strong&gt; L'athéisme a pris de l'importance pendant la période de la philosophie moderne avec des penseurs tels que Spinoza, qui a élaboré une vision panthéiste du divin, et Diderot, qui a ouvertement professé l'athéisme dans son Encyclopédie. Il ne faut pas oublier Meslier, prêtre athé du 17 ème qui apporta beaucoup aux Lumières.&lt;/dd&gt; &lt;dd&gt;&lt;strong&gt;Arguments athées :&lt;/strong&gt; Les philosophes athées ont avancé divers arguments comme l'absence de preuves empiriques de l'existence de Dieu, tandis que d'autres ont soulevé des questions sur la cohérence des concepts de dieu ou de divinité. &lt;/dd&gt; &lt;dd&gt;&lt;strong&gt;Le problème du mal :&lt;/strong&gt; Les athées demandent comment un dieu tout-puissant, omniscient et bon peut permettre l'existence du mal et de la souffrance dans le monde. &lt;/dd&gt; &lt;dd&gt;&lt;strong&gt;Athéisme contemporain :&lt;/strong&gt; Au cours des derniers siècles, l'athéisme est devenu plus répandu, notamment avec la montée du mouvement humaniste séculier. Des philosophes contemporains tels que Dawkins, Hitchens ont promu l'athéisme en critiquant la religion et en défendant la rationalité scientifique et la séparation entre la religion et la politique. &lt;/dd&gt; &lt;dd&gt; &lt;strong&gt;Agnosticisme :&lt;/strong&gt; Certains athées sont agnostiques, ils ne croient pas en Dieu mais ne prétendent pas qu'il est impossible de prouver ou de réfuter l'existence de Dieu. &lt;/dd&gt; &lt;p&gt; L'athéisme en philosophie englobe une variété de positions allant de l'athéisme fort (affirmant qu'il n'y a pas de dieux) à l'athéisme faible (simplement l'absence de croyance en Dieu). Il existe également des athées qui considérent l'existence de Dieu comme improbable mais non impossible. &lt;/p&gt;
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ath%C3%A9isme"  title=" Wikipedia"&gt;L'Athéisme&lt;/a&gt; est une position métaphysique qui nie l'existence de Dieu ou de divinités.&lt;/p&gt; &lt;p&gt;  C'est une perspective qui a été explorée et discutée par de nombreux philosophes à travers l'histoire de la philosophie occidentale et orientale. &lt;/p&gt; &lt;p&gt; Les premières traces de pensée athée se trouvent dans la Grèce antique, notamment avec des philosophes présocratiques tels que Diagoras de Mélos et Protagoras. Ils remettaient en question l'existence des dieux olympiens et avaient des doutes quant à leur réalité. &lt;/p&gt; &lt;p&gt;&lt;strong&gt;Matérialisme :&lt;/strong&gt; L'athéisme a pris de l'importance pendant la période de la philosophie moderne avec des penseurs tels que Spinoza, qui a élaboré une vision panthéiste du divin, et Diderot, qui a ouvertement professé l'athéisme dans son Encyclopédie. Il ne faut pas oublier Meslier, prêtre athé du 17 ème qui apporta beaucoup aux Lumières.&lt;/p&gt; &lt;p&gt;&lt;strong&gt;Arguments athées :&lt;/strong&gt; Les philosophes athées ont avancé divers arguments comme l'absence de preuves empiriques de l'existence de Dieu, tandis que d'autres ont soulevé des questions sur la cohérence des concepts de dieu ou de divinité. &lt;/p&gt; &lt;p&gt;&lt;strong&gt;Le problème du mal :&lt;/strong&gt; Les athées demandent comment un dieu tout-puissant, omniscient et bon peut permettre l'existence du mal et de la souffrance dans le monde. &lt;/p&gt; &lt;p&gt;&lt;strong&gt;Athéisme contemporain :&lt;/strong&gt; Au cours des derniers siècles, l'athéisme est devenu plus répandu, notamment avec la montée du mouvement humaniste séculier. Des philosophes contemporains tels que Dawkins, Hitchens ont promu l'athéisme en critiquant la religion et en défendant la rationalité scientifique et la séparation entre la religion et la politique. &lt;/p&gt; &lt;p&gt; &lt;strong&gt;Agnosticisme :&lt;/strong&gt; Certains athées sont agnostiques, ils ne croient pas en Dieu mais ne prétendent pas qu'il est impossible de prouver ou de réfuter l'existence de Dieu. &lt;/p&gt; &lt;p&gt; L'athéisme en philosophie englobe une variété de positions allant de l'athéisme fort (affirmant qu'il n'y a pas de dieux) à l'athéisme faible (simplement l'absence de croyance en Dieu). Il existe également des athées qui considérent l'existence de Dieu comme improbable mais non impossible. &lt;/p&gt;
 &lt;audio controls title="Dieu, un homme en trop ?  "L'athéisme aujourd'hui" par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/inter/sons/2013/03/s13/NET_FI_28bd824f-f8fe-491a-9bae-e5a5bd5a6a51.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
@@ -6991,8 +7073,14 @@
       <c r="D64" s="12" t="s">
         <v>346</v>
       </c>
-      <c r="E64" s="13" t="s">
-        <v>347</v>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/D%C3%A9isme"  style="color:#d35400"  title=" Wikipedia"&gt; Le Déisme&lt;/a&gt; est une perspective qui examine la nature de Dieu et son rôle dans le monde à travers le prisme de la raison et de la logique. Il s'agit d'une approche théologique et métaphysique qui tente de comprendre l'existence et les attributs de Dieu en utilisant la réflexion philosophique plutôt que la révélation religieuse ou les dogmes. &lt;/p&gt; &lt;p&gt; 
+Les philosophes déistes tels que Voltaire s'interrogent sur des questions fondamentales comme l'existence de Dieu, sa nature, la relation entre Dieu et l'univers, et le problème du mal. Ils cherchent à comprendre si son l'existence peut être prouvée par des arguments rationnels et si la logique et la raison peuvent nous fournir des informations. &lt;/p&gt; &lt;p&gt;  
+Un argument souvent avancé est celui du dessein, également connu sous le nom d'argument téléologique qui soutient que l'ordre et la complexité de l'univers sont des indications de l'existence d'un concepteur intelligent et s'appuyent sur des arguments cosmologiques, métaphysiques et moraux pour étayer leur croyance en un Dieu. &lt;/p&gt; &lt;p&gt; 
+Les philosophes déistes ont également exploré la question de la relation entre Dieu et l'humanité. Certains déistes soutiennent que Dieu a créé l'univers et a ensuite abandonné toute intervention directe, laissant l'humanité agir selon sa propre volonté et utiliser la raison pour découvrir la vérité. D'autres affirment que Dieu interagit avec l'humanité d'une manière indirecte, en influençant les lois naturelles ou en inspirant les facultés humaines. &lt;/p&gt; &lt;p&gt; 
+le déisme en philosophie ne se limite pas à une seule perspective ou à une seule série de croyances. Les philosophes déistes peuvent présenter une variété de points de vue sur la nature de Dieu et la relation entre Dieu et l'univers. Certains peuvent s'approcher davantage du théisme, en soutenant une vision plus active de l'intervention divine, tandis que d'autres peuvent se rapprocher de l'agnosticisme, en reconnaissant l'existence possible de Dieu, mais sans prétendre avoir une connaissance certaine de cette réalité. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F64" s="11" t="s">
         <v>348</v>
@@ -7037,8 +7125,15 @@
       <c r="D65" s="15" t="s">
         <v>352</v>
       </c>
-      <c r="E65" s="16" t="s">
-        <v>353</v>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a  href="https://fr.wikipedia.org/wiki/Lib%C3%A9ralisme#:~:text=Le%20n%C3%A9ologisme%20lib%C3%A9ralisme%20est%20forg%C3%A9,favorable%20au%20d%C3%A9veloppement%20des%20libert%C3%A9s%20%C2%BB."  style="color:#d35400"  title=" Wikipedia"&gt; Le Libéralisme&lt;/a&gt; est une philosophie politique et sociale qui met l'accent sur la liberté individuelle, les droits de l'homme et la primauté de l'individu. Il repose sur plusieurs principes fondamentaux, tels que la liberté individuelle, l'égalité des droits, la justice, la tolérance, la responsabilité individuelle et la primauté de la loi. &lt;/p&gt; &lt;p&gt; 
+L'un des principes centraux du libéralisme est la liberté individuelle. Les libéraux considèrent que chaque individu possède des droits fondamentaux inhérents, tels que la liberté d'expression, la liberté de conscience, la liberté de religion, la liberté de réunion et la liberté de propriété. Ils soutiennent que ces libertés doivent être protégées par l'État et que les individus doivent être libres de mener leur vie comme ils le souhaitent, tant que cela n'empiète pas sur les droits et les libertés des autres. &lt;/p&gt; &lt;p&gt;
+Un autre aspect important du libéralisme est l'idée d'égalité des droits. Les libéraux considèrent que tous les individus sont égaux en dignité et en valeur, et qu'ils doivent être traités de manière égale devant la loi. Cela implique l'égalité des chances, l'accès aux mêmes droits et opportunités pour tous, indépendamment de leur origine sociale, de leur race, de leur religion ou de leur sexe. Le libéralisme promeut également l'idée d'une société inclusive, où la diversité est valorisée et respectée. &lt;/p&gt; &lt;p&gt;
+Le libéralisme prône également la tolérance et le pluralisme. Les libéraux reconnaissent que les sociétés sont composées de personnes ayant des croyances, des valeurs et des modes de vie différents. Ils défendent le droit des individus à exprimer leurs opinions, même si celles-ci sont en désaccord avec la majorité, et soutiennent la coexistence pacifique des différentes visions du monde au sein d'une société pluraliste. &lt;/p&gt; &lt;p&gt; 
+En ce qui concerne l'économie, le libéralisme est souvent associé à la promotion de l'économie de marché et à la liberté économique. Les libéraux soutiennent généralement que les échanges économiques devraient être basés sur le libre choix et la concurrence, avec une intervention minimale de l'État dans les affaires économiques. Cela se traduit souvent par la défense du droit de propriété privée, de la libre entreprise et de la liberté contractuelle. &lt;/p&gt; &lt;p&gt; 
+Il convient de noter que le libéralisme se décline en différentes variantes et qu'il existe des débats et des nuances au sein de cette tradition philosophique. On trouve notamment le libéralisme classique, le libéralisme social, le libéralisme politique et d'autres courants qui mettent l'accent sur différents aspects de la philosophie libérale. &lt;/p&gt;  &lt;audio controls title="Les penseurs du libéralisme au XVIIIe par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2015/01/s02/NET_FC_f8ff59de-a76a-443d-9dcf-1cc6f2af7538.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
+        </is>
       </c>
       <c r="F65" s="14" t="s">
         <v>354</v>
@@ -7613,8 +7708,10 @@
       <c r="D76" s="12" t="s">
         <v>405</v>
       </c>
-      <c r="E76" s="13" t="s">
-        <v>406</v>
+      <c r="E76" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Libertarianisme" title=" Wikipedia"&gt;Le Libertarianisme&lt;/a&gt;  ou Libertarisme est un courant politique et philosophique qui met l'accent sur la liberté individuelle et la primauté de l'individu sur l'État. Ses origines remontent aux idées du siècle des Lumières et ont été développées plus tard par des penseurs comme John Locke, Adam Smith, et plus récemment par des figures comme Friedrich Hayek, Robert Nozick et Murray Rothbard. &lt;/p&gt; &lt;p&gt;Les libertariens croient en un gouvernement minimal, dont le rôle se limiterait à protéger les droits naturels des individus, limité, à la défense nationale et l'application des contrats. Ils s'opposent aux interventions gouvernementales dans des domaines tels que la santé, l'éducation et la moralité individuelle.tels que la vie, la liberté et la propriété. Ils prônent généralement une réduction drastique du rôle de l'État dans l'économie, préférant les mécanismes du marché libre pour réguler les échanges et allouer les ressources considérant la liberté individuelle comme étant de la plus haute importance. Ils soutiennent que les individus devraient avoir le droit de vivre leur vie comme ils l'entendent, tant qu'ils ne violent pas les droits des autres. &lt;/p&gt; &lt;p&gt;Ils défendent le droit à la propriété privée. Ils estiment que les individus ont le droit de posséder et de disposer de leurs biens comme bon leur semble, sans ingérence injustifiée de l'État et ils  favorisent généralement une économie de marché non réglementée, où l'offre et la demande déterminent les prix et les allocations de ressources. Ils soutiennent que les interventions gouvernementales dans l'économie, telles que les taxes excessives ou les réglementations strictes, entravent la liberté et nuisent à la prospérité économique. &lt;/p&gt; &lt;p&gt;Le principe de non-agression est central pour les libertariens. Cela signifie qu'ils s'opposent à l'utilisation de la force ou de la coercition, sauf en légitime défense. Ils considèrent toute action initiée par l'État qui viole les droits individuels comme illégitime. &lt;/p&gt; &lt;p&gt;Le libertarisme est souvent perçu comme un spectre politique qui s'étend du libertarianisme de gauche, qui accorde plus d'importance aux droits sociaux et à l'égalité, au libertarianisme de droite, qui met davantage l'accent sur les droits individuels et la primauté du marché libre. Ces variations peuvent conduire à des désaccords internes sur des questions spécifiques, mais tous les libertariens partagent généralement un engagement envers la liberté individuelle et la limitation du pouvoir gouvernemental. &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F76" s="11" t="s">
         <v>407</v>
@@ -7814,8 +7911,11 @@
       <c r="D80" s="15" t="s">
         <v>427</v>
       </c>
-      <c r="E80" s="16" t="s">
-        <v>428</v>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_(%C3%A9pist%C3%A9mologie)"  title=" Wikipedia"&gt; Le Constructivisme &lt;/a&gt; est un courant de pensée multidisciplinaire postulant que nos connaissances et notre vision du monde ne sont pas un reflet passif de la réalité, mais une construction active élaborée par l'esprit humain. Dans cette approche, le sujet connaissant interagit avec son environnement pour structurer ses propres modèles mentaux, intégrant de nouvelles expériences à des structures cognitives déjà existantes. &lt;/p&gt;&lt;p&gt; Emmanuel Kant a joué un rôle charnière au XVIIIe siècle, en proposant dans sa Critique de la raison pure une vision où l'expérience naît de l'interaction entre les impressions sensibles et la structure propre à l'esprit humain. Cette perspective a posé les jalons d'un constructivisme empirique qui rejette l'idée d'une perception passive et directe de la réalité. &lt;/p&gt; &lt;p&gt; Dans le domaine de la philosophie politique et du libéralisme, le « rationalisme constructiviste » est souvent dénoncé comme une volonté d'édifier la société selon un dessein rationnel préconçu. Les critiques, notamment Friedrich Hayek, soutiennent que cette approche tend à imposer des plans collectifs par la coercition, négligeant la liberté individuelle et les mécanismes d'ordre spontané issus des interactions humaines. &lt;/p&gt; &lt;p&gt; À l'inverse, en relations internationales, le constructivisme est une théorie scientifique qui analyse la réalité mondiale comme une construction sociale. Pour ses partisans, les intérêts des États et les structures du système international ne sont pas des données fixes ou matérielles, mais le fruit de normes, d'idées et d'interactions partagées entre les acteurs. &lt;/p&gt; 
+</t>
+        </is>
       </c>
       <c r="F80" s="14" t="s">
         <v>429</v>
@@ -7911,8 +8011,10 @@
       <c r="D82" s="15" t="s">
         <v>438</v>
       </c>
-      <c r="E82" s="16" t="s">
-        <v>439</v>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Panenth%C3%A9isme"  title=" Wikipedia"&gt;Le Panenthéisme&lt;/a&gt;  est une doctrine philosophique et théologique affirmant que Dieu englobe et interpénètre tout l'univers, tout en le dépassant par sa transcendance, formant une médiation entre panthéisme (Dieu identifié à l'univers) et théisme classique (Dieu extérieur). Introduit par le philosophe allemand Karl Christian Friedrich Krause au début du XIXe siècle (vers 1828), il postule que le monde est contenu en Dieu comme une partie de son être, sans s'y réduire, influençant des courants comme la théologie du processus ou certaines interprétations de Spinoza. &lt;/p&gt; &lt;p&gt; Forgé par Krause pour dépasser le panthéisme spinoziste, le panenthéisme puise dans des idées anciennes : néoplatonisme (Plotin), hindouisme védantique (Brahman immanent et transcendant), ou kabbalah juive (Tsimtsoum). Au XXe siècle, il inspire Alfred North Whitehead  et des théologiens protestants comme Jürgen Moltmann. &lt;/p&gt; &lt;p&gt; Concepts centraux : Immanence et transcendance : Dieu est dans tout (immanence) mais plus grand que le cosmos, qui n'est qu'une manifestation partielle de sa réalité infinie. Dynamisme divin : Contrairement au déisme statique, Dieu évolue avec l'univers, influencé par ses changements (théologie du processus). Critiques : Accusé de diluer la transcendance divine ou de verser dans un vague mysticisme naturaliste. &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F82" s="14" t="s">
         <v>440</v>
@@ -8059,8 +8161,12 @@
       <c r="D85" s="15" t="s">
         <v>454</v>
       </c>
-      <c r="E85" s="16" t="s">
-        <v>455</v>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Conservatisme"  title=" Wikipedia"&gt;Le Conservatisme&lt;/a&gt;  est un courant philosophique et politique qui valorise la préservation des traditions, des institutions établies et de l'ordre social organique contre les changements radicaux ou utopiques. Il met l'accent sur la sagesse accumulée par l'expérience historique plutôt que sur des théories abstraites, prônant une évolution prudente de la société. &lt;/p&gt; &lt;p&gt; Né comme réaction à la Révolution française (1789), le conservatisme trouve son expression fondatrice chez Edmund Burke dans Réflexions sur la Révolution de France (1790), qui dénonce la rupture brutale avec le passé au nom de la raison pure. Au XIXe siècle, il se développe en Angleterre avec des penseurs comme Samuel Taylor Coleridge et en Europe continentale via Joseph de Maistre, défendant la religion, la famille et la hiérarchie naturelle contre l'égalitarisme révolutionnaire. &lt;/p&gt; &lt;p&gt; Les principaux fondements sont : Tradition comme sagesse : La société est un héritage complexe, non un contrat rationnel ; les réformes doivent être graduelles pour éviter le chaos. Primauté de l'ordre : Liberté individuelle liée à la propriété privée et aux devoirs moraux, avec rôle de l'État pour protéger la stabilité. Scepticisme envers l'abstraction : Méfiance envers les idéologies universalistes (libéralisme extrême, socialisme) qui ignorent les contextes locaux. &lt;/p&gt; 
+ &lt;audio controls title=" Quand le conservatisme devient populiste par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23497-28.03.2025-ITEMA_24077783-2025F49012S0089-NET_MFI_26E2E121-D064-4F2B-B604-612240DE65AA-27.m4a" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;
+​</t>
+        </is>
       </c>
       <c r="F85" s="14" t="s">
         <v>456</v>
@@ -8314,8 +8420,11 @@
       <c r="D90" s="15" t="s">
         <v>482</v>
       </c>
-      <c r="E90" s="16" t="s">
-        <v>483</v>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pessimisme_(philosophie)"  title=" Wikipedia"&gt; Le Pessimisme&lt;/a&gt;  est une perspective philosophique qui considère que la vie et le monde sont fondamentalement marqués par la souffrance, la douleur et l'insatisfaction. Les philosophes pessimistes remettent en question l'idée que la vie a une valeur intrinsèque positive ou qu'elle conduit inévitablement au bonheur. Au lieu de cela, ils soutiennent que la souffrance est omniprésente et inhérente à l'existence humaine.  Il se distingue de l'optimisme, qui soutient que la vie a une valeur intrinsèque positive et que le bonheur est atteignable malgré les difficultés. Les philosophes pessimistes rejettent généralement cette vision optimiste et soulignent plutôt la réalité de la souffrance, de l'incertitude et de la finitude de la condition humaine. &lt;/p&gt; &lt;p&gt; L'une des figures les plus célèbres du pessimisme philosophique est Arthur Schopenhauer qui considérait que la vie était une lutte perpétuelle et que la souffrance était le fondement même de l'existence. Selon lui, la volonté de vivre, un désir insatiable et sans fin, est à l'origine de nos besoins, de nos désirs et de notre insatisfaction perpétuelle. Il croyait que l'accomplissement de ces désirs était éphémère et qu'il était suivi par une nouvelle recherche insatiable de satisfaction, créant ainsi un cycle de souffrance inévitable. &lt;/p&gt; &lt;p&gt;
+Un autre philosophe pessimiste influent est Friedrich Nietzsche. Bien qu'il ne soit pas strictement considéré comme un pessimiste, il a abordé la question de la souffrance et de l'existence humaine d'une manière qui mettait en évidence les aspects sombres et douloureux de la vie. Il a remis en question les croyances traditionnelles et les valeurs morales et a souligné l'importance de faire face à la réalité de manière lucide. &lt;/p&gt; &lt;p&gt; Cependant, le pessimisme philosophique ne se limite pas à une seule vision unifiée. Il existe différentes nuances allant d'un pessimisme radical et absolu à des formes plus modérées qui reconnaissent également des aspects positifs dans la vie. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F90" s="14" t="s">
         <v>484</v>
@@ -8567,8 +8676,14 @@
       <c r="D95" s="15" t="s">
         <v>510</v>
       </c>
-      <c r="E95" s="16" t="s">
-        <v>511</v>
+      <c r="E95" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Anarchisme"  style="color:#d35400"  title=" Wikipedia"&gt; L'Anarchisme &lt;/a&gt; est un courant de pensée politique et social qui prône la suppression de toutes les formes d'autorité et de hiérarchie, qu'elles soient politiques, économiques ou sociales. L'idéologie anarchiste est née au XIXe siècle, en réaction aux injustices et aux oppressions engendrées par le capitalisme et l'État.&lt;/p&gt; &lt;p&gt;
+Les premiers théoriciens de l'anarchisme étaient Pierre-Joseph Proudhon, Mikhail Bakounine et Pierre Kropotkine. Proudhon est considéré comme le fondateur de l'anarchisme, avec son ouvrage "Qu'est-ce que la propriété ?", publié en 1840. Dans cet ouvrage, Proudhon développe l'idée que la propriété est un vol et que le droit à la propriété ne peut exister que si tous les individus ont les mêmes opportunités pour y accéder.&lt;/p&gt; &lt;p&gt;
+Mikhail Bakounine, quant à lui, a élaboré une critique radicale de l'État et du capitalisme. Il a affirmé que l'État était une institution oppressive, qui devait être détruite pour que les individus puissent être libres. Bakounine a également développé l'idée de la "révolution sociale", qui consiste à renverser le système capitaliste par la force, en mobilisant les masses populaires.&lt;/p&gt; &lt;p&gt;
+Enfin, Pierre Kropotkine a développé une vision de l'anarchisme qui met l'accent sur la coopération et l'entraide. Dans son ouvrage "L'Entraide, un facteur de l'évolution", publié en 1902, Kropotkine a affirmé que la coopération et l'entraide étaient des forces essentielles de la vie sociale, qui pouvaient remplacer la compétition et l'exploitation.&lt;/p&gt; &lt;p&gt;
+&lt;p&gt; L'anarchisme a inspiré de nombreux mouvements sociaux et politiques à travers le monde, le mouvement anarchiste espagnol de la guerre civile, les Zapatistes du Mexique et les mouvements autonomes en Europe.&lt;/p&gt;   &lt;audio controls title="Naissance du mouvement anarchiste par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10076-28.08.2017-ITEMA_21417855-1.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
+        </is>
       </c>
       <c r="F95" s="14" t="s">
         <v>512</v>
@@ -9033,8 +9148,15 @@
       <c r="D104" s="15" t="s">
         <v>566</v>
       </c>
-      <c r="E104" s="16" t="s">
-        <v>567</v>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Nihilisme" title=" Wikipedia"&gt; Le Nihilisme&lt;/a&gt; est une position philosophique qui remet en question ou nie la valeur et la signification de la vie, de la connaissance, de la morale et d'autres concepts fondamentaux. Les nihilistes affirment que la réalité est dépourvue de sens intrinsèque, de valeurs objectives ou de vérités ultimes et que rien n'a de valeur ou d'importance réelle, et que toutes les croyances, les systèmes moraux et les vérités sont des constructions arbitraires et illusoires. &lt;/p&gt; &lt;p&gt;
+Il peut prendre différentes formes et être appliqué à différents domaines de la philosophie. Le nihilisme métaphysique, par exemple, nie l'existence de toute réalité objective ou transcendante. Il n'y a pas de Dieu, d'âme, de monde spirituel ou de finalité ultime dans l'univers. &lt;/p&gt; &lt;p&gt;
+Le nihilisme épistémologique remet en question la possibilité de connaître la réalité telle qu'elle est en soi et soutient que nos perceptions et nos croyances sont toujours limitées et subjectives, et qu'il est impossible d'atteindre une connaissance objective et complète. &lt;/p&gt; &lt;p&gt;
+Le nihilisme moral rejette l'idée de valeurs morales objectives et que les notions de bien et de mal sont des constructions humaines sans fondement réel, que la morale est une illusion et que chaque individu est libre de créer ses propres valeurs ou d'adopter l'absence totale de valeurs. &lt;/p&gt; &lt;p&gt;
+le nihilisme n'est pas nécessairement une position que l'on adopte activement, mais plutôt une perspective critique qui remet en question les systèmes de croyances et les valeurs établies. Certains philosophes ont même fait valoir que le nihilisme peut être un point de départ pour la construction d'une nouvelle signification et de nouvelles valeurs. &lt;/p&gt;   &lt;audio controls title="Le nihilisme et la mort de l'homme par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2015/08/s35/WL-ITE_00075081_RSCE-10.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+</t>
+        </is>
       </c>
       <c r="F104" s="14" t="s">
         <v>568</v>
@@ -9309,8 +9431,10 @@
       <c r="D109" s="15" t="s">
         <v>587</v>
       </c>
-      <c r="E109" s="16" t="s">
-        <v>588</v>
+      <c r="E109" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Perspectivisme" title=" Wikipedia"&gt;Le Perspectivisme&lt;/a&gt; est un courant philosophique affirmant que toute connaissance ou perception de la réalité est nécessairement relative à un point de vue spécifique, sans accès à une vérité objective absolue indépendante des perspectives individuelles ou culturelles. Développé principalement par Friedrich Nietzsche au XIXe siècle, il rejette l'idée d'une "vue de nulle part" et insiste sur la multiplicité des interprétations comme constitutive de la réalité. &lt;/p&gt; &lt;p&gt; Le terme émerge explicitement avec Nietzsche, qui s'appuie sur Gustav Teichmüller dans les années 1870, pour critiquer le réalisme métaphysique platonicien. Chez Leibniz (XVIIe siècle), l'univers est vu comme un ensemble de monades, chacune offrant une perspective unique sur le tout. Nietzsche en fait une "antimétaphysique réaliste" dès Humain, trop humain (1878) et Généalogie de la morale (1887), où la vérité résulte d'une comparaison asymptotique des perspectives. &lt;/p&gt; &lt;p&gt; Les principes clés : Relativité des vérités : Aucun fait n'a de sens hors d'une perspective subjective ou corporelle, liée à des forces vitales. Rejet du relativisme pur : Toutes les perspectives ne se valent pas ; certaines favorisent l'épanouissement humain plus que d'autres, Pluralisme épistémique : La réalité est la somme des points de vue, sans fondement transcendant. &lt;p&gt;</t>
+        </is>
       </c>
       <c r="F109" s="14" t="s">
         <v>589</v>
@@ -9363,8 +9487,11 @@
       <c r="D110" s="12" t="s">
         <v>592</v>
       </c>
-      <c r="E110" s="13" t="s">
-        <v>593</v>
+      <c r="E110" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89cologisme" title=" Wikipedia"&gt;L'Ècologisme&lt;/a&gt;  ou environnementalisme, est un courant philosophique et idéologique qui place la préservation de la nature et des écosystèmes au centre des valeurs humaines, critiquant l'anthropocentrisme dominant de la modernité industrielle. Il prône une rupture avec la croissance illimitée et l'exploitation des ressources, favorisant une éthique biocentrée où la diversité biologique possède une valeur intrinsèque indépendante des besoins humains. &lt;/p&gt; &lt;p&gt; Émergé au XXe siècle, l'écologisme s'ancre dans les travaux d'Alexander von Humboldt (fin XVIIIe-XIXe) sur l'interdépendance des écosystèmes, et se radicalise dans les années 1960-1970 avec Rachel Carson (Silent Spring, 1962) et Arne Naess, fondateur de l'écologie profonde (1973). En France, Bernard Charbonneau et Jacques Ellul dénoncent dès les années 1930 la "technique" destructrice, influençant les mouvements anti-nucléaires et anti-croissance des années 1970. &lt;/p&gt; &lt;p&gt; L'écologisme repose sur huit piliers inspirés de Naess pour l'écologie profonde : Valeur intrinsèque de toute vie humaine et non humaine. Richesse et diversité biologique comme fins en soi. Limitation humaine aux besoins vitaux pour ne pas réduire cette diversité. Compatibilité de l'épanouissement humain avec une décroissance démographique. Priorité à la qualité de vie sur l'accumulation matérielle. Engagement personnel pour des changements politiques et culturels. &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=" L'écologisme, une révolution politique par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/16260-15.02.2014-ITEMA_20589182-2014C6260E0005-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;
+</t>
+        </is>
       </c>
       <c r="F110" s="11" t="s">
         <v>594</v>
@@ -9501,8 +9628,13 @@
       <c r="D113" s="15" t="s">
         <v>608</v>
       </c>
-      <c r="E113" s="16" t="s">
-        <v>609</v>
+      <c r="E113" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pragmatisme"   title=" Wikipedia"&gt; Le Pragmatisme&lt;/a&gt; est un courant philosophique qui a émergé aux États-Unis avec des penseurs tels que William James ou John Dewey. Il met l'accent sur la pratique, l'action et les conséquences concrètes de nos idées et croyances et rejette les approches philosophiques abstraites et spéculatives en mettant plutôt l'accent sur l'expérience vécue, l'action et les résultats pratiques. La vérité et la signification des idées et des théories doivent être évaluées en fonction de leur utilité pratique et de leur capacité à produire des résultats positifs dans la réalité. &lt;/p&gt; &lt;p&gt;
+Le pragmatisme propose une méthode d'enquête appelée "méthode pragmatique", qui consiste à considérer les idées et les théories comme des outils pratiques pour résoudre les problèmes et guider l'action. Selon cette approche, une idée est vraie si elle fonctionne efficacement dans la pratique et si elle permet de résoudre les problèmes concrets auxquels nous sommes confrontés. &lt;/p&gt; &lt;p&gt;
+Il met également l'accent sur le contexte social et la dimension collective de la connaissance en soutenant que nos croyances et nos idées sont forgées en interaction avec notre environnement social, et qu'elles doivent être évaluées en fonction de leur impact sur la société et sur les individus. Ainsi, il souligne l'importance de la démocratie, de l'action sociale et de l'amélioration de la condition humaine. &lt;/p&gt; &lt;p&gt;
+Il a également eu une influence importante dans le domaine de l'éducation. Les pragmatistes, tels que John Dewey, ont mis l'accent sur l'apprentissage par l'expérience, l'interaction sociale et la résolution de problèmes concrets. Ils ont également souligné l'importance d'une éducation démocratique qui prépare les individus à devenir des membres actifs et responsables de la société. &lt;/p&gt; &lt;audio controls title="la vérité dans le pragmatisme chez Dewey par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2012/10/s43/les_nouveaux_chemins--Pensee_americaine_4_4_Action_ou_Verite__La_verite_--NET_ffccd5c0-ae35-43ec-b4bf-4d1139fad30b_FC.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
+        </is>
       </c>
       <c r="F113" s="14" t="s">
         <v>610</v>
@@ -9604,8 +9736,11 @@
       <c r="D115" s="15" t="s">
         <v>618</v>
       </c>
-      <c r="E115" s="16" t="s">
-        <v>619</v>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/N%C3%A9othomisme"   title=" Wikipedia"&gt; Le Néothomisme&lt;/a&gt; est un renouveau de la philosophie thomiste, initié par l'Église catholique à la fin du XIXe siècle pour répondre aux défis de la modernité. Il vise à adapter la pensée de saint Thomas d'Aquin aux questions contemporaines tout en préservant son réalisme métaphysique.  Promu par l'encyclique Æterni Patris du pape Léon XIII en 1879, ce courant devient la philosophie officielle de l'Église contre le modernisme et le kantisme. Pie X le renforce en 1904 via Pascendi dominici gregis, en faisant un rempart doctrinal.  Il s'agit d'un "néoscolastique" qui réactualise Aristote via Thomas pour une théologie rationnelle.&lt;/p&gt; &lt;p&gt; Fondé sur l'analogie de l'Être, la distinction essence-existence et la primauté de l'intelligence sur la volonté. Il défend une métaphysique réaliste : l'être est acte, Dieu premier moteur, accessible par la raison naturelle. Contrairement au thomisme originel, il intègre des problématiques post-kantiennes comme la critique de l'idéalisme. &lt;/p&gt; &lt;p&gt; Les figures majeures sont : Jacques Maritain : applique à la politique et l'art (humanisme intégral). Étienne Gilson : historien de la philosophie, met l'accent sur l'existence chrétienne. Marie-Dominique Chenu : ouvre vers une théologie historique. Autres : Réginald Garrigou-Lagrange, Joseph Maréchal (transcendantal). &lt;/p&gt; &lt;p&gt; Dominant jusqu'au Concile Vatican II (1962-65), il influence l'enseignement catholique mondial via des universités comme Louvain. Aujourd'hui, il persiste dans des cercles traditionalistes et dialogue avec la phénoménologie ou la science. &lt;/p&gt; 
+</t>
+        </is>
       </c>
       <c r="F115" s="14" t="s">
         <v>620</v>
@@ -9866,8 +10001,10 @@
       <c r="D120" s="12" t="s">
         <v>645</v>
       </c>
-      <c r="E120" s="13" t="s">
-        <v>646</v>
+      <c r="E120" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/M%C3%A9r%C3%A9ologie"  style="color:#d35400"  title=" Wikipedia"&gt;Méréologie&lt;/a&gt;  est la branche de la logique et de la métaphysique qui étudie de manière formelle les relations entre parties et touts, en alternative (ou complément) à la théorie des ensembles. Elle fournit un langage précis pour parler de composition, de décomposition et de structure des objets matériels, des événements, voire d’entités plus abstraites. &lt;/p&gt; &lt;p&gt; La méréologie définit d’abord ce que signifie “être une partie de” quelque chose. Une partie est ce qui compose un tout, comme une roue pour une voiture, une scène pour une pièce de théâtre ou un chapitre pour un livre. Le tout est l’entité composée de ces parties, et la relation fondamentale étudiée est “x est partie de y”. &lt;/p&gt; &lt;p&gt; La “méréologie extensionnelle” ajoute le principe que deux objets qui ont exactement les mêmes parties sont identiques (extensionalité). Cela donne un système très proche de la théorie des ensembles, mais exprimé en termes de parties et de fusions plutôt qu’en termes d’appartenance. Une conséquence importante: pour tout ensemble de choses, il existe une somme méréologique (une fusion) qui les compose. &lt;/p&gt; &lt;p&gt; La méréologie est devenue un outil central de l’ontologie formelle et de la métaphysique contemporaine. Elle intervient dans le débat sur la composition des objets matériels: quand des particules composent‑elles un objet unique (par exemple une table) plutôt qu’un simple “amas” ? &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F120" s="11" t="s">
         <v>647</v>
@@ -10444,9 +10581,7 @@
       </c>
       <c r="E132" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Empirisme_logique"  title=" Wikipedia"&gt;Le positivisme logique&lt;/a&gt;, également connu sous le nom "d'empirisme logique" est un courant philosophique majeur qui a cherché à définir les critères de la connaissance scientifique et à éliminer la métaphysique jugée dépourvue de sens. Né au sein du Cercle de Vienne, il a eu une influence considérable sur la philosophie des sciences et la philosophie analytique. Voici les points essentiels: &lt;/p&gt; &lt;p&gt; - Le principe de vérification (ou vérifiabilité) : C'est le critère central du positivisme logique pour déterminer la signification d'un énoncé. Selon ce principe, un énoncé n'a de sens que s'il est : &lt;/p&gt; 
-&lt;dd&gt; - Analytiquement vrai : vrai en vertu de sa structure logique ou de la définition de ses termes (par exemple, "Tous les célibataires sont non mariés"). Ces énoncés sont tautologiques et n'apportent pas d'information sur le monde. &lt;/dd&gt; 
-&lt;dd&gt; - Empiriquement vérifiable : sa vérité ou sa fausseté peut être établie par l'observation et l'expérience sensorielle (par exemple, "Cette table est marron"). &lt;/dd&gt; &lt;p&gt; - Le rejet de la métaphysique : Les énoncés qui ne sont ni analytiques ni empiriquement vérifiables sont considérés comme dépourvus de sens cognitif. Cela inclut la plupart des affirmations traditionnelles de la métaphysique (sur l'existence de Dieu, l'âme, le sens de la vie, etc.), de l'éthique normative (les jugements de valeur ne pouvant être vérifiés empiriquement) et de la théologie. Pour les positivistes logiques, ces énoncés peuvent avoir une valeur émotive ou poétique, mais pas une valeur de vérité. &lt;/p&gt; &lt;p&gt; - L'empirisme radical : Toute connaissance du monde provient de l'expérience sensorielle. La science est considérée comme le modèle de la connaissance rationnelle. &lt;/p&gt; &lt;p&gt; - La logique et les mathématiques comme outils : La logique et les mathématiques sont vues comme des outils formels essentiels pour analyser et structurer la connaissance scientifique. Leurs énoncés sont analytiques. &lt;/p&gt; &lt;p&gt;  - L'unité de la science : Les positivistes logiques aspiraient à unifier toutes les sciences (physique, biologie, psychologie, sciences sociales) sur la base d'un langage commun (idéalement le langage de la physique) et d'une méthodologie commune fondée sur la vérification empirique. &lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Empirisme_logique"  title=" Wikipedia"&gt;Le positivisme logique&lt;/a&gt;, également connu sous le nom "d'empirisme logique" est un courant philosophique majeur qui a cherché à définir les critères de la connaissance scientifique et à éliminer la métaphysique jugée dépourvue de sens. Né au sein du Cercle de Vienne, il a eu une influence considérable sur la philosophie des sciences et la philosophie analytique. &lt;/p&gt; &lt;p&gt;Le principe de vérification (ou vérifiabilité) : C'est le critère central du positivisme logique pour déterminer la signification d'un énoncé. Selon ce principe, un énoncé n'a de sens que s'il est : &lt;/p&gt; &lt;p&gt;Analytiquement vrai : vrai en vertu de sa structure logique ou de la définition de ses termes (par exemple, "Tous les célibataires sont non mariés"). Ces énoncés sont tautologiques et n'apportent pas d'information sur le monde. &lt;/p&gt; &lt;p&gt;Empiriquement vérifiable : sa vérité ou sa fausseté peut être établie par l'observation et l'expérience sensorielle (par exemple, "Cette table est marron"). &lt;/p&gt; &lt;p&gt;Le rejet de la métaphysique : Les énoncés qui ne sont ni analytiques ni empiriquement vérifiables sont considérés comme dépourvus de sens cognitif. Cela inclut la plupart des affirmations traditionnelles de la métaphysique (sur l'existence de Dieu, l'âme, le sens de la vie, etc.), de l'éthique normative (les jugements de valeur ne pouvant être vérifiés empiriquement) et de la théologie. Pour les positivistes logiques, ces énoncés peuvent avoir une valeur émotive ou poétique, mais pas une valeur de vérité. &lt;/p&gt; &lt;p&gt;L'empirisme radical : Toute connaissance du monde provient de l'expérience sensorielle. La science est considérée comme le modèle de la connaissance rationnelle. &lt;/p&gt; &lt;p&gt;La logique et les mathématiques comme outils : La logique et les mathématiques sont vues comme des outils formels essentiels pour analyser et structurer la connaissance scientifique. Leurs énoncés sont analytiques. &lt;/p&gt; &lt;p&gt;L'unité de la science : Les positivistes logiques aspiraient à unifier toutes les sciences (physique, biologie, psychologie, sciences sociales) sur la base d'un langage commun (idéalement le langage de la physique) et d'une méthodologie commune fondée sur la vérification empirique. &lt;/p&gt;</t>
         </is>
       </c>
       <c r="F132" s="14" t="s">
@@ -10737,8 +10872,13 @@
       <c r="D138" s="12" t="s">
         <v>742</v>
       </c>
-      <c r="E138" s="13" t="s">
-        <v>743</v>
+      <c r="E138" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Objectivisme_(Ayn_Rand)"  title=" Wikipedia"&gt; L'Objectivisme&lt;/a&gt;  est une philosophie développée par la philosophe américaine Ayn Rand. Elle a exposé ses principes fondamentaux dans plusieurs de ses œuvres, notamment dans son roman philosophique "La Grève" et dans son ouvrage non-fictionnel "La Vertu d'égoïsme". &lt;/p&gt; &lt;p&gt;  Au cœur de l'objectivisme se trouve la conviction que la réalité existe indépendamment de notre conscience et qu'il est possible d'accéder à la connaissance objective. Selon cette perspective, il existe des vérités objectives qui peuvent être découvertes par la raison humaine en prônant un réalisme métaphysique, affirmant que la réalité est objective, absolue et cohérente. Il rejette les idées de relativisme et de subjectivisme, qui soutiennent que la vérité dépend de l'individu ou du contexte. Selon l'objectivisme, la réalité est gouvernée par des lois naturelles et universelles qui ne peuvent pas être modifiées par nos opinions ou nos désirs. &lt;/p&gt; &lt;p&gt;
+Sur le plan éthique, il promeut une éthique de l'égoïsme rationnel, soutenant que l'égoïsme, compris comme la poursuite rationnelle de son propre intérêt à long terme, est moralement juste et bénéfique pour l'individu et pour la société dans son ensemble. Rand défend le droit individuel à la vie, à la liberté et à la poursuite du bonheur, ainsi que la propriété privée et la libre entreprise. &lt;/p&gt; &lt;p&gt;
+En politique, l'objectivisme préconise un système de capitalisme de laissez-faire. Selon cette vision, l'économie doit être basée sur le respect des droits individuels et sur des échanges volontaires entre les personnes. L'État devrait être limité à la protection des droits individuels, tels que la sécurité et la justice, sans s'immiscer dans l'économie ou dans les affaires privées.  &lt;/p&gt;
+</t>
+        </is>
       </c>
       <c r="F138" s="11" t="s">
         <v>744</v>
@@ -10949,8 +11089,10 @@
       <c r="D142" s="12" t="s">
         <v>764</v>
       </c>
-      <c r="E142" s="13" t="s">
-        <v>765</v>
+      <c r="E142" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Essentialisme" title=" Wikipedia"&gt;L'Essentialisme&lt;/a&gt;  est une doctrine qui soutient que les objets, les êtres ou les concepts possèdent une essence, c'est-à-dire un ensemble de propriétés fondamentales et immuables qui définissent ce qu'ils sont. Cette essence précède leur existence et détermine leur nature. &lt;/p&gt; &lt;p&gt;Nature Intrinsèque : L'essentialisme postule qu'il existe une nature intrinsèque aux choses, indépendante de la perception ou de la construction sociale. Par exemple, un essentialiste pourrait affirmer qu'il existe une essence de "l'être humain" qui définit ce que c'est d'être humain, quelles que soient les variations culturelles ou individuelles. &lt;/p&gt; &lt;p&gt;Propriétés Nécessaires vs. Accidentelles : Il distingue les propriétés essentielles, celles qu'une chose doit posséder pour être ce qu'elle est, des propriétés accidentelles, qui peuvent changer sans altérer l'identité fondamentale de la chose. Par exemple, avoir trois côtés est une propriété essentielle d'un triangle, tandis que sa couleur ou sa taille sont des propriétés accidentelles. &lt;/p&gt; &lt;p&gt;Stabilité et Permanence : L'essence est considérée comme stable et permanente. Même si les apparences ou les manifestations d'une chose peuvent changer, son essence demeure. &lt;/p&gt; &lt;p&gt;  L'essentialisme peut s'appliquer à divers domaines  comme la Métaphysique, la nature fondamentale de la réalité et des entités mais aussi la Biologie ou l'idée que les espèces ont des caractéristiques fixes et définissables (bien que cette vision soit largement remise en question par la théorie de l'évolution). L' Identité avec les débats sur l'existence d'une essence de l'identité de genre, de l'identité nationale, etc et pour finir Éthique ou certaines théories morales peuvent reposer sur une conception essentialiste de la nature humaine pour déterminer ce qui est bon ou mauvais. &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F142" s="11" t="s">
         <v>766</v>
@@ -11303,9 +11445,7 @@
       </c>
       <c r="E149" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/D%C3%A9construction_(analyse_de_texte)#:~:text=La%20d%C3%A9construction%20(ou%20le%20d%C3%A9constructionnisme,sous%2Dentendus%20et%20les%20omissions."   title=" Wikipedia"&gt;Le Déconstructionnisme&lt;/a&gt;, tel que développé principalement par Jacques Derrida, n'est pas une doctrine ou une méthode fixe, mais plutôt une approche critique et philosophique qui vise à déconstruire les systèmes de pensée et les textes en révélant les tensions, les contradictions et les hiérarchies cachées qui les sous-tendent. Pour le comprendre, imaginez un bâtiment que vous analysez non seulement pour sa structure apparente, mais aussi pour les fondations invisibles, les matériaux utilisés, les fissures potentielles et les différentes manières dont il pourrait être interprété ou utilisé. Le déconstructionnisme fait quelque chose d'analogue avec les idées et les textes.  Voici les principaux aspects du déconstructionnisme : &lt;/p&gt; &lt;p&gt; 
--  Déconstruction des Oppositions Binaires : La pensée occidentale est souvent structurée autour d'oppositions binaires (par exemple, bien/mal, vrai/faux). Le déconstructionnisme ne cherche pas simplement à inverser ces oppositions, mais à montrer comment chaque terme d'une paire dépend de l'autre pour sa définition et comment la hiérarchie implicite entre eux est instable et arbitraire. &lt;/p&gt; &lt;p&gt; -  Mise en Lumière de l'Instabilité du Sens : Le déconstructionnisme souligne que le sens n'est pas fixe et transparent, mais qu'il est toujours en jeu, différé et dépendant du contexte et des interprétations. Le concept clé de différance (un néologisme de Derrida) exprime cette idée : il combine à la fois la "différence" (le sens émerge des distinctions entre les éléments) et le "différer" (le sens est toujours renvoyé à plus tard, à d'autres contextes et interprétations). &lt;/p&gt; &lt;p&gt; 
-- Révélation des Tensions Internes : Les textes et les systèmes de pensée contiennent souvent des contradictions internes, des non-dits et des présupposés implicites qui minent leur cohérence apparente. Le déconstructionnisme cherche à identifier ces tensions et à montrer comment elles déstabilisent les affirmations centrales du texte ou du système. &lt;/p&gt; &lt;p&gt; - Attention au Langage : Le langage n'est pas un outil neutre pour transmettre des idées, mais il est intrinsèquement ambigu et porteur d'une histoire et de préjugés. Le déconstructionnisme examine attentivement le langage utilisé dans un texte pour révéler les jeux de sens, les métaphores et les implications qui peuvent échapper à une lecture superficielle. &lt;/p&gt; &lt;p&gt; -  Pas une Méthode, mais une Stratégie de Lecture :  Derrida insistait sur le fait que la déconstruction n'est pas une méthode que l'on peut appliquer mécaniquement. C'est plutôt une attitude critique, une manière d'aborder les textes et les idées avec une sensibilité aux complexités et aux non-dits. &lt;/p&gt; &lt;p&gt; Il est important de noter que le déconstructionnisme a souvent été mal compris et critiqué pour son apparente négation du sens ou son relativisme. Cependant, pour Derrida, il ne s'agissait pas de détruire le sens, mais de montrer sa complexité et de nous rendre plus conscients des forces qui le façonnent. &lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/D%C3%A9construction_(analyse_de_texte)#:~:text=La%20d%C3%A9construction%20(ou%20le%20d%C3%A9constructionnisme,sous%2Dentendus%20et%20les%20omissions."   title=" Wikipedia"&gt;Le Déconstructionnisme&lt;/a&gt;, tel que développé principalement par Jacques Derrida, n'est pas une doctrine ou une méthode fixe, mais plutôt une approche critique et philosophique qui vise à déconstruire les systèmes de pensée et les textes en révélant les tensions, les contradictions et les hiérarchies cachées qui les sous-tendent. Pour le comprendre, imaginez un bâtiment que vous analysez non seulement pour sa structure apparente, mais aussi pour les fondations invisibles, les matériaux utilisés, les fissures potentielles et les différentes manières dont il pourrait être interprété ou utilisé. Le déconstructionnisme fait quelque chose d'analogue avec les idées et les textes.  &lt;/p&gt; &lt;p&gt;Déconstruction des Oppositions Binaires : La pensée occidentale est souvent structurée autour d'oppositions binaires (par exemple, bien/mal, vrai/faux). Le déconstructionnisme ne cherche pas simplement à inverser ces oppositions, mais à montrer comment chaque terme d'une paire dépend de l'autre pour sa définition et comment la hiérarchie implicite entre eux est instable et arbitraire. &lt;/p&gt; &lt;p&gt;Mise en Lumière de l'Instabilité du Sens : Le déconstructionnisme souligne que le sens n'est pas fixe et transparent, mais qu'il est toujours en jeu, différé et dépendant du contexte et des interprétations. Le concept clé de différance (un néologisme de Derrida) exprime cette idée : il combine à la fois la "différence" (le sens émerge des distinctions entre les éléments) et le "différer" (le sens est toujours renvoyé à plus tard, à d'autres contextes et interprétations). &lt;/p&gt; &lt;p&gt;Révélation des Tensions Internes : Les textes et les systèmes de pensée contiennent souvent des contradictions internes, des non-dits et des présupposés implicites qui minent leur cohérence apparente. Le déconstructionnisme cherche à identifier ces tensions et à montrer comment elles déstabilisent les affirmations centrales du texte ou du système. &lt;/p&gt; &lt;p&gt;Attention au Langage : Le langage n'est pas un outil neutre pour transmettre des idées, mais il est intrinsèquement ambigu et porteur d'une histoire et de préjugés. Le déconstructionnisme examine attentivement le langage utilisé dans un texte pour révéler les jeux de sens, les métaphores et les implications qui peuvent échapper à une lecture superficielle. &lt;/p&gt; &lt;p&gt;Pas une Méthode, mais une Stratégie de Lecture :  Derrida insistait sur le fait que la déconstruction n'est pas une méthode que l'on peut appliquer mécaniquement. C'est plutôt une attitude critique, une manière d'aborder les textes et les idées avec une sensibilité aux complexités et aux non-dits. &lt;/p&gt; &lt;p&gt; le déconstructionnisme a souvent été mal compris et critiqué pour son apparente négation du sens ou son relativisme. Cependant, pour Derrida, il ne s'agissait pas de détruire le sens, mais de montrer sa complexité et de nous rendre plus conscients des forces qui le façonnent. &lt;/p&gt;</t>
         </is>
       </c>
       <c r="F149" s="11" t="s">
@@ -11570,8 +11710,10 @@
       <c r="D154" s="12" t="s">
         <v>823</v>
       </c>
-      <c r="E154" s="13" t="s">
-        <v>824</v>
+      <c r="E154" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Post-structuralisme" title=" Wikipedia"&gt;Le Post-structuralisme&lt;/a&gt;  est un courant philosophique et critique qui prolonge et critique le structuralisme en remettant en question les structures fixes, les significations stables et les vérités absolues. Il insiste sur l'instabilité des signes, le rôle du pouvoir dans les discours et la fluidité des identités, influençant les sciences humaines, la littérature et l'anthropologie. &lt;/p&gt; &lt;p&gt; Émergé après le structuralisme de Lévi-Strauss ou Saussure, qui analysait les systèmes sous-jacents (langage, mythes), le post-structuralisme dénonce leur rigidité. Jacques Derrida introduit la déconstruction dès De la grammatologie (1967), montrant que les textes sont polysémiques et indéterminés. Michel Foucault explore dans Les Mots et les choses (1966) comment le savoir est un effet de pouvoir, historicisé en épistémès. &lt;/p&gt; &lt;p&gt; Il rejette les fondations universelles : la vérité est construite par des discours instables, le sujet est éclaté (pas d'ego unifié), et le langage précède la réalité (signifiant sans signifié fixe). Il privilégie l'analyse critique des hiérarchies implicites et des exclusions. Les principaux penseurs sont : Jacques Derrida : Déconstruction des binaires (présence/absence), différance comme jeu infini des signes. Michel Foucault : Généalogie du pouvoir, discours comme dispositifs disciplinaires (Surveiller et punir, 1975). &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F154" s="11" t="s">
         <v>825</v>
@@ -11717,8 +11859,11 @@
       <c r="D157" s="15" t="s">
         <v>839</v>
       </c>
-      <c r="E157" s="16" t="s">
-        <v>840</v>
+      <c r="E157" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/French_Theory"    title=" Wikipedia"&gt;La French Theory&lt;/a&gt; : Une Révolution des Idées à la française. &lt;/p&gt; &lt;p&gt; Dans les années 1960, une vague de penseurs français secoue les fondements de la philosophie et des sciences humaines. Leurs idées, souvent complexes mais toujours provocantes, traversent l’Atlantique pour influencer profondément les universités américaines. On les regroupe sous le nom de French Theory, un courant qui n’est pas une école organisée, mais plutôt une constellation d’esprits brillants remettant en question les certitudes de l’Occident. &lt;/p&gt; &lt;p&gt; Au cœur de ce mouvement, Michel Foucault explore les mécanismes du pouvoir, révélant comment les prisons, les hôpitaux et même la sexualité sont des instruments de contrôle. Son contemporain, Jacques Derrida, ébranle la philosophie avec sa déconstruction, montrant que le langage est toujours instable, que les mots ne captent jamais tout à fait le réel. Tandis que Gilles Deleuze et Félix Guattari imaginent un monde où le désir ne serait pas réprimé, où la pensée ne suivrait pas des lignes droites, mais se déploierait en rhizomes, comme des racines souterraines et imprévisibles. Pendant ce temps, Jean-François Lyotard annonce la fin des grands récits – plus de croyance absolue dans le Progrès, la Science ou la Révolution. Roland Barthes, lui, dissèque les mythes modernes, révélant comment la publicité, le cinéma ou la politique fabriquent du sens à notre insu. Julia Kristeva, entre psychanalyse et linguistique, explore les frontières mouvantes de l’identité. Enfin, Jean Baudrillard pousse la critique plus loin : et si notre époque n’était plus qu’un jeu de simulations, où le réel a disparu sous les images ? &lt;/p&gt;
+&lt;p&gt; Ces idées ont bouleversé les études littéraires, la sociologie, et même les mouvements militants. Aux États-Unis, elles ont nourri les Gender Studies, les théories queer, et une remise en question radicale des normes. Mais la French Theory a aussi suscité des rejets. Certains lui reprochent son jargon, son obscurité, ou son relativisme excessif. L’affaire Sokal, où un physicien a piégé une revue en publiant un texte absurde sous couvert de postmodernisme, a marqué un tournant dans cette critique. &lt;/p&gt; &lt;p&gt; Pourtant, aujourd’hui encore, ces penseurs continuent d’inspirer. Leurs questions – Qu’est-ce que le pouvoir ? Comment le langage nous influence ? Peut-on échapper aux normes ? – restent brûlantes.  La French Theory, finalement, n’est pas qu’un moment de l’histoire des idées, c’est une boîte à outils pour démonter les évidences et imaginer d’autres mondes possibles.&lt;/p&gt;   &lt;audio controls title="La French theory, what else ?  par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-07.09.2016-ITEMA_21069154-2016C12410S0251-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; &lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F157" s="14" t="s">
         <v>841</v>
@@ -12289,8 +12434,13 @@
       <c r="D169" s="12" t="s">
         <v>902</v>
       </c>
-      <c r="E169" s="13" t="s">
-        <v>903</v>
+      <c r="E169" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Nouveau_r%C3%A9alisme"  title=" Wikipedia"&gt; Le Nouveau Réalisme&lt;/a&gt; est un courant philosophique contemporain qui cherche à réaffirmer l'importance de la réalité et de l'expérience directe dans la philosophie, en s'opposant à certaines tendances du postmodernisme. &lt;/p&gt; &lt;p&gt; 
+Les Nouveaux Réalistes mettent l'accent sur l'existence d'un monde réel indépendant de notre perception ou de notre représentation de celui-ci. Ils rejettent l'idée que la réalité est entièrement construite socialement ou linguistiquement, et insistent sur l'objectivité de certains phénomènes et faits. Selon eux, il existe des réalités objectives qui existent en dehors de notre conscience et qui peuvent être étudiées et décrites de manière impartiale. &lt;/p&gt; &lt;p&gt; 
+Il s'intéresse également aux aspects pratiques et concrets de la vie quotidienne en s'attachant à étudier des objets ou des phénomènes ordinaires, souvent négligés par la philosophie traditionnelle. Ils accordent de l'importance à la matérialité et à la corporeité, et mettent en avant la dimension sensorielle de l'expérience. &lt;/p&gt; &lt;p&gt; 
+Parmi les principaux représentants du Nouveau Réalisme, on peut citer le philosophe français Bruno Latour, qui s'intéresse notamment aux relations entre la science, la société et la politique. Le sociologue et philosophe allemand Hartmut Rosa est également associé à ce courant, en mettant l'accent sur la relation entre l'accélération sociale et la perte de contact avec la réalité. &lt;/p&gt; </t>
+        </is>
       </c>
       <c r="F169" s="11" t="s">
         <v>904</v>
@@ -12537,7 +12687,7 @@
       </c>
       <c r="E174" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Woke#:~:text=Par%20exemple%2C%20MTV%20News%20l,ne%20l'es%20pas%20%C2%BB."  style="color:#d35400"  title=" Wikipedia"&gt;Le Wokisme&lt;/a&gt;, diré du mot "woke" (éveillé en anglais) était utilisé dans les communautés afro-américaines pour désigner une prise de conscience des injustices raciales et sociales. Il invitait à rester vigilant face aux discriminations. &lt;/p&gt;  Aujourd'hui, le terme "wokisme" a pris une connotation plus large et plus complexe. Il est souvent utilisé pour décrire les questions d'injustice sociale, Il encourage à remettre en question les normes sociales et les stéréotypes, en particulier ceux liés à la race, au genre, à l'orientation sexuelle. Les personnes considérées comme "woke" cherchent à créer une société plus juste et équitable pour tous, en dénonçant les discriminations et en promouvant la diversité. Ils s'intéressent aux mécanismes qui perpétuent les inégalités, comme le racisme systémique, le sexisme, l'homophobie. &lt;/p&gt; &lt;p&gt; Certains accusent les personnes "woke" d'être trop radicales et de vouloir censurer les opinions dissidentes. On leur reproche de diviser la société en groupes identitaires et de nier l'existence d'une humanité universelle. Ses détracteurs estiment que les personnes "woke" exagèrent les problèmes et se présentent comme des victimes. &lt;/p&gt;  &lt;p&gt;  &lt;p&gt; Il remet en question les valeurs traditionnelles et propose une vision plus inclusive de la société, contribuant à l'émergence de nouveaux mots et expressions pour décrire les expériences des personnes marginalisées. &lt;/p&gt;   &lt;p&gt; Des philosophes comme Judith Butler, philosophe féministe et queer qui a développé la théorie du genre et a questionné les normes de genre et de sexualité. Michel Foucault, historien et philosophe, il a analysé les rapports de pouvoir et les mécanismes de domination dans la société. Kimberlé Crenshaw, juriste et théoricienne féministe, elle a développé le concept d'intersectionnalité, qui permet d'analyser les différentes formes de discrimination qui se croisent et s'additionnent. &lt;/p&gt; &lt;audio controls title="Dieu, un homme en trop ?  "Qu'est ce que le Wokisme? " par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13397-11.06.2022-ITEMA_23055745-2022C3397E0022-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Woke"  style="color:#d35400"  title=" Wikipedia"&gt;Le Wokisme&lt;/a&gt;, dérivé du mot "woke" (éveillé en anglais) était utilisé dans les communautés afro-américaines pour désigner une prise de conscience des injustices raciales et sociales. Il invitait à rester vigilant face aux discriminations. &lt;/p&gt;  Aujourd'hui, le terme "wokisme" a pris une connotation plus large et plus complexe. Il est souvent utilisé pour décrire les questions d'injustice sociale, Il encourage à remettre en question les normes sociales et les stéréotypes, en particulier ceux liés à la race, au genre, à l'orientation sexuelle. Les personnes considérées comme "woke" cherchent à créer une société plus juste et équitable pour tous, en dénonçant les discriminations et en promouvant la diversité. Ils s'intéressent aux mécanismes qui perpétuent les inégalités, comme le racisme systémique, le sexisme, l'homophobie. &lt;/p&gt; &lt;p&gt; Certains accusent les personnes "woke" d'être trop radicales et de vouloir censurer les opinions dissidentes. On leur reproche de diviser la société en groupes identitaires et de nier l'existence d'une humanité universelle. Ses détracteurs estiment que les personnes "woke" exagèrent les problèmes et se présentent comme des victimes. &lt;/p&gt; &lt;p&gt;  &lt;p&gt; Il remet en question les valeurs traditionnelles et propose une vision plus inclusive de la société, contribuant à l'émergence de nouveaux mots et expressions pour décrire les expériences des personnes marginalisées. &lt;/p&gt; &lt;p&gt; Des philosophes comme Judith Butler, philosophe féministe et queer qui a développé la théorie du genre et a questionné les normes de genre et de sexualité. Michel Foucault, historien et philosophe, il a analysé les rapports de pouvoir et les mécanismes de domination dans la société. Kimberlé Crenshaw, juriste et théoricienne féministe, elle a développé le concept d'intersectionnalité, qui permet d'analyser les différentes formes de discrimination qui se croisent et s'additionnent. &lt;/p&gt; &lt;audio controls title="Dieu, un homme en trop ?  "Qu'est ce que le Wokisme? " par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13397-11.06.2022-ITEMA_23055745-2022C3397E0022-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
       <c r="F174" s="11" t="s">

</xml_diff>

<commit_message>
Fiches — 2 fiches modifiées : Charlotte WERNDL, Nihilisme (courant) ; 1 image
Publié depuis l'éditeur des fiches.
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-occidental.xlsx
+++ b/data/frise-courant-pensee-occidental.xlsx
@@ -7293,81 +7293,93 @@
         </is>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="11">
+    <row r="68" customFormat="false" ht="165.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="14" t="n">
+        <v>1860</v>
+      </c>
+      <c r="B68" s="14"/>
+      <c r="C68" s="14" t="s">
+        <v>565</v>
+      </c>
+      <c r="D68" s="15" t="s">
+        <v>566</v>
+      </c>
+      <c r="E68" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Nihilisme" title=" Wikipedia"&gt; Le Nihilisme&lt;/a&gt; est une position philosophique qui remet en question ou nie la valeur et la signification de la vie, de la connaissance, de la morale et d'autres concepts fondamentaux. Les nihilistes affirment que la réalité est dépourvue de sens intrinsèque, de valeurs objectives ou de vérités ultimes et que rien n'a de valeur ou d'importance réelle, et que toutes les croyances, les systèmes moraux et les vérités sont des constructions arbitraires et illusoires. &lt;/p&gt; &lt;p&gt;
+Il peut prendre différentes formes et être appliqué à différents domaines de la philosophie. Le nihilisme métaphysique, par exemple, nie l'existence de toute réalité objective ou transcendante. Il n'y a pas de Dieu, d'âme, de monde spirituel ou de finalité ultime dans l'univers. &lt;/p&gt; &lt;p&gt;
+Le nihilisme épistémologique remet en question la possibilité de connaître la réalité telle qu'elle est en soi et soutient que nos perceptions et nos croyances sont toujours limitées et subjectives, et qu'il est impossible d'atteindre une connaissance objective et complète. &lt;/p&gt; &lt;p&gt;
+Le nihilisme moral rejette l'idée de valeurs morales objectives et que les notions de bien et de mal sont des constructions humaines sans fondement réel, que la morale est une illusion et que chaque individu est libre de créer ses propres valeurs ou d'adopter l'absence totale de valeurs. &lt;/p&gt; &lt;p&gt;
+le nihilisme n'est pas nécessairement une position que l'on adopte activement, mais plutôt une perspective critique qui remet en question les systèmes de croyances et les valeurs établies. Certains philosophes ont même fait valoir que le nihilisme peut être un point de départ pour la construction d'une nouvelle signification et de nouvelles valeurs. &lt;/p&gt;  &lt;audio controls title="Le nouveau Nihilisme par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/12014-16.11.2015-ITEMA_20842008-2015C18009S0320-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
+      </c>
+      <c r="F68" s="14" t="s">
+        <v>568</v>
+      </c>
+      <c r="G68" s="16" t="s">
+        <v>569</v>
+      </c>
+      <c r="H68" s="14"/>
+      <c r="I68" s="16"/>
+      <c r="J68" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="K68" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Slavophiles, occidentalistes et nihilistes</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matérialisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="153" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="11">
         <v>1871</v>
-      </c>
-      <c r="B68" s="11"/>
-      <c r="C68" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1871</t>
-        </is>
-      </c>
-      <c r="D68" s="23" t="s">
-        <v>362</v>
-      </c>
-      <c r="E68" s="24" t="s">
-        <v>363</v>
-      </c>
-      <c r="F68" s="11" t="s">
-        <v>364</v>
-      </c>
-      <c r="G68" s="13" t="s">
-        <v>365</v>
-      </c>
-      <c r="H68" s="11"/>
-      <c r="I68" s="11"/>
-      <c r="J68" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ontologie où humains et non-humains partagent une même intériorité, une âme, mais diffèrent par leur corps (Descola).</t>
-        </is>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">position</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comment les sociétés pensent-elles la nature ? (Descola)</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="11">
-        <v>1869</v>
       </c>
       <c r="B69" s="11"/>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1869</t>
+          <t xml:space="preserve">1871</t>
         </is>
       </c>
       <c r="D69" s="23" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E69" s="24" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="G69" s="13" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="H69" s="11"/>
       <c r="I69" s="11"/>
       <c r="J69" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">ontologie où un groupe humain et une espèce animale ou végétale partagent les mêmes qualités, physiques et morales (Descola).</t>
+          <t xml:space="preserve">ontologie où humains et non-humains partagent une même intériorité, une âme, mais diffèrent par leur corps (Descola).</t>
         </is>
       </c>
       <c r="K69" s="1" t="s">
@@ -7389,33 +7401,33 @@
         </is>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="117" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="11">
-        <v>2005</v>
+        <v>1869</v>
       </c>
       <c r="B70" s="11"/>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">2005</t>
+          <t xml:space="preserve">1869</t>
         </is>
       </c>
       <c r="D70" s="23" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="E70" s="24" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="F70" s="11" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
       <c r="G70" s="13" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="H70" s="11"/>
       <c r="I70" s="11"/>
       <c r="J70" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">ontologie qui voit le monde comme une multitude d’êtres tous différents, reliés par un réseau de correspondances (Descola).</t>
+          <t xml:space="preserve">ontologie où un groupe humain et une espèce animale ou végétale partagent les mêmes qualités, physiques et morales (Descola).</t>
         </is>
       </c>
       <c r="K70" s="1" t="s">
@@ -7437,7 +7449,7 @@
         </is>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="117" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11">
         <v>2005</v>
       </c>
@@ -7448,22 +7460,22 @@
         </is>
       </c>
       <c r="D71" s="23" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="E71" s="24" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="G71" s="13" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="H71" s="11"/>
       <c r="I71" s="11"/>
       <c r="J71" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">ontologie moderne où tous les êtres partagent une même nature physique, mais où seuls les humains ont une intériorité (Descola).</t>
+          <t xml:space="preserve">ontologie qui voit le monde comme une multitude d’êtres tous différents, reliés par un réseau de correspondances (Descola).</t>
         </is>
       </c>
       <c r="K71" s="1" t="s">
@@ -7485,37 +7497,37 @@
         </is>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="11" t="n">
-        <v>1728</v>
+    <row r="72" customFormat="false" ht="176.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="11">
+        <v>2005</v>
       </c>
       <c r="B72" s="11"/>
-      <c r="C72" s="11" t="n">
-        <v>1728</v>
-      </c>
-      <c r="D72" s="12" t="s">
-        <v>383</v>
-      </c>
-      <c r="E72" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pluralisme_(philosophie)"  title=" Wikipedia"&gt;Le Pluralisme&lt;/a&gt; désigne, en philosophie, la thèse selon laquelle la réalité est faite de plusieurs principes, êtres ou valeurs irréductibles les uns aux autres. Il s’oppose au monisme, qui ramène tout à un seul principe, et au dualisme, qui en compte deux. Le mot est forgé vers 1720 par le philosophe allemand Christian Wolff, mais l’idée est bien plus ancienne.&lt;/p&gt; &lt;p&gt;Chez les présocratiques, &lt;a href="https://fr.wikipedia.org/wiki/Emp%C3%A9docle" title=" Wikipedia"&gt;Empédocle&lt;/a&gt; explique le monde par quatre éléments, la terre, l’eau, l’air et le feu, que l’Amour unit et que la Haine sépare ; Anaxagore pose une infinité de « semences » mêlées en toute chose, et les atomistes une infinité d’atomes. Leibniz, avec ses monades innombrables, propose un pluralisme métaphysique. Au début du XXe siècle, &lt;a href="https://fr.wikipedia.org/wiki/William_James" title=" Wikipedia"&gt;William James&lt;/a&gt; défend dans &lt;em&gt;Un univers pluraliste&lt;/em&gt; (1909) un monde ouvert, inachevé, où la nouveauté et la liberté sont réelles, contre l’idéalisme qui fait de tout un seul bloc. Le pluralisme s’étend ensuite à la connaissance : plusieurs théories ou méthodes peuvent éclairer chacune une part du réel, sans qu’aucune n’épuise la vérité.&lt;/p&gt; &lt;p&gt;En morale et en politique, &lt;a href="https://fr.wikipedia.org/wiki/Isaiah_Berlin" title=" Wikipedia"&gt;Isaiah Berlin&lt;/a&gt; soutient que les valeurs humaines, liberté, égalité, justice ou pitié, sont multiples et parfois incompatibles : il n’existe pas de solution unique et parfaite. Cette idée nourrit le libéralisme et la réflexion sur la tolérance dans les sociétés démocratiques. Michael Walzer la prolonge : chaque sphère de la vie sociale, le marché, la politique, l’école ou la famille, obéit à ses propres règles de justice.&lt;/p&gt;</t>
-        </is>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2005</t>
+        </is>
+      </c>
+      <c r="D72" s="23" t="s">
+        <v>378</v>
+      </c>
+      <c r="E72" s="24" t="s">
+        <v>379</v>
       </c>
       <c r="F72" s="11" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="G72" s="13" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="H72" s="11"/>
-      <c r="I72" s="13"/>
-      <c r="J72" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thèse selon laquelle le réel est fait de plusieurs substances ou principes, irréductibles les uns aux autres.</t>
-        </is>
-      </c>
-      <c r="K72" s="3" t="s">
-        <v>27</v>
+      <c r="I72" s="11"/>
+      <c r="J72" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ontologie moderne où tous les êtres partagent une même nature physique, mais où seuls les humains ont une intériorité (Descola).</t>
+        </is>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="M72" t="inlineStr">
         <is>
@@ -7529,11 +7541,11 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le réel est-il un ou multiple ?</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="266.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+          <t xml:space="preserve">Comment les sociétés pensent-elles la nature ? (Descola)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="n">
         <v>1728</v>
       </c>
@@ -7542,22 +7554,24 @@
         <v>1728</v>
       </c>
       <c r="D73" s="12" t="s">
-        <v>388</v>
-      </c>
-      <c r="E73" s="26" t="s">
-        <v>389</v>
+        <v>383</v>
+      </c>
+      <c r="E73" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pluralisme_(philosophie)"  title=" Wikipedia"&gt;Le Pluralisme&lt;/a&gt; désigne, en philosophie, la thèse selon laquelle la réalité est faite de plusieurs principes, êtres ou valeurs irréductibles les uns aux autres. Il s’oppose au monisme, qui ramène tout à un seul principe, et au dualisme, qui en compte deux. Le mot est forgé vers 1720 par le philosophe allemand Christian Wolff, mais l’idée est bien plus ancienne.&lt;/p&gt; &lt;p&gt;Chez les présocratiques, &lt;a href="https://fr.wikipedia.org/wiki/Emp%C3%A9docle" title=" Wikipedia"&gt;Empédocle&lt;/a&gt; explique le monde par quatre éléments, la terre, l’eau, l’air et le feu, que l’Amour unit et que la Haine sépare ; Anaxagore pose une infinité de « semences » mêlées en toute chose, et les atomistes une infinité d’atomes. Leibniz, avec ses monades innombrables, propose un pluralisme métaphysique. Au début du XXe siècle, &lt;a href="https://fr.wikipedia.org/wiki/William_James" title=" Wikipedia"&gt;William James&lt;/a&gt; défend dans &lt;em&gt;Un univers pluraliste&lt;/em&gt; (1909) un monde ouvert, inachevé, où la nouveauté et la liberté sont réelles, contre l’idéalisme qui fait de tout un seul bloc. Le pluralisme s’étend ensuite à la connaissance : plusieurs théories ou méthodes peuvent éclairer chacune une part du réel, sans qu’aucune n’épuise la vérité.&lt;/p&gt; &lt;p&gt;En morale et en politique, &lt;a href="https://fr.wikipedia.org/wiki/Isaiah_Berlin" title=" Wikipedia"&gt;Isaiah Berlin&lt;/a&gt; soutient que les valeurs humaines, liberté, égalité, justice ou pitié, sont multiples et parfois incompatibles : il n’existe pas de solution unique et parfaite. Cette idée nourrit le libéralisme et la réflexion sur la tolérance dans les sociétés démocratiques. Michael Walzer la prolonge : chaque sphère de la vie sociale, le marché, la politique, l’école ou la famille, obéit à ses propres règles de justice.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F73" s="11" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="G73" s="13" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="H73" s="11"/>
       <c r="I73" s="13"/>
-      <c r="J73" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">doctrine selon laquelle nous ne connaissons que des phénomènes, c’est-à-dire les choses telles qu’elles nous apparaissent.</t>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thèse selon laquelle le réel est fait de plusieurs substances ou principes, irréductibles les uns aux autres.</t>
         </is>
       </c>
       <c r="K73" s="3" t="s">
@@ -7575,24 +7589,70 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
+          <t xml:space="preserve">Le réel est-il un ou multiple ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="266.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="11" t="n">
+        <v>1728</v>
+      </c>
+      <c r="B74" s="11"/>
+      <c r="C74" s="11" t="n">
+        <v>1728</v>
+      </c>
+      <c r="D74" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="E74" s="26" t="s">
+        <v>389</v>
+      </c>
+      <c r="F74" s="11" t="s">
+        <v>390</v>
+      </c>
+      <c r="G74" s="13" t="s">
+        <v>391</v>
+      </c>
+      <c r="H74" s="11"/>
+      <c r="I74" s="13"/>
+      <c r="J74" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">doctrine selon laquelle nous ne connaissons que des phénomènes, c’est-à-dire les choses telles qu’elles nous apparaissent.</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
           <t xml:space="preserve">Que pouvons-nous connaître ?</t>
         </is>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="202.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="14" t="n">
+    <row r="75" customFormat="false" ht="202.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="14" t="n">
         <v>1735</v>
       </c>
-      <c r="B74" s="14"/>
-      <c r="C74" s="14" t="s">
+      <c r="B75" s="14"/>
+      <c r="C75" s="14" t="s">
         <v>393</v>
       </c>
-      <c r="D74" s="15" t="inlineStr">
+      <c r="D75" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Lumières</t>
         </is>
       </c>
-      <c r="E74" s="16" t="inlineStr">
+      <c r="E75" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Lumi%C3%A8res_(philosophie)" title=" Wikipedia"&gt;Les Lumières&lt;/a&gt; sont un mouvement intellectuel et philosophique qui s'est développé en Europe aux XVIIe et XVIIIe siècles. Leurs penseurs remettaient en question les dogmes religieux et l'autorité absolue des monarchies, tout en prônant la raison, la science et la tolérance. &lt;/p&gt; &lt;p&gt;
 Ils cherchaient à éclairer l'esprit des individus en promouvant les idées de liberté, d'égalité, de démocratie, de progrès et de droits de l'homme et ils s'opposaient aux préjugés, à l'obscurantisme et à l'intolérance, et plaçaient la raison au centre de leurs réflexions. &lt;/p&gt; &lt;p&gt;
@@ -7602,633 +7662,584 @@
 </t>
         </is>
       </c>
-      <c r="F74" s="14" t="s">
+      <c r="F75" s="14" t="s">
         <v>396</v>
       </c>
-      <c r="G74" s="16" t="s">
+      <c r="G75" s="16" t="s">
         <v>397</v>
-      </c>
-      <c r="H74" s="14"/>
-      <c r="I74" s="16"/>
-      <c r="J74" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement philosophique européen du XVIIIe siècle qui prône la raison, la tolérance, la liberté et le progrès contre les préjugés et l'arbitraire.</t>
-        </is>
-      </c>
-      <c r="K74" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Philosophie politique;Épistémologie</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VOLTAIRE;Denis DIDEROT;MONTESQUIEU;Emmanuel KANT</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lumières et pensée politique moderne</t>
-        </is>
-      </c>
-      <c r="Q74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cartésianisme;Empirisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="162.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="14" t="n">
-        <v>1740</v>
-      </c>
-      <c r="B75" s="14"/>
-      <c r="C75" s="14" t="n">
-        <v>1740</v>
-      </c>
-      <c r="D75" s="15" t="s">
-        <v>399</v>
-      </c>
-      <c r="E75" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Monisme"  title=" Wikipedia"&gt;Le Monisme&lt;/a&gt; désigne toute doctrine qui ramène la diversité du réel à une seule substance ou à un seul principe. Le mot est forgé en 1734 par le philosophe allemand Christian Wolff dans sa &lt;em&gt;Psychologia rationalis&lt;/em&gt;, pour désigner ceux qui n’admettent qu’une seule sorte de substance, par opposition au &lt;a href="https://fr.wikipedia.org/wiki/Dualisme_%28philosophie_de_l%27esprit%29" title=" Wikipedia"&gt;dualisme&lt;/a&gt; de Descartes, qui distinguait l’âme et le corps. Il entre en français à la fin du XIXe siècle.&lt;/p&gt; &lt;p&gt;Les idées monistes sont pourtant bien plus anciennes. Parménide affirme que l’Être est un, éternel et immobile ; Héraclite voit dans le Logos l’unité des contraires. En Inde, l’Advaita Védanta enseigne que l’âme individuelle et l’absolu, le Brahman, ne font qu’un. Le premier grand monisme moderne est celui de Spinoza : dans l’&lt;em&gt;Éthique&lt;/em&gt; (1677), il n’existe qu’une seule substance infinie, « Dieu, c’est-à-dire la Nature », dont la pensée et l’étendue ne sont que deux attributs. On distingue ensuite plusieurs formes de monisme : matérialiste, quand tout se ramène à la matière, comme chez d’Holbach ou chez le biologiste &lt;a href="https://fr.wikipedia.org/wiki/Ernst_Haeckel" title=" Wikipedia"&gt;Ernst Haeckel&lt;/a&gt;, qui fonde en 1906 une Ligue moniste ; idéaliste, quand tout est esprit, comme chez Hegel, pour qui le réel est le déploiement de l’Esprit absolu ; ou neutre, quand matière et esprit sont deux aspects d’une réalité plus fondamentale, comme chez William James ou Bertrand Russell.&lt;/p&gt; &lt;p&gt;En philosophie de l’esprit, le débat entre monisme et dualisme reste vif : la plupart des philosophes contemporains sont monistes et cherchent à expliquer la conscience comme un phénomène naturel, tandis que d’autres jugent cette réduction impossible. Le monisme s’oppose ainsi au dualisme, qui admet deux principes, et au pluralisme, qui en admet plusieurs.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F75" s="14" t="s">
-        <v>401</v>
-      </c>
-      <c r="G75" s="16" t="s">
-        <v>402</v>
       </c>
       <c r="H75" s="14"/>
       <c r="I75" s="16"/>
       <c r="J75" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">mouvement philosophique européen du XVIIIe siècle qui prône la raison, la tolérance, la liberté et le progrès contre les préjugés et l'arbitraire.</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique;Épistémologie</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VOLTAIRE;Denis DIDEROT;MONTESQUIEU;Emmanuel KANT</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cartésianisme;Empirisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="162.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="14" t="n">
+        <v>1740</v>
+      </c>
+      <c r="B76" s="14"/>
+      <c r="C76" s="14" t="n">
+        <v>1740</v>
+      </c>
+      <c r="D76" s="15" t="s">
+        <v>399</v>
+      </c>
+      <c r="E76" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Monisme"  title=" Wikipedia"&gt;Le Monisme&lt;/a&gt; désigne toute doctrine qui ramène la diversité du réel à une seule substance ou à un seul principe. Le mot est forgé en 1734 par le philosophe allemand Christian Wolff dans sa &lt;em&gt;Psychologia rationalis&lt;/em&gt;, pour désigner ceux qui n’admettent qu’une seule sorte de substance, par opposition au &lt;a href="https://fr.wikipedia.org/wiki/Dualisme_%28philosophie_de_l%27esprit%29" title=" Wikipedia"&gt;dualisme&lt;/a&gt; de Descartes, qui distinguait l’âme et le corps. Il entre en français à la fin du XIXe siècle.&lt;/p&gt; &lt;p&gt;Les idées monistes sont pourtant bien plus anciennes. Parménide affirme que l’Être est un, éternel et immobile ; Héraclite voit dans le Logos l’unité des contraires. En Inde, l’Advaita Védanta enseigne que l’âme individuelle et l’absolu, le Brahman, ne font qu’un. Le premier grand monisme moderne est celui de Spinoza : dans l’&lt;em&gt;Éthique&lt;/em&gt; (1677), il n’existe qu’une seule substance infinie, « Dieu, c’est-à-dire la Nature », dont la pensée et l’étendue ne sont que deux attributs. On distingue ensuite plusieurs formes de monisme : matérialiste, quand tout se ramène à la matière, comme chez d’Holbach ou chez le biologiste &lt;a href="https://fr.wikipedia.org/wiki/Ernst_Haeckel" title=" Wikipedia"&gt;Ernst Haeckel&lt;/a&gt;, qui fonde en 1906 une Ligue moniste ; idéaliste, quand tout est esprit, comme chez Hegel, pour qui le réel est le déploiement de l’Esprit absolu ; ou neutre, quand matière et esprit sont deux aspects d’une réalité plus fondamentale, comme chez William James ou Bertrand Russell.&lt;/p&gt; &lt;p&gt;En philosophie de l’esprit, le débat entre monisme et dualisme reste vif : la plupart des philosophes contemporains sont monistes et cherchent à expliquer la conscience comme un phénomène naturel, tandis que d’autres jugent cette réduction impossible. Le monisme s’oppose ainsi au dualisme, qui admet deux principes, et au pluralisme, qui en admet plusieurs.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F76" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="G76" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="H76" s="14"/>
+      <c r="I76" s="16"/>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">doctrine selon laquelle toute la réalité se ramène à une seule substance ou à un seul principe (Parménide, Spinoza).</t>
         </is>
       </c>
-      <c r="K75" s="3" t="s">
+      <c r="K76" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="N75" t="inlineStr">
+      <c r="M76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
         <is>
           <t xml:space="preserve">russe;sud</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr">
+      <c r="O76" t="inlineStr">
         <is>
           <t xml:space="preserve">position</t>
         </is>
       </c>
-      <c r="P75" t="inlineStr">
+      <c r="P76" t="inlineStr">
         <is>
           <t xml:space="preserve">Le réel est-il un ou multiple ?</t>
         </is>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="11" t="n">
+    <row r="77" customFormat="false" ht="272.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="11" t="n">
         <v>1750</v>
       </c>
-      <c r="B76" s="11"/>
-      <c r="C76" s="11" t="s">
+      <c r="B77" s="11"/>
+      <c r="C77" s="11" t="s">
         <v>404</v>
       </c>
-      <c r="D76" s="12" t="s">
+      <c r="D77" s="12" t="s">
         <v>405</v>
       </c>
-      <c r="E76" s="13" t="inlineStr">
+      <c r="E77" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Libertarianisme" title=" Wikipedia"&gt;Le Libertarianisme&lt;/a&gt;  ou Libertarisme est un courant politique et philosophique qui met l'accent sur la liberté individuelle et la primauté de l'individu sur l'État. Ses origines remontent aux idées du siècle des Lumières et ont été développées plus tard par des penseurs comme John Locke, Adam Smith, et plus récemment par des figures comme Friedrich Hayek, Robert Nozick et Murray Rothbard. &lt;/p&gt; &lt;p&gt;Les libertariens croient en un gouvernement minimal, dont le rôle se limiterait à protéger les droits naturels des individus, limité, à la défense nationale et l'application des contrats. Ils s'opposent aux interventions gouvernementales dans des domaines tels que la santé, l'éducation et la moralité individuelle.tels que la vie, la liberté et la propriété. Ils prônent généralement une réduction drastique du rôle de l'État dans l'économie, préférant les mécanismes du marché libre pour réguler les échanges et allouer les ressources considérant la liberté individuelle comme étant de la plus haute importance. Ils soutiennent que les individus devraient avoir le droit de vivre leur vie comme ils l'entendent, tant qu'ils ne violent pas les droits des autres. &lt;/p&gt; &lt;p&gt;Ils défendent le droit à la propriété privée. Ils estiment que les individus ont le droit de posséder et de disposer de leurs biens comme bon leur semble, sans ingérence injustifiée de l'État et ils  favorisent généralement une économie de marché non réglementée, où l'offre et la demande déterminent les prix et les allocations de ressources. Ils soutiennent que les interventions gouvernementales dans l'économie, telles que les taxes excessives ou les réglementations strictes, entravent la liberté et nuisent à la prospérité économique. &lt;/p&gt; &lt;p&gt;Le principe de non-agression est central pour les libertariens. Cela signifie qu'ils s'opposent à l'utilisation de la force ou de la coercition, sauf en légitime défense. Ils considèrent toute action initiée par l'État qui viole les droits individuels comme illégitime. &lt;/p&gt; &lt;p&gt;Le libertarisme est souvent perçu comme un spectre politique qui s'étend du libertarianisme de gauche, qui accorde plus d'importance aux droits sociaux et à l'égalité, au libertarianisme de droite, qui met davantage l'accent sur les droits individuels et la primauté du marché libre. Ces variations peuvent conduire à des désaccords internes sur des questions spécifiques, mais tous les libertariens partagent généralement un engagement envers la liberté individuelle et la limitation du pouvoir gouvernemental. &lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F76" s="11" t="s">
+      <c r="F77" s="11" t="s">
         <v>407</v>
       </c>
-      <c r="G76" s="13" t="s">
+      <c r="G77" s="13" t="s">
         <v>408</v>
       </c>
-      <c r="H76" s="11"/>
-      <c r="I76" s="13"/>
-      <c r="J76" s="3" t="s">
+      <c r="H77" s="11"/>
+      <c r="I77" s="13"/>
+      <c r="J77" s="3" t="s">
         <v>409</v>
-      </c>
-      <c r="K76" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="M76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pensées économiques et libertariennes</t>
-        </is>
-      </c>
-      <c r="Q76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Libéralisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="14" t="n">
-        <v>1750</v>
-      </c>
-      <c r="B77" s="14"/>
-      <c r="C77" s="14" t="s">
-        <v>404</v>
-      </c>
-      <c r="D77" s="15" t="s">
-        <v>410</v>
-      </c>
-      <c r="E77" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Anticolonialisme" title=" Wikipedia"&gt;L’Anticolonialisme&lt;/a&gt; désigne l’ensemble des pensées et des luttes qui contestent la colonisation, c’est-à-dire la domination d’un peuple par une puissance étrangère qui s’empare de ses terres, exploite ses ressources et lui impose ses lois. Il en conteste la légitimité morale, au nom de l’égalité des êtres humains, mais aussi l’utilité économique et les justifications culturelles, comme la prétendue « mission civilisatrice ».&lt;/p&gt; &lt;p&gt;Dès le XVIe siècle, &lt;a href="https://fr.wikipedia.org/wiki/Bartolom%C3%A9_de_las_Casas" title=" Wikipedia"&gt;Bartolomé de las Casas&lt;/a&gt; dénonce les massacres des Indiens d’Amérique et, lors de la controverse de Valladolid (1550), défend leur pleine humanité. Au XVIIIe siècle, les Lumières s’en prennent à l’esclavage et aux conquêtes : l’&lt;em&gt;Histoire des deux Indes&lt;/em&gt; de l’abbé Raynal, à laquelle &lt;a href="https://fr.wikipedia.org/wiki/Denis_Diderot" title=" Wikipedia"&gt;Diderot&lt;/a&gt; prête ses pages les plus violentes, appelle les colonisés à la révolte, et la révolution haïtienne, menée par Toussaint Louverture, fonde en 1804 la première république noire. Au XIXe siècle, des libéraux comme Bastiat jugent les colonies ruineuses, tandis que des socialistes et des anarchistes dénoncent leur violence. Au XXe siècle, Lénine lie l’impérialisme au capitalisme, et Gandhi oppose à l’Empire britannique la résistance non violente. Après 1945, l’anticolonialisme porte les luttes d’indépendance, en Asie puis en Afrique.&lt;/p&gt; &lt;p&gt;Ses grands textes sont le &lt;em&gt;Discours sur le colonialisme&lt;/em&gt; (1950) d’&lt;a href="https://fr.wikipedia.org/wiki/Aim%C3%A9_C%C3%A9saire" title=" Wikipedia"&gt;Aimé Césaire&lt;/a&gt; et &lt;em&gt;Les Damnés de la terre&lt;/em&gt; (1961) de &lt;a href="https://fr.wikipedia.org/wiki/Frantz_Fanon" title=" Wikipedia"&gt;Frantz Fanon&lt;/a&gt;. Les études postcoloniales et la pensée décoloniale prolongent aujourd’hui son analyse des effets durables de la colonisation.&lt;/p&gt;  &lt;audio controls title=" "Fanon": le biopic sur la figure de l'anticolonialisme est peu diffusé dans les cinémas mais agite les réseaux par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23694-08.04.2025-ITEMA_24096522-2025J49319S0098-NET_MLM_8C70D14C-38CF-46CE-811B-6AFD802BAF4A-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
-        </is>
-      </c>
-      <c r="F77" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1E_GadDJvKI</t>
-        </is>
-      </c>
-      <c r="G77" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">"Le Temps des archives / 1950 : le Discours sur le colonialisme d'Aimé Césaire" par France Culture</t>
-        </is>
-      </c>
-      <c r="H77" s="14"/>
-      <c r="I77" s="16"/>
-      <c r="J77" s="3" t="s">
-        <v>414</v>
       </c>
       <c r="K77" s="3" t="s">
         <v>251</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées économiques et libertariennes</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Libéralisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="14" t="n">
+        <v>1750</v>
+      </c>
+      <c r="B78" s="14"/>
+      <c r="C78" s="14" t="s">
+        <v>404</v>
+      </c>
+      <c r="D78" s="15" t="s">
+        <v>410</v>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Anticolonialisme" title=" Wikipedia"&gt;L’Anticolonialisme&lt;/a&gt; désigne l’ensemble des pensées et des luttes qui contestent la colonisation, c’est-à-dire la domination d’un peuple par une puissance étrangère qui s’empare de ses terres, exploite ses ressources et lui impose ses lois. Il en conteste la légitimité morale, au nom de l’égalité des êtres humains, mais aussi l’utilité économique et les justifications culturelles, comme la prétendue « mission civilisatrice ».&lt;/p&gt; &lt;p&gt;Dès le XVIe siècle, &lt;a href="https://fr.wikipedia.org/wiki/Bartolom%C3%A9_de_las_Casas" title=" Wikipedia"&gt;Bartolomé de las Casas&lt;/a&gt; dénonce les massacres des Indiens d’Amérique et, lors de la controverse de Valladolid (1550), défend leur pleine humanité. Au XVIIIe siècle, les Lumières s’en prennent à l’esclavage et aux conquêtes : l’&lt;em&gt;Histoire des deux Indes&lt;/em&gt; de l’abbé Raynal, à laquelle &lt;a href="https://fr.wikipedia.org/wiki/Denis_Diderot" title=" Wikipedia"&gt;Diderot&lt;/a&gt; prête ses pages les plus violentes, appelle les colonisés à la révolte, et la révolution haïtienne, menée par Toussaint Louverture, fonde en 1804 la première république noire. Au XIXe siècle, des libéraux comme Bastiat jugent les colonies ruineuses, tandis que des socialistes et des anarchistes dénoncent leur violence. Au XXe siècle, Lénine lie l’impérialisme au capitalisme, et Gandhi oppose à l’Empire britannique la résistance non violente. Après 1945, l’anticolonialisme porte les luttes d’indépendance, en Asie puis en Afrique.&lt;/p&gt; &lt;p&gt;Ses grands textes sont le &lt;em&gt;Discours sur le colonialisme&lt;/em&gt; (1950) d’&lt;a href="https://fr.wikipedia.org/wiki/Aim%C3%A9_C%C3%A9saire" title=" Wikipedia"&gt;Aimé Césaire&lt;/a&gt; et &lt;em&gt;Les Damnés de la terre&lt;/em&gt; (1961) de &lt;a href="https://fr.wikipedia.org/wiki/Frantz_Fanon" title=" Wikipedia"&gt;Frantz Fanon&lt;/a&gt;. Les études postcoloniales et la pensée décoloniale prolongent aujourd’hui son analyse des effets durables de la colonisation.&lt;/p&gt;  &lt;audio controls title=" "Fanon": le biopic sur la figure de l'anticolonialisme est peu diffusé dans les cinémas mais agite les réseaux par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23694-08.04.2025-ITEMA_24096522-2025J49319S0098-NET_MLM_8C70D14C-38CF-46CE-811B-6AFD802BAF4A-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
+      </c>
+      <c r="F78" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1E_GadDJvKI</t>
+        </is>
+      </c>
+      <c r="G78" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Le Temps des archives / 1950 : le Discours sur le colonialisme d'Aimé Césaire" par France Culture</t>
+        </is>
+      </c>
+      <c r="H78" s="14"/>
+      <c r="I78" s="16"/>
+      <c r="J78" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="K78" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
           <t xml:space="preserve">sud</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr">
+      <c r="N78" t="inlineStr">
         <is>
           <t xml:space="preserve">islam-juif</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr">
+      <c r="O78" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P77" t="inlineStr">
+      <c r="P78" t="inlineStr">
         <is>
           <t xml:space="preserve">Anticolonialisme et décolonisation</t>
         </is>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="11" t="n">
+    <row r="79" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="11" t="n">
         <v>1750</v>
       </c>
-      <c r="B78" s="11"/>
-      <c r="C78" s="11" t="s">
+      <c r="B79" s="11"/>
+      <c r="C79" s="11" t="s">
         <v>404</v>
       </c>
-      <c r="D78" s="12" t="s">
+      <c r="D79" s="12" t="s">
         <v>415</v>
       </c>
-      <c r="E78" s="26" t="inlineStr">
+      <c r="E79" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Vitalisme"  title=" Wikipedia"&gt;Le Vitalisme&lt;/a&gt; est une doctrine philosophique et médicale selon laquelle la vie ne s’explique pas seulement par les lois de la physique et de la chimie : les êtres vivants seraient animés par un principe propre, une « force vitale », qui les distingue de la matière inerte. Il s’oppose au mécanisme de Descartes, pour qui l’animal n’est qu’une machine, plus compliquée qu’une horloge. Le vivant, au contraire, se développe, se répare, se reproduit et résiste à sa propre destruction ; en lui, c’est le tout qui commande aux parties.&lt;/p&gt; &lt;p&gt;L’idée remonte à Aristote, pour qui l’âme est le principe qui organise le corps vivant. Le vitalisme moderne naît au XVIIIe siècle à l’école de médecine de Montpellier, avec Théophile de Bordeu puis Paul-Joseph Barthez, qui parle en 1778 d’un « principe vital » distinct à la fois de l’âme et du corps. &lt;a href="https://fr.wikipedia.org/wiki/Xavier_Bichat" title=" Wikipedia"&gt;Xavier Bichat&lt;/a&gt; définit la vie comme « l’ensemble des fonctions qui résistent à la mort ». Au XIXe siècle, la chimie l’affaiblit : en 1828, Friedrich Wöhler fabrique en laboratoire l’urée, qu’on croyait réservée aux êtres vivants. Le biologiste Hans Driesch le relance pourtant vers 1900 sous le nom d’« entéléchie ». En 1907, dans &lt;em&gt;L’Évolution créatrice&lt;/em&gt;, &lt;a href="https://fr.wikipedia.org/wiki/Henri_Bergson" title=" Wikipedia"&gt;Henri Bergson&lt;/a&gt; en donne une version philosophique avec l’« élan vital », poussée créatrice et imprévisible qui traverse toute l’évolution.&lt;/p&gt; &lt;p&gt;Rejeté par la biologie moderne, le vitalisme a été réhabilité comme attitude par &lt;a href="https://fr.wikipedia.org/wiki/Georges_Canguilhem" title=" Wikipedia"&gt;Georges Canguilhem&lt;/a&gt;, qui y voit l’exigence de respecter l’originalité du vivant face au réductionnisme.&lt;/p&gt;  &lt;audio controls title="Qu’est ce que le vitalisme par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-02.04.2013-ITEMA_20465724-2013C12410S0092-NET_FC_A749DB22-ACB1-4BF2-9A16-61DE07750CA9-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
-      <c r="F78" s="11" t="s">
+      <c r="F79" s="11" t="s">
         <v>417</v>
       </c>
-      <c r="G78" s="13" t="s">
+      <c r="G79" s="13" t="s">
         <v>418</v>
       </c>
-      <c r="H78" s="11"/>
-      <c r="I78" s="13"/>
-      <c r="J78" s="3" t="inlineStr">
+      <c r="H79" s="11"/>
+      <c r="I79" s="13"/>
+      <c r="J79" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">doctrine selon laquelle la vie ne s’explique pas par la seule physique-chimie, mais par un principe propre aux êtres vivants.</t>
         </is>
       </c>
-      <c r="K78" s="3" t="s">
+      <c r="K79" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O78" t="inlineStr">
+      <c r="M79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
         <is>
           <t xml:space="preserve">position</t>
         </is>
       </c>
-      <c r="P78" t="inlineStr">
+      <c r="P79" t="inlineStr">
         <is>
           <t xml:space="preserve">Matière ou esprit ?</t>
         </is>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="14" t="n">
+    <row r="80" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="14" t="n">
         <v>1760</v>
       </c>
-      <c r="B79" s="14"/>
-      <c r="C79" s="14" t="s">
+      <c r="B80" s="14"/>
+      <c r="C80" s="14" t="s">
         <v>421</v>
       </c>
-      <c r="D79" s="15" t="s">
+      <c r="D80" s="15" t="s">
         <v>422</v>
       </c>
-      <c r="E79" s="16" t="s">
+      <c r="E80" s="16" t="s">
         <v>423</v>
       </c>
-      <c r="F79" s="14" t="s">
+      <c r="F80" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="G79" s="16" t="s">
+      <c r="G80" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="H79" s="14"/>
-      <c r="I79" s="16"/>
-      <c r="J79" s="3" t="s">
+      <c r="H80" s="14"/>
+      <c r="I80" s="16"/>
+      <c r="J80" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="K79" s="3" t="s">
+      <c r="K80" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="M79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O79" t="inlineStr">
+      <c r="M80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P79" t="inlineStr">
+      <c r="P80" t="inlineStr">
         <is>
           <t xml:space="preserve">Idéalisme allemand et romantisme</t>
         </is>
       </c>
-      <c r="Q79" t="inlineStr">
+      <c r="Q80" t="inlineStr">
         <is>
           <t xml:space="preserve">Rationalisme;Empirisme</t>
         </is>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="182.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="14" t="n">
+    <row r="81" customFormat="false" ht="182.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="14" t="n">
         <v>1770</v>
       </c>
-      <c r="B80" s="14"/>
-      <c r="C80" s="14" t="n">
+      <c r="B81" s="14"/>
+      <c r="C81" s="14" t="n">
         <v>1770</v>
       </c>
-      <c r="D80" s="15" t="s">
+      <c r="D81" s="15" t="s">
         <v>427</v>
       </c>
-      <c r="E80" s="16" t="inlineStr">
+      <c r="E81" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_(%C3%A9pist%C3%A9mologie)"  title=" Wikipedia"&gt; Le Constructivisme &lt;/a&gt; est un courant de pensée multidisciplinaire postulant que nos connaissances et notre vision du monde ne sont pas un reflet passif de la réalité, mais une construction active élaborée par l'esprit humain. Dans cette approche, le sujet connaissant interagit avec son environnement pour structurer ses propres modèles mentaux, intégrant de nouvelles expériences à des structures cognitives déjà existantes. &lt;/p&gt;&lt;p&gt; Emmanuel Kant a joué un rôle charnière au XVIIIe siècle, en proposant dans sa Critique de la raison pure une vision où l'expérience naît de l'interaction entre les impressions sensibles et la structure propre à l'esprit humain. Cette perspective a posé les jalons d'un constructivisme empirique qui rejette l'idée d'une perception passive et directe de la réalité. &lt;/p&gt; &lt;p&gt; Dans le domaine de la philosophie politique et du libéralisme, le « rationalisme constructiviste » est souvent dénoncé comme une volonté d'édifier la société selon un dessein rationnel préconçu. Les critiques, notamment Friedrich Hayek, soutiennent que cette approche tend à imposer des plans collectifs par la coercition, négligeant la liberté individuelle et les mécanismes d'ordre spontané issus des interactions humaines. &lt;/p&gt; &lt;p&gt; À l'inverse, en relations internationales, le constructivisme est une théorie scientifique qui analyse la réalité mondiale comme une construction sociale. Pour ses partisans, les intérêts des États et les structures du système international ne sont pas des données fixes ou matérielles, mais le fruit de normes, d'idées et d'interactions partagées entre les acteurs. &lt;/p&gt; 
 </t>
         </is>
       </c>
-      <c r="F80" s="14" t="s">
+      <c r="F81" s="14" t="s">
         <v>429</v>
       </c>
-      <c r="G80" s="16" t="s">
+      <c r="G81" s="16" t="s">
         <v>430</v>
       </c>
-      <c r="H80" s="14"/>
-      <c r="I80" s="16"/>
-      <c r="J80" s="3" t="inlineStr">
+      <c r="H81" s="14"/>
+      <c r="I81" s="16"/>
+      <c r="J81" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">position selon laquelle nos connaissances ne reflètent pas le réel mais sont construites activement par l’esprit (Piaget).</t>
         </is>
       </c>
-      <c r="K80" s="3" t="s">
+      <c r="K81" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="M80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O80" t="inlineStr">
+      <c r="M81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
         <is>
           <t xml:space="preserve">position</t>
         </is>
       </c>
-      <c r="P80" t="inlineStr">
+      <c r="P81" t="inlineStr">
         <is>
           <t xml:space="preserve">Que pouvons-nous connaître ?</t>
         </is>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="11" t="n">
+    <row r="82" customFormat="false" ht="159.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="11" t="n">
         <v>1780</v>
       </c>
-      <c r="B81" s="11"/>
-      <c r="C81" s="11" t="s">
+      <c r="B82" s="11"/>
+      <c r="C82" s="11" t="s">
         <v>432</v>
       </c>
-      <c r="D81" s="12" t="s">
+      <c r="D82" s="12" t="s">
         <v>433</v>
       </c>
-      <c r="E81" s="13" t="s">
+      <c r="E82" s="13" t="s">
         <v>434</v>
       </c>
-      <c r="F81" s="11" t="s">
+      <c r="F82" s="11" t="s">
         <v>435</v>
       </c>
-      <c r="G81" s="13" t="s">
+      <c r="G82" s="13" t="s">
         <v>436</v>
       </c>
-      <c r="H81" s="11"/>
-      <c r="I81" s="13"/>
-      <c r="J81" s="3" t="inlineStr">
+      <c r="H82" s="11"/>
+      <c r="I82" s="13"/>
+      <c r="J82" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">morale selon laquelle la bonne action est celle qui produit le plus grand bonheur pour le plus grand nombre (Bentham, Mill).</t>
         </is>
       </c>
-      <c r="K81" s="3" t="s">
+      <c r="K82" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O81" t="inlineStr">
+      <c r="M82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
         <is>
           <t xml:space="preserve">position</t>
         </is>
       </c>
-      <c r="P81" t="inlineStr">
+      <c r="P82" t="inlineStr">
         <is>
           <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
         </is>
       </c>
-      <c r="Q81" t="inlineStr">
+      <c r="Q82" t="inlineStr">
         <is>
           <t xml:space="preserve">Hédonisme</t>
         </is>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="222" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="14" t="n">
+    <row r="83" customFormat="false" ht="222" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="14" t="n">
         <v>1780</v>
       </c>
-      <c r="B82" s="14"/>
-      <c r="C82" s="14" t="s">
+      <c r="B83" s="14"/>
+      <c r="C83" s="14" t="s">
         <v>432</v>
       </c>
-      <c r="D82" s="15" t="s">
+      <c r="D83" s="15" t="s">
         <v>438</v>
       </c>
-      <c r="E82" s="16" t="inlineStr">
+      <c r="E83" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Panenth%C3%A9isme"  title=" Wikipedia"&gt;Le Panenthéisme&lt;/a&gt;, « tout en Dieu », est une doctrine philosophique et théologique selon laquelle le monde est contenu en Dieu, sans que Dieu se réduise au monde. Il se situe entre le panthéisme, qui identifie Dieu et l’univers, et le théisme classique, qui fait de Dieu un créateur extérieur à sa création : Dieu pénètre toute chose, mais il dépasse le cosmos par sa transcendance.&lt;/p&gt; &lt;p&gt;Le mot est forgé vers 1828 par le philosophe allemand Karl Christian Friedrich Krause, disciple de Schelling, pour distinguer sa doctrine du panthéisme de Spinoza. L’idée est pourtant plus ancienne : on la retrouve chez Plotin, pour qui tout procède de l’Un, dans certains textes hindous où le Brahman est à la fois immanent et transcendant, ou dans la kabbale d’Isaac Louria, où Dieu se retire en lui-même pour faire place au monde (&lt;em&gt;tsimtsoum&lt;/em&gt;). En Espagne, Julián Sanz del Río diffuse la pensée de Krause, et le « krausisme » inspire la réforme de l’enseignement.&lt;/p&gt; &lt;p&gt;Au XXe siècle, il est renouvelé par la théologie du processus d’Alfred North Whitehead et de Charles Hartshorne : Dieu n’y est pas immuable, il est affecté par ce qui arrive dans le monde et en garde éternellement la mémoire. Des théologiens comme Jürgen Moltmann ou Sallie McFague, qui pense le monde comme le « corps de Dieu », s’en inspirent. Ses partisans citent souvent la parole de Paul aux Athéniens : « En lui nous avons la vie, le mouvement et l’être. » Ses critiques lui reprochent de diluer la transcendance divine.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F82" s="14" t="s">
+      <c r="F83" s="14" t="s">
         <v>440</v>
       </c>
-      <c r="G82" s="16" t="s">
+      <c r="G83" s="16" t="s">
         <v>441</v>
       </c>
-      <c r="H82" s="14"/>
-      <c r="I82" s="16"/>
-      <c r="J82" s="3" t="inlineStr">
+      <c r="H83" s="14"/>
+      <c r="I83" s="16"/>
+      <c r="J83" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">doctrine selon laquelle le monde est en Dieu, mais Dieu dépasse le monde.</t>
         </is>
       </c>
-      <c r="K82" s="3" t="s">
+      <c r="K83" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O82" t="inlineStr">
+      <c r="M83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
         <is>
           <t xml:space="preserve">position</t>
         </is>
       </c>
-      <c r="P82" t="inlineStr">
+      <c r="P83" t="inlineStr">
         <is>
           <t xml:space="preserve">Dieu, les dieux ou aucun ?</t>
         </is>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="195" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="11" t="n">
+    <row r="84" customFormat="false" ht="195" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="11" t="n">
         <v>1780</v>
       </c>
-      <c r="B83" s="11"/>
-      <c r="C83" s="11" t="n">
+      <c r="B84" s="11"/>
+      <c r="C84" s="11" t="n">
         <v>1780</v>
       </c>
-      <c r="D83" s="12" t="s">
+      <c r="D84" s="12" t="s">
         <v>443</v>
       </c>
-      <c r="E83" s="28" t="s">
+      <c r="E84" s="28" t="s">
         <v>444</v>
       </c>
-      <c r="F83" s="11" t="s">
+      <c r="F84" s="11" t="s">
         <v>445</v>
       </c>
-      <c r="G83" s="13" t="s">
+      <c r="G84" s="13" t="s">
         <v>446</v>
-      </c>
-      <c r="H83" s="11"/>
-      <c r="I83" s="13"/>
-      <c r="J83" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">famille de morales selon lesquelles la valeur d’une action dépend uniquement de ses conséquences.</t>
-        </is>
-      </c>
-      <c r="K83" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="M83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">position</t>
-        </is>
-      </c>
-      <c r="P83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
-        </is>
-      </c>
-      <c r="Q83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Utilitarisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="222" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="11" t="n">
-        <v>1790</v>
-      </c>
-      <c r="B84" s="11"/>
-      <c r="C84" s="11" t="s">
-        <v>448</v>
-      </c>
-      <c r="D84" s="12" t="s">
-        <v>449</v>
-      </c>
-      <c r="E84" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Saint-simonisme"  title=" Wikipedia"&gt;Le Saint-simonisme&lt;/a&gt; est un courant de pensée politique, économique et religieux né des idées de Claude-Henri de Rouvroy, comte de &lt;a href="https://fr.wikipedia.org/wiki/Claude-Henri_de_Rouvroy_de_Saint-Simon" title=" Wikipedia"&gt;Saint-Simon&lt;/a&gt; (1760-1825), et développé après sa mort par ses disciples. Aristocrate ruiné, ancien combattant de la guerre d’indépendance américaine, Saint-Simon voit naître la révolution industrielle et en tire une conviction : la société doit être dirigée par ceux qui produisent, les « industriels », savants, ingénieurs, banquiers, artisans et ouvriers, et non plus par les nobles, les militaires et les rentiers, qu’il appelle les « oisifs ».&lt;/p&gt; &lt;p&gt;Dans sa célèbre « parabole » de 1819, il montre que la France perdrait tout si disparaissaient ses trois mille meilleurs savants, artistes et producteurs, mais rien si mouraient les princes et les grands dignitaires. La politique doit devenir une science de la production, qui remplace le gouvernement des hommes par l’administration des choses. Dans le &lt;em&gt;Nouveau Christianisme&lt;/em&gt; (1825), il propose une religion sans dogme, tournée vers l’amélioration du sort de « la classe la plus pauvre ». Ses disciples Saint-Amand Bazard et Prosper Enfantin en font une doctrine : « à chacun selon sa capacité, à chaque capacité selon ses œuvres », suppression de l’héritage, crédit organisé, émancipation des femmes. Enfantin fonde même en 1832 une communauté à Ménilmontant, vite condamnée par la justice.&lt;/p&gt; &lt;p&gt;Les saint-simoniens ont surtout bâti la France industrielle : chemins de fer, banques comme le Crédit mobilier des frères Pereire, libre-échange avec Michel Chevalier, projet du &lt;a href="https://fr.wikipedia.org/wiki/Canal_de_Suez" title=" Wikipedia"&gt;canal de Suez&lt;/a&gt;. Auguste Comte, secrétaire de Saint-Simon, et Marx leur doivent beaucoup.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F84" s="11" t="s">
-        <v>451</v>
-      </c>
-      <c r="G84" s="13" t="s">
-        <v>452</v>
       </c>
       <c r="H84" s="11"/>
       <c r="I84" s="13"/>
-      <c r="J84" s="3" t="s">
+      <c r="J84" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">famille de morales selon lesquelles la valeur d’une action dépend uniquement de ses conséquences.</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comment bien vivre et bien agir ?</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utilitarisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="222" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="11" t="n">
+        <v>1790</v>
+      </c>
+      <c r="B85" s="11"/>
+      <c r="C85" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="D85" s="12" t="s">
+        <v>449</v>
+      </c>
+      <c r="E85" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Saint-simonisme"  title=" Wikipedia"&gt;Le Saint-simonisme&lt;/a&gt; est un courant de pensée politique, économique et religieux né des idées de Claude-Henri de Rouvroy, comte de &lt;a href="https://fr.wikipedia.org/wiki/Claude-Henri_de_Rouvroy_de_Saint-Simon" title=" Wikipedia"&gt;Saint-Simon&lt;/a&gt; (1760-1825), et développé après sa mort par ses disciples. Aristocrate ruiné, ancien combattant de la guerre d’indépendance américaine, Saint-Simon voit naître la révolution industrielle et en tire une conviction : la société doit être dirigée par ceux qui produisent, les « industriels », savants, ingénieurs, banquiers, artisans et ouvriers, et non plus par les nobles, les militaires et les rentiers, qu’il appelle les « oisifs ».&lt;/p&gt; &lt;p&gt;Dans sa célèbre « parabole » de 1819, il montre que la France perdrait tout si disparaissaient ses trois mille meilleurs savants, artistes et producteurs, mais rien si mouraient les princes et les grands dignitaires. La politique doit devenir une science de la production, qui remplace le gouvernement des hommes par l’administration des choses. Dans le &lt;em&gt;Nouveau Christianisme&lt;/em&gt; (1825), il propose une religion sans dogme, tournée vers l’amélioration du sort de « la classe la plus pauvre ». Ses disciples Saint-Amand Bazard et Prosper Enfantin en font une doctrine : « à chacun selon sa capacité, à chaque capacité selon ses œuvres », suppression de l’héritage, crédit organisé, émancipation des femmes. Enfantin fonde même en 1832 une communauté à Ménilmontant, vite condamnée par la justice.&lt;/p&gt; &lt;p&gt;Les saint-simoniens ont surtout bâti la France industrielle : chemins de fer, banques comme le Crédit mobilier des frères Pereire, libre-échange avec Michel Chevalier, projet du &lt;a href="https://fr.wikipedia.org/wiki/Canal_de_Suez" title=" Wikipedia"&gt;canal de Suez&lt;/a&gt;. Auguste Comte, secrétaire de Saint-Simon, et Marx leur doivent beaucoup.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F85" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="G85" s="13" t="s">
+        <v>452</v>
+      </c>
+      <c r="H85" s="11"/>
+      <c r="I85" s="13"/>
+      <c r="J85" s="3" t="s">
         <v>453</v>
       </c>
-      <c r="K84" s="3" t="s">
+      <c r="K85" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="M84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O84" t="inlineStr">
+      <c r="M85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P84" t="inlineStr">
+      <c r="P85" t="inlineStr">
         <is>
           <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
         </is>
       </c>
-      <c r="Q84" t="inlineStr">
+      <c r="Q85" t="inlineStr">
         <is>
           <t xml:space="preserve">Lumières</t>
         </is>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="14" t="n">
+    <row r="86" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="14" t="n">
         <v>1790</v>
       </c>
-      <c r="B85" s="14"/>
-      <c r="C85" s="14" t="n">
+      <c r="B86" s="14"/>
+      <c r="C86" s="14" t="n">
         <v>1790</v>
       </c>
-      <c r="D85" s="15" t="s">
+      <c r="D86" s="15" t="s">
         <v>454</v>
       </c>
-      <c r="E85" s="16" t="inlineStr">
+      <c r="E86" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Conservatisme"  title=" Wikipedia"&gt;Le Conservatisme&lt;/a&gt;  est un courant philosophique et politique qui valorise la préservation des traditions, des institutions établies et de l'ordre social organique contre les changements radicaux ou utopiques. Il met l'accent sur la sagesse accumulée par l'expérience historique plutôt que sur des théories abstraites, prônant une évolution prudente de la société. &lt;/p&gt; &lt;p&gt; Né comme réaction à la Révolution française (1789), le conservatisme trouve son expression fondatrice chez Edmund Burke dans Réflexions sur la Révolution de France (1790), qui dénonce la rupture brutale avec le passé au nom de la raison pure. Au XIXe siècle, il se développe en Angleterre avec des penseurs comme Samuel Taylor Coleridge et en Europe continentale via Joseph de Maistre, défendant la religion, la famille et la hiérarchie naturelle contre l'égalitarisme révolutionnaire. &lt;/p&gt; &lt;p&gt; Ses principes sont la confiance dans la tradition, sagesse accumulée par les générations, plutôt que dans la raison abstraite ; la préférence pour des réformes graduelles ; l’attachement aux institutions intermédiaires, la famille, la commune, l’Église, qui protègent la liberté ; et la méfiance envers les idéologies qui prétendent refaire la société d’après un plan. Au XXe siècle, Michael Oakeshott le définit comme une disposition plutôt qu’une doctrine : « préférer le familier à l’inconnu, l’éprouvé à l’inexpérimenté ». Roger Scruton en a été un défenseur contemporain. &lt;/p&gt; 
  &lt;audio controls title=" Quand le conservatisme devient populiste par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23497-28.03.2025-ITEMA_24077783-2025F49012S0089-NET_MFI_26E2E121-D064-4F2B-B604-612240DE65AA-27.m4a" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;
 ​</t>
         </is>
       </c>
-      <c r="F85" s="14" t="s">
+      <c r="F86" s="14" t="s">
         <v>456</v>
       </c>
-      <c r="G85" s="16" t="s">
+      <c r="G86" s="16" t="s">
         <v>457</v>
-      </c>
-      <c r="H85" s="14"/>
-      <c r="I85" s="16"/>
-      <c r="J85" s="20" t="s">
-        <v>458</v>
-      </c>
-      <c r="K85" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="M85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">russe</t>
-        </is>
-      </c>
-      <c r="O85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lumières et pensée politique moderne</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="136.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="14" t="n">
-        <v>1790</v>
-      </c>
-      <c r="B86" s="14"/>
-      <c r="C86" s="14" t="n">
-        <v>1790</v>
-      </c>
-      <c r="D86" s="15" t="s">
-        <v>459</v>
-      </c>
-      <c r="E86" s="21" t="s">
-        <v>460</v>
-      </c>
-      <c r="F86" s="14" t="s">
-        <v>461</v>
-      </c>
-      <c r="G86" s="16" t="s">
-        <v>462</v>
       </c>
       <c r="H86" s="14"/>
       <c r="I86" s="16"/>
-      <c r="J86" s="22" t="s">
-        <v>463</v>
+      <c r="J86" s="20" t="s">
+        <v>458</v>
       </c>
       <c r="K86" s="3" t="s">
         <v>251</v>
@@ -8240,445 +8251,494 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lumières et pensée politique moderne</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="136.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="14" t="n">
+        <v>1790</v>
+      </c>
+      <c r="B87" s="14"/>
+      <c r="C87" s="14" t="n">
+        <v>1790</v>
+      </c>
+      <c r="D87" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="E87" s="21" t="s">
+        <v>460</v>
+      </c>
+      <c r="F87" s="14" t="s">
+        <v>461</v>
+      </c>
+      <c r="G87" s="16" t="s">
+        <v>462</v>
+      </c>
+      <c r="H87" s="14"/>
+      <c r="I87" s="16"/>
+      <c r="J87" s="22" t="s">
+        <v>463</v>
+      </c>
+      <c r="K87" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
           <t xml:space="preserve">asie-est</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr">
+      <c r="O87" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P86" t="inlineStr">
+      <c r="P87" t="inlineStr">
         <is>
           <t xml:space="preserve">Lumières et pensée politique moderne</t>
         </is>
       </c>
-      <c r="Q86" t="inlineStr">
+      <c r="Q87" t="inlineStr">
         <is>
           <t xml:space="preserve">Lumières</t>
         </is>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="151.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="1" t="n">
+    <row r="88" customFormat="false" ht="151.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="n">
         <v>1794</v>
       </c>
-      <c r="C87" s="1" t="s">
+      <c r="C88" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="D87" s="2" t="s">
+      <c r="D88" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="E87" s="3" t="inlineStr">
+      <c r="E88" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Id%C3%A9alisme_allemand" style="color:#d35400" title=" Wikipedia"&gt;L’Idéalisme allemand&lt;/a&gt; est le grand mouvement philosophique né en Allemagne à la fin du XVIIIe siècle, en réponse à la philosophie critique de Kant. Celui-ci avait montré que nous ne connaissons les choses que telles qu’elles nous apparaissent, la « chose en soi » restant hors d’atteinte. Ses successeurs veulent surmonter ce partage entre le sujet et l’objet, et bâtir un système où la réalité tout entière se comprend comme l’œuvre de l’esprit. Vers 1800, l’université d’Iéna, où enseignent Fichte, Schelling et Hegel, en est le premier foyer, aux côtés des romantiques.&lt;/p&gt; &lt;p&gt;Dans sa &lt;em&gt;Doctrine de la science&lt;/em&gt; (1794), &lt;a href="https://fr.wikipedia.org/wiki/Johann_Gottlieb_Fichte" title=" Wikipedia"&gt;Fichte&lt;/a&gt; fait du Moi, activité libre qui se pose elle-même et pose le monde comme ce qui lui résiste, le principe de tout savoir. &lt;a href="https://fr.wikipedia.org/wiki/Friedrich_Wilhelm_Joseph_von_Schelling" title=" Wikipedia"&gt;Schelling&lt;/a&gt; lui reproche d’oublier la nature, qu’il conçoit comme un esprit encore endormi : nature et esprit sont deux faces d’un même Absolu. &lt;a href="https://fr.wikipedia.org/wiki/Georg_Wilhelm_Friedrich_Hegel" title=" Wikipedia"&gt;Hegel&lt;/a&gt;, avec la &lt;em&gt;Phénoménologie de l’esprit&lt;/em&gt; (1807) et la &lt;em&gt;Science de la logique&lt;/em&gt;, porte le mouvement à son sommet : l’Absolu n’est pas donné d’emblée, il se réalise dans l’histoire, à travers le droit, l’art, la religion et la philosophie, par un mouvement dialectique où chaque contradiction est dépassée.&lt;/p&gt; &lt;p&gt;Après la mort de Hegel en 1831, ses disciples se divisent. Marx renverse sa dialectique sur une base matérialiste, Kierkegaard lui oppose l’existence individuelle, Schopenhauer la volonté aveugle, tandis que le néo-kantisme prône un retour à Kant. Le mouvement reste une référence majeure de la métaphysique et de la philosophie politique.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F87" s="1" t="s">
+      <c r="F88" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="G87" s="3" t="s">
+      <c r="G88" s="3" t="s">
         <v>468</v>
       </c>
-      <c r="I87" s="1"/>
-      <c r="J87" s="3" t="s">
+      <c r="I88" s="1"/>
+      <c r="J88" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="K87" s="3" t="s">
+      <c r="K88" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="N87" t="inlineStr">
+      <c r="M88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
         <is>
           <t xml:space="preserve">russe</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr">
+      <c r="O88" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P87" t="inlineStr">
+      <c r="P88" t="inlineStr">
         <is>
           <t xml:space="preserve">Idéalisme allemand et romantisme</t>
         </is>
       </c>
-      <c r="Q87" t="inlineStr">
+      <c r="Q88" t="inlineStr">
         <is>
           <t xml:space="preserve">Criticisme</t>
         </is>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="11" t="n">
+    <row r="89" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="11" t="n">
         <v>1800</v>
       </c>
-      <c r="B88" s="11"/>
-      <c r="C88" s="11" t="s">
+      <c r="B89" s="11"/>
+      <c r="C89" s="11" t="s">
         <v>470</v>
       </c>
-      <c r="D88" s="12" t="s">
+      <c r="D89" s="12" t="s">
         <v>471</v>
       </c>
-      <c r="E88" s="13" t="s">
+      <c r="E89" s="13" t="s">
         <v>472</v>
       </c>
-      <c r="F88" s="11" t="s">
+      <c r="F89" s="11" t="s">
         <v>473</v>
       </c>
-      <c r="G88" s="13" t="s">
+      <c r="G89" s="13" t="s">
         <v>474</v>
       </c>
-      <c r="H88" s="11"/>
-      <c r="I88" s="13"/>
-      <c r="J88" s="3" t="s">
+      <c r="H89" s="11"/>
+      <c r="I89" s="13"/>
+      <c r="J89" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="K88" s="3" t="s">
+      <c r="K89" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="M88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O88" t="inlineStr">
+      <c r="M89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P88" t="inlineStr">
+      <c r="P89" t="inlineStr">
         <is>
           <t xml:space="preserve">Idéalisme allemand et romantisme</t>
         </is>
       </c>
-      <c r="Q88" t="inlineStr">
+      <c r="Q89" t="inlineStr">
         <is>
           <t xml:space="preserve">Idéalisme allemand</t>
         </is>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="11">
+    <row r="90" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="11">
         <v>1932</v>
       </c>
-      <c r="B89" s="11"/>
-      <c r="C89" s="11" t="inlineStr">
+      <c r="B90" s="11"/>
+      <c r="C90" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">1932</t>
         </is>
       </c>
-      <c r="D89" s="12" t="s">
+      <c r="D90" s="12" t="s">
         <v>476</v>
       </c>
-      <c r="E89" s="13" t="inlineStr">
+      <c r="E90" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Personnalisme"  title=" Wikipedia"&gt; Le Personnalisme&lt;/a&gt; est un courant philosophique qui place la personne humaine au centre de toute réflexion. Il affirme que chaque être humain possède une dignité propre, irréductible à sa fonction sociale, à son utilité économique ou à une simple appartenance au groupe. &lt;/p&gt; &lt;p&gt; Ce courant s’est développé surtout au début du XXe siècle, dans un contexte de crise des valeurs et de montée des idéologies qui tendaient à écraser l’individu, comme certaines formes de collectivisme ou de matérialisme. Il s’agit donc d’une réaction contre tout ce qui réduit l’être humain à un rouage, un objet ou un numéro. &lt;/p&gt; &lt;p&gt; Le personnalisme insiste sur le fait que la personne n’est pas un individu isolé. Elle est au contraire un être libre, conscient, responsable et fondamentalement relationnel, c’est-à-dire défini aussi par ses liens avec autrui. Cette idée mène à une éthique de la solidarité, du respect et de la reconnaissance de l’autre. &lt;/p&gt; &lt;p&gt; En France, Emmanuel Mounier est la figure la plus connue du personnalisme chrétien. Il a donné à ce courant une portée morale et politique en défendant une société plus humaine, où l’économie et les institutions doivent rester au service de la personne. Le personnalisme propose une vision de l’homme qui refuse à la fois l’individualisme absolu et le collectivisme excessif. Son message essentiel est simple : la personne humaine a une valeur absolue et doit toujours être traitée comme une fin, jamais comme un moyen.  &lt;/p&gt;  
 </t>
         </is>
       </c>
-      <c r="F89" s="11" t="s">
+      <c r="F90" s="11" t="s">
         <v>478</v>
       </c>
-      <c r="G89" s="13" t="s">
+      <c r="G90" s="13" t="s">
         <v>479</v>
       </c>
-      <c r="H89" s="11"/>
-      <c r="I89" s="13"/>
-      <c r="J89" s="20" t="s">
+      <c r="H90" s="11"/>
+      <c r="I90" s="13"/>
+      <c r="J90" s="20" t="s">
         <v>480</v>
       </c>
-      <c r="K89" s="3" t="s">
+      <c r="K90" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="M89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O89" t="inlineStr">
+      <c r="M90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P89" t="inlineStr">
+      <c r="P90" t="inlineStr">
         <is>
           <t xml:space="preserve">Pensée chrétienne moderne</t>
         </is>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="14" t="n">
+    <row r="91" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="14" t="n">
         <v>1820</v>
       </c>
-      <c r="B90" s="14"/>
-      <c r="C90" s="14" t="s">
+      <c r="B91" s="14"/>
+      <c r="C91" s="14" t="s">
         <v>481</v>
       </c>
-      <c r="D90" s="15" t="s">
+      <c r="D91" s="15" t="s">
         <v>482</v>
       </c>
-      <c r="E90" s="16" t="inlineStr">
+      <c r="E91" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pessimisme_(philosophie)"  title=" Wikipedia"&gt; Le Pessimisme&lt;/a&gt;  est une perspective philosophique qui considère que la vie et le monde sont fondamentalement marqués par la souffrance, la douleur et l'insatisfaction. Les philosophes pessimistes remettent en question l'idée que la vie a une valeur intrinsèque positive ou qu'elle conduit inévitablement au bonheur. Au lieu de cela, ils soutiennent que la souffrance est omniprésente et inhérente à l'existence humaine.  Il se distingue de l'optimisme, qui soutient que la vie a une valeur intrinsèque positive et que le bonheur est atteignable malgré les difficultés. Les philosophes pessimistes rejettent généralement cette vision optimiste et soulignent plutôt la réalité de la souffrance, de l'incertitude et de la finitude de la condition humaine. &lt;/p&gt; &lt;p&gt; L'une des figures les plus célèbres du pessimisme philosophique est Arthur Schopenhauer qui considérait que la vie était une lutte perpétuelle et que la souffrance était le fondement même de l'existence. Selon lui, la volonté de vivre, un désir insatiable et sans fin, est à l'origine de nos besoins, de nos désirs et de notre insatisfaction perpétuelle. Il croyait que l'accomplissement de ces désirs était éphémère et qu'il était suivi par une nouvelle recherche insatiable de satisfaction, créant ainsi un cycle de souffrance inévitable. &lt;/p&gt; &lt;p&gt;
 Un autre philosophe pessimiste influent est Friedrich Nietzsche. Bien qu'il ne soit pas strictement considéré comme un pessimiste, il a abordé la question de la souffrance et de l'existence humaine d'une manière qui mettait en évidence les aspects sombres et douloureux de la vie. Il a remis en question les croyances traditionnelles et les valeurs morales et a souligné l'importance de faire face à la réalité de manière lucide. &lt;/p&gt; &lt;p&gt; Cependant, le pessimisme philosophique ne se limite pas à une seule vision unifiée. Il existe différentes nuances allant d'un pessimisme radical et absolu à des formes plus modérées qui reconnaissent également des aspects positifs dans la vie. &lt;/p&gt; </t>
         </is>
       </c>
-      <c r="F90" s="14" t="s">
+      <c r="F91" s="14" t="s">
         <v>484</v>
       </c>
-      <c r="G90" s="16" t="s">
+      <c r="G91" s="16" t="s">
         <v>485</v>
       </c>
-      <c r="H90" s="14"/>
-      <c r="I90" s="16"/>
-      <c r="J90" s="3" t="s">
+      <c r="H91" s="14"/>
+      <c r="I91" s="16"/>
+      <c r="J91" s="3" t="s">
         <v>486</v>
       </c>
-      <c r="K90" s="3" t="s">
+      <c r="K91" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="M90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O90" t="inlineStr">
+      <c r="M91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P90" t="inlineStr">
+      <c r="P91" t="inlineStr">
         <is>
           <t xml:space="preserve">Volonté, vie et soupçon</t>
         </is>
       </c>
-      <c r="Q90" t="inlineStr">
+      <c r="Q91" t="inlineStr">
         <is>
           <t xml:space="preserve">Idéalisme allemand;Bouddhisme</t>
         </is>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="11" t="n">
+    <row r="92" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="11" t="n">
         <v>1823</v>
       </c>
-      <c r="B91" s="11"/>
-      <c r="C91" s="11" t="s">
+      <c r="B92" s="11"/>
+      <c r="C92" s="11" t="s">
         <v>487</v>
       </c>
-      <c r="D91" s="12" t="s">
+      <c r="D92" s="12" t="s">
         <v>488</v>
       </c>
-      <c r="E91" s="13" t="s">
+      <c r="E92" s="13" t="s">
         <v>489</v>
       </c>
-      <c r="F91" s="11" t="s">
+      <c r="F92" s="11" t="s">
         <v>490</v>
       </c>
-      <c r="G91" s="13" t="s">
+      <c r="G92" s="13" t="s">
         <v>491</v>
-      </c>
-      <c r="H91" s="11"/>
-      <c r="I91" s="13"/>
-      <c r="J91" s="3" t="s">
-        <v>492</v>
-      </c>
-      <c r="K91" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="M91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="N91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">russe</t>
-        </is>
-      </c>
-      <c r="O91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Positivismes</t>
-        </is>
-      </c>
-      <c r="Q91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Saint-Simonisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="99" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="11" t="n">
-        <v>1830</v>
-      </c>
-      <c r="B92" s="11"/>
-      <c r="C92" s="11" t="n">
-        <v>1830</v>
-      </c>
-      <c r="D92" s="12" t="s">
-        <v>493</v>
-      </c>
-      <c r="E92" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Orientalisme"  title=" Wikipedia"&gt;L’Orientalisme&lt;/a&gt; désigne d’abord, au XIXe siècle, l’étude savante des langues, des textes et des civilisations de l’« Orient », du Maghreb à la Chine, ainsi qu’un goût artistique et littéraire pour ces mondes jugés exotiques. Depuis 1978, le mot désigne aussi la critique de ce regard : dans &lt;em&gt;L’Orientalisme. L’Orient créé par l’Occident&lt;/em&gt;, l’universitaire palestino-américain &lt;a href="https://fr.wikipedia.org/wiki/Edward_Sa%C3%AFd" title=" Wikipedia"&gt;Edward Saïd&lt;/a&gt; montre que l’Occident a construit une image de l’Orient qui servait sa domination.&lt;/p&gt; &lt;p&gt;L’expédition d’Égypte de Bonaparte (1798-1801), avec ses savants et sa monumentale &lt;em&gt;Description de l’Égypte&lt;/em&gt;, ouvre l’âge d’or de l’orientalisme. Champollion déchiffre les hiéroglyphes, Silvestre de Sacy enseigne l’arabe et le persan, Ernest Renan étudie les langues sémitiques. Les peintres, de Delacroix, qui voyage au Maroc en 1832, à Ingres et Gérôme, multiplient harems, bazars et déserts ; les écrivains, de Chateaubriand à Flaubert, font le voyage en Orient. Pour Saïd, ce savoir n’est pas neutre : en décrivant l’Orient comme immobile, irrationnel, sensuel et despotique, il en fait l’envers de l’Occident rationnel et justifie la colonisation. S’inspirant de Michel Foucault, il analyse les récits de voyage, la littérature et les rapports administratifs pour montrer comment savoir et pouvoir se renforcent.&lt;/p&gt; &lt;p&gt;Son livre fonde les études postcoloniales. Il a aussi été discuté : l’historien Bernard Lewis lui reproche d’ignorer la valeur scientifique de nombreux orientalistes. Le livre a changé la manière dont les historiens, les musées et les écrivains représentent les autres cultures.&lt;/p&gt;  &lt;audio controls title="l’Orientalisme d’Edward Saîd par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/17362-15.07.2024-ITEMA_23802909-2024C35448E0017-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
-        </is>
-      </c>
-      <c r="F92" s="11" t="s">
-        <v>495</v>
-      </c>
-      <c r="G92" s="13" t="s">
-        <v>496</v>
       </c>
       <c r="H92" s="11"/>
       <c r="I92" s="13"/>
       <c r="J92" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="K92" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Positivismes</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saint-Simonisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="99" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="11" t="n">
+        <v>1830</v>
+      </c>
+      <c r="B93" s="11"/>
+      <c r="C93" s="11" t="n">
+        <v>1830</v>
+      </c>
+      <c r="D93" s="12" t="s">
+        <v>493</v>
+      </c>
+      <c r="E93" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Orientalisme"  title=" Wikipedia"&gt;L’Orientalisme&lt;/a&gt; désigne d’abord, au XIXe siècle, l’étude savante des langues, des textes et des civilisations de l’« Orient », du Maghreb à la Chine, ainsi qu’un goût artistique et littéraire pour ces mondes jugés exotiques. Depuis 1978, le mot désigne aussi la critique de ce regard : dans &lt;em&gt;L’Orientalisme. L’Orient créé par l’Occident&lt;/em&gt;, l’universitaire palestino-américain &lt;a href="https://fr.wikipedia.org/wiki/Edward_Sa%C3%AFd" title=" Wikipedia"&gt;Edward Saïd&lt;/a&gt; montre que l’Occident a construit une image de l’Orient qui servait sa domination.&lt;/p&gt; &lt;p&gt;L’expédition d’Égypte de Bonaparte (1798-1801), avec ses savants et sa monumentale &lt;em&gt;Description de l’Égypte&lt;/em&gt;, ouvre l’âge d’or de l’orientalisme. Champollion déchiffre les hiéroglyphes, Silvestre de Sacy enseigne l’arabe et le persan, Ernest Renan étudie les langues sémitiques. Les peintres, de Delacroix, qui voyage au Maroc en 1832, à Ingres et Gérôme, multiplient harems, bazars et déserts ; les écrivains, de Chateaubriand à Flaubert, font le voyage en Orient. Pour Saïd, ce savoir n’est pas neutre : en décrivant l’Orient comme immobile, irrationnel, sensuel et despotique, il en fait l’envers de l’Occident rationnel et justifie la colonisation. S’inspirant de Michel Foucault, il analyse les récits de voyage, la littérature et les rapports administratifs pour montrer comment savoir et pouvoir se renforcent.&lt;/p&gt; &lt;p&gt;Son livre fonde les études postcoloniales. Il a aussi été discuté : l’historien Bernard Lewis lui reproche d’ignorer la valeur scientifique de nombreux orientalistes. Le livre a changé la manière dont les historiens, les musées et les écrivains représentent les autres cultures.&lt;/p&gt;  &lt;audio controls title="l’Orientalisme d’Edward Saîd par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/17362-15.07.2024-ITEMA_23802909-2024C35448E0017-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
+      </c>
+      <c r="F93" s="11" t="s">
+        <v>495</v>
+      </c>
+      <c r="G93" s="13" t="s">
+        <v>496</v>
+      </c>
+      <c r="H93" s="11"/>
+      <c r="I93" s="13"/>
+      <c r="J93" s="3" t="s">
         <v>497</v>
       </c>
-      <c r="K92" s="3" t="s">
+      <c r="K93" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="M92" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O92" t="inlineStr">
+      <c r="M93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P92" t="inlineStr">
+      <c r="P93" t="inlineStr">
         <is>
           <t xml:space="preserve">Idéalisme allemand et romantisme</t>
         </is>
       </c>
-      <c r="Q92" t="inlineStr">
+      <c r="Q93" t="inlineStr">
         <is>
           <t xml:space="preserve">Romantisme</t>
         </is>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="14">
+    <row r="94" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="14">
         <v>1910</v>
       </c>
-      <c r="B93" s="14"/>
-      <c r="C93" s="14" t="inlineStr">
+      <c r="B94" s="14"/>
+      <c r="C94" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">1910</t>
         </is>
       </c>
-      <c r="D93" s="15" t="s">
+      <c r="D94" s="15" t="s">
         <v>499</v>
       </c>
-      <c r="E93" s="29" t="inlineStr">
+      <c r="E94" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C5%92cum%C3%A9nisme"  title=" Wikipedia"&gt;L'Oecuménisme&lt;/a&gt;  désigne le mouvement au sein du christianisme visant à promouvoir l'unité visible entre les différentes Églises et confessions chrétiennes, en surmontant les divisions historiques et doctrinales. Issu du grec oikoumenê "terre habitée" ou "monde entier", il s'agit d'un effort spirituel et pratique pour réaliser la prière de Jésus « que tous soient un » (Jean 17:21), en favorisant le dialogue, la prière commune et la coopération. &lt;/p&gt; &lt;p&gt; Le mouvement moderne émerge avec des initiatives protestantes comme la Conférence missionnaire mondiale d'Édimbourg en 1910. Le Conseil œcuménique des Églises (COE) est fondé en 1948 à Amsterdam, regroupant protestants, anglicans et orthodoxes. L'Église catholique s'engage officiellement lors du Concile Vatican II (1962-1965), avec le décret Unitatis redintegratio qui définit l'œcuménisme comme une priorité. &lt;/p&gt; &lt;p&gt; Le COE réunit aujourd'hui plus de 350 Églises, tandis que des organismes bilatéraux comme le Groupe des Dombes (catholiques-protestants) avancent sur des consensus. Les obstacles persistent : divergences sur le rôle du pape, l'ordination des femmes ou le mariage homosexuel, mais des progrès marquent 2025, comme des déclarations conjointes sur la synodalité. &lt;/p&gt; &lt;p&gt;Le rêve de l’unité des chrétiens est pourtant plus ancien. Après les déchirements de la Réforme, des penseurs « iréniques » cherchent la paix entre les confessions : Hugo Grotius, Comenius, ou &lt;a href="https://fr.wikipedia.org/wiki/Gottfried_Wilhelm_Leibniz" title=" Wikipedia"&gt;Leibniz&lt;/a&gt;, qui négocie avec Bossuet, à la fin du XVIIe siècle, un projet de réunion des catholiques et des protestants. En Russie, Vladimir Soloviev plaide pour l’union de l’Église orthodoxe et de Rome. Au XXe siècle, des théologiens orthodoxes de l’émigration, comme Sergueï Boulgakov et &lt;a href="https://fr.wikipedia.org/wiki/Georges_Florovsky" title=" Wikipedia"&gt;Georges Florovsky&lt;/a&gt;, deviennent des acteurs majeurs du dialogue avec les anglicans et les protestants, et Florovsky participe à la fondation du COE.&lt;/p&gt; </t>
         </is>
       </c>
-      <c r="F93" s="14" t="s">
+      <c r="F94" s="14" t="s">
         <v>501</v>
       </c>
-      <c r="G93" s="16" t="s">
+      <c r="G94" s="16" t="s">
         <v>502</v>
       </c>
-      <c r="H93" s="14"/>
-      <c r="I93" s="16"/>
-      <c r="J93" s="3" t="s">
+      <c r="H94" s="14"/>
+      <c r="I94" s="16"/>
+      <c r="J94" s="3" t="s">
         <v>503</v>
       </c>
-      <c r="K93" s="3" t="s">
+      <c r="K94" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="L93" t="inlineStr">
+      <c r="L94" t="inlineStr">
         <is>
           <t xml:space="preserve">Vladimir SOLOVIEV;Sergueï BOULGAKOV;Georges FLOROVSKY</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O93" t="inlineStr">
+      <c r="M94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P93" t="inlineStr">
+      <c r="P94" t="inlineStr">
         <is>
           <t xml:space="preserve">Pensée chrétienne moderne</t>
         </is>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="11" t="n">
+    <row r="95" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="11" t="n">
         <v>1830</v>
       </c>
-      <c r="B94" s="11"/>
-      <c r="C94" s="11" t="s">
+      <c r="B95" s="11"/>
+      <c r="C95" s="11" t="s">
         <v>498</v>
       </c>
-      <c r="D94" s="12" t="s">
+      <c r="D95" s="12" t="s">
         <v>504</v>
       </c>
-      <c r="E94" s="13" t="inlineStr">
+      <c r="E95" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Populisme_(politique)"  style="color:#d35400"  title=" Wikipedia"&gt;Le Populisme&lt;/a&gt; désigne une conception de la politique qui oppose un « peuple » vertueux et uni à des « élites » jugées corrompues, et prétend exprimer directement la volonté populaire. Pour le politologue Cas Mudde, c’est une « idéologie mince » : elle ne propose pas de programme complet et se combine avec d’autres doctrines, le nationalisme à droite, le socialisme à gauche.&lt;/p&gt; &lt;p&gt;Le mot a d’abord désigné, en Russie, les &lt;a href="https://fr.wikipedia.org/wiki/Narodniki" title=" Wikipedia"&gt;narodniki&lt;/a&gt; des années 1860-1870 : de jeunes intellectuels qui « allaient au peuple » pour éveiller les paysans et fonder un socialisme sur la commune rurale, sans passer par le capitalisme. Aux États-Unis, le People’s Party des années 1890 défend les fermiers contre les banques et les compagnies de chemin de fer. Au XXe siècle, le péronisme, en Argentine, associe autour de &lt;a href="https://fr.wikipedia.org/wiki/Juan_Per%C3%B3n" title=" Wikipedia"&gt;Juan Perón&lt;/a&gt; un chef charismatique, les masses ouvrières et un nationalisme social. Depuis les années 1990, et plus encore après la crise de 2008, des partis populistes progressent en Europe et en Amérique. Leurs traits communs sont la méfiance envers les institutions représentatives, les médias et les experts, le goût du référendum et du lien direct entre le chef et le peuple, et une conception du peuple comme un tout homogène.&lt;/p&gt; &lt;p&gt;Pour Jan-Werner Müller, le populisme est dangereux parce qu’il refuse le pluralisme : ses adversaires sont exclus du « vrai peuple ». À l’inverse, &lt;a href="https://fr.wikipedia.org/wiki/Ernesto_Laclau" title=" Wikipedia"&gt;Ernesto Laclau&lt;/a&gt; y voit la logique même de toute construction politique d’un « nous ».&lt;/p&gt;  &lt;audio controls title=" Le populiste par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/23497-01.09.2023-ITEMA_23473557-2023F49012S0245-27.m4a" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
-      <c r="F94" s="11" t="s">
+      <c r="F95" s="11" t="s">
         <v>506</v>
       </c>
-      <c r="G94" s="13" t="s">
+      <c r="G95" s="13" t="s">
         <v>507</v>
       </c>
-      <c r="H94" s="11"/>
-      <c r="I94" s="13"/>
-      <c r="J94" s="3" t="s">
+      <c r="H95" s="11"/>
+      <c r="I95" s="13"/>
+      <c r="J95" s="3" t="s">
         <v>508</v>
       </c>
-      <c r="K94" s="3" t="s">
+      <c r="K95" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="M94" t="inlineStr">
+      <c r="M95" t="inlineStr">
         <is>
           <t xml:space="preserve">russe</t>
         </is>
       </c>
-      <c r="O94" t="inlineStr">
+      <c r="O95" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P94" t="inlineStr">
+      <c r="P95" t="inlineStr">
         <is>
           <t xml:space="preserve">Lumières et pensée politique moderne</t>
         </is>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="14" t="n">
+    <row r="96" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A96" s="14" t="n">
         <v>1835</v>
       </c>
-      <c r="B95" s="14"/>
-      <c r="C95" s="14" t="s">
+      <c r="B96" s="14"/>
+      <c r="C96" s="14" t="s">
         <v>509</v>
       </c>
-      <c r="D95" s="15" t="s">
+      <c r="D96" s="15" t="s">
         <v>510</v>
       </c>
-      <c r="E95" s="16" t="inlineStr">
+      <c r="E96" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Anarchisme"  style="color:#d35400"  title=" Wikipedia"&gt; L'Anarchisme &lt;/a&gt; est un courant de pensée politique et social qui prône la suppression de toutes les formes d'autorité et de hiérarchie, qu'elles soient politiques, économiques ou sociales. L'idéologie anarchiste est née au XIXe siècle, en réaction aux injustices et aux oppressions engendrées par le capitalisme et l'État.&lt;/p&gt; &lt;p&gt;
 Les premiers théoriciens de l'anarchisme étaient Pierre-Joseph Proudhon, Mikhail Bakounine et Pierre Kropotkine. Proudhon est considéré comme le fondateur de l'anarchisme, avec son ouvrage "Qu'est-ce que la propriété ?", publié en 1840. Dans cet ouvrage, Proudhon développe l'idée que la propriété est un vol et que le droit à la propriété ne peut exister que si tous les individus ont les mêmes opportunités pour y accéder.&lt;/p&gt; &lt;p&gt;
@@ -8687,336 +8747,285 @@
 &lt;p&gt; L'anarchisme a inspiré de nombreux mouvements sociaux et politiques à travers le monde, le mouvement anarchiste espagnol de la guerre civile, les Zapatistes du Mexique et les mouvements autonomes en Europe.&lt;/p&gt;   &lt;audio controls title="Naissance du mouvement anarchiste par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10076-28.08.2017-ITEMA_21417855-1.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
-      <c r="F95" s="14" t="s">
+      <c r="F96" s="14" t="s">
         <v>512</v>
       </c>
-      <c r="G95" s="16" t="inlineStr">
+      <c r="G96" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">"La philosophie de l'anarchisme" par Parole de Philosophe</t>
         </is>
       </c>
-      <c r="H95" s="14"/>
-      <c r="I95" s="16"/>
-      <c r="J95" s="3" t="s">
+      <c r="H96" s="14"/>
+      <c r="I96" s="16"/>
+      <c r="J96" s="3" t="s">
         <v>514</v>
       </c>
-      <c r="K95" s="3" t="s">
+      <c r="K96" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="M95" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="N95" t="inlineStr">
+      <c r="M96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
         <is>
           <t xml:space="preserve">russe</t>
         </is>
       </c>
-      <c r="O95" t="inlineStr">
+      <c r="O96" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P95" t="inlineStr">
+      <c r="P96" t="inlineStr">
         <is>
           <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
         </is>
       </c>
-      <c r="Q95" t="inlineStr">
+      <c r="Q96" t="inlineStr">
         <is>
           <t xml:space="preserve">Jeunes hégéliens</t>
         </is>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A96" s="11" t="n">
+    <row r="97" customFormat="false" ht="141" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A97" s="11" t="n">
         <v>1836</v>
       </c>
-      <c r="B96" s="11"/>
-      <c r="C96" s="11" t="s">
+      <c r="B97" s="11"/>
+      <c r="C97" s="11" t="s">
         <v>515</v>
       </c>
-      <c r="D96" s="12" t="s">
+      <c r="D97" s="12" t="s">
         <v>516</v>
       </c>
-      <c r="E96" s="13" t="inlineStr">
+      <c r="E97" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Transcendantalisme_(%C3%89tats-Unis)"  style="color:#d35400"  title=" Wikipedia"&gt;Le Transcendantalisme&lt;/a&gt; est un mouvement philosophique, littéraire et spirituel né en Nouvelle-Angleterre dans les années 1830, autour de &lt;a href="https://fr.wikipedia.org/wiki/Ralph_Waldo_Emerson" title=" Wikipedia"&gt;Ralph Waldo Emerson&lt;/a&gt;. Il réagit contre le rationalisme de l’Église unitarienne et contre l’empirisme de Locke, pour qui toute connaissance vient des sens. Les transcendantalistes affirment au contraire, en s’inspirant de Kant, de l’idéalisme allemand, du romantisme anglais et même des textes sacrés de l’Inde, que l’esprit humain a une intuition directe des vérités spirituelles.&lt;/p&gt; &lt;p&gt;Son manifeste est l’essai &lt;em&gt;Nature&lt;/em&gt; d’Emerson (1836) : la nature est le langage de l’esprit, et chacun peut y rencontrer le divin sans passer par les Églises ni les dogmes. Emerson parle d’une « surâme » (&lt;em&gt;Over-Soul&lt;/em&gt;), âme universelle à laquelle participent tous les êtres. Il en tire une éthique de la « confiance en soi » : chacun doit suivre sa voix intérieure plutôt que la tradition et le conformisme. Le « Transcendental Club » fonde une revue, &lt;em&gt;The Dial&lt;/em&gt;, dirigée par la féministe &lt;a href="https://fr.wikipedia.org/wiki/Margaret_Fuller" title=" Wikipedia"&gt;Margaret Fuller&lt;/a&gt;, et des communautés utopiques comme Brook Farm. &lt;a href="https://fr.wikipedia.org/wiki/Henry_David_Thoreau" title=" Wikipedia"&gt;Henry David Thoreau&lt;/a&gt;, ami d’Emerson, vit deux ans dans une cabane au bord de l’étang de Walden, expérience racontée dans &lt;em&gt;Walden ou la Vie dans les bois&lt;/em&gt; (1854) ; il refuse de payer l’impôt qui finance l’esclavage et la guerre, et en tire &lt;a href="https://fr.wikipedia.org/wiki/La_D%C3%A9sob%C3%A9issance_civile" title=" Wikipedia"&gt;&lt;em&gt;La Désobéissance civile&lt;/em&gt;&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Mouvement bref, qui décline après 1850, le transcendantalisme a pourtant profondément marqué la culture américaine : il a nourri l’abolitionnisme, inspiré Walt Whitman et, plus tard, Gandhi, Martin Luther King et la pensée écologique.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F96" s="11" t="s">
+      <c r="F97" s="11" t="s">
         <v>518</v>
       </c>
-      <c r="G96" s="13" t="inlineStr">
+      <c r="G97" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">"Le transcendantalisme : définition, exemples." par Le Savoir Partagé</t>
         </is>
       </c>
-      <c r="H96" s="11"/>
-      <c r="I96" s="13"/>
-      <c r="J96" s="3" t="s">
+      <c r="H97" s="11"/>
+      <c r="I97" s="13"/>
+      <c r="J97" s="3" t="s">
         <v>520</v>
       </c>
-      <c r="K96" s="3" t="s">
+      <c r="K97" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="M96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O96" t="inlineStr">
+      <c r="M97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P96" t="inlineStr">
+      <c r="P97" t="inlineStr">
         <is>
           <t xml:space="preserve">Idéalisme allemand et romantisme</t>
         </is>
       </c>
-      <c r="Q96" t="inlineStr">
+      <c r="Q97" t="inlineStr">
         <is>
           <t xml:space="preserve">Romantisme;Idéalisme allemand</t>
         </is>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A97" s="14" t="n">
+    <row r="98" customFormat="false" ht="137.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="14" t="n">
         <v>1840</v>
       </c>
-      <c r="B97" s="14"/>
-      <c r="C97" s="14" t="s">
+      <c r="B98" s="14"/>
+      <c r="C98" s="14" t="s">
         <v>521</v>
       </c>
-      <c r="D97" s="15" t="s">
+      <c r="D98" s="15" t="s">
         <v>522</v>
       </c>
-      <c r="E97" s="16" t="s">
+      <c r="E98" s="16" t="s">
         <v>523</v>
       </c>
-      <c r="F97" s="14" t="s">
+      <c r="F98" s="14" t="s">
         <v>524</v>
       </c>
-      <c r="G97" s="16" t="s">
+      <c r="G98" s="16" t="s">
         <v>525</v>
       </c>
-      <c r="H97" s="14"/>
-      <c r="I97" s="16"/>
-      <c r="J97" s="3" t="s">
+      <c r="H98" s="14"/>
+      <c r="I98" s="16"/>
+      <c r="J98" s="3" t="s">
         <v>526</v>
       </c>
-      <c r="K97" s="3" t="s">
+      <c r="K98" s="3" t="s">
         <v>527</v>
       </c>
-      <c r="L97" s="1" t="s">
+      <c r="L98" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="M97" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="N97" s="1" t="inlineStr">
+      <c r="M98" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N98" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">russe</t>
         </is>
       </c>
-      <c r="O97" s="1" t="inlineStr">
+      <c r="O98" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P97" s="1" t="inlineStr">
+      <c r="P98" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Phénoménologie, existence et herméneutique</t>
         </is>
       </c>
-      <c r="Q97" s="1" t="inlineStr">
+      <c r="Q98" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Idéalisme allemand</t>
         </is>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="191.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="11" t="n">
+    <row r="99" customFormat="false" ht="191.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="11" t="n">
         <v>1845</v>
       </c>
-      <c r="B98" s="11"/>
-      <c r="C98" s="11" t="s">
+      <c r="B99" s="11"/>
+      <c r="C99" s="11" t="s">
         <v>529</v>
       </c>
-      <c r="D98" s="12" t="s">
+      <c r="D99" s="12" t="s">
         <v>530</v>
       </c>
-      <c r="E98" s="13" t="s">
+      <c r="E99" s="13" t="s">
         <v>531</v>
       </c>
-      <c r="F98" s="11" t="s">
+      <c r="F99" s="11" t="s">
         <v>532</v>
       </c>
-      <c r="G98" s="13" t="s">
+      <c r="G99" s="13" t="s">
         <v>533</v>
       </c>
-      <c r="H98" s="11"/>
-      <c r="I98" s="13"/>
-      <c r="J98" s="3" t="s">
+      <c r="H99" s="11"/>
+      <c r="I99" s="13"/>
+      <c r="J99" s="3" t="s">
         <v>534</v>
       </c>
-      <c r="K98" s="3" t="s">
+      <c r="K99" s="3" t="s">
         <v>535</v>
       </c>
-      <c r="L98" s="1" t="s">
+      <c r="L99" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="M98" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="N98" s="1" t="inlineStr">
+      <c r="M99" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="N99" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">russe;asie-est</t>
         </is>
       </c>
-      <c r="O98" s="1" t="inlineStr">
+      <c r="O99" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P98" s="1" t="inlineStr">
+      <c r="P99" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
         </is>
       </c>
-      <c r="Q98" s="1" t="inlineStr">
+      <c r="Q99" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Jeunes hégéliens;Saint-Simonisme</t>
         </is>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="1" t="n">
+    <row r="100" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1" t="n">
         <v>1848</v>
       </c>
-      <c r="C99" s="1" t="s">
+      <c r="C100" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D99" s="2" t="s">
+      <c r="D100" s="2" t="s">
         <v>538</v>
       </c>
-      <c r="E99" s="3" t="inlineStr">
+      <c r="E100" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Utopie"  title=" Wikipedia"&gt;L’Utopisme&lt;/a&gt; désigne la pensée qui imagine une société idéale, radicalement différente de l’ordre existant, pour juger le présent et inviter à le transformer. Le mot vient de l’&lt;em&gt;Utopia&lt;/em&gt; (1516) de &lt;a href="https://fr.wikipedia.org/wiki/Thomas_More" title=" Wikipedia"&gt;Thomas More&lt;/a&gt;, récit d’une île sans propriété privée dont le nom grec signifie à la fois « nulle part » et « lieu heureux ». Platon, avec sa &lt;em&gt;République&lt;/em&gt;, en avait donné le modèle ; Campanella et Bacon prolongent le genre.&lt;/p&gt; &lt;p&gt;Au XIXe siècle, l’utopie quitte la fiction pour devenir projet social. Saint-Simon rêve d’une société gouvernée par les savants et les industriels, Robert Owen fonde des communautés ouvrières en Écosse puis aux États-Unis, et &lt;a href="https://fr.wikipedia.org/wiki/Charles_Fourier" title=" Wikipedia"&gt;Charles Fourier&lt;/a&gt; imagine des phalanstères où le travail, librement choisi, deviendrait attrayant. Marx et Engels les appellent « socialistes utopiques » pour leur opposer un socialisme qu’ils disent scientifique. Au XXe siècle, &lt;a href="https://fr.wikipedia.org/wiki/Ernst_Bloch" title=" Wikipedia"&gt;Ernst Bloch&lt;/a&gt; fait de l’utopie une catégorie philosophique : dans &lt;em&gt;Le Principe Espérance&lt;/em&gt; (1954-1959), l’être est inachevé, tendu vers un « pas encore » que les rêves éveillés, les arts et les religions anticipent.&lt;/p&gt; &lt;p&gt;Après les totalitarismes, l’utopie inquiète, et les contre-utopies de Zamiatine, Huxley ou Orwell en montrent le revers. Pour Paul Ricœur, elle reste pourtant une fonction essentielle de l’imagination sociale : penser que le monde pourrait être autrement. Les « utopies concrètes » d’aujourd’hui, coopératives, écovillages ou monnaies locales, en gardent l’esprit, sans prétendre bâtir d’un coup la cité parfaite.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F99" s="1" t="s">
+      <c r="F100" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G99" s="3" t="inlineStr">
+      <c r="G100" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">l’utopie par Culture Philo</t>
         </is>
       </c>
-      <c r="I99" s="1"/>
-      <c r="J99" s="3" t="s">
+      <c r="I100" s="1"/>
+      <c r="J100" s="3" t="s">
         <v>542</v>
       </c>
-      <c r="K99" s="3" t="s">
+      <c r="K100" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="M99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O99" t="inlineStr">
+      <c r="M100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P99" t="inlineStr">
+      <c r="P100" t="inlineStr">
         <is>
           <t xml:space="preserve">Socialismes, marxismes et anarchismes</t>
         </is>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="11" t="n">
+    <row r="101" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="11" t="n">
         <v>1848</v>
       </c>
-      <c r="B100" s="11"/>
-      <c r="C100" s="11" t="n">
+      <c r="B101" s="11"/>
+      <c r="C101" s="11" t="n">
         <v>1848</v>
       </c>
-      <c r="D100" s="12" t="s">
+      <c r="D101" s="12" t="s">
         <v>543</v>
       </c>
-      <c r="E100" s="28" t="s">
+      <c r="E101" s="28" t="s">
         <v>544</v>
       </c>
-      <c r="F100" s="11" t="s">
+      <c r="F101" s="11" t="s">
         <v>545</v>
       </c>
-      <c r="G100" s="13" t="s">
+      <c r="G101" s="13" t="s">
         <v>546</v>
       </c>
-      <c r="H100" s="11"/>
-      <c r="I100" s="13"/>
-      <c r="J100" s="3" t="s">
+      <c r="H101" s="11"/>
+      <c r="I101" s="13"/>
+      <c r="J101" s="3" t="s">
         <v>547</v>
-      </c>
-      <c r="K100" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="M100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pensée chrétienne moderne</t>
-        </is>
-      </c>
-      <c r="Q100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Occasionalisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A101" s="14" t="n">
-        <v>1850</v>
-      </c>
-      <c r="B101" s="14"/>
-      <c r="C101" s="14" t="s">
-        <v>548</v>
-      </c>
-      <c r="D101" s="15" t="s">
-        <v>549</v>
-      </c>
-      <c r="E101" s="16" t="s">
-        <v>550</v>
-      </c>
-      <c r="F101" s="14" t="s">
-        <v>551</v>
-      </c>
-      <c r="G101" s="16" t="s">
-        <v>552</v>
-      </c>
-      <c r="H101" s="14"/>
-      <c r="I101" s="16"/>
-      <c r="J101" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">position selon laquelle il existe une réalité indépendante de notre esprit et de nos perceptions.</t>
-        </is>
       </c>
       <c r="K101" s="3" t="s">
         <v>27</v>
@@ -9028,175 +9037,165 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée chrétienne moderne</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Occasionalisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="14" t="n">
+        <v>1850</v>
+      </c>
+      <c r="B102" s="14"/>
+      <c r="C102" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D102" s="15" t="s">
+        <v>549</v>
+      </c>
+      <c r="E102" s="16" t="s">
+        <v>550</v>
+      </c>
+      <c r="F102" s="14" t="s">
+        <v>551</v>
+      </c>
+      <c r="G102" s="16" t="s">
+        <v>552</v>
+      </c>
+      <c r="H102" s="14"/>
+      <c r="I102" s="16"/>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position selon laquelle il existe une réalité indépendante de notre esprit et de nos perceptions.</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
           <t xml:space="preserve">position</t>
         </is>
       </c>
-      <c r="P101" t="inlineStr">
+      <c r="P102" t="inlineStr">
         <is>
           <t xml:space="preserve">Qu’est-ce qui existe vraiment ?</t>
         </is>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="11" t="n">
+    <row r="103" customFormat="false" ht="171.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="11" t="n">
         <v>1850</v>
       </c>
-      <c r="B102" s="11"/>
-      <c r="C102" s="11" t="s">
+      <c r="B103" s="11"/>
+      <c r="C103" s="11" t="s">
         <v>548</v>
       </c>
-      <c r="D102" s="12" t="s">
+      <c r="D103" s="12" t="s">
         <v>554</v>
       </c>
-      <c r="E102" s="13" t="inlineStr">
+      <c r="E103" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Fonctionnalisme_(philosophie)"  title=" Wikipedia"&gt;Le Fonctionnalisme&lt;/a&gt; est une théorie de la philosophie de l’esprit selon laquelle un état mental se définit par son rôle fonctionnel, c’est-à-dire par ses relations causales avec les stimuli, les autres états mentaux et les comportements, et non par la matière dont il est fait. Une douleur, par exemple, est ce qui est causé par une lésion, provoque de la détresse et le désir qu’elle cesse, et fait crier ou retirer la main.&lt;/p&gt; &lt;p&gt;Il apparaît dans les années 1960 avec Hilary Putnam, Jerry Fodor et David Lewis, contre la théorie de l’identité, qui identifiait chaque état mental à un état précis du cerveau. Son argument principal est celui de la « réalisabilité multiple » : une pieuvre, un extraterrestre ou un ordinateur pourraient avoir des douleurs ou des croyances avec un tout autre support que nos neurones. Comme un logiciel peut tourner sur des machines différentes, l’esprit serait une organisation, non une substance. Compatible avec le matérialisme, le fonctionnalisme refuse pourtant de réduire le mental à la biologie, et il a fourni leur cadre aux sciences cognitives.&lt;/p&gt; &lt;p&gt;Ses critiques objectent qu’il laisse échapper la conscience vécue, les &lt;em&gt;qualia&lt;/em&gt;, et John Searle soutient, avec l’argument de la « chambre chinoise », qu’un programme peut manipuler des symboles sans rien comprendre. Le mot désigne aussi, en psychologie (William James) et en sciences sociales (Durkheim, Malinowski, Parsons), l’étude des fonctions que remplissent les processus mentaux ou les institutions.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F102" s="11" t="s">
+      <c r="F103" s="11" t="s">
         <v>556</v>
       </c>
-      <c r="G102" s="13" t="s">
+      <c r="G103" s="13" t="s">
         <v>557</v>
-      </c>
-      <c r="H102" s="11"/>
-      <c r="I102" s="13"/>
-      <c r="J102" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">thèse selon laquelle un état mental se définit par son rôle, par ce qu’il fait, et non par la matière qui le réalise (Putnam).</t>
-        </is>
-      </c>
-      <c r="K102" s="3" t="s">
-        <v>559</v>
-      </c>
-      <c r="M102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">position</t>
-        </is>
-      </c>
-      <c r="P102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Qu’est-ce que l’esprit ?</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="288" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A103" s="11" t="n">
-        <v>1855</v>
-      </c>
-      <c r="B103" s="11"/>
-      <c r="C103" s="11" t="n">
-        <v>1855</v>
-      </c>
-      <c r="D103" s="12" t="s">
-        <v>560</v>
-      </c>
-      <c r="E103" s="13" t="s">
-        <v>561</v>
-      </c>
-      <c r="F103" s="11" t="s">
-        <v>562</v>
-      </c>
-      <c r="G103" s="13" t="s">
-        <v>563</v>
       </c>
       <c r="H103" s="11"/>
       <c r="I103" s="13"/>
-      <c r="J103" s="3" t="s">
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thèse selon laquelle un état mental se définit par son rôle, par ce qu’il fait, et non par la matière qui le réalise (Putnam).</t>
+        </is>
+      </c>
+      <c r="K103" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">position</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qu’est-ce que l’esprit ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="288" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="11" t="n">
+        <v>1855</v>
+      </c>
+      <c r="B104" s="11"/>
+      <c r="C104" s="11" t="n">
+        <v>1855</v>
+      </c>
+      <c r="D104" s="12" t="s">
+        <v>560</v>
+      </c>
+      <c r="E104" s="13" t="s">
+        <v>561</v>
+      </c>
+      <c r="F104" s="11" t="s">
+        <v>562</v>
+      </c>
+      <c r="G104" s="13" t="s">
+        <v>563</v>
+      </c>
+      <c r="H104" s="11"/>
+      <c r="I104" s="13"/>
+      <c r="J104" s="3" t="s">
         <v>564</v>
       </c>
-      <c r="K103" s="3" t="s">
+      <c r="K104" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="L103" t="inlineStr">
+      <c r="L104" t="inlineStr">
         <is>
           <t xml:space="preserve">Ernest RENAN</t>
         </is>
       </c>
-      <c r="M103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O103" t="inlineStr">
+      <c r="M104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
         <is>
           <t xml:space="preserve">mouvement</t>
         </is>
       </c>
-      <c r="P103" t="inlineStr">
+      <c r="P104" t="inlineStr">
         <is>
           <t xml:space="preserve">Positivismes</t>
         </is>
       </c>
-      <c r="Q103" t="inlineStr">
+      <c r="Q104" t="inlineStr">
         <is>
           <t xml:space="preserve">Positivisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" customFormat="false" ht="165.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A104" s="14" t="n">
-        <v>1860</v>
-      </c>
-      <c r="B104" s="14"/>
-      <c r="C104" s="14" t="s">
-        <v>565</v>
-      </c>
-      <c r="D104" s="15" t="s">
-        <v>566</v>
-      </c>
-      <c r="E104" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Nihilisme" title=" Wikipedia"&gt; Le Nihilisme&lt;/a&gt; est une position philosophique qui remet en question ou nie la valeur et la signification de la vie, de la connaissance, de la morale et d'autres concepts fondamentaux. Les nihilistes affirment que la réalité est dépourvue de sens intrinsèque, de valeurs objectives ou de vérités ultimes et que rien n'a de valeur ou d'importance réelle, et que toutes les croyances, les systèmes moraux et les vérités sont des constructions arbitraires et illusoires. &lt;/p&gt; &lt;p&gt;
-Il peut prendre différentes formes et être appliqué à différents domaines de la philosophie. Le nihilisme métaphysique, par exemple, nie l'existence de toute réalité objective ou transcendante. Il n'y a pas de Dieu, d'âme, de monde spirituel ou de finalité ultime dans l'univers. &lt;/p&gt; &lt;p&gt;
-Le nihilisme épistémologique remet en question la possibilité de connaître la réalité telle qu'elle est en soi et soutient que nos perceptions et nos croyances sont toujours limitées et subjectives, et qu'il est impossible d'atteindre une connaissance objective et complète. &lt;/p&gt; &lt;p&gt;
-Le nihilisme moral rejette l'idée de valeurs morales objectives et que les notions de bien et de mal sont des constructions humaines sans fondement réel, que la morale est une illusion et que chaque individu est libre de créer ses propres valeurs ou d'adopter l'absence totale de valeurs. &lt;/p&gt; &lt;p&gt;
-le nihilisme n'est pas nécessairement une position que l'on adopte activement, mais plutôt une perspective critique qui remet en question les systèmes de croyances et les valeurs établies. Certains philosophes ont même fait valoir que le nihilisme peut être un point de départ pour la construction d'une nouvelle signification et de nouvelles valeurs. &lt;/p&gt;   &lt;audio controls title="Le nihilisme et la mort de l'homme par France Culture"&gt; &lt;source src="https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2015/08/s35/WL-ITE_00075081_RSCE-10.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
-</t>
-        </is>
-      </c>
-      <c r="F104" s="14" t="s">
-        <v>568</v>
-      </c>
-      <c r="G104" s="16" t="s">
-        <v>569</v>
-      </c>
-      <c r="H104" s="14"/>
-      <c r="I104" s="16"/>
-      <c r="J104" s="3" t="s">
-        <v>570</v>
-      </c>
-      <c r="K104" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="M104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">russe</t>
-        </is>
-      </c>
-      <c r="N104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-      <c r="O104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Slavophiles, occidentalistes et nihilistes</t>
-        </is>
-      </c>
-      <c r="Q104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Matérialisme</t>
         </is>
       </c>
     </row>
@@ -12817,18 +12816,18 @@
     <hyperlink ref="E55" r:id="rId9" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Cart%C3%A9sianisme&quot;   title=&quot; Wikipedia&quot;&gt; Le Cartésianisme&lt;/a&gt; est un courant de pensée issu de René Descartes, qui place la raison au centre de la connaissance. Il cherche à fonder le savoir sur des bases certaines, en rompant avec la simple autorité des traditions ou des dogmes. &lt;/p&gt; &lt;p&gt; Au cœur de cette philosophie se trouve le doute méthodique : on met en question tout ce qui peut être contesté afin de découvrir une vérité absolument indubitable. C’est ainsi que Descartes formule son célèbre « je pense, donc je suis », qui devient le point de départ de la certitude. &lt;/p&gt; &lt;p&gt;  Il défend aussi l’idée d’une distinction entre l’âme et le corps, souvent appelée dualisme. Pour Descartes et ses successeurs, l’esprit relève de la pensée, tandis que le corps appartient au monde matériel soumis à des lois mécaniques. &lt;/p&gt; &lt;p&gt; Ce courant a encouragé une méthode rigoureuse fondée sur l’analyse, la déduction et la recherche de lois générales. Il a ainsi profondément influencé la philosophie moderne et la manière de concevoir les sciences &lt;/p&gt; &lt;p&gt; Il  a eu une grande postérité, avec des penseurs comme Malebranche, Spinoza ou Leibniz, qui s’en sont inspirés tout en le transformant. Aujourd’hui encore, il reste associé à l’exigence de clarté, de méthode et de confiance dans la raison, même s’il a aussi été critiqué pour son dualisme. &lt;/p&gt; &#10;  .&#10;&#10;&#10;"/>
     <hyperlink ref="E62" r:id="rId10" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/D%C3%A9terminisme&quot; title=&quot; Wikipedia&quot;&gt; Le Déterminisme &lt;/a&gt;  est une théorie philosophique selon laquelle tous les événements de l'univers, y compris les actions humaines, sont causalement déterminés par des causes antérieures. Selon cette perspective, chaque événement est la conséquence inévitable de conditions initiales et de lois de la nature. En d'autres termes, si nous connaissions toutes les conditions présentes à un moment donné et toutes les lois de la nature qui régissent ces conditions, nous pourrions prédire avec certitude tous les événements futurs. &lt;/p&gt; &lt;p&gt;  Son origine remonte à l'Antiquité, où des philosophes comme Leucippe et Démocrite en Grèce, ainsi que certains penseurs indiens, ont formulé des idées préliminaires sur la nature déterministe de l'univers mais c'est principalement avec la montée du rationalisme et du matérialisme scientifique au XVIIe siècle avec des philosophes comme Spinoza qu'il est devenu une question centrale dans la philosophie occidentale. &lt;/p&gt; &lt;p&gt;&#10;L'idée fondamentale du déterminisme est liée à la notion de causalité. Elle suppose que chaque effet est produit par une cause précise et que cet effet devait nécessairement se produire compte tenu des circonstances existantes. Il soutient que les actions humaines sont également soumises à cette causalité déterministe et que même si nous avons l'impression de faire des choix libres, ces choix sont en réalité déterminés par des facteurs préexistants, tels que notre éducation, notre environnement, notre héritage génétique, etc et que le résultat est une série de causes et d'effets qui remontent à l'origine de l'univers. &lt;/p&gt; &lt;p&gt; &#10;Cela soulève des questions profondes, notamment en ce qui concerne le libre arbitre et la responsabilité morale. Si tout est déterminé, cela signifie-t-il que nous n'avons aucun contrôle réel sur nos actions et que nous ne pouvons être tenus responsables de nos actes ? Cette question a suscité de nombreux débats philosophiques, et différentes positions ont été développées pour tenter de concilier le déterminisme avec l'idée du libre arbitre. &lt;/p&gt; &#10;  &lt;audio controls title=&quot;Le monde : entre déterminisme et liberté par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22095-26.04.2021-ITEMA_22651648-2016C12410S0284.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &#10;"/>
     <hyperlink ref="E63" r:id="rId11" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Occasionnalisme&quot;  title=&quot; Wikipedia&quot;&gt;L'occasionalisme&lt;/a&gt; est une théorie philosophique qui émerge principalement au XVIIe siècle, en réponse aux problèmes posés par la métaphysique cartésienne, notamment la question de l'interaction entre l'âme et le corps. Cette doctrine soutient que Dieu est la seule cause véritable de tous les événements dans le monde, et que les causes naturelles ne sont que des &quot;occasions&quot; pour Dieu d'intervenir.  trouve ses racines dans la philosophie de René Descartes, qui a introduit une distinction radicale entre l'âme (la substance pensante) et le corps (la substance étendue). Cette dualité pose un problème majeur : comment l'âme, qui est immatérielle, peut-elle agir sur le corps, qui est matériel, et vice versa ? &lt;/p&gt; &lt;p&gt; Selon l'occasionalisme, Dieu est la seule cause efficiente dans l'univers. Les événements naturels (comme une boule de billard qui en frappe une autre) ne sont pas causés par les objets eux-mêmes, mais par l'intervention directe de Dieu. Les causes naturelles ne sont que des &quot;occasions&quot; qui déclenchent l'action divine. Ils soutiennent que Dieu a établi une harmonie entre les événements du monde. Par exemple, quand je décide de lever mon bras (action de l'âme), Dieu intervient pour faire en sorte que mon bras se lève (action du corps). Il n'y a pas de causalité directe entre l'âme et le corps, mais une coordination divine. L'occasionalisme résout le problème cartésien de l'interaction entre l'âme et le corps en niant toute causalité directe entre les deux. Dieu agit comme médiateur entre les deux substances. Ils s'appuient sur l'idée que Dieu doit continuellement maintenir l'existence du monde. Si Dieu doit constamment soutenir l'univers, il est cohérent de penser qu'il intervient aussi dans chaque événement. &lt;/p&gt; &lt;p&gt; Malebranche est le plus célèbre des occasionalistes. Dans De la recherche de la vérité, il développe une version sophistiquée de l'occasionalisme, en insistant sur la &quot;vision en Dieu&quot; (l'idée que nous percevons les objets à travers les idées divines). &lt;/p&gt;"/>
-    <hyperlink ref="E72" r:id="rId12" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Pluralisme_(philosophie)&quot;  title=&quot; Wikipedia&quot;&gt; Le Pluralisme&lt;/a&gt; apparaît en philosophie au début du XVIIIe siècle, introduit vers 1720 par le philosophe allemand Christian Wolff. Il n'entre dans les dictionnaires français qu'en 1932, mais l'idée de multiplicité existe bien avant.https://fr.wikipedia.org/wiki/Pluralisme &lt;/p&gt; &lt;p&gt; Dès l'Antiquité grecque, des présocratiques comme Empédocle (Ve siècle av. J.-C.) proposent un pluralisme cosmologique avec les quatre éléments (terre, air, feu, eau), irréductibles entre eux.https://www.philosophes.org/glossaire/pluralisme/ Anaxagore va plus loin avec une infinité de &quot;semences&quot; primordiales, fondant un pluralisme radical.https://www.philosophes.org/glossaire/pluralisme/ Ces idées s'opposent déjà au monisme des milésiens comme Thalès.https://www.philosophes.org/glossaire/pluralisme/ &lt;/p&gt; &lt;p&gt; Au XIXe-XXe siècle, William James (1909) défend un &quot;univers pluraliste&quot; contre l'idéalisme moniste, voyant un &quot;multiverse&quot; ouvert à la nouveauté et à la liberté.https://www.philosophes.org/glossaire/pluralisme/  Isaiah Berlin (1958) popularise le pluralisme des valeurs en philosophie morale, influençant le libéralisme contemporain. En épistémologie, il émerge au XXe siècle contre le réductionnisme, reconnaissant plusieurs approches scientifiques valides, &lt;/p&gt;  &#10;&#10;"/>
-    <hyperlink ref="E76" r:id="rId13" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Libertarianisme&quot; title=&quot; Wikipedia&quot;&gt;Le Libertarianisme&lt;/a&gt;  ou Libertarisme est un courant politique et philosophique qui met l'accent sur la liberté individuelle et la primauté de l'individu sur l'État. Ses origines remontent aux idées du siècle des Lumières et ont été développées plus tard par des penseurs comme John Locke, Adam Smith, et plus récemment par des figures comme Friedrich Hayek, Robert Nozick et Murray Rothbard. &lt;/p&gt; &lt;p&gt;Les libertariens croient en un gouvernement minimal, dont le rôle se limiterait à protéger les droits naturels des individus, limité, à la défense nationale et l'application des contrats. Ils s'opposent aux interventions gouvernementales dans des domaines tels que la santé, l'éducation et la moralité individuelle.tels que la vie, la liberté et la propriété. Ils prônent généralement une réduction drastique du rôle de l'État dans l'économie, préférant les mécanismes du marché libre pour réguler les échanges et allouer les ressources considérant la liberté individuelle comme étant de la plus haute importance. Ils soutiennent que les individus devraient avoir le droit de vivre leur vie comme ils l'entendent, tant qu'ils ne violent pas les droits des autres. &lt;/p&gt; &#10;&lt;p&gt;Ils défendent le droit à la propriété privée. Ils estiment que les individus ont le droit de posséder et de disposer de leurs biens comme bon leur semble, sans ingérence injustifiée de l'État et ils  favorisent généralement une économie de marché non réglementée, où l'offre et la demande déterminent les prix et les allocations de ressources. Ils soutiennent que les interventions gouvernementales dans l'économie, telles que les taxes excessives ou les réglementations strictes, entravent la liberté et nuisent à la prospérité économique. &lt;/p&gt; &lt;p&gt;Le principe de non-agression est central pour les libertariens. Cela signifie qu'ils s'opposent à l'utilisation de la force ou de la coercition, sauf en légitime défense. Ils considèrent toute action initiée par l'État qui viole les droits individuels comme illégitime. &lt;/p&gt; &#10;&lt;p&gt;Le libertarisme est souvent perçu comme un spectre politique qui s'étend du libertarianisme de gauche, qui accorde plus d'importance aux droits sociaux et à l'égalité, au libertarianisme de droite, qui met davantage l'accent sur les droits individuels et la primauté du marché libre. Ces variations peuvent conduire à des désaccords internes sur des questions spécifiques, mais tous les libertariens partagent généralement un engagement envers la liberté individuelle et la limitation du pouvoir gouvernemental. &lt;/p&gt;"/>
-    <hyperlink ref="E77" r:id="rId14" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Anticolonialisme&quot; title=&quot; Wikipedia&quot;&gt;L'anticolonialisme&lt;/a&gt; est un courant de pensée philosophique et politique qui s'oppose à la colonisation, en contestant sa légitimité morale, économique et culturelle.  Ce mouvement rejette l'établissement, le maintien et l'expansion des colonies par une puissance étrangère, critiquant l'exploitation des ressources, l'esclavage et l'imposition de lois ou coutumes étrangères. Il repose sur des principes d'égalité humaine et de droit des peuples à l'autodétermination, remettant en cause les hiérarchies raciales justifiant le colonialisme. &lt;/p&gt; &lt;p&gt; Dès le XVIe siècle, des figures comme Bartolomé de las Casas dénoncent les abus en Amérique, plaidant pour la liberté des Indiens et contre l'esclavage. Au XIXe siècle, des libéraux comme Frédéric Bastiat critiquent le colonialisme comme une erreur économique et étatiste, tandis que l'abolition de l'esclavage en 1848 marque une victoire anticoloniale en France. &lt;/p&gt; &lt;p&gt; Au XXe siècle, l'anticolonialisme s'intensifie avec Lénine liant colonialisme et capitalisme, puis les mouvements indépendantistes post-1945 mêlant extrême gauche, intellectuels et catholiques. Il mène à la décolonisation, influençant des penseurs comme Frantz Fanon, et se distingue du postcolonialisme par son focus sur la lutte active contre les structures coloniales. &lt;/p&gt;   &lt;p&gt; &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=&quot; &quot;Fanon&quot;: le biopic sur la figure de l'anticolonialisme est peu diffusé dans les cinémas mais agite les réseaux par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/23694-08.04.2025-ITEMA_24096522-2025J49319S0098-NET_MLM_8C70D14C-38CF-46CE-811B-6AFD802BAF4A-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;"/>
-    <hyperlink ref="E79" r:id="rId15" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Criticisme&quot; title=&quot; Wikipedia&quot;&gt; Le Criticisme&lt;/a&gt;  est une approche philosophique qui se concentre sur l'examen critique des idées, des croyances et des concepts. Il s'agit d'une méthode de réflexion qui remet en question les fondements et les présuppositions des connaissances établies, afin de déterminer leur validité et leur légitimité. Il cherche à évaluer de manière rigoureuse les arguments, les théories et les systèmes de pensée, dans le but de découvrir leurs éventuelles incohérences, erreurs ou limites. &lt;/p&gt; &lt;p&gt;  Le criticisme trouve ses origines dans la philosophie des Lumières, notamment avec les travaux d'Emmanuel Kant. Kant qui a développé une approche critique de la connaissance dans son ouvrage majeur, la &quot;Critique de la raison pure&quot;. Il a soutenu que la connaissance n'est pas simplement une accumulation passive de faits, mais qu'elle nécessite une réflexion critique sur les concepts et les catégories qui structurent notre compréhension du monde. &lt;/p&gt; &lt;p&gt; &#10;Le criticisme implique une remise en question systématique des présuppositions, des hypothèses et des normes établies. Il cherche à analyser les raisonnements, les preuves et les arguments pour déterminer leur solidité et leur validité. Il exige une rigueur intellectuelle et une évaluation objective, en évitant les biais et les préjugés. &lt;/p&gt; &lt;p&gt; Une des contributions majeures du criticisme est sa capacité à identifier les limites de la connaissance humaine. En reconnaissant que nos perceptions et nos concepts sont filtrés par nos sens et notre cognition, il souligne les frontières de notre compréhension et nous invite à rester humbles face à l'étendue du savoir. Il nous rappelle également que les connaissances établies ne sont pas immuables et qu'elles doivent être constamment remises en question et réévaluées à la lumière de nouvelles preuves et de nouvelles perspectives. &lt;/p&gt;&#10;&#10;"/>
-    <hyperlink ref="E81" r:id="rId16" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Utilitarisme&quot;  title=&quot; Wikipedia&quot;&gt; L'Utilitarisme&lt;/a&gt;  est une théorie éthique qui propose que l'action morale est celle qui produit le plus grand bonheur pour le plus grand nombre de personnes. Elle est souvent associée au philosophe britannique Jeremy Bentham, et à son disciple John Stuart Mill. &lt;/p&gt; &lt;p&gt;&#10;Selon l'utilitarisme, le bonheur est l'objectif ultime de la moralité, et l'éthique doit être basée sur la maximisation du bonheur. Il cherche à évaluer les actions, les politiques et les systèmes moraux en termes de leurs conséquences sur le bien-être des individus en se concentrant sur les résultats, plutôt que sur les intentions ou les devoirs. &lt;/p&gt; &lt;p&gt;&#10;Cette théorie repose sur le principe du &quot;principe d'utilité&quot; ou &quot;principe du plus grand bonheur&quot; où une action est considérée comme morale si elle tend à maximiser le bonheur global et à minimiser la souffrance. Le bonheur est généralement compris comme la satisfaction des désirs, le bien-être, le plaisir ou la prévention de la douleur. &lt;/p&gt; &lt;p&gt;&#10;Il se distingue sous deux formes principales : l'utilitarisme actuel et l'utilitarisme règle. L'utilitarisme actuel évalue chaque action individuelle en fonction de ses conséquences pour le bonheur. Par exemple, si mentir dans une situation particulière produit plus de bonheur global que dire la vérité, l'utilitarisme actuel soutiendrait que mentir est la meilleure action morale dans ce cas précis. &lt;/p&gt; &lt;p&gt;&#10;En revanche, l'utilitarisme règle propose d'établir des règles générales pour guider les actions individuelles. Ces règles sont conçues pour maximiser le bonheur global lorsqu'elles sont suivies de manière cohérente. Cela signifie que, même si une règle particulière peut ne pas maximiser le bonheur dans un cas particulier, elle est considérée comme juste lorsqu'elle est suivie de manière générale. &lt;/p&gt; &#10;&lt;/p&gt; &lt;audio controls title=&quot;L'utilitarisme par France Culture&quot;&gt; &lt;source src=&quot;https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2011/09/s36/Les_nouveaux_chemins_de_la_connaissance--France_Culture_1--NET_f48812fe-a9e8-46ae-b628-4850e35e439e_DF.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E82" r:id="rId17" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Panenth%C3%A9isme&quot;  title=&quot; Wikipedia&quot;&gt;Le Panenthéisme&lt;/a&gt;  est une doctrine philosophique et théologique affirmant que Dieu englobe et interpénètre tout l'univers, tout en le dépassant par sa transcendance, formant une médiation entre panthéisme (Dieu identifié à l'univers) et théisme classique (Dieu extérieur). Introduit par le philosophe allemand Karl Christian Friedrich Krause au début du XIXe siècle (vers 1828), il postule que le monde est contenu en Dieu comme une partie de son être, sans s'y réduire, influençant des courants comme la théologie du processus ou certaines interprétations de Spinoza. &lt;/p&gt; &lt;p&gt; Forgé par Krause pour dépasser le panthéisme spinoziste, le panenthéisme puise dans des idées anciennes : néoplatonisme (Plotin), hindouisme védantique (Brahman immanent et transcendant), ou kabbalah juive (Tsimtsoum). Au XXe siècle, il inspire Alfred North Whitehead  et des théologiens protestants comme Jürgen Moltmann. &lt;/p&gt; &lt;p&gt; Concepts centraux : - Immanence et transcendance : Dieu est dans tout (immanence) mais plus grand que le cosmos, qui n'est qu'une manifestation partielle de sa réalité infinie. - Dynamisme divin : Contrairement au déisme statique, Dieu évolue avec l'univers, influencé par ses changements (théologie du processus). - Critiques : Accusé de diluer la transcendance divine ou de verser dans un vague mysticisme naturaliste. &lt;/p&gt;"/>
-    <hyperlink ref="E85" r:id="rId18" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Conservatisme&quot;  title=&quot; Wikipedia&quot;&gt;Le Conservatisme&lt;/a&gt;  est un courant philosophique et politique qui valorise la préservation des traditions, des institutions établies et de l'ordre social organique contre les changements radicaux ou utopiques. Il met l'accent sur la sagesse accumulée par l'expérience historique plutôt que sur des théories abstraites, prônant une évolution prudente de la société. &lt;/p&gt; &lt;p&gt; Né comme réaction à la Révolution française (1789), le conservatisme trouve son expression fondatrice chez Edmund Burke dans Réflexions sur la Révolution de France (1790), qui dénonce la rupture brutale avec le passé au nom de la raison pure. Au XIXe siècle, il se développe en Angleterre avec des penseurs comme Samuel Taylor Coleridge et en Europe continentale via Joseph de Maistre, défendant la religion, la famille et la hiérarchie naturelle contre l'égalitarisme révolutionnaire. &lt;/p&gt; &lt;p&gt; Les principaux fondements sont : - Tradition comme sagesse : La société est un héritage complexe, non un contrat rationnel ; les réformes doivent être graduelles pour éviter le chaos. - Primauté de l'ordre : Liberté individuelle liée à la propriété privée et aux devoirs moraux, avec rôle de l'État pour protéger la stabilité. - Scepticisme envers l'abstraction : Méfiance envers les idéologies universalistes (libéralisme extrême, socialisme) qui ignorent les contextes locaux. &lt;/p&gt; &#10; &lt;audio controls title=&quot; Quand le conservatisme devient populiste par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/23497-28.03.2025-ITEMA_24077783-2025F49012S0089-NET_MFI_26E2E121-D064-4F2B-B604-612240DE65AA-27.m4a&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;&#10;​"/>
-    <hyperlink ref="E93" r:id="rId19" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/%C5%92cum%C3%A9nisme&quot;  title=&quot; Wikipedia&quot;&gt;L'Oecuménisme&lt;/a&gt;  désigne le mouvement au sein du christianisme visant à promouvoir l'unité visible entre les différentes Églises et confessions chrétiennes, en surmontant les divisions historiques et doctrinales. Issu du grec oikoumenê &quot;terre habitée&quot; ou &quot;monde entier&quot;, il s'agit d'un effort spirituel et pratique pour réaliser la prière de Jésus « que tous soient un » (Jean 17:21), en favorisant le dialogue, la prière commune et la coopération. &lt;/p&gt; &lt;p&gt; Le mouvement moderne émerge avec des initiatives protestantes comme la Conférence missionnaire mondiale d'Édimbourg en 1910. Le Conseil œcuménique des Églises (COE) est fondé en 1948 à Amsterdam, regroupant protestants, anglicans et orthodoxes. L'Église catholique s'engage officiellement lors du Concile Vatican II (1962-1965), avec le décret Unitatis redintegratio qui définit l'œcuménisme comme une priorité. &lt;/p&gt; &lt;p&gt; Le COE réunit aujourd'hui plus de 350 Églises, tandis que des organismes bilatéraux comme le Groupe des Dombes (catholiques-protestants) avancent sur des consensus. Les obstacles persistent : divergences sur le rôle du pape, l'ordination des femmes ou le mariage homosexuel, mais des progrès marquent 2025, comme des déclarations conjointes sur la synodalité. &lt;/p&gt; L'orientalisme comme courant de pensée n'est pas une simple étude de l'Orient, mais un discours de pouvoir qui façonne la perception de l'Orient pour légitimer la domination occidentale. &lt;/p&gt; "/>
-    <hyperlink ref="E96" r:id="rId20" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Transcendantalisme_(%C3%89tats-Unis)&quot;  style=&quot;color:#d35400&quot;  title=&quot; Wikipedia&quot;&gt;Le Transcendantalisme&lt;/a&gt; est un mouvement philosophique et littéraire américain, plus particulièrement dans la Nouvelle-Angleterre, et qui met l'accent sur l'intuition, l'individualisme et l'unité spirituelle entre l'humain, la nature et le divin et réagit ainsi  contre le rationalisme et l'unitéarisme institutionnel en privilégiant une connaissance a priori issue de la conscience intérieure plutôt que des sens ou des dogmes, &lt;/p&gt; &lt;p&gt; Influencé par l'idéalisme allemand de Kant et les romantiques européens, il émerge avec des intellectuels comme Ralph Waldo Emerson, dont l'essai Nature paru en 1836 pose ses bases. Il s'oppose au matérialisme et valorise une &quot;surâme&quot; (Over-Soul) universelle, immanente à la nature, accessible par contemplation et intuition. &lt;/p&gt; &lt;p&gt; Ce mouvement inspire l'abolitionnisme, l'écologie et la Beat Generation, influençant Whitman ou Melville. Bien que bref (1830-1850), il marque la littérature américaine par son mysticisme optimiste et son appel à transcender le matériel pour l'esprit. &lt;/p&gt;"/>
-    <hyperlink ref="E97" r:id="rId21" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Existentialisme#:~:text=L'existentialisme%20est%20un%20courant,doctrines%20th%C3%A9ologiques%2C%20philosophiques%20ou%20morales.&quot;  style=&quot;color:#d35400&quot;  title=&quot; Wikipedia&quot;&gt; L'existentialisme&lt;/a&gt;  est un courant philosophique qui met l'accent sur l'existence individuelle, la liberté et la responsabilité de chaque être humain. Il explore des questions fondamentales telles que le sens de la vie, la liberté, la morale et la nature de l'existence humaine. &lt;/p&gt; &lt;p&gt;&#10;L'existentialisme a émergé principalement en réaction aux systèmes philosophiques antérieurs, tels que le positivisme et le rationalisme, qui tendaient à réduire l'individu à une simple partie d'un système plus vaste. Les philosophes existentialistes se sont concentrés sur l'expérience subjective de l'individu et ont cherché à comprendre la condition humaine telle qu'elle est vécue par chaque personne.  &lt;/p&gt; &lt;p&gt;&#10;De nombreux philosophes ont contribué à ce courant, notamment Soren Kierkegaard qui fut le premier et par la suite, Camus, Martin Heidegger mais le plus influent est Jean-Paul Sartre, dont les idées sont exposées dans son œuvre majeure, &quot;L'Être et le Néant&quot;. Sartre soutient que l'existence précède l'essence, ce qui signifie que les individus ne sont pas définis par une nature ou une essence préalable, mais qu'ils sont libres de se créer et de donner un sens à leur propre existence par leurs choix et leurs actions.  &lt;/p&gt; &lt;p&gt;&#10;L'existentialisme insiste également sur la responsabilité individuelle. Les existentialistes considèrent que chaque individu est responsable de ses choix et de ses actions, et qu'il est confronté à l'angoisse existentielle découlant de la liberté. Cette liberté implique également la responsabilité de créer ses propres valeurs et de donner un sens à sa vie, plutôt que de s'appuyer sur des systèmes de croyances préétablis ou des normes sociales. Il ne propose pas un ensemble de doctrines fixes, mais plutôt une approche philosophique qui encourage l'exploration personnelle et individuelle de la condition humaine &lt;/p&gt;  &lt;audio controls title=&quot;Qu'est ce que l'existentialisme ? par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22788-22.09.2021-ITEMA_22782644-2021C45539E0018-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
-    <hyperlink ref="E99" r:id="rId22" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Utopie&quot;  title=&quot; Wikipedia&quot;&gt;L'Utopisme philosophique&lt;/a&gt; désigne la pensée qui projette une société idéale radicalement différente de l'ordre existant, et qui fait de cette projection un levier de transformation sociale et politique. Le terme vient de Thomas More (&lt;em&gt;Utopia&lt;/em&gt;, 1516), mais comme courant philosophique structuré, l'utopisme s'affirme  avec les socialistes utopistes (Saint-Simon, Fourier, Owen) et atteint sa maturité philosophique avec Ernst Bloch.&lt;/p&gt;&lt;p&gt;Ernst Bloch, dans &lt;em&gt;Le Principe Espérance&lt;/em&gt; (1954-1959), élève l'utopisme au rang d'une ontologie du &quot;pas encore&quot; : l'être est fondamentalement inachevé, tendu vers un futur meilleur. Pour Bloch, les rêves diurnes, les mythes, les arts et les grandes religions sont autant d'expressions de cette &quot;fonction utopique&quot; inscrite dans la conscience humaine. L'utopie n'est pas une fuite hors du réel, mais une anticipation concrète de possibilités réelles.&lt;/p&gt;&lt;p&gt;L'utopisme se distingue du simple idéalisme par son ancrage dans les conditions historiques et sociales de son époque. Il a nourri les grandes idéologies émancipatrices du XXe siècle et continue d'irriguer la philosophie politique contemporaine, notamment les théories de la justice sociale et les courants écosocialistes.&lt;/p&gt;"/>
-    <hyperlink ref="E103" r:id="rId23" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Scientisme&quot;  title=&quot; Wikipedia&quot;&gt;Le Scientisme&lt;/a&gt;  est une position philosophique qui affirme que la science expérimentale constitue la seule source fiable de connaissance sur le monde. Ce courant soutient que les méthodes scientifiques, fondées sur l’observation et l’expérimentation, doivent être étendues à tous les domaines de la pensée, y compris la morale et la politique. &lt;/p&gt; &lt;p&gt; En plaçant la science au sommet de la hiérarchie des savoirs, le scientisme rejette souvent les autres formes d'interprétation, telles que la religion, la philosophie métaphysique ou les traditions, qu'il perçoit comme irrationnelles. Pour ses partisans, les progrès technologiques et scientifiques sont destinés à résoudre les problèmes humains fondamentaux et à dissiper l'inconnu. &lt;/p&gt; &lt;p&gt; Le terme est néanmoins fréquemment utilisé de manière critique par les philosophes pour dénoncer une confiance excessive, voire dogmatique, envers la science. Cette « religion de la science » est souvent accusée de réductionnisme, car elle évacue les questions existentielles sur le sens de la vie, l'éthique ou l'esthétique, considérant qu'elles ne relèvent pas du champ de la connaissance authentique. &lt;/p&gt; &lt;p&gt; Il continue de faire débat, illustrant la tension entre le besoin humain de réponses rationnelles et la complexité des questions sur les valeurs et le sens. Bien que largement critiqué pour son impérialisme intellectuel, il reste une influence marquante dans notre vision contemporaine du progrès et de la maîtrise technique de notre environnement. &lt;/p&gt; &#10;&#10;"/>
+    <hyperlink ref="E73" r:id="rId12" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Pluralisme_(philosophie)&quot;  title=&quot; Wikipedia&quot;&gt; Le Pluralisme&lt;/a&gt; apparaît en philosophie au début du XVIIIe siècle, introduit vers 1720 par le philosophe allemand Christian Wolff. Il n'entre dans les dictionnaires français qu'en 1932, mais l'idée de multiplicité existe bien avant.https://fr.wikipedia.org/wiki/Pluralisme &lt;/p&gt; &lt;p&gt; Dès l'Antiquité grecque, des présocratiques comme Empédocle (Ve siècle av. J.-C.) proposent un pluralisme cosmologique avec les quatre éléments (terre, air, feu, eau), irréductibles entre eux.https://www.philosophes.org/glossaire/pluralisme/ Anaxagore va plus loin avec une infinité de &quot;semences&quot; primordiales, fondant un pluralisme radical.https://www.philosophes.org/glossaire/pluralisme/ Ces idées s'opposent déjà au monisme des milésiens comme Thalès.https://www.philosophes.org/glossaire/pluralisme/ &lt;/p&gt; &lt;p&gt; Au XIXe-XXe siècle, William James (1909) défend un &quot;univers pluraliste&quot; contre l'idéalisme moniste, voyant un &quot;multiverse&quot; ouvert à la nouveauté et à la liberté.https://www.philosophes.org/glossaire/pluralisme/  Isaiah Berlin (1958) popularise le pluralisme des valeurs en philosophie morale, influençant le libéralisme contemporain. En épistémologie, il émerge au XXe siècle contre le réductionnisme, reconnaissant plusieurs approches scientifiques valides, &lt;/p&gt;  &#10;&#10;"/>
+    <hyperlink ref="E77" r:id="rId13" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Libertarianisme&quot; title=&quot; Wikipedia&quot;&gt;Le Libertarianisme&lt;/a&gt;  ou Libertarisme est un courant politique et philosophique qui met l'accent sur la liberté individuelle et la primauté de l'individu sur l'État. Ses origines remontent aux idées du siècle des Lumières et ont été développées plus tard par des penseurs comme John Locke, Adam Smith, et plus récemment par des figures comme Friedrich Hayek, Robert Nozick et Murray Rothbard. &lt;/p&gt; &lt;p&gt;Les libertariens croient en un gouvernement minimal, dont le rôle se limiterait à protéger les droits naturels des individus, limité, à la défense nationale et l'application des contrats. Ils s'opposent aux interventions gouvernementales dans des domaines tels que la santé, l'éducation et la moralité individuelle.tels que la vie, la liberté et la propriété. Ils prônent généralement une réduction drastique du rôle de l'État dans l'économie, préférant les mécanismes du marché libre pour réguler les échanges et allouer les ressources considérant la liberté individuelle comme étant de la plus haute importance. Ils soutiennent que les individus devraient avoir le droit de vivre leur vie comme ils l'entendent, tant qu'ils ne violent pas les droits des autres. &lt;/p&gt; &#10;&lt;p&gt;Ils défendent le droit à la propriété privée. Ils estiment que les individus ont le droit de posséder et de disposer de leurs biens comme bon leur semble, sans ingérence injustifiée de l'État et ils  favorisent généralement une économie de marché non réglementée, où l'offre et la demande déterminent les prix et les allocations de ressources. Ils soutiennent que les interventions gouvernementales dans l'économie, telles que les taxes excessives ou les réglementations strictes, entravent la liberté et nuisent à la prospérité économique. &lt;/p&gt; &lt;p&gt;Le principe de non-agression est central pour les libertariens. Cela signifie qu'ils s'opposent à l'utilisation de la force ou de la coercition, sauf en légitime défense. Ils considèrent toute action initiée par l'État qui viole les droits individuels comme illégitime. &lt;/p&gt; &#10;&lt;p&gt;Le libertarisme est souvent perçu comme un spectre politique qui s'étend du libertarianisme de gauche, qui accorde plus d'importance aux droits sociaux et à l'égalité, au libertarianisme de droite, qui met davantage l'accent sur les droits individuels et la primauté du marché libre. Ces variations peuvent conduire à des désaccords internes sur des questions spécifiques, mais tous les libertariens partagent généralement un engagement envers la liberté individuelle et la limitation du pouvoir gouvernemental. &lt;/p&gt;"/>
+    <hyperlink ref="E78" r:id="rId14" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Anticolonialisme&quot; title=&quot; Wikipedia&quot;&gt;L'anticolonialisme&lt;/a&gt; est un courant de pensée philosophique et politique qui s'oppose à la colonisation, en contestant sa légitimité morale, économique et culturelle.  Ce mouvement rejette l'établissement, le maintien et l'expansion des colonies par une puissance étrangère, critiquant l'exploitation des ressources, l'esclavage et l'imposition de lois ou coutumes étrangères. Il repose sur des principes d'égalité humaine et de droit des peuples à l'autodétermination, remettant en cause les hiérarchies raciales justifiant le colonialisme. &lt;/p&gt; &lt;p&gt; Dès le XVIe siècle, des figures comme Bartolomé de las Casas dénoncent les abus en Amérique, plaidant pour la liberté des Indiens et contre l'esclavage. Au XIXe siècle, des libéraux comme Frédéric Bastiat critiquent le colonialisme comme une erreur économique et étatiste, tandis que l'abolition de l'esclavage en 1848 marque une victoire anticoloniale en France. &lt;/p&gt; &lt;p&gt; Au XXe siècle, l'anticolonialisme s'intensifie avec Lénine liant colonialisme et capitalisme, puis les mouvements indépendantistes post-1945 mêlant extrême gauche, intellectuels et catholiques. Il mène à la décolonisation, influençant des penseurs comme Frantz Fanon, et se distingue du postcolonialisme par son focus sur la lutte active contre les structures coloniales. &lt;/p&gt;   &lt;p&gt; &lt;/p&gt; &lt;p&gt;  &lt;audio controls title=&quot; &quot;Fanon&quot;: le biopic sur la figure de l'anticolonialisme est peu diffusé dans les cinémas mais agite les réseaux par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/23694-08.04.2025-ITEMA_24096522-2025J49319S0098-NET_MLM_8C70D14C-38CF-46CE-811B-6AFD802BAF4A-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;"/>
+    <hyperlink ref="E80" r:id="rId15" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Criticisme&quot; title=&quot; Wikipedia&quot;&gt; Le Criticisme&lt;/a&gt;  est une approche philosophique qui se concentre sur l'examen critique des idées, des croyances et des concepts. Il s'agit d'une méthode de réflexion qui remet en question les fondements et les présuppositions des connaissances établies, afin de déterminer leur validité et leur légitimité. Il cherche à évaluer de manière rigoureuse les arguments, les théories et les systèmes de pensée, dans le but de découvrir leurs éventuelles incohérences, erreurs ou limites. &lt;/p&gt; &lt;p&gt;  Le criticisme trouve ses origines dans la philosophie des Lumières, notamment avec les travaux d'Emmanuel Kant. Kant qui a développé une approche critique de la connaissance dans son ouvrage majeur, la &quot;Critique de la raison pure&quot;. Il a soutenu que la connaissance n'est pas simplement une accumulation passive de faits, mais qu'elle nécessite une réflexion critique sur les concepts et les catégories qui structurent notre compréhension du monde. &lt;/p&gt; &lt;p&gt; &#10;Le criticisme implique une remise en question systématique des présuppositions, des hypothèses et des normes établies. Il cherche à analyser les raisonnements, les preuves et les arguments pour déterminer leur solidité et leur validité. Il exige une rigueur intellectuelle et une évaluation objective, en évitant les biais et les préjugés. &lt;/p&gt; &lt;p&gt; Une des contributions majeures du criticisme est sa capacité à identifier les limites de la connaissance humaine. En reconnaissant que nos perceptions et nos concepts sont filtrés par nos sens et notre cognition, il souligne les frontières de notre compréhension et nous invite à rester humbles face à l'étendue du savoir. Il nous rappelle également que les connaissances établies ne sont pas immuables et qu'elles doivent être constamment remises en question et réévaluées à la lumière de nouvelles preuves et de nouvelles perspectives. &lt;/p&gt;&#10;&#10;"/>
+    <hyperlink ref="E82" r:id="rId16" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Utilitarisme&quot;  title=&quot; Wikipedia&quot;&gt; L'Utilitarisme&lt;/a&gt;  est une théorie éthique qui propose que l'action morale est celle qui produit le plus grand bonheur pour le plus grand nombre de personnes. Elle est souvent associée au philosophe britannique Jeremy Bentham, et à son disciple John Stuart Mill. &lt;/p&gt; &lt;p&gt;&#10;Selon l'utilitarisme, le bonheur est l'objectif ultime de la moralité, et l'éthique doit être basée sur la maximisation du bonheur. Il cherche à évaluer les actions, les politiques et les systèmes moraux en termes de leurs conséquences sur le bien-être des individus en se concentrant sur les résultats, plutôt que sur les intentions ou les devoirs. &lt;/p&gt; &lt;p&gt;&#10;Cette théorie repose sur le principe du &quot;principe d'utilité&quot; ou &quot;principe du plus grand bonheur&quot; où une action est considérée comme morale si elle tend à maximiser le bonheur global et à minimiser la souffrance. Le bonheur est généralement compris comme la satisfaction des désirs, le bien-être, le plaisir ou la prévention de la douleur. &lt;/p&gt; &lt;p&gt;&#10;Il se distingue sous deux formes principales : l'utilitarisme actuel et l'utilitarisme règle. L'utilitarisme actuel évalue chaque action individuelle en fonction de ses conséquences pour le bonheur. Par exemple, si mentir dans une situation particulière produit plus de bonheur global que dire la vérité, l'utilitarisme actuel soutiendrait que mentir est la meilleure action morale dans ce cas précis. &lt;/p&gt; &lt;p&gt;&#10;En revanche, l'utilitarisme règle propose d'établir des règles générales pour guider les actions individuelles. Ces règles sont conçues pour maximiser le bonheur global lorsqu'elles sont suivies de manière cohérente. Cela signifie que, même si une règle particulière peut ne pas maximiser le bonheur dans un cas particulier, elle est considérée comme juste lorsqu'elle est suivie de manière générale. &lt;/p&gt; &#10;&lt;/p&gt; &lt;audio controls title=&quot;L'utilitarisme par France Culture&quot;&gt; &lt;source src=&quot;https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2011/09/s36/Les_nouveaux_chemins_de_la_connaissance--France_Culture_1--NET_f48812fe-a9e8-46ae-b628-4850e35e439e_DF.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E83" r:id="rId17" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Panenth%C3%A9isme&quot;  title=&quot; Wikipedia&quot;&gt;Le Panenthéisme&lt;/a&gt;  est une doctrine philosophique et théologique affirmant que Dieu englobe et interpénètre tout l'univers, tout en le dépassant par sa transcendance, formant une médiation entre panthéisme (Dieu identifié à l'univers) et théisme classique (Dieu extérieur). Introduit par le philosophe allemand Karl Christian Friedrich Krause au début du XIXe siècle (vers 1828), il postule que le monde est contenu en Dieu comme une partie de son être, sans s'y réduire, influençant des courants comme la théologie du processus ou certaines interprétations de Spinoza. &lt;/p&gt; &lt;p&gt; Forgé par Krause pour dépasser le panthéisme spinoziste, le panenthéisme puise dans des idées anciennes : néoplatonisme (Plotin), hindouisme védantique (Brahman immanent et transcendant), ou kabbalah juive (Tsimtsoum). Au XXe siècle, il inspire Alfred North Whitehead  et des théologiens protestants comme Jürgen Moltmann. &lt;/p&gt; &lt;p&gt; Concepts centraux : - Immanence et transcendance : Dieu est dans tout (immanence) mais plus grand que le cosmos, qui n'est qu'une manifestation partielle de sa réalité infinie. - Dynamisme divin : Contrairement au déisme statique, Dieu évolue avec l'univers, influencé par ses changements (théologie du processus). - Critiques : Accusé de diluer la transcendance divine ou de verser dans un vague mysticisme naturaliste. &lt;/p&gt;"/>
+    <hyperlink ref="E86" r:id="rId18" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Conservatisme&quot;  title=&quot; Wikipedia&quot;&gt;Le Conservatisme&lt;/a&gt;  est un courant philosophique et politique qui valorise la préservation des traditions, des institutions établies et de l'ordre social organique contre les changements radicaux ou utopiques. Il met l'accent sur la sagesse accumulée par l'expérience historique plutôt que sur des théories abstraites, prônant une évolution prudente de la société. &lt;/p&gt; &lt;p&gt; Né comme réaction à la Révolution française (1789), le conservatisme trouve son expression fondatrice chez Edmund Burke dans Réflexions sur la Révolution de France (1790), qui dénonce la rupture brutale avec le passé au nom de la raison pure. Au XIXe siècle, il se développe en Angleterre avec des penseurs comme Samuel Taylor Coleridge et en Europe continentale via Joseph de Maistre, défendant la religion, la famille et la hiérarchie naturelle contre l'égalitarisme révolutionnaire. &lt;/p&gt; &lt;p&gt; Les principaux fondements sont : - Tradition comme sagesse : La société est un héritage complexe, non un contrat rationnel ; les réformes doivent être graduelles pour éviter le chaos. - Primauté de l'ordre : Liberté individuelle liée à la propriété privée et aux devoirs moraux, avec rôle de l'État pour protéger la stabilité. - Scepticisme envers l'abstraction : Méfiance envers les idéologies universalistes (libéralisme extrême, socialisme) qui ignorent les contextes locaux. &lt;/p&gt; &#10; &lt;audio controls title=&quot; Quand le conservatisme devient populiste par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/23497-28.03.2025-ITEMA_24077783-2025F49012S0089-NET_MFI_26E2E121-D064-4F2B-B604-612240DE65AA-27.m4a&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;&#10;​"/>
+    <hyperlink ref="E94" r:id="rId19" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/%C5%92cum%C3%A9nisme&quot;  title=&quot; Wikipedia&quot;&gt;L'Oecuménisme&lt;/a&gt;  désigne le mouvement au sein du christianisme visant à promouvoir l'unité visible entre les différentes Églises et confessions chrétiennes, en surmontant les divisions historiques et doctrinales. Issu du grec oikoumenê &quot;terre habitée&quot; ou &quot;monde entier&quot;, il s'agit d'un effort spirituel et pratique pour réaliser la prière de Jésus « que tous soient un » (Jean 17:21), en favorisant le dialogue, la prière commune et la coopération. &lt;/p&gt; &lt;p&gt; Le mouvement moderne émerge avec des initiatives protestantes comme la Conférence missionnaire mondiale d'Édimbourg en 1910. Le Conseil œcuménique des Églises (COE) est fondé en 1948 à Amsterdam, regroupant protestants, anglicans et orthodoxes. L'Église catholique s'engage officiellement lors du Concile Vatican II (1962-1965), avec le décret Unitatis redintegratio qui définit l'œcuménisme comme une priorité. &lt;/p&gt; &lt;p&gt; Le COE réunit aujourd'hui plus de 350 Églises, tandis que des organismes bilatéraux comme le Groupe des Dombes (catholiques-protestants) avancent sur des consensus. Les obstacles persistent : divergences sur le rôle du pape, l'ordination des femmes ou le mariage homosexuel, mais des progrès marquent 2025, comme des déclarations conjointes sur la synodalité. &lt;/p&gt; L'orientalisme comme courant de pensée n'est pas une simple étude de l'Orient, mais un discours de pouvoir qui façonne la perception de l'Orient pour légitimer la domination occidentale. &lt;/p&gt; "/>
+    <hyperlink ref="E97" r:id="rId20" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Transcendantalisme_(%C3%89tats-Unis)&quot;  style=&quot;color:#d35400&quot;  title=&quot; Wikipedia&quot;&gt;Le Transcendantalisme&lt;/a&gt; est un mouvement philosophique et littéraire américain, plus particulièrement dans la Nouvelle-Angleterre, et qui met l'accent sur l'intuition, l'individualisme et l'unité spirituelle entre l'humain, la nature et le divin et réagit ainsi  contre le rationalisme et l'unitéarisme institutionnel en privilégiant une connaissance a priori issue de la conscience intérieure plutôt que des sens ou des dogmes, &lt;/p&gt; &lt;p&gt; Influencé par l'idéalisme allemand de Kant et les romantiques européens, il émerge avec des intellectuels comme Ralph Waldo Emerson, dont l'essai Nature paru en 1836 pose ses bases. Il s'oppose au matérialisme et valorise une &quot;surâme&quot; (Over-Soul) universelle, immanente à la nature, accessible par contemplation et intuition. &lt;/p&gt; &lt;p&gt; Ce mouvement inspire l'abolitionnisme, l'écologie et la Beat Generation, influençant Whitman ou Melville. Bien que bref (1830-1850), il marque la littérature américaine par son mysticisme optimiste et son appel à transcender le matériel pour l'esprit. &lt;/p&gt;"/>
+    <hyperlink ref="E98" r:id="rId21" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Existentialisme#:~:text=L'existentialisme%20est%20un%20courant,doctrines%20th%C3%A9ologiques%2C%20philosophiques%20ou%20morales.&quot;  style=&quot;color:#d35400&quot;  title=&quot; Wikipedia&quot;&gt; L'existentialisme&lt;/a&gt;  est un courant philosophique qui met l'accent sur l'existence individuelle, la liberté et la responsabilité de chaque être humain. Il explore des questions fondamentales telles que le sens de la vie, la liberté, la morale et la nature de l'existence humaine. &lt;/p&gt; &lt;p&gt;&#10;L'existentialisme a émergé principalement en réaction aux systèmes philosophiques antérieurs, tels que le positivisme et le rationalisme, qui tendaient à réduire l'individu à une simple partie d'un système plus vaste. Les philosophes existentialistes se sont concentrés sur l'expérience subjective de l'individu et ont cherché à comprendre la condition humaine telle qu'elle est vécue par chaque personne.  &lt;/p&gt; &lt;p&gt;&#10;De nombreux philosophes ont contribué à ce courant, notamment Soren Kierkegaard qui fut le premier et par la suite, Camus, Martin Heidegger mais le plus influent est Jean-Paul Sartre, dont les idées sont exposées dans son œuvre majeure, &quot;L'Être et le Néant&quot;. Sartre soutient que l'existence précède l'essence, ce qui signifie que les individus ne sont pas définis par une nature ou une essence préalable, mais qu'ils sont libres de se créer et de donner un sens à leur propre existence par leurs choix et leurs actions.  &lt;/p&gt; &lt;p&gt;&#10;L'existentialisme insiste également sur la responsabilité individuelle. Les existentialistes considèrent que chaque individu est responsable de ses choix et de ses actions, et qu'il est confronté à l'angoisse existentielle découlant de la liberté. Cette liberté implique également la responsabilité de créer ses propres valeurs et de donner un sens à sa vie, plutôt que de s'appuyer sur des systèmes de croyances préétablis ou des normes sociales. Il ne propose pas un ensemble de doctrines fixes, mais plutôt une approche philosophique qui encourage l'exploration personnelle et individuelle de la condition humaine &lt;/p&gt;  &lt;audio controls title=&quot;Qu'est ce que l'existentialisme ? par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/22788-22.09.2021-ITEMA_22782644-2021C45539E0018-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; "/>
+    <hyperlink ref="E100" r:id="rId22" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Utopie&quot;  title=&quot; Wikipedia&quot;&gt;L'Utopisme philosophique&lt;/a&gt; désigne la pensée qui projette une société idéale radicalement différente de l'ordre existant, et qui fait de cette projection un levier de transformation sociale et politique. Le terme vient de Thomas More (&lt;em&gt;Utopia&lt;/em&gt;, 1516), mais comme courant philosophique structuré, l'utopisme s'affirme  avec les socialistes utopistes (Saint-Simon, Fourier, Owen) et atteint sa maturité philosophique avec Ernst Bloch.&lt;/p&gt;&lt;p&gt;Ernst Bloch, dans &lt;em&gt;Le Principe Espérance&lt;/em&gt; (1954-1959), élève l'utopisme au rang d'une ontologie du &quot;pas encore&quot; : l'être est fondamentalement inachevé, tendu vers un futur meilleur. Pour Bloch, les rêves diurnes, les mythes, les arts et les grandes religions sont autant d'expressions de cette &quot;fonction utopique&quot; inscrite dans la conscience humaine. L'utopie n'est pas une fuite hors du réel, mais une anticipation concrète de possibilités réelles.&lt;/p&gt;&lt;p&gt;L'utopisme se distingue du simple idéalisme par son ancrage dans les conditions historiques et sociales de son époque. Il a nourri les grandes idéologies émancipatrices du XXe siècle et continue d'irriguer la philosophie politique contemporaine, notamment les théories de la justice sociale et les courants écosocialistes.&lt;/p&gt;"/>
+    <hyperlink ref="E104" r:id="rId23" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Scientisme&quot;  title=&quot; Wikipedia&quot;&gt;Le Scientisme&lt;/a&gt;  est une position philosophique qui affirme que la science expérimentale constitue la seule source fiable de connaissance sur le monde. Ce courant soutient que les méthodes scientifiques, fondées sur l’observation et l’expérimentation, doivent être étendues à tous les domaines de la pensée, y compris la morale et la politique. &lt;/p&gt; &lt;p&gt; En plaçant la science au sommet de la hiérarchie des savoirs, le scientisme rejette souvent les autres formes d'interprétation, telles que la religion, la philosophie métaphysique ou les traditions, qu'il perçoit comme irrationnelles. Pour ses partisans, les progrès technologiques et scientifiques sont destinés à résoudre les problèmes humains fondamentaux et à dissiper l'inconnu. &lt;/p&gt; &lt;p&gt; Le terme est néanmoins fréquemment utilisé de manière critique par les philosophes pour dénoncer une confiance excessive, voire dogmatique, envers la science. Cette « religion de la science » est souvent accusée de réductionnisme, car elle évacue les questions existentielles sur le sens de la vie, l'éthique ou l'esthétique, considérant qu'elles ne relèvent pas du champ de la connaissance authentique. &lt;/p&gt; &lt;p&gt; Il continue de faire débat, illustrant la tension entre le besoin humain de réponses rationnelles et la complexité des questions sur les valeurs et le sens. Bien que largement critiqué pour son impérialisme intellectuel, il reste une influence marquante dans notre vision contemporaine du progrès et de la maîtrise technique de notre environnement. &lt;/p&gt; &#10;&#10;"/>
     <hyperlink ref="E105" r:id="rId24" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Volontarisme_(courant_politique)&quot; title=&quot; Wikipedia&quot;&gt;Le Volontarisme&lt;/a&gt; en tant que courant politique libertarian, est une philosophie avec Auberon Herbert, qui prône un État financé exclusivement sur une base volontaire, sans imposition coercitive. Ce courant, également appelé voluntaryism en anglais, rejette l'usage de la force pour lever l'impôt et défend un « État volontaire ». &lt;/p&gt; &lt;p&gt; Les principes fondamentaux du volontarisme reposent sur les droits naturels, l'égalité, la non-coercition et le principe de non-agression. Dans la pratique, il implique un respect strict du pacifisme, des droits civiques, et le recours à l'arbitrage ou à des systèmes juridiques de résolution des conflits librement acceptés par les individus. &lt;/p&gt; &lt;p&gt; À la fin du XXᵉ siècle, il a retrouvé une popularité surtout au sein du courant libertarien aux États-Unis, où il est associé à l'anarcho-capitalisme. Les volontaristes prônent des stratégies non politiques pour établir une société libre, rejettant la politique électorale comme incompatible avec les objectifs libertariens. Pour eux, les méthodes politiques renforcent inévitablement la légitimité de gouvernements coercitifs ; ils cherchent plutôt à délégitimer l'État par l'éducation et préconisent le retrait de la coopération et du consentement tacite sur lesquels repose la puissance de l'État. Cette approche s'approprie le terme au nom du libertarianisme de droite. &lt;/p&gt; &lt;p&gt; Il existe une autre acception du volontarisme, plus répandue en France, qui désigne l'interventionnisme étatique : une attitude consistant à soumettre la réalité à une volonté politique, favorisant des politiques publiques fortes et appliquées rapidement. Dans ce sens sociopolitique, le volontarisme devient un euphémisme pour le dirigisme, donnant à l'État un rôle prépondérant, comme dans le colbertisme. &lt;/p&gt; "/>
     <hyperlink ref="E107" r:id="rId25" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Agnosticisme&quot; title=&quot; Wikipedia&quot;&gt; L’Agnosticisme&lt;/a&gt;  est une position philosophique qui affirme que l'existence ou l'inexistence de Dieu, ou plus largement toute réalité métaphysique absolue, est inconnaissable par l'esprit humain. Il ne s'agit ni d'une croyance en Dieu ni d'un athéisme affirmant son absence, mais d'une suspension du jugement faute de preuves accessibles à la raison ou à l'expérience. Cette doctrine préconise ainsi un refus de toute affirmation dogmatique sur les questions ultimes. &lt;/p&gt; &lt;p&gt; Le mot « agnosticisme » a été forgé en 1869 par le naturaliste anglais Thomas Huxley (1825-1895), ami de Charles Darwin, lors d'un débat sur la science et la religion. Inspiré du grec a-gnôstos (« inconnu » ou « inconnaissable »), Huxley l'opposait au « gnosticisme » des certitudes religieuses. Cette création s'inscrivait dans le contexte des avancées scientifiques du XIXe siècle, qui remettaient en cause les dogmes traditionnels. &lt;/p&gt; &lt;p&gt; Il  s'est ensuite développé aux XVIIIe et XIXe siècles, influencé par des philosophes comme David Hume et Emmanuel Kant, qui questionnaient les limites de la connaissance. Il représente une forme de scepticisme appliqué à la théologie, affirmant que Dieu, s'il existe, reste hors de portée empirique ou rationnelle. Aujourd'hui, il influence débats modernes sur foi, science et athéisme. &lt;/p&gt; &#10;&#10;"/>
     <hyperlink ref="E120" r:id="rId26" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/M%C3%A9r%C3%A9ologie&quot;  style=&quot;color:#d35400&quot;  title=&quot; Wikipedia&quot;&gt;Méréologie&lt;/a&gt;  est la branche de la logique et de la métaphysique qui étudie de manière formelle les relations entre parties et touts, en alternative (ou complément) à la théorie des ensembles. Elle fournit un langage précis pour parler de composition, de décomposition et de structure des objets matériels, des événements, voire d’entités plus abstraites. &lt;/p&gt; &lt;p&gt; La méréologie définit d’abord ce que signifie “être une partie de” quelque chose. - Une partie est ce qui compose un tout, comme une roue pour une voiture, une scène pour une pièce de théâtre ou un chapitre pour un livre. - Le tout est l’entité composée de ces parties, et la relation fondamentale étudiée est “x est partie de y”. &lt;/p&gt; &lt;p&gt; La “méréologie extensionnelle” ajoute le principe que deux objets qui ont exactement les mêmes parties sont identiques (extensionalité). - Cela donne un système très proche de la théorie des ensembles, mais exprimé en termes de parties et de fusions plutôt qu’en termes d’appartenance. - Une conséquence importante: pour tout ensemble de choses, il existe une somme méréologique (une fusion) qui les compose. &lt;/p&gt; &lt;p&gt; La méréologie est devenue un outil central de l’ontologie formelle et de la métaphysique contemporaine. Elle intervient dans le débat sur la composition des objets matériels: quand des particules composent‑elles un objet unique (par exemple une table) plutôt qu’un simple “amas” ? &lt;/p&gt;"/>

</xml_diff>